<commit_message>
Cleanup and fixed column name typos
</commit_message>
<xml_diff>
--- a/data/mapping_config_files/nwss_to_odm_v2_mapping.xlsx
+++ b/data/mapping_config_files/nwss_to_odm_v2_mapping.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/martinwellman/Documents/Health/Wastewater/PHES-ODM-MapGenerator/PHES-ODM-MapGenerator/data/mapping_config_files/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7CE17CF6-4E3F-5241-AEC0-B0C17D9F9EE0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{AD817F65-1D3B-0046-97B6-DAE4445D7E46}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="500" windowWidth="28800" windowHeight="15840" activeTab="1" xr2:uid="{77810E24-F86B-BC44-A0D5-8790E6EC60B4}"/>
   </bookViews>
@@ -26,9 +26,9 @@
   </externalReferences>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">enums!$A$1:$J$41</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">maps!$A$1:$K$10</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">maps!$A$1:$K$11</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="6" hidden="1">'maps original'!$A$1:$L$87</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">wide_measures!$A$1:$T$24</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">wide_measures!$A$1:$S$24</definedName>
     <definedName name="partID">[1]parts!$A:$A</definedName>
     <definedName name="partLabel">[1]parts!$B:$B</definedName>
   </definedNames>
@@ -52,7 +52,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2797" uniqueCount="883">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2787" uniqueCount="886">
   <si>
     <t>Reporter</t>
   </si>
@@ -2682,13 +2682,7 @@
     <t>{{id:measureRepID_pcr_target_avg_conc}}</t>
   </si>
   <si>
-    <t>purposeID_value</t>
-  </si>
-  <si>
     <t>norm</t>
-  </si>
-  <si>
-    <t>reflink_value</t>
   </si>
   <si>
     <t>{{hum_frac_target_chem_ref}}</t>
@@ -2748,6 +2742,21 @@
   </si>
   <si>
     <t>Is ml OR grams for unit_value correct?</t>
+  </si>
+  <si>
+    <t>purpose_value</t>
+  </si>
+  <si>
+    <t>refLink_value</t>
+  </si>
+  <si>
+    <t>compartment</t>
+  </si>
+  <si>
+    <t>"wat"</t>
+  </si>
+  <si>
+    <t>summ</t>
   </si>
 </sst>
 </file>
@@ -14192,7 +14201,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{3154BFCE-06D9-9649-B340-B23DCF20DD83}">
-  <dimension ref="A1:K68"/>
+  <dimension ref="A1:K71"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="2" max="2" width="13" bestFit="1" customWidth="1"/>
@@ -14343,27 +14352,24 @@
         <v>709</v>
       </c>
     </row>
-    <row r="8" spans="1:11" s="25" customFormat="1" x14ac:dyDescent="0.2"/>
-    <row r="9" spans="1:11" s="25" customFormat="1" x14ac:dyDescent="0.2">
-      <c r="A9" s="25" t="b">
-        <v>1</v>
-      </c>
-      <c r="B9" s="25" t="s">
-        <v>631</v>
-      </c>
-      <c r="C9" s="25" t="s">
-        <v>73</v>
-      </c>
-      <c r="E9" s="25" t="s">
-        <v>475</v>
-      </c>
-      <c r="F9" s="25" t="s">
-        <v>472</v>
-      </c>
-      <c r="G9" s="25" t="s">
-        <v>710</v>
-      </c>
-    </row>
+    <row r="8" spans="1:11" s="25" customFormat="1" x14ac:dyDescent="0.2">
+      <c r="A8" s="25" t="b">
+        <v>1</v>
+      </c>
+      <c r="B8" s="25" t="s">
+        <v>631</v>
+      </c>
+      <c r="E8" s="25" t="s">
+        <v>114</v>
+      </c>
+      <c r="F8" s="25" t="s">
+        <v>883</v>
+      </c>
+      <c r="H8" s="31" t="s">
+        <v>884</v>
+      </c>
+    </row>
+    <row r="9" spans="1:11" s="25" customFormat="1" x14ac:dyDescent="0.2"/>
     <row r="10" spans="1:11" s="25" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A10" s="25" t="b">
         <v>1</v>
@@ -14372,68 +14378,70 @@
         <v>631</v>
       </c>
       <c r="C10" s="25" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="E10" s="25" t="s">
         <v>475</v>
       </c>
       <c r="F10" s="25" t="s">
-        <v>474</v>
+        <v>472</v>
       </c>
       <c r="G10" s="25" t="s">
+        <v>710</v>
+      </c>
+    </row>
+    <row r="11" spans="1:11" s="25" customFormat="1" x14ac:dyDescent="0.2">
+      <c r="A11" s="25" t="b">
+        <v>1</v>
+      </c>
+      <c r="B11" s="25" t="s">
+        <v>631</v>
+      </c>
+      <c r="C11" s="25" t="s">
+        <v>74</v>
+      </c>
+      <c r="E11" s="25" t="s">
+        <v>475</v>
+      </c>
+      <c r="F11" s="25" t="s">
+        <v>885</v>
+      </c>
+      <c r="G11" s="25" t="s">
         <v>711</v>
       </c>
-      <c r="K10" s="17"/>
-    </row>
-    <row r="11" spans="1:11" s="25" customFormat="1" x14ac:dyDescent="0.2"/>
-    <row r="12" spans="1:11" s="25" customFormat="1" x14ac:dyDescent="0.2">
-      <c r="A12" s="25" t="b">
-        <v>1</v>
-      </c>
-      <c r="B12" s="25" t="s">
-        <v>631</v>
-      </c>
-      <c r="C12" s="25" t="s">
+      <c r="K11" s="17"/>
+    </row>
+    <row r="12" spans="1:11" s="25" customFormat="1" x14ac:dyDescent="0.2"/>
+    <row r="13" spans="1:11" s="25" customFormat="1" x14ac:dyDescent="0.2">
+      <c r="A13" s="25" t="b">
+        <v>1</v>
+      </c>
+      <c r="B13" s="25" t="s">
+        <v>631</v>
+      </c>
+      <c r="C13" s="25" t="s">
         <v>53</v>
       </c>
-      <c r="E12" s="25" t="s">
+      <c r="E13" s="25" t="s">
         <v>146</v>
       </c>
-      <c r="F12" s="25" t="s">
+      <c r="F13" s="25" t="s">
         <v>139</v>
       </c>
-      <c r="G12" s="42" t="s">
+      <c r="G13" s="42" t="s">
         <v>707</v>
       </c>
-      <c r="H12" s="30"/>
-      <c r="I12" s="30"/>
-      <c r="K12" s="16" t="s">
-        <v>806</v>
-      </c>
-    </row>
-    <row r="13" spans="1:11" s="25" customFormat="1" x14ac:dyDescent="0.2">
-      <c r="G13" s="30"/>
       <c r="H13" s="30"/>
       <c r="I13" s="30"/>
-      <c r="K13" s="17"/>
-    </row>
-    <row r="14" spans="1:11" s="25" customFormat="1" ht="16" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A14" s="25" t="b">
-        <v>1</v>
-      </c>
-      <c r="B14" s="25" t="s">
-        <v>631</v>
-      </c>
-      <c r="E14" s="25" t="s">
-        <v>117</v>
-      </c>
-      <c r="F14" s="25" t="s">
-        <v>676</v>
-      </c>
+      <c r="K13" s="16" t="s">
+        <v>806</v>
+      </c>
+    </row>
+    <row r="14" spans="1:11" s="25" customFormat="1" x14ac:dyDescent="0.2">
       <c r="G14" s="30"/>
-      <c r="H14" s="32" t="s">
-        <v>698</v>
-      </c>
+      <c r="H14" s="30"/>
+      <c r="I14" s="30"/>
+      <c r="K14" s="17"/>
     </row>
     <row r="15" spans="1:11" s="25" customFormat="1" ht="16" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A15" s="25" t="b">
@@ -14442,40 +14450,37 @@
       <c r="B15" s="25" t="s">
         <v>631</v>
       </c>
-      <c r="C15" s="31"/>
-      <c r="D15" s="33"/>
       <c r="E15" s="25" t="s">
         <v>117</v>
       </c>
       <c r="F15" s="25" t="s">
-        <v>118</v>
-      </c>
+        <v>676</v>
+      </c>
+      <c r="G15" s="30"/>
       <c r="H15" s="32" t="s">
-        <v>699</v>
-      </c>
-    </row>
-    <row r="16" spans="1:11" s="25" customFormat="1" x14ac:dyDescent="0.2">
+        <v>698</v>
+      </c>
+    </row>
+    <row r="16" spans="1:11" s="25" customFormat="1" ht="16" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A16" s="25" t="b">
         <v>1</v>
       </c>
       <c r="B16" s="25" t="s">
         <v>631</v>
       </c>
-      <c r="C16" s="25" t="s">
-        <v>23</v>
-      </c>
+      <c r="C16" s="31"/>
       <c r="D16" s="33"/>
       <c r="E16" s="25" t="s">
         <v>117</v>
       </c>
       <c r="F16" s="25" t="s">
-        <v>119</v>
-      </c>
-      <c r="G16" s="25" t="s">
-        <v>706</v>
-      </c>
-    </row>
-    <row r="17" spans="1:10" s="25" customFormat="1" x14ac:dyDescent="0.2">
+        <v>118</v>
+      </c>
+      <c r="H16" s="32" t="s">
+        <v>699</v>
+      </c>
+    </row>
+    <row r="17" spans="1:11" s="25" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A17" s="25" t="b">
         <v>1</v>
       </c>
@@ -14483,19 +14488,20 @@
         <v>631</v>
       </c>
       <c r="C17" s="25" t="s">
-        <v>56</v>
-      </c>
+        <v>23</v>
+      </c>
+      <c r="D17" s="33"/>
       <c r="E17" s="25" t="s">
         <v>117</v>
       </c>
       <c r="F17" s="25" t="s">
-        <v>144</v>
-      </c>
-      <c r="H17" s="25" t="s">
-        <v>881</v>
-      </c>
-    </row>
-    <row r="18" spans="1:10" s="25" customFormat="1" x14ac:dyDescent="0.2">
+        <v>119</v>
+      </c>
+      <c r="G17" s="25" t="s">
+        <v>706</v>
+      </c>
+    </row>
+    <row r="18" spans="1:11" s="25" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A18" s="25" t="b">
         <v>1</v>
       </c>
@@ -14503,19 +14509,19 @@
         <v>631</v>
       </c>
       <c r="C18" s="25" t="s">
-        <v>54</v>
+        <v>56</v>
       </c>
       <c r="E18" s="25" t="s">
         <v>117</v>
       </c>
       <c r="F18" s="25" t="s">
-        <v>143</v>
-      </c>
-      <c r="G18" s="25" t="s">
-        <v>708</v>
-      </c>
-    </row>
-    <row r="19" spans="1:10" s="25" customFormat="1" x14ac:dyDescent="0.2">
+        <v>144</v>
+      </c>
+      <c r="H18" s="25" t="s">
+        <v>879</v>
+      </c>
+    </row>
+    <row r="19" spans="1:11" s="25" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A19" s="25" t="b">
         <v>1</v>
       </c>
@@ -14523,152 +14529,144 @@
         <v>631</v>
       </c>
       <c r="C19" s="25" t="s">
-        <v>53</v>
+        <v>54</v>
       </c>
       <c r="E19" s="25" t="s">
         <v>117</v>
       </c>
       <c r="F19" s="25" t="s">
+        <v>143</v>
+      </c>
+      <c r="G19" s="25" t="s">
+        <v>708</v>
+      </c>
+    </row>
+    <row r="20" spans="1:11" s="25" customFormat="1" x14ac:dyDescent="0.2">
+      <c r="A20" s="25" t="b">
+        <v>1</v>
+      </c>
+      <c r="B20" s="25" t="s">
+        <v>631</v>
+      </c>
+      <c r="C20" s="25" t="s">
+        <v>7</v>
+      </c>
+      <c r="E20" s="25" t="s">
+        <v>117</v>
+      </c>
+      <c r="F20" s="25" t="s">
+        <v>720</v>
+      </c>
+      <c r="G20" s="25" t="s">
+        <v>700</v>
+      </c>
+      <c r="K20" s="17"/>
+    </row>
+    <row r="21" spans="1:11" s="25" customFormat="1" x14ac:dyDescent="0.2">
+      <c r="A21" s="25" t="b">
+        <v>1</v>
+      </c>
+      <c r="B21" s="25" t="s">
+        <v>631</v>
+      </c>
+      <c r="C21" s="25" t="s">
+        <v>53</v>
+      </c>
+      <c r="E21" s="25" t="s">
+        <v>117</v>
+      </c>
+      <c r="F21" s="25" t="s">
         <v>139</v>
       </c>
-      <c r="G19" s="25" t="s">
+      <c r="G21" s="25" t="s">
         <v>707</v>
       </c>
     </row>
-    <row r="20" spans="1:10" s="25" customFormat="1" x14ac:dyDescent="0.2"/>
-    <row r="21" spans="1:10" s="17" customFormat="1" ht="17" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A21" s="17" t="b">
+    <row r="22" spans="1:11" s="25" customFormat="1" x14ac:dyDescent="0.2">
+      <c r="A22" s="25" t="b">
+        <v>1</v>
+      </c>
+      <c r="B22" s="25" t="s">
+        <v>631</v>
+      </c>
+      <c r="C22" s="25" t="s">
+        <v>8</v>
+      </c>
+      <c r="E22" s="25" t="s">
+        <v>117</v>
+      </c>
+      <c r="F22" s="25" t="s">
+        <v>77</v>
+      </c>
+      <c r="G22" s="25" t="s">
+        <v>701</v>
+      </c>
+    </row>
+    <row r="23" spans="1:11" s="25" customFormat="1" x14ac:dyDescent="0.2"/>
+    <row r="24" spans="1:11" s="17" customFormat="1" ht="17" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A24" s="17" t="b">
         <v>0</v>
       </c>
-      <c r="B21" s="17" t="s">
-        <v>631</v>
-      </c>
-      <c r="C21" s="27" t="s">
+      <c r="B24" s="17" t="s">
+        <v>631</v>
+      </c>
+      <c r="C24" s="27" t="s">
         <v>44</v>
       </c>
-      <c r="E21" s="17" t="s">
+      <c r="E24" s="17" t="s">
         <v>117</v>
       </c>
-      <c r="F21" s="17" t="s">
+      <c r="F24" s="17" t="s">
         <v>137</v>
       </c>
-      <c r="H21" s="28"/>
-      <c r="J21" s="17" t="s">
+      <c r="H24" s="28"/>
+      <c r="J24" s="17" t="s">
         <v>138</v>
       </c>
     </row>
-    <row r="22" spans="1:10" s="17" customFormat="1" ht="16" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A22" s="17" t="b">
+    <row r="25" spans="1:11" s="17" customFormat="1" ht="16" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A25" s="17" t="b">
         <v>0</v>
       </c>
-      <c r="B22" s="17" t="s">
-        <v>631</v>
-      </c>
-      <c r="C22" s="17" t="s">
+      <c r="B25" s="17" t="s">
+        <v>631</v>
+      </c>
+      <c r="C25" s="17" t="s">
         <v>45</v>
       </c>
-      <c r="E22" s="17" t="s">
+      <c r="E25" s="17" t="s">
         <v>117</v>
       </c>
-      <c r="F22" s="17" t="s">
+      <c r="F25" s="17" t="s">
         <v>137</v>
       </c>
-      <c r="H22" s="28"/>
-      <c r="J22" s="17" t="s">
+      <c r="H25" s="28"/>
+      <c r="J25" s="17" t="s">
         <v>138</v>
       </c>
     </row>
-    <row r="23" spans="1:10" s="17" customFormat="1" x14ac:dyDescent="0.2">
-      <c r="A23" s="17" t="b">
+    <row r="26" spans="1:11" s="17" customFormat="1" x14ac:dyDescent="0.2">
+      <c r="A26" s="17" t="b">
         <v>0</v>
       </c>
-      <c r="B23" s="17" t="s">
-        <v>631</v>
-      </c>
-      <c r="C23" s="17" t="s">
+      <c r="B26" s="17" t="s">
+        <v>631</v>
+      </c>
+      <c r="C26" s="17" t="s">
         <v>46</v>
       </c>
-      <c r="E23" s="17" t="s">
+      <c r="E26" s="17" t="s">
         <v>117</v>
       </c>
-      <c r="F23" s="17" t="s">
+      <c r="F26" s="17" t="s">
         <v>137</v>
       </c>
-      <c r="J23" s="17" t="s">
+      <c r="J26" s="17" t="s">
         <v>138</v>
       </c>
     </row>
-    <row r="24" spans="1:10" s="25" customFormat="1" x14ac:dyDescent="0.2"/>
-    <row r="25" spans="1:10" s="25" customFormat="1" x14ac:dyDescent="0.2">
-      <c r="A25" s="25" t="b">
-        <v>1</v>
-      </c>
-      <c r="B25" s="25" t="s">
-        <v>631</v>
-      </c>
-      <c r="C25" s="25" t="s">
-        <v>24</v>
-      </c>
-      <c r="D25" s="34" t="s">
-        <v>121</v>
-      </c>
-      <c r="E25" s="25" t="s">
-        <v>117</v>
-      </c>
-      <c r="F25" s="25" t="s">
-        <v>129</v>
-      </c>
-      <c r="G25" s="25" t="s">
-        <v>136</v>
-      </c>
-    </row>
-    <row r="26" spans="1:10" s="25" customFormat="1" x14ac:dyDescent="0.2">
-      <c r="A26" s="25" t="b">
-        <v>1</v>
-      </c>
-      <c r="B26" s="25" t="s">
-        <v>631</v>
-      </c>
-      <c r="C26" s="25" t="s">
-        <v>24</v>
-      </c>
-      <c r="D26" s="33" t="s">
-        <v>122</v>
-      </c>
-      <c r="E26" s="25" t="s">
-        <v>117</v>
-      </c>
-      <c r="F26" s="25" t="s">
-        <v>129</v>
-      </c>
-      <c r="G26" s="25" t="s">
-        <v>134</v>
-      </c>
-    </row>
-    <row r="27" spans="1:10" s="25" customFormat="1" x14ac:dyDescent="0.2">
-      <c r="A27" s="25" t="b">
-        <v>1</v>
-      </c>
-      <c r="B27" s="25" t="s">
-        <v>631</v>
-      </c>
-      <c r="C27" s="25" t="s">
-        <v>24</v>
-      </c>
-      <c r="D27" s="33" t="s">
-        <v>123</v>
-      </c>
-      <c r="E27" s="25" t="s">
-        <v>117</v>
-      </c>
-      <c r="F27" s="25" t="s">
-        <v>129</v>
-      </c>
-      <c r="G27" s="25" t="s">
-        <v>130</v>
-      </c>
-    </row>
-    <row r="28" spans="1:10" s="25" customFormat="1" x14ac:dyDescent="0.2">
+    <row r="27" spans="1:11" s="25" customFormat="1" x14ac:dyDescent="0.2"/>
+    <row r="28" spans="1:11" s="25" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A28" s="25" t="b">
         <v>1</v>
       </c>
@@ -14678,8 +14676,8 @@
       <c r="C28" s="25" t="s">
         <v>24</v>
       </c>
-      <c r="D28" s="33" t="s">
-        <v>124</v>
+      <c r="D28" s="34" t="s">
+        <v>121</v>
       </c>
       <c r="E28" s="25" t="s">
         <v>117</v>
@@ -14688,10 +14686,10 @@
         <v>129</v>
       </c>
       <c r="G28" s="25" t="s">
-        <v>131</v>
-      </c>
-    </row>
-    <row r="29" spans="1:10" s="25" customFormat="1" x14ac:dyDescent="0.2">
+        <v>136</v>
+      </c>
+    </row>
+    <row r="29" spans="1:11" s="25" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A29" s="25" t="b">
         <v>1</v>
       </c>
@@ -14702,7 +14700,7 @@
         <v>24</v>
       </c>
       <c r="D29" s="33" t="s">
-        <v>125</v>
+        <v>122</v>
       </c>
       <c r="E29" s="25" t="s">
         <v>117</v>
@@ -14711,10 +14709,10 @@
         <v>129</v>
       </c>
       <c r="G29" s="25" t="s">
-        <v>132</v>
-      </c>
-    </row>
-    <row r="30" spans="1:10" s="25" customFormat="1" x14ac:dyDescent="0.2">
+        <v>134</v>
+      </c>
+    </row>
+    <row r="30" spans="1:11" s="25" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A30" s="25" t="b">
         <v>1</v>
       </c>
@@ -14725,7 +14723,7 @@
         <v>24</v>
       </c>
       <c r="D30" s="33" t="s">
-        <v>126</v>
+        <v>123</v>
       </c>
       <c r="E30" s="25" t="s">
         <v>117</v>
@@ -14734,10 +14732,10 @@
         <v>129</v>
       </c>
       <c r="G30" s="25" t="s">
-        <v>133</v>
-      </c>
-    </row>
-    <row r="31" spans="1:10" s="25" customFormat="1" x14ac:dyDescent="0.2">
+        <v>130</v>
+      </c>
+    </row>
+    <row r="31" spans="1:11" s="25" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A31" s="25" t="b">
         <v>1</v>
       </c>
@@ -14748,7 +14746,7 @@
         <v>24</v>
       </c>
       <c r="D31" s="33" t="s">
-        <v>127</v>
+        <v>124</v>
       </c>
       <c r="E31" s="25" t="s">
         <v>117</v>
@@ -14757,10 +14755,10 @@
         <v>129</v>
       </c>
       <c r="G31" s="25" t="s">
-        <v>127</v>
-      </c>
-    </row>
-    <row r="32" spans="1:10" s="25" customFormat="1" x14ac:dyDescent="0.2">
+        <v>131</v>
+      </c>
+    </row>
+    <row r="32" spans="1:11" s="25" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A32" s="25" t="b">
         <v>1</v>
       </c>
@@ -14771,7 +14769,7 @@
         <v>24</v>
       </c>
       <c r="D32" s="33" t="s">
-        <v>128</v>
+        <v>125</v>
       </c>
       <c r="E32" s="25" t="s">
         <v>117</v>
@@ -14780,11 +14778,31 @@
         <v>129</v>
       </c>
       <c r="G32" s="25" t="s">
-        <v>135</v>
+        <v>132</v>
       </c>
     </row>
     <row r="33" spans="1:10" s="25" customFormat="1" x14ac:dyDescent="0.2">
-      <c r="D33" s="33"/>
+      <c r="A33" s="25" t="b">
+        <v>1</v>
+      </c>
+      <c r="B33" s="25" t="s">
+        <v>631</v>
+      </c>
+      <c r="C33" s="25" t="s">
+        <v>24</v>
+      </c>
+      <c r="D33" s="33" t="s">
+        <v>126</v>
+      </c>
+      <c r="E33" s="25" t="s">
+        <v>117</v>
+      </c>
+      <c r="F33" s="25" t="s">
+        <v>129</v>
+      </c>
+      <c r="G33" s="25" t="s">
+        <v>133</v>
+      </c>
     </row>
     <row r="34" spans="1:10" s="25" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A34" s="25" t="b">
@@ -14794,16 +14812,19 @@
         <v>631</v>
       </c>
       <c r="C34" s="25" t="s">
-        <v>9</v>
-      </c>
-      <c r="E34" s="42" t="s">
-        <v>76</v>
-      </c>
-      <c r="F34" s="42" t="s">
-        <v>120</v>
-      </c>
-      <c r="H34" s="31" t="s">
-        <v>729</v>
+        <v>24</v>
+      </c>
+      <c r="D34" s="33" t="s">
+        <v>127</v>
+      </c>
+      <c r="E34" s="25" t="s">
+        <v>117</v>
+      </c>
+      <c r="F34" s="25" t="s">
+        <v>129</v>
+      </c>
+      <c r="G34" s="25" t="s">
+        <v>127</v>
       </c>
     </row>
     <row r="35" spans="1:10" s="25" customFormat="1" x14ac:dyDescent="0.2">
@@ -14814,37 +14835,23 @@
         <v>631</v>
       </c>
       <c r="C35" s="25" t="s">
-        <v>11</v>
+        <v>24</v>
+      </c>
+      <c r="D35" s="33" t="s">
+        <v>128</v>
       </c>
       <c r="E35" s="25" t="s">
-        <v>76</v>
+        <v>117</v>
       </c>
       <c r="F35" s="25" t="s">
-        <v>80</v>
+        <v>129</v>
       </c>
       <c r="G35" s="25" t="s">
-        <v>703</v>
+        <v>135</v>
       </c>
     </row>
     <row r="36" spans="1:10" s="25" customFormat="1" x14ac:dyDescent="0.2">
-      <c r="A36" s="25" t="b">
-        <v>1</v>
-      </c>
-      <c r="B36" s="25" t="s">
-        <v>631</v>
-      </c>
-      <c r="C36" s="25" t="s">
-        <v>8</v>
-      </c>
-      <c r="E36" s="25" t="s">
-        <v>76</v>
-      </c>
-      <c r="F36" s="25" t="s">
-        <v>77</v>
-      </c>
-      <c r="G36" s="25" t="s">
-        <v>701</v>
-      </c>
+      <c r="D36" s="33"/>
     </row>
     <row r="37" spans="1:10" s="25" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A37" s="25" t="b">
@@ -14854,16 +14861,16 @@
         <v>631</v>
       </c>
       <c r="C37" s="25" t="s">
-        <v>19</v>
-      </c>
-      <c r="E37" s="25" t="s">
+        <v>9</v>
+      </c>
+      <c r="E37" s="42" t="s">
         <v>76</v>
       </c>
-      <c r="F37" s="25" t="s">
-        <v>719</v>
-      </c>
-      <c r="G37" s="25" t="s">
-        <v>705</v>
+      <c r="F37" s="42" t="s">
+        <v>120</v>
+      </c>
+      <c r="H37" s="31" t="s">
+        <v>729</v>
       </c>
     </row>
     <row r="38" spans="1:10" s="25" customFormat="1" x14ac:dyDescent="0.2">
@@ -14874,20 +14881,39 @@
         <v>631</v>
       </c>
       <c r="C38" s="25" t="s">
-        <v>18</v>
+        <v>11</v>
       </c>
       <c r="E38" s="25" t="s">
         <v>76</v>
       </c>
       <c r="F38" s="25" t="s">
-        <v>115</v>
+        <v>80</v>
       </c>
       <c r="G38" s="25" t="s">
-        <v>704</v>
-      </c>
-    </row>
-    <row r="39" spans="1:10" s="25" customFormat="1" x14ac:dyDescent="0.2"/>
-    <row r="40" spans="1:10" s="17" customFormat="1" ht="17" customHeight="1" x14ac:dyDescent="0.2">
+        <v>703</v>
+      </c>
+    </row>
+    <row r="39" spans="1:10" s="25" customFormat="1" x14ac:dyDescent="0.2">
+      <c r="A39" s="25" t="b">
+        <v>1</v>
+      </c>
+      <c r="B39" s="25" t="s">
+        <v>631</v>
+      </c>
+      <c r="C39" s="25" t="s">
+        <v>8</v>
+      </c>
+      <c r="E39" s="25" t="s">
+        <v>76</v>
+      </c>
+      <c r="F39" s="25" t="s">
+        <v>77</v>
+      </c>
+      <c r="G39" s="25" t="s">
+        <v>701</v>
+      </c>
+    </row>
+    <row r="40" spans="1:10" s="25" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A40" s="25" t="b">
         <v>1</v>
       </c>
@@ -14895,23 +14921,17 @@
         <v>631</v>
       </c>
       <c r="C40" s="25" t="s">
-        <v>15</v>
-      </c>
-      <c r="D40" s="34" t="s">
-        <v>84</v>
+        <v>19</v>
       </c>
       <c r="E40" s="25" t="s">
         <v>76</v>
       </c>
       <c r="F40" s="25" t="s">
-        <v>100</v>
+        <v>719</v>
       </c>
       <c r="G40" s="25" t="s">
-        <v>75</v>
-      </c>
-      <c r="H40" s="25"/>
-      <c r="I40" s="25"/>
-      <c r="J40" s="25"/>
+        <v>705</v>
+      </c>
     </row>
     <row r="41" spans="1:10" s="25" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A41" s="25" t="b">
@@ -14921,45 +14941,20 @@
         <v>631</v>
       </c>
       <c r="C41" s="25" t="s">
-        <v>15</v>
-      </c>
-      <c r="D41" s="34" t="s">
-        <v>85</v>
+        <v>18</v>
       </c>
       <c r="E41" s="25" t="s">
         <v>76</v>
       </c>
       <c r="F41" s="25" t="s">
-        <v>100</v>
+        <v>115</v>
       </c>
       <c r="G41" s="25" t="s">
-        <v>101</v>
-      </c>
-    </row>
-    <row r="42" spans="1:10" s="25" customFormat="1" x14ac:dyDescent="0.2">
-      <c r="A42" s="25" t="b">
-        <v>1</v>
-      </c>
-      <c r="B42" s="25" t="s">
-        <v>631</v>
-      </c>
-      <c r="C42" s="25" t="s">
-        <v>15</v>
-      </c>
-      <c r="D42" s="35" t="s">
-        <v>86</v>
-      </c>
-      <c r="E42" s="25" t="s">
-        <v>76</v>
-      </c>
-      <c r="F42" s="25" t="s">
-        <v>100</v>
-      </c>
-      <c r="G42" s="25" t="s">
-        <v>102</v>
-      </c>
-    </row>
-    <row r="43" spans="1:10" s="25" customFormat="1" x14ac:dyDescent="0.2">
+        <v>704</v>
+      </c>
+    </row>
+    <row r="42" spans="1:10" s="25" customFormat="1" x14ac:dyDescent="0.2"/>
+    <row r="43" spans="1:10" s="17" customFormat="1" ht="17" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A43" s="25" t="b">
         <v>1</v>
       </c>
@@ -14969,8 +14964,8 @@
       <c r="C43" s="25" t="s">
         <v>15</v>
       </c>
-      <c r="D43" s="35" t="s">
-        <v>87</v>
+      <c r="D43" s="34" t="s">
+        <v>84</v>
       </c>
       <c r="E43" s="25" t="s">
         <v>76</v>
@@ -14979,8 +14974,11 @@
         <v>100</v>
       </c>
       <c r="G43" s="25" t="s">
-        <v>103</v>
-      </c>
+        <v>75</v>
+      </c>
+      <c r="H43" s="25"/>
+      <c r="I43" s="25"/>
+      <c r="J43" s="25"/>
     </row>
     <row r="44" spans="1:10" s="25" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A44" s="25" t="b">
@@ -14992,8 +14990,8 @@
       <c r="C44" s="25" t="s">
         <v>15</v>
       </c>
-      <c r="D44" s="35" t="s">
-        <v>88</v>
+      <c r="D44" s="34" t="s">
+        <v>85</v>
       </c>
       <c r="E44" s="25" t="s">
         <v>76</v>
@@ -15002,7 +15000,7 @@
         <v>100</v>
       </c>
       <c r="G44" s="25" t="s">
-        <v>104</v>
+        <v>101</v>
       </c>
     </row>
     <row r="45" spans="1:10" s="25" customFormat="1" x14ac:dyDescent="0.2">
@@ -15015,8 +15013,8 @@
       <c r="C45" s="25" t="s">
         <v>15</v>
       </c>
-      <c r="D45" s="33" t="s">
-        <v>89</v>
+      <c r="D45" s="35" t="s">
+        <v>86</v>
       </c>
       <c r="E45" s="25" t="s">
         <v>76</v>
@@ -15025,7 +15023,7 @@
         <v>100</v>
       </c>
       <c r="G45" s="25" t="s">
-        <v>113</v>
+        <v>102</v>
       </c>
     </row>
     <row r="46" spans="1:10" s="25" customFormat="1" x14ac:dyDescent="0.2">
@@ -15038,8 +15036,8 @@
       <c r="C46" s="25" t="s">
         <v>15</v>
       </c>
-      <c r="D46" s="33" t="s">
-        <v>90</v>
+      <c r="D46" s="35" t="s">
+        <v>87</v>
       </c>
       <c r="E46" s="25" t="s">
         <v>76</v>
@@ -15048,7 +15046,7 @@
         <v>100</v>
       </c>
       <c r="G46" s="25" t="s">
-        <v>112</v>
+        <v>103</v>
       </c>
     </row>
     <row r="47" spans="1:10" s="25" customFormat="1" x14ac:dyDescent="0.2">
@@ -15061,8 +15059,8 @@
       <c r="C47" s="25" t="s">
         <v>15</v>
       </c>
-      <c r="D47" s="34" t="s">
-        <v>91</v>
+      <c r="D47" s="35" t="s">
+        <v>88</v>
       </c>
       <c r="E47" s="25" t="s">
         <v>76</v>
@@ -15071,7 +15069,7 @@
         <v>100</v>
       </c>
       <c r="G47" s="25" t="s">
-        <v>109</v>
+        <v>104</v>
       </c>
     </row>
     <row r="48" spans="1:10" s="25" customFormat="1" x14ac:dyDescent="0.2">
@@ -15084,8 +15082,8 @@
       <c r="C48" s="25" t="s">
         <v>15</v>
       </c>
-      <c r="D48" s="34" t="s">
-        <v>92</v>
+      <c r="D48" s="33" t="s">
+        <v>89</v>
       </c>
       <c r="E48" s="25" t="s">
         <v>76</v>
@@ -15094,7 +15092,7 @@
         <v>100</v>
       </c>
       <c r="G48" s="25" t="s">
-        <v>108</v>
+        <v>113</v>
       </c>
     </row>
     <row r="49" spans="1:11" s="25" customFormat="1" x14ac:dyDescent="0.2">
@@ -15108,7 +15106,7 @@
         <v>15</v>
       </c>
       <c r="D49" s="33" t="s">
-        <v>93</v>
+        <v>90</v>
       </c>
       <c r="E49" s="25" t="s">
         <v>76</v>
@@ -15117,7 +15115,7 @@
         <v>100</v>
       </c>
       <c r="G49" s="25" t="s">
-        <v>107</v>
+        <v>112</v>
       </c>
     </row>
     <row r="50" spans="1:11" s="25" customFormat="1" x14ac:dyDescent="0.2">
@@ -15130,8 +15128,8 @@
       <c r="C50" s="25" t="s">
         <v>15</v>
       </c>
-      <c r="D50" s="33" t="s">
-        <v>94</v>
+      <c r="D50" s="34" t="s">
+        <v>91</v>
       </c>
       <c r="E50" s="25" t="s">
         <v>76</v>
@@ -15140,7 +15138,7 @@
         <v>100</v>
       </c>
       <c r="G50" s="25" t="s">
-        <v>106</v>
+        <v>109</v>
       </c>
     </row>
     <row r="51" spans="1:11" s="25" customFormat="1" x14ac:dyDescent="0.2">
@@ -15153,8 +15151,8 @@
       <c r="C51" s="25" t="s">
         <v>15</v>
       </c>
-      <c r="D51" s="33" t="s">
-        <v>95</v>
+      <c r="D51" s="34" t="s">
+        <v>92</v>
       </c>
       <c r="E51" s="25" t="s">
         <v>76</v>
@@ -15163,7 +15161,7 @@
         <v>100</v>
       </c>
       <c r="G51" s="25" t="s">
-        <v>105</v>
+        <v>108</v>
       </c>
     </row>
     <row r="52" spans="1:11" s="25" customFormat="1" x14ac:dyDescent="0.2">
@@ -15177,7 +15175,7 @@
         <v>15</v>
       </c>
       <c r="D52" s="33" t="s">
-        <v>96</v>
+        <v>93</v>
       </c>
       <c r="E52" s="25" t="s">
         <v>76</v>
@@ -15186,7 +15184,7 @@
         <v>100</v>
       </c>
       <c r="G52" s="25" t="s">
-        <v>110</v>
+        <v>107</v>
       </c>
     </row>
     <row r="53" spans="1:11" s="25" customFormat="1" x14ac:dyDescent="0.2">
@@ -15200,7 +15198,7 @@
         <v>15</v>
       </c>
       <c r="D53" s="33" t="s">
-        <v>97</v>
+        <v>94</v>
       </c>
       <c r="E53" s="25" t="s">
         <v>76</v>
@@ -15209,7 +15207,7 @@
         <v>100</v>
       </c>
       <c r="G53" s="25" t="s">
-        <v>97</v>
+        <v>106</v>
       </c>
     </row>
     <row r="54" spans="1:11" s="25" customFormat="1" x14ac:dyDescent="0.2">
@@ -15223,7 +15221,7 @@
         <v>15</v>
       </c>
       <c r="D54" s="33" t="s">
-        <v>98</v>
+        <v>95</v>
       </c>
       <c r="E54" s="25" t="s">
         <v>76</v>
@@ -15232,7 +15230,7 @@
         <v>100</v>
       </c>
       <c r="G54" s="25" t="s">
-        <v>111</v>
+        <v>105</v>
       </c>
     </row>
     <row r="55" spans="1:11" s="25" customFormat="1" x14ac:dyDescent="0.2">
@@ -15246,7 +15244,7 @@
         <v>15</v>
       </c>
       <c r="D55" s="33" t="s">
-        <v>99</v>
+        <v>96</v>
       </c>
       <c r="E55" s="25" t="s">
         <v>76</v>
@@ -15254,20 +15252,34 @@
       <c r="F55" s="25" t="s">
         <v>100</v>
       </c>
-      <c r="G55" s="42" t="s">
-        <v>531</v>
-      </c>
-      <c r="H55" s="30"/>
-      <c r="I55" s="30"/>
-      <c r="K55" s="42"/>
+      <c r="G55" s="25" t="s">
+        <v>110</v>
+      </c>
     </row>
     <row r="56" spans="1:11" s="25" customFormat="1" x14ac:dyDescent="0.2">
-      <c r="D56" s="33"/>
-      <c r="G56" s="30"/>
-      <c r="H56" s="30"/>
-      <c r="I56" s="30"/>
-    </row>
-    <row r="57" spans="1:11" s="25" customFormat="1" ht="17" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A56" s="25" t="b">
+        <v>1</v>
+      </c>
+      <c r="B56" s="25" t="s">
+        <v>631</v>
+      </c>
+      <c r="C56" s="25" t="s">
+        <v>15</v>
+      </c>
+      <c r="D56" s="33" t="s">
+        <v>97</v>
+      </c>
+      <c r="E56" s="25" t="s">
+        <v>76</v>
+      </c>
+      <c r="F56" s="25" t="s">
+        <v>100</v>
+      </c>
+      <c r="G56" s="25" t="s">
+        <v>97</v>
+      </c>
+    </row>
+    <row r="57" spans="1:11" s="25" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A57" s="25" t="b">
         <v>1</v>
       </c>
@@ -15275,87 +15287,79 @@
         <v>631</v>
       </c>
       <c r="C57" s="25" t="s">
-        <v>13</v>
-      </c>
-      <c r="D57" s="33"/>
+        <v>15</v>
+      </c>
+      <c r="D57" s="33" t="s">
+        <v>98</v>
+      </c>
       <c r="E57" s="25" t="s">
         <v>76</v>
       </c>
       <c r="F57" s="25" t="s">
+        <v>100</v>
+      </c>
+      <c r="G57" s="25" t="s">
+        <v>111</v>
+      </c>
+    </row>
+    <row r="58" spans="1:11" s="25" customFormat="1" x14ac:dyDescent="0.2">
+      <c r="A58" s="25" t="b">
+        <v>1</v>
+      </c>
+      <c r="B58" s="25" t="s">
+        <v>631</v>
+      </c>
+      <c r="C58" s="25" t="s">
+        <v>15</v>
+      </c>
+      <c r="D58" s="33" t="s">
+        <v>99</v>
+      </c>
+      <c r="E58" s="25" t="s">
+        <v>76</v>
+      </c>
+      <c r="F58" s="25" t="s">
+        <v>100</v>
+      </c>
+      <c r="G58" s="42" t="s">
+        <v>531</v>
+      </c>
+      <c r="H58" s="30"/>
+      <c r="I58" s="30"/>
+      <c r="K58" s="42"/>
+    </row>
+    <row r="59" spans="1:11" s="25" customFormat="1" x14ac:dyDescent="0.2">
+      <c r="D59" s="33"/>
+      <c r="G59" s="30"/>
+      <c r="H59" s="30"/>
+      <c r="I59" s="30"/>
+    </row>
+    <row r="60" spans="1:11" s="25" customFormat="1" ht="17" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A60" s="25" t="b">
+        <v>1</v>
+      </c>
+      <c r="B60" s="25" t="s">
+        <v>631</v>
+      </c>
+      <c r="C60" s="25" t="s">
+        <v>13</v>
+      </c>
+      <c r="D60" s="33"/>
+      <c r="E60" s="25" t="s">
+        <v>76</v>
+      </c>
+      <c r="F60" s="25" t="s">
         <v>83</v>
       </c>
-      <c r="H57" s="43" t="s">
-        <v>879</v>
-      </c>
-    </row>
-    <row r="58" spans="1:11" s="25" customFormat="1" x14ac:dyDescent="0.2">
-      <c r="G58" s="30"/>
-      <c r="H58" s="42"/>
-      <c r="I58" s="30"/>
-      <c r="K58" s="17"/>
-    </row>
-    <row r="59" spans="1:11" s="25" customFormat="1" x14ac:dyDescent="0.2">
-      <c r="A59" s="25" t="b">
-        <v>1</v>
-      </c>
-      <c r="B59" s="25" t="s">
-        <v>631</v>
-      </c>
-      <c r="C59" s="25" t="s">
-        <v>782</v>
-      </c>
-      <c r="E59" s="25" t="s">
-        <v>78</v>
-      </c>
-      <c r="F59" s="25" t="s">
-        <v>732</v>
-      </c>
-      <c r="G59" s="25" t="str">
-        <f>"{{"&amp;C59&amp;"}}"</f>
-        <v>{{id:datasetID}}</v>
-      </c>
-    </row>
-    <row r="60" spans="1:11" s="25" customFormat="1" x14ac:dyDescent="0.2">
-      <c r="A60" s="25" t="b">
-        <v>1</v>
-      </c>
-      <c r="B60" s="25" t="s">
-        <v>631</v>
-      </c>
-      <c r="C60" s="25" t="s">
-        <v>787</v>
-      </c>
-      <c r="E60" s="25" t="s">
-        <v>78</v>
-      </c>
-      <c r="F60" s="25" t="s">
-        <v>736</v>
-      </c>
-      <c r="G60" s="25" t="str">
-        <f t="shared" ref="G60" si="0">"{{"&amp;C60&amp;"}}"</f>
-        <v>{{id:addressID}}</v>
+      <c r="H60" s="43" t="s">
+        <v>877</v>
       </c>
     </row>
     <row r="61" spans="1:11" s="25" customFormat="1" x14ac:dyDescent="0.2">
-      <c r="A61" s="25" t="b">
-        <v>1</v>
-      </c>
-      <c r="B61" s="25" t="s">
-        <v>631</v>
-      </c>
-      <c r="C61" s="25" t="s">
-        <v>782</v>
-      </c>
-      <c r="E61" s="25" t="s">
-        <v>114</v>
-      </c>
-      <c r="F61" s="25" t="s">
-        <v>732</v>
-      </c>
-      <c r="G61" s="25" t="str">
-        <f t="shared" ref="G61:G67" si="1">"{{"&amp;C61&amp;"}}"</f>
-        <v>{{id:datasetID}}</v>
-      </c>
+      <c r="G61" s="30"/>
+      <c r="H61" s="42"/>
+      <c r="I61" s="30"/>
+      <c r="K61" s="17"/>
     </row>
     <row r="62" spans="1:11" s="25" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A62" s="25" t="b">
@@ -15365,17 +15369,17 @@
         <v>631</v>
       </c>
       <c r="C62" s="25" t="s">
-        <v>783</v>
+        <v>782</v>
       </c>
       <c r="E62" s="25" t="s">
-        <v>114</v>
+        <v>78</v>
       </c>
       <c r="F62" s="25" t="s">
-        <v>733</v>
+        <v>732</v>
       </c>
       <c r="G62" s="25" t="str">
-        <f t="shared" si="1"/>
-        <v>{{id:measureSetRepID}}</v>
+        <f>"{{"&amp;C62&amp;"}}"</f>
+        <v>{{id:datasetID}}</v>
       </c>
     </row>
     <row r="63" spans="1:11" s="25" customFormat="1" x14ac:dyDescent="0.2">
@@ -15386,17 +15390,17 @@
         <v>631</v>
       </c>
       <c r="C63" s="25" t="s">
-        <v>782</v>
+        <v>787</v>
       </c>
       <c r="E63" s="25" t="s">
-        <v>475</v>
+        <v>78</v>
       </c>
       <c r="F63" s="25" t="s">
-        <v>732</v>
+        <v>736</v>
       </c>
       <c r="G63" s="25" t="str">
-        <f t="shared" si="1"/>
-        <v>{{id:datasetID}}</v>
+        <f t="shared" ref="G63" si="0">"{{"&amp;C63&amp;"}}"</f>
+        <v>{{id:addressID}}</v>
       </c>
     </row>
     <row r="64" spans="1:11" s="25" customFormat="1" x14ac:dyDescent="0.2">
@@ -15407,17 +15411,17 @@
         <v>631</v>
       </c>
       <c r="C64" s="25" t="s">
-        <v>785</v>
+        <v>782</v>
       </c>
       <c r="E64" s="25" t="s">
-        <v>151</v>
+        <v>114</v>
       </c>
       <c r="F64" s="25" t="s">
-        <v>742</v>
+        <v>732</v>
       </c>
       <c r="G64" s="25" t="str">
-        <f t="shared" si="1"/>
-        <v>{{id:instrumentID}}</v>
+        <f t="shared" ref="G64:G70" si="1">"{{"&amp;C64&amp;"}}"</f>
+        <v>{{id:datasetID}}</v>
       </c>
     </row>
     <row r="65" spans="1:7" s="25" customFormat="1" x14ac:dyDescent="0.2">
@@ -15431,7 +15435,7 @@
         <v>783</v>
       </c>
       <c r="E65" s="25" t="s">
-        <v>146</v>
+        <v>114</v>
       </c>
       <c r="F65" s="25" t="s">
         <v>733</v>
@@ -15452,7 +15456,7 @@
         <v>782</v>
       </c>
       <c r="E66" s="25" t="s">
-        <v>117</v>
+        <v>475</v>
       </c>
       <c r="F66" s="25" t="s">
         <v>732</v>
@@ -15470,20 +15474,83 @@
         <v>631</v>
       </c>
       <c r="C67" s="25" t="s">
-        <v>782</v>
+        <v>785</v>
       </c>
       <c r="E67" s="25" t="s">
-        <v>76</v>
+        <v>151</v>
       </c>
       <c r="F67" s="25" t="s">
-        <v>732</v>
+        <v>742</v>
       </c>
       <c r="G67" s="25" t="str">
         <f t="shared" si="1"/>
+        <v>{{id:instrumentID}}</v>
+      </c>
+    </row>
+    <row r="68" spans="1:7" s="25" customFormat="1" x14ac:dyDescent="0.2">
+      <c r="A68" s="25" t="b">
+        <v>1</v>
+      </c>
+      <c r="B68" s="25" t="s">
+        <v>631</v>
+      </c>
+      <c r="C68" s="25" t="s">
+        <v>783</v>
+      </c>
+      <c r="E68" s="25" t="s">
+        <v>146</v>
+      </c>
+      <c r="F68" s="25" t="s">
+        <v>733</v>
+      </c>
+      <c r="G68" s="25" t="str">
+        <f t="shared" si="1"/>
+        <v>{{id:measureSetRepID}}</v>
+      </c>
+    </row>
+    <row r="69" spans="1:7" s="25" customFormat="1" x14ac:dyDescent="0.2">
+      <c r="A69" s="25" t="b">
+        <v>1</v>
+      </c>
+      <c r="B69" s="25" t="s">
+        <v>631</v>
+      </c>
+      <c r="C69" s="25" t="s">
+        <v>782</v>
+      </c>
+      <c r="E69" s="25" t="s">
+        <v>117</v>
+      </c>
+      <c r="F69" s="25" t="s">
+        <v>732</v>
+      </c>
+      <c r="G69" s="25" t="str">
+        <f t="shared" si="1"/>
         <v>{{id:datasetID}}</v>
       </c>
     </row>
-    <row r="68" spans="1:7" s="25" customFormat="1" x14ac:dyDescent="0.2"/>
+    <row r="70" spans="1:7" s="25" customFormat="1" x14ac:dyDescent="0.2">
+      <c r="A70" s="25" t="b">
+        <v>1</v>
+      </c>
+      <c r="B70" s="25" t="s">
+        <v>631</v>
+      </c>
+      <c r="C70" s="25" t="s">
+        <v>782</v>
+      </c>
+      <c r="E70" s="25" t="s">
+        <v>76</v>
+      </c>
+      <c r="F70" s="25" t="s">
+        <v>732</v>
+      </c>
+      <c r="G70" s="25" t="str">
+        <f t="shared" si="1"/>
+        <v>{{id:datasetID}}</v>
+      </c>
+    </row>
+    <row r="71" spans="1:7" s="25" customFormat="1" x14ac:dyDescent="0.2"/>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" horizontalDpi="0" verticalDpi="0"/>
@@ -15492,7 +15559,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B39AC7DD-3F73-2C47-925D-21E5B4EBE6FC}">
-  <dimension ref="A1:T26"/>
+  <dimension ref="A1:S26"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="2" max="2" width="13" bestFit="1" customWidth="1"/>
@@ -15505,16 +15572,15 @@
     <col min="9" max="9" width="21.83203125" customWidth="1"/>
     <col min="10" max="10" width="16.83203125" bestFit="1" customWidth="1"/>
     <col min="11" max="11" width="22" bestFit="1" customWidth="1"/>
-    <col min="12" max="12" width="14.5" bestFit="1" customWidth="1"/>
-    <col min="13" max="13" width="23.5" bestFit="1" customWidth="1"/>
-    <col min="14" max="14" width="23.5" customWidth="1"/>
-    <col min="15" max="15" width="20.1640625" bestFit="1" customWidth="1"/>
-    <col min="16" max="16" width="18.5" bestFit="1" customWidth="1"/>
-    <col min="17" max="19" width="21.83203125" customWidth="1"/>
-    <col min="20" max="20" width="27.6640625" customWidth="1"/>
+    <col min="12" max="12" width="23.5" bestFit="1" customWidth="1"/>
+    <col min="13" max="13" width="23.5" customWidth="1"/>
+    <col min="14" max="14" width="20.1640625" bestFit="1" customWidth="1"/>
+    <col min="15" max="15" width="18.5" bestFit="1" customWidth="1"/>
+    <col min="16" max="18" width="21.83203125" customWidth="1"/>
+    <col min="19" max="19" width="27.6640625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:20" s="40" customFormat="1" ht="19" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:19" s="40" customFormat="1" ht="19" x14ac:dyDescent="0.25">
       <c r="A1" s="40" t="s">
         <v>673</v>
       </c>
@@ -15540,7 +15606,7 @@
         <v>818</v>
       </c>
       <c r="I1" s="40" t="s">
-        <v>867</v>
+        <v>881</v>
       </c>
       <c r="J1" s="41" t="s">
         <v>810</v>
@@ -15549,34 +15615,31 @@
         <v>811</v>
       </c>
       <c r="L1" s="41" t="s">
-        <v>812</v>
+        <v>813</v>
       </c>
       <c r="M1" s="41" t="s">
-        <v>813</v>
+        <v>858</v>
       </c>
       <c r="N1" s="41" t="s">
-        <v>858</v>
+        <v>814</v>
       </c>
       <c r="O1" s="41" t="s">
-        <v>814</v>
-      </c>
-      <c r="P1" s="41" t="s">
         <v>815</v>
       </c>
+      <c r="P1" s="40" t="s">
+        <v>882</v>
+      </c>
       <c r="Q1" s="40" t="s">
-        <v>869</v>
+        <v>873</v>
       </c>
       <c r="R1" s="40" t="s">
-        <v>875</v>
-      </c>
-      <c r="S1" s="40" t="s">
         <v>863</v>
       </c>
-      <c r="T1" s="41" t="s">
+      <c r="S1" s="41" t="s">
         <v>120</v>
       </c>
     </row>
-    <row r="2" spans="1:20" s="25" customFormat="1" x14ac:dyDescent="0.2">
+    <row r="2" spans="1:19" s="25" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A2" s="25" t="b">
         <v>1</v>
       </c>
@@ -15603,19 +15666,16 @@
         <v>160</v>
       </c>
       <c r="L2" s="25" t="s">
-        <v>646</v>
-      </c>
-      <c r="M2" s="25" t="s">
         <v>648</v>
       </c>
+      <c r="N2" s="25" t="s">
+        <v>161</v>
+      </c>
       <c r="O2" s="25" t="s">
-        <v>161</v>
-      </c>
-      <c r="P2" s="25" t="s">
         <v>154</v>
       </c>
     </row>
-    <row r="3" spans="1:20" s="25" customFormat="1" x14ac:dyDescent="0.2">
+    <row r="3" spans="1:19" s="25" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A3" s="25" t="b">
         <v>1</v>
       </c>
@@ -15642,19 +15702,16 @@
         <v>167</v>
       </c>
       <c r="L3" s="25" t="s">
-        <v>646</v>
-      </c>
-      <c r="M3" s="25" t="s">
         <v>652</v>
       </c>
+      <c r="N3" s="25" t="s">
+        <v>168</v>
+      </c>
       <c r="O3" s="25" t="s">
-        <v>168</v>
-      </c>
-      <c r="P3" s="25" t="s">
         <v>154</v>
       </c>
     </row>
-    <row r="4" spans="1:20" s="25" customFormat="1" x14ac:dyDescent="0.2">
+    <row r="4" spans="1:19" s="25" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A4" s="25" t="b">
         <v>1</v>
       </c>
@@ -15681,19 +15738,16 @@
         <v>166</v>
       </c>
       <c r="L4" s="25" t="s">
-        <v>646</v>
-      </c>
-      <c r="M4" s="25" t="s">
         <v>651</v>
       </c>
+      <c r="N4" s="25" t="s">
+        <v>157</v>
+      </c>
       <c r="O4" s="25" t="s">
-        <v>157</v>
-      </c>
-      <c r="P4" s="25" t="s">
         <v>154</v>
       </c>
     </row>
-    <row r="5" spans="1:20" s="25" customFormat="1" x14ac:dyDescent="0.2">
+    <row r="5" spans="1:19" s="25" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A5" s="25" t="b">
         <v>1</v>
       </c>
@@ -15720,19 +15774,16 @@
         <v>176</v>
       </c>
       <c r="L5" s="25" t="s">
-        <v>646</v>
-      </c>
-      <c r="M5" s="25" t="s">
         <v>665</v>
       </c>
+      <c r="N5" s="25" t="s">
+        <v>168</v>
+      </c>
       <c r="O5" s="25" t="s">
-        <v>168</v>
-      </c>
-      <c r="P5" s="25" t="s">
         <v>154</v>
       </c>
     </row>
-    <row r="6" spans="1:20" s="25" customFormat="1" x14ac:dyDescent="0.2">
+    <row r="6" spans="1:19" s="25" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A6" s="25" t="b">
         <v>1</v>
       </c>
@@ -15759,19 +15810,16 @@
         <v>172</v>
       </c>
       <c r="L6" s="25" t="s">
-        <v>646</v>
-      </c>
-      <c r="M6" s="25" t="s">
         <v>663</v>
       </c>
+      <c r="N6" s="25" t="s">
+        <v>173</v>
+      </c>
       <c r="O6" s="25" t="s">
-        <v>173</v>
-      </c>
-      <c r="P6" s="25" t="s">
         <v>154</v>
       </c>
     </row>
-    <row r="7" spans="1:20" s="25" customFormat="1" x14ac:dyDescent="0.2">
+    <row r="7" spans="1:19" s="25" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A7" s="25" t="b">
         <v>1</v>
       </c>
@@ -15798,22 +15846,19 @@
         <v>177</v>
       </c>
       <c r="L7" s="25" t="s">
-        <v>646</v>
-      </c>
-      <c r="M7" s="25" t="s">
         <v>666</v>
       </c>
+      <c r="N7" s="25" t="s">
+        <v>175</v>
+      </c>
       <c r="O7" s="25" t="s">
-        <v>175</v>
-      </c>
-      <c r="P7" s="25" t="s">
         <v>154</v>
       </c>
-      <c r="T7" s="26" t="s">
-        <v>882</v>
-      </c>
-    </row>
-    <row r="8" spans="1:20" s="25" customFormat="1" x14ac:dyDescent="0.2">
+      <c r="S7" s="26" t="s">
+        <v>880</v>
+      </c>
+    </row>
+    <row r="8" spans="1:19" s="25" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A8" s="25" t="b">
         <v>1</v>
       </c>
@@ -15840,19 +15885,16 @@
         <v>170</v>
       </c>
       <c r="L8" s="25" t="s">
-        <v>646</v>
-      </c>
-      <c r="M8" s="25" t="s">
         <v>661</v>
       </c>
+      <c r="N8" s="25" t="s">
+        <v>161</v>
+      </c>
       <c r="O8" s="25" t="s">
-        <v>161</v>
-      </c>
-      <c r="P8" s="25" t="s">
         <v>158</v>
       </c>
     </row>
-    <row r="9" spans="1:20" s="25" customFormat="1" x14ac:dyDescent="0.2">
+    <row r="9" spans="1:19" s="25" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A9" s="25" t="b">
         <v>1</v>
       </c>
@@ -15879,22 +15921,19 @@
         <v>640</v>
       </c>
       <c r="L9" s="25" t="s">
-        <v>646</v>
-      </c>
-      <c r="M9" s="25" t="s">
         <v>671</v>
       </c>
+      <c r="N9" s="25" t="s">
+        <v>644</v>
+      </c>
       <c r="O9" s="25" t="s">
-        <v>644</v>
+        <v>158</v>
       </c>
       <c r="P9" s="25" t="s">
-        <v>158</v>
-      </c>
-      <c r="Q9" s="25" t="s">
-        <v>870</v>
-      </c>
-    </row>
-    <row r="10" spans="1:20" s="25" customFormat="1" x14ac:dyDescent="0.2">
+        <v>868</v>
+      </c>
+    </row>
+    <row r="10" spans="1:19" s="25" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A10" s="25" t="b">
         <v>1</v>
       </c>
@@ -15921,22 +15960,19 @@
         <v>639</v>
       </c>
       <c r="L10" s="25" t="s">
-        <v>646</v>
-      </c>
-      <c r="M10" s="25" t="s">
         <v>670</v>
       </c>
+      <c r="N10" s="25" t="s">
+        <v>643</v>
+      </c>
       <c r="O10" s="25" t="s">
-        <v>643</v>
+        <v>158</v>
       </c>
       <c r="P10" s="25" t="s">
-        <v>158</v>
-      </c>
-      <c r="Q10" s="25" t="s">
-        <v>871</v>
-      </c>
-    </row>
-    <row r="11" spans="1:20" s="25" customFormat="1" x14ac:dyDescent="0.2">
+        <v>869</v>
+      </c>
+    </row>
+    <row r="11" spans="1:19" s="25" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A11" s="25" t="b">
         <v>1</v>
       </c>
@@ -15963,19 +15999,16 @@
         <v>162</v>
       </c>
       <c r="L11" s="25" t="s">
-        <v>646</v>
-      </c>
-      <c r="M11" s="25" t="s">
         <v>649</v>
       </c>
+      <c r="N11" s="25" t="s">
+        <v>163</v>
+      </c>
       <c r="O11" s="25" t="s">
-        <v>163</v>
-      </c>
-      <c r="P11" s="25" t="s">
         <v>158</v>
       </c>
     </row>
-    <row r="12" spans="1:20" s="25" customFormat="1" x14ac:dyDescent="0.2">
+    <row r="12" spans="1:19" s="25" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A12" s="25" t="b">
         <v>1</v>
       </c>
@@ -16002,13 +16035,10 @@
         <v>165</v>
       </c>
       <c r="L12" s="25" t="s">
-        <v>646</v>
-      </c>
-      <c r="M12" s="25" t="s">
         <v>650</v>
       </c>
     </row>
-    <row r="13" spans="1:20" s="25" customFormat="1" x14ac:dyDescent="0.2">
+    <row r="13" spans="1:19" s="25" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A13" s="25" t="b">
         <v>1</v>
       </c>
@@ -16035,22 +16065,19 @@
         <v>596</v>
       </c>
       <c r="L13" s="25" t="s">
-        <v>646</v>
-      </c>
-      <c r="M13" s="25" t="s">
         <v>668</v>
       </c>
+      <c r="N13" s="25" t="s">
+        <v>642</v>
+      </c>
       <c r="O13" s="25" t="s">
-        <v>642</v>
+        <v>158</v>
       </c>
       <c r="P13" s="25" t="s">
-        <v>158</v>
-      </c>
-      <c r="Q13" s="25" t="s">
-        <v>872</v>
-      </c>
-    </row>
-    <row r="14" spans="1:20" s="25" customFormat="1" x14ac:dyDescent="0.2">
+        <v>870</v>
+      </c>
+    </row>
+    <row r="14" spans="1:19" s="25" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A14" s="25" t="b">
         <v>1</v>
       </c>
@@ -16071,7 +16098,7 @@
         <v>831</v>
       </c>
       <c r="I14" s="25" t="s">
-        <v>868</v>
+        <v>867</v>
       </c>
       <c r="J14" s="25" t="s">
         <v>164</v>
@@ -16080,22 +16107,19 @@
         <v>641</v>
       </c>
       <c r="L14" s="25" t="s">
-        <v>646</v>
-      </c>
-      <c r="M14" s="25" t="s">
         <v>672</v>
       </c>
+      <c r="N14" s="25" t="s">
+        <v>645</v>
+      </c>
       <c r="O14" s="25" t="s">
-        <v>645</v>
+        <v>158</v>
       </c>
       <c r="P14" s="25" t="s">
-        <v>158</v>
-      </c>
-      <c r="Q14" s="25" t="s">
-        <v>873</v>
-      </c>
-    </row>
-    <row r="15" spans="1:20" s="25" customFormat="1" x14ac:dyDescent="0.2">
+        <v>871</v>
+      </c>
+    </row>
+    <row r="15" spans="1:19" s="25" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A15" s="25" t="b">
         <v>1</v>
       </c>
@@ -16122,25 +16146,22 @@
         <v>638</v>
       </c>
       <c r="L15" s="25" t="s">
-        <v>646</v>
-      </c>
-      <c r="M15" s="25" t="s">
         <v>667</v>
       </c>
-      <c r="O15" t="s">
+      <c r="N15" t="s">
         <v>642</v>
       </c>
+      <c r="O15" s="25" t="s">
+        <v>158</v>
+      </c>
       <c r="P15" s="25" t="s">
-        <v>158</v>
+        <v>872</v>
       </c>
       <c r="Q15" s="25" t="s">
         <v>874</v>
       </c>
-      <c r="R15" s="25" t="s">
-        <v>876</v>
-      </c>
-    </row>
-    <row r="16" spans="1:20" s="25" customFormat="1" x14ac:dyDescent="0.2">
+    </row>
+    <row r="16" spans="1:19" s="25" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A16" s="25" t="b">
         <v>1</v>
       </c>
@@ -16166,26 +16187,23 @@
       <c r="K16" s="25" t="s">
         <v>638</v>
       </c>
-      <c r="L16" s="25" t="s">
-        <v>646</v>
+      <c r="M16" s="25" t="s">
+        <v>860</v>
       </c>
       <c r="N16" s="25" t="s">
-        <v>860</v>
+        <v>642</v>
       </c>
       <c r="O16" s="25" t="s">
-        <v>642</v>
+        <v>591</v>
       </c>
       <c r="P16" s="25" t="s">
-        <v>591</v>
-      </c>
-      <c r="Q16" s="25" t="s">
-        <v>874</v>
-      </c>
-      <c r="T16" s="26" t="s">
+        <v>872</v>
+      </c>
+      <c r="S16" s="26" t="s">
         <v>862</v>
       </c>
     </row>
-    <row r="17" spans="1:20" s="25" customFormat="1" x14ac:dyDescent="0.2">
+    <row r="17" spans="1:19" s="25" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A17" s="25" t="b">
         <v>1</v>
       </c>
@@ -16211,26 +16229,23 @@
       <c r="K17" s="25" t="s">
         <v>638</v>
       </c>
-      <c r="L17" s="25" t="s">
-        <v>646</v>
+      <c r="M17" s="25" t="s">
+        <v>861</v>
       </c>
       <c r="N17" s="25" t="s">
-        <v>861</v>
+        <v>642</v>
       </c>
       <c r="O17" s="25" t="s">
-        <v>642</v>
+        <v>592</v>
       </c>
       <c r="P17" s="25" t="s">
-        <v>592</v>
-      </c>
-      <c r="Q17" s="25" t="s">
-        <v>874</v>
-      </c>
-      <c r="T17" s="26" t="s">
+        <v>872</v>
+      </c>
+      <c r="S17" s="26" t="s">
         <v>862</v>
       </c>
     </row>
-    <row r="18" spans="1:20" s="25" customFormat="1" x14ac:dyDescent="0.2">
+    <row r="18" spans="1:19" s="25" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A18" s="25" t="b">
         <v>1</v>
       </c>
@@ -16256,26 +16271,23 @@
       <c r="K18" s="25" t="s">
         <v>638</v>
       </c>
-      <c r="L18" s="25" t="s">
-        <v>646</v>
+      <c r="M18" s="25" t="s">
+        <v>859</v>
       </c>
       <c r="N18" s="25" t="s">
-        <v>859</v>
+        <v>642</v>
       </c>
       <c r="O18" s="25" t="s">
-        <v>642</v>
+        <v>590</v>
       </c>
       <c r="P18" s="25" t="s">
-        <v>590</v>
-      </c>
-      <c r="Q18" s="25" t="s">
-        <v>874</v>
-      </c>
-      <c r="T18" s="26" t="s">
+        <v>872</v>
+      </c>
+      <c r="S18" s="26" t="s">
         <v>862</v>
       </c>
     </row>
-    <row r="19" spans="1:20" s="25" customFormat="1" x14ac:dyDescent="0.2">
+    <row r="19" spans="1:19" s="25" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A19" s="25" t="b">
         <v>1</v>
       </c>
@@ -16302,19 +16314,16 @@
         <v>48</v>
       </c>
       <c r="L19" s="25" t="s">
-        <v>646</v>
-      </c>
-      <c r="M19" s="25" t="s">
         <v>662</v>
       </c>
+      <c r="N19" s="25" t="s">
+        <v>171</v>
+      </c>
       <c r="O19" s="25" t="s">
-        <v>171</v>
-      </c>
-      <c r="P19" s="25" t="s">
         <v>154</v>
       </c>
     </row>
-    <row r="20" spans="1:20" s="25" customFormat="1" x14ac:dyDescent="0.2">
+    <row r="20" spans="1:19" s="25" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A20" s="25" t="b">
         <v>1</v>
       </c>
@@ -16341,16 +16350,13 @@
         <v>169</v>
       </c>
       <c r="L20" s="25" t="s">
-        <v>646</v>
-      </c>
-      <c r="M20" s="25" t="s">
         <v>637</v>
       </c>
-      <c r="S20" s="25" t="s">
-        <v>877</v>
-      </c>
-    </row>
-    <row r="21" spans="1:20" s="25" customFormat="1" x14ac:dyDescent="0.2">
+      <c r="R20" s="25" t="s">
+        <v>875</v>
+      </c>
+    </row>
+    <row r="21" spans="1:19" s="25" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A21" s="25" t="b">
         <v>1</v>
       </c>
@@ -16377,19 +16383,16 @@
         <v>597</v>
       </c>
       <c r="L21" s="25" t="s">
-        <v>646</v>
-      </c>
-      <c r="M21" s="25" t="s">
         <v>669</v>
       </c>
+      <c r="N21" s="25" t="s">
+        <v>163</v>
+      </c>
       <c r="O21" s="25" t="s">
-        <v>163</v>
-      </c>
-      <c r="P21" s="25" t="s">
         <v>158</v>
       </c>
     </row>
-    <row r="22" spans="1:20" s="25" customFormat="1" x14ac:dyDescent="0.2">
+    <row r="22" spans="1:19" s="25" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A22" s="25" t="b">
         <v>1</v>
       </c>
@@ -16416,19 +16419,16 @@
         <v>579</v>
       </c>
       <c r="L22" s="25" t="s">
-        <v>646</v>
-      </c>
-      <c r="M22" s="25" t="s">
         <v>659</v>
       </c>
+      <c r="N22" s="25" t="s">
+        <v>580</v>
+      </c>
       <c r="O22" s="25" t="s">
-        <v>580</v>
-      </c>
-      <c r="P22" s="25" t="s">
         <v>154</v>
       </c>
     </row>
-    <row r="23" spans="1:20" s="25" customFormat="1" x14ac:dyDescent="0.2">
+    <row r="23" spans="1:19" s="25" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A23" s="25" t="b">
         <v>1</v>
       </c>
@@ -16455,20 +16455,17 @@
         <v>159</v>
       </c>
       <c r="L23" s="29" t="s">
-        <v>646</v>
-      </c>
-      <c r="M23" s="29" t="s">
         <v>647</v>
       </c>
-      <c r="N23" s="29"/>
+      <c r="M23" s="29"/>
+      <c r="N23" s="29" t="s">
+        <v>157</v>
+      </c>
       <c r="O23" s="29" t="s">
-        <v>157</v>
-      </c>
-      <c r="P23" s="29" t="s">
         <v>158</v>
       </c>
     </row>
-    <row r="24" spans="1:20" s="25" customFormat="1" x14ac:dyDescent="0.2">
+    <row r="24" spans="1:19" s="25" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A24" s="25" t="b">
         <v>1</v>
       </c>
@@ -16495,26 +16492,23 @@
         <v>50</v>
       </c>
       <c r="L24" s="25" t="s">
-        <v>646</v>
-      </c>
-      <c r="M24" s="25" t="s">
         <v>664</v>
       </c>
+      <c r="N24" s="25" t="s">
+        <v>174</v>
+      </c>
       <c r="O24" s="25" t="s">
-        <v>174</v>
-      </c>
-      <c r="P24" s="25" t="s">
         <v>154</v>
       </c>
     </row>
-    <row r="25" spans="1:20" s="25" customFormat="1" x14ac:dyDescent="0.2">
+    <row r="25" spans="1:19" s="25" customFormat="1" x14ac:dyDescent="0.2">
       <c r="G25"/>
     </row>
-    <row r="26" spans="1:20" s="25" customFormat="1" x14ac:dyDescent="0.2">
+    <row r="26" spans="1:19" s="25" customFormat="1" x14ac:dyDescent="0.2">
       <c r="G26"/>
     </row>
   </sheetData>
-  <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:T26">
+  <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:S26">
     <sortCondition ref="C1:C26"/>
   </sortState>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -16600,7 +16594,7 @@
         <v>797</v>
       </c>
       <c r="K2" s="36" t="s">
-        <v>880</v>
+        <v>878</v>
       </c>
       <c r="L2" s="36" t="s">
         <v>864</v>
@@ -16939,7 +16933,7 @@
         <v>815</v>
       </c>
       <c r="O1" s="41" t="s">
-        <v>869</v>
+        <v>882</v>
       </c>
       <c r="P1" s="41" t="s">
         <v>120</v>
@@ -19126,7 +19120,7 @@
         <v>683</v>
       </c>
       <c r="O78" s="25" t="s">
-        <v>878</v>
+        <v>876</v>
       </c>
     </row>
     <row r="79" spans="1:15" s="25" customFormat="1" x14ac:dyDescent="0.2">

</xml_diff>

<commit_message>
Added dat0 binding for ID generation code, that does not replace empty values with "Empty"
</commit_message>
<xml_diff>
--- a/data/mapping_config_files/nwss_to_odm_v2_mapping.xlsx
+++ b/data/mapping_config_files/nwss_to_odm_v2_mapping.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/martinwellman/Documents/Health/Wastewater/PHES-ODM-MapGenerator/PHES-ODM-MapGenerator/data/mapping_config_files/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{753AD274-237D-8148-A5C6-BC44D4EDCFAC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C5389CD7-1A3A-0242-923B-0879027E46CC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="500" windowWidth="40960" windowHeight="20860" xr2:uid="{77810E24-F86B-BC44-A0D5-8790E6EC60B4}"/>
   </bookViews>
@@ -53,7 +53,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3240" uniqueCount="987">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3228" uniqueCount="986">
   <si>
     <t>Reporter</t>
   </si>
@@ -2468,9 +2468,6 @@
   </si>
   <si>
     <t>&lt;empty&gt;</t>
-  </si>
-  <si>
-    <t>Added by Martin</t>
   </si>
   <si>
     <t>qualityFlag_expr</t>
@@ -3159,7 +3156,7 @@
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="8">
+  <fills count="7">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -3193,12 +3190,6 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor theme="0" tint="-0.14999847407452621"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="7" tint="0.59999389629810485"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -3302,7 +3293,6 @@
     <xf numFmtId="0" fontId="0" fillId="6" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="6" fillId="7" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" quotePrefix="1" applyFont="1"/>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment wrapText="1"/>
@@ -3339,6 +3329,7 @@
       <alignment wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="6" fillId="6" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -14506,7 +14497,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{3154BFCE-06D9-9649-B340-B23DCF20DD83}">
-  <dimension ref="A1:K107"/>
+  <dimension ref="A1:K104"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="2" max="2" width="13" bestFit="1" customWidth="1"/>
@@ -14520,35 +14511,35 @@
     <col min="11" max="11" width="47.6640625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:10" s="40" customFormat="1" ht="19" x14ac:dyDescent="0.25">
-      <c r="A1" s="40" t="s">
+    <row r="1" spans="1:10" s="39" customFormat="1" ht="19" x14ac:dyDescent="0.25">
+      <c r="A1" s="39" t="s">
         <v>666</v>
       </c>
-      <c r="B1" s="40" t="s">
+      <c r="B1" s="39" t="s">
         <v>629</v>
       </c>
-      <c r="C1" s="40" t="s">
+      <c r="C1" s="39" t="s">
         <v>631</v>
       </c>
-      <c r="D1" s="40" t="s">
+      <c r="D1" s="39" t="s">
         <v>632</v>
       </c>
-      <c r="E1" s="40" t="s">
+      <c r="E1" s="39" t="s">
         <v>633</v>
       </c>
-      <c r="F1" s="40" t="s">
+      <c r="F1" s="39" t="s">
         <v>634</v>
       </c>
-      <c r="G1" s="40" t="s">
+      <c r="G1" s="39" t="s">
         <v>635</v>
       </c>
-      <c r="H1" s="40" t="s">
-        <v>806</v>
-      </c>
-      <c r="I1" s="40" t="s">
+      <c r="H1" s="39" t="s">
+        <v>805</v>
+      </c>
+      <c r="I1" s="39" t="s">
         <v>668</v>
       </c>
-      <c r="J1" s="40" t="s">
+      <c r="J1" s="39" t="s">
         <v>120</v>
       </c>
     </row>
@@ -14589,7 +14580,7 @@
         <v>725</v>
       </c>
       <c r="G3" s="25" t="s">
-        <v>876</v>
+        <v>875</v>
       </c>
     </row>
     <row r="4" spans="1:10" s="25" customFormat="1" x14ac:dyDescent="0.2">
@@ -14609,7 +14600,7 @@
         <v>729</v>
       </c>
       <c r="G4" s="25" t="s">
-        <v>877</v>
+        <v>876</v>
       </c>
     </row>
     <row r="5" spans="1:10" s="25" customFormat="1" x14ac:dyDescent="0.2"/>
@@ -14650,7 +14641,7 @@
         <v>725</v>
       </c>
       <c r="G7" s="25" t="s">
-        <v>876</v>
+        <v>875</v>
       </c>
     </row>
     <row r="8" spans="1:10" s="25" customFormat="1" x14ac:dyDescent="0.2">
@@ -14684,7 +14675,7 @@
         <v>739</v>
       </c>
       <c r="F9" s="25" t="s">
-        <v>880</v>
+        <v>879</v>
       </c>
     </row>
     <row r="10" spans="1:10" s="25" customFormat="1" x14ac:dyDescent="0.2">
@@ -14698,7 +14689,7 @@
         <v>739</v>
       </c>
       <c r="F10" s="25" t="s">
-        <v>881</v>
+        <v>880</v>
       </c>
     </row>
     <row r="11" spans="1:10" s="25" customFormat="1" x14ac:dyDescent="0.2">
@@ -14712,7 +14703,7 @@
         <v>739</v>
       </c>
       <c r="F11" s="25" t="s">
-        <v>882</v>
+        <v>881</v>
       </c>
     </row>
     <row r="12" spans="1:10" s="25" customFormat="1" x14ac:dyDescent="0.2">
@@ -14726,7 +14717,7 @@
         <v>739</v>
       </c>
       <c r="F12" s="25" t="s">
-        <v>883</v>
+        <v>882</v>
       </c>
     </row>
     <row r="13" spans="1:10" s="25" customFormat="1" x14ac:dyDescent="0.2">
@@ -14740,7 +14731,7 @@
         <v>739</v>
       </c>
       <c r="F13" s="25" t="s">
-        <v>884</v>
+        <v>883</v>
       </c>
     </row>
     <row r="14" spans="1:10" s="25" customFormat="1" x14ac:dyDescent="0.2">
@@ -14754,7 +14745,7 @@
         <v>739</v>
       </c>
       <c r="F14" s="25" t="s">
-        <v>875</v>
+        <v>874</v>
       </c>
     </row>
     <row r="15" spans="1:10" s="25" customFormat="1" x14ac:dyDescent="0.2">
@@ -14790,7 +14781,7 @@
         <v>725</v>
       </c>
       <c r="G17" s="25" t="s">
-        <v>876</v>
+        <v>875</v>
       </c>
     </row>
     <row r="18" spans="1:11" x14ac:dyDescent="0.2">
@@ -14820,7 +14811,7 @@
         <v>725</v>
       </c>
       <c r="G19" s="25" t="s">
-        <v>876</v>
+        <v>875</v>
       </c>
     </row>
     <row r="20" spans="1:11" s="25" customFormat="1" x14ac:dyDescent="0.2">
@@ -14860,7 +14851,7 @@
         <v>735</v>
       </c>
       <c r="G21" s="25" t="s">
-        <v>879</v>
+        <v>878</v>
       </c>
     </row>
     <row r="22" spans="1:11" s="25" customFormat="1" x14ac:dyDescent="0.2">
@@ -14901,7 +14892,7 @@
         <v>725</v>
       </c>
       <c r="G24" s="25" t="s">
-        <v>876</v>
+        <v>875</v>
       </c>
     </row>
     <row r="25" spans="1:11" s="25" customFormat="1" x14ac:dyDescent="0.2">
@@ -14921,7 +14912,7 @@
         <v>726</v>
       </c>
       <c r="G25" s="25" t="s">
-        <v>878</v>
+        <v>877</v>
       </c>
     </row>
     <row r="26" spans="1:11" s="25" customFormat="1" x14ac:dyDescent="0.2">
@@ -15004,9 +14995,7 @@
       <c r="G29" s="25" t="s">
         <v>700</v>
       </c>
-      <c r="K29" s="26" t="s">
-        <v>796</v>
-      </c>
+      <c r="K29" s="44"/>
     </row>
     <row r="30" spans="1:11" s="25" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A30" s="25" t="b">
@@ -15039,14 +15028,14 @@
         <v>114</v>
       </c>
       <c r="F31" s="25" t="s">
+        <v>866</v>
+      </c>
+      <c r="H31" s="30" t="s">
         <v>867</v>
       </c>
-      <c r="H31" s="31" t="s">
-        <v>868</v>
-      </c>
     </row>
     <row r="32" spans="1:11" s="25" customFormat="1" x14ac:dyDescent="0.2">
-      <c r="H32" s="31"/>
+      <c r="H32" s="30"/>
     </row>
     <row r="33" spans="1:8" s="25" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A33" s="25" t="b">
@@ -15065,9 +15054,9 @@
         <v>726</v>
       </c>
       <c r="G33" s="25" t="s">
-        <v>878</v>
-      </c>
-      <c r="H33" s="31"/>
+        <v>877</v>
+      </c>
+      <c r="H33" s="30"/>
     </row>
     <row r="34" spans="1:8" s="25" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A34" s="25" t="b">
@@ -15088,7 +15077,7 @@
       <c r="G34" s="25" t="s">
         <v>703</v>
       </c>
-      <c r="H34" s="31"/>
+      <c r="H34" s="30"/>
     </row>
     <row r="35" spans="1:8" s="25" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A35" s="25" t="b">
@@ -15109,7 +15098,7 @@
       <c r="G35" s="25" t="s">
         <v>701</v>
       </c>
-      <c r="H35" s="31"/>
+      <c r="H35" s="30"/>
     </row>
     <row r="36" spans="1:8" s="25" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A36" s="25" t="b">
@@ -15130,10 +15119,10 @@
       <c r="G36" s="25" t="s">
         <v>693</v>
       </c>
-      <c r="H36" s="31"/>
+      <c r="H36" s="30"/>
     </row>
     <row r="37" spans="1:8" s="25" customFormat="1" x14ac:dyDescent="0.2">
-      <c r="H37" s="31"/>
+      <c r="H37" s="30"/>
     </row>
     <row r="38" spans="1:8" s="25" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A38" s="25" t="b">
@@ -15180,7 +15169,7 @@
         <v>723</v>
       </c>
       <c r="F40" s="25" t="s">
-        <v>871</v>
+        <v>870</v>
       </c>
     </row>
     <row r="41" spans="1:8" s="25" customFormat="1" x14ac:dyDescent="0.2">
@@ -15200,7 +15189,7 @@
         <v>729</v>
       </c>
       <c r="G41" s="25" t="s">
-        <v>877</v>
+        <v>876</v>
       </c>
     </row>
     <row r="42" spans="1:8" s="25" customFormat="1" x14ac:dyDescent="0.2">
@@ -15220,7 +15209,7 @@
         <v>725</v>
       </c>
       <c r="G42" s="25" t="s">
-        <v>876</v>
+        <v>875</v>
       </c>
     </row>
     <row r="43" spans="1:8" s="25" customFormat="1" x14ac:dyDescent="0.2">
@@ -15234,7 +15223,7 @@
         <v>723</v>
       </c>
       <c r="F43" s="25" t="s">
-        <v>872</v>
+        <v>871</v>
       </c>
     </row>
     <row r="44" spans="1:8" s="25" customFormat="1" x14ac:dyDescent="0.2">
@@ -15248,7 +15237,7 @@
         <v>723</v>
       </c>
       <c r="F44" s="25" t="s">
-        <v>873</v>
+        <v>872</v>
       </c>
     </row>
     <row r="45" spans="1:8" s="25" customFormat="1" x14ac:dyDescent="0.2">
@@ -15262,7 +15251,7 @@
         <v>723</v>
       </c>
       <c r="F45" s="25" t="s">
-        <v>874</v>
+        <v>873</v>
       </c>
     </row>
     <row r="46" spans="1:8" s="25" customFormat="1" x14ac:dyDescent="0.2">
@@ -15276,7 +15265,7 @@
         <v>723</v>
       </c>
       <c r="F46" s="25" t="s">
-        <v>875</v>
+        <v>874</v>
       </c>
     </row>
     <row r="47" spans="1:8" s="25" customFormat="1" x14ac:dyDescent="0.2">
@@ -15311,7 +15300,7 @@
         <v>725</v>
       </c>
       <c r="G49" s="25" t="s">
-        <v>876</v>
+        <v>875</v>
       </c>
     </row>
     <row r="50" spans="1:11" s="25" customFormat="1" x14ac:dyDescent="0.2">
@@ -15368,7 +15357,7 @@
         <v>474</v>
       </c>
       <c r="F52" s="25" t="s">
-        <v>869</v>
+        <v>868</v>
       </c>
       <c r="G52" s="25" t="s">
         <v>704</v>
@@ -15454,96 +15443,106 @@
         <v>735</v>
       </c>
       <c r="G57" s="25" t="s">
-        <v>879</v>
+        <v>878</v>
       </c>
     </row>
     <row r="58" spans="1:11" s="25" customFormat="1" x14ac:dyDescent="0.2"/>
-    <row r="59" spans="1:11" s="25" customFormat="1" x14ac:dyDescent="0.2">
+    <row r="59" spans="1:11" s="25" customFormat="1" ht="16" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A59" s="25" t="b">
         <v>1</v>
       </c>
       <c r="B59" s="25" t="s">
         <v>630</v>
       </c>
-      <c r="C59" s="25" t="s">
-        <v>53</v>
-      </c>
       <c r="E59" s="25" t="s">
-        <v>146</v>
+        <v>117</v>
       </c>
       <c r="F59" s="25" t="s">
-        <v>139</v>
-      </c>
-      <c r="G59" s="42" t="s">
-        <v>700</v>
-      </c>
-      <c r="H59" s="30"/>
-      <c r="I59" s="30"/>
-      <c r="K59" s="16" t="s">
-        <v>796</v>
-      </c>
-    </row>
-    <row r="60" spans="1:11" s="25" customFormat="1" x14ac:dyDescent="0.2">
+        <v>669</v>
+      </c>
+      <c r="G59" s="29"/>
+      <c r="H59" s="31" t="s">
+        <v>691</v>
+      </c>
+    </row>
+    <row r="60" spans="1:11" s="25" customFormat="1" ht="16" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A60" s="25" t="b">
         <v>1</v>
       </c>
       <c r="B60" s="25" t="s">
         <v>630</v>
       </c>
-      <c r="C60" s="25" t="s">
-        <v>773</v>
-      </c>
+      <c r="C60" s="30"/>
+      <c r="D60" s="32"/>
       <c r="E60" s="25" t="s">
-        <v>146</v>
+        <v>117</v>
       </c>
       <c r="F60" s="25" t="s">
-        <v>726</v>
-      </c>
-      <c r="G60" s="25" t="s">
-        <v>878</v>
+        <v>118</v>
+      </c>
+      <c r="H60" s="31" t="s">
+        <v>692</v>
       </c>
     </row>
     <row r="61" spans="1:11" s="25" customFormat="1" x14ac:dyDescent="0.2">
-      <c r="G61" s="30"/>
-      <c r="H61" s="30"/>
-      <c r="I61" s="30"/>
-      <c r="K61" s="17"/>
-    </row>
-    <row r="62" spans="1:11" s="25" customFormat="1" ht="16" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A61" s="25" t="b">
+        <v>1</v>
+      </c>
+      <c r="B61" s="25" t="s">
+        <v>630</v>
+      </c>
+      <c r="C61" s="25" t="s">
+        <v>23</v>
+      </c>
+      <c r="D61" s="32"/>
+      <c r="E61" s="25" t="s">
+        <v>117</v>
+      </c>
+      <c r="F61" s="25" t="s">
+        <v>119</v>
+      </c>
+      <c r="G61" s="25" t="s">
+        <v>699</v>
+      </c>
+    </row>
+    <row r="62" spans="1:11" s="25" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A62" s="25" t="b">
         <v>1</v>
       </c>
       <c r="B62" s="25" t="s">
         <v>630</v>
+      </c>
+      <c r="C62" s="25" t="s">
+        <v>56</v>
       </c>
       <c r="E62" s="25" t="s">
         <v>117</v>
       </c>
       <c r="F62" s="25" t="s">
-        <v>669</v>
-      </c>
-      <c r="G62" s="30"/>
-      <c r="H62" s="32" t="s">
-        <v>691</v>
-      </c>
-    </row>
-    <row r="63" spans="1:11" s="25" customFormat="1" ht="16" customHeight="1" x14ac:dyDescent="0.2">
+        <v>144</v>
+      </c>
+      <c r="H62" s="25" t="s">
+        <v>922</v>
+      </c>
+    </row>
+    <row r="63" spans="1:11" s="25" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A63" s="25" t="b">
         <v>1</v>
       </c>
       <c r="B63" s="25" t="s">
         <v>630</v>
       </c>
-      <c r="C63" s="31"/>
-      <c r="D63" s="33"/>
+      <c r="C63" s="25" t="s">
+        <v>54</v>
+      </c>
       <c r="E63" s="25" t="s">
         <v>117</v>
       </c>
       <c r="F63" s="25" t="s">
-        <v>118</v>
-      </c>
-      <c r="H63" s="32" t="s">
-        <v>692</v>
+        <v>143</v>
+      </c>
+      <c r="G63" s="25" t="s">
+        <v>701</v>
       </c>
     </row>
     <row r="64" spans="1:11" s="25" customFormat="1" x14ac:dyDescent="0.2">
@@ -15554,20 +15553,20 @@
         <v>630</v>
       </c>
       <c r="C64" s="25" t="s">
-        <v>23</v>
-      </c>
-      <c r="D64" s="33"/>
+        <v>7</v>
+      </c>
       <c r="E64" s="25" t="s">
         <v>117</v>
       </c>
       <c r="F64" s="25" t="s">
-        <v>119</v>
+        <v>713</v>
       </c>
       <c r="G64" s="25" t="s">
-        <v>699</v>
-      </c>
-    </row>
-    <row r="65" spans="1:11" s="25" customFormat="1" x14ac:dyDescent="0.2">
+        <v>693</v>
+      </c>
+      <c r="K64" s="17"/>
+    </row>
+    <row r="65" spans="1:10" s="25" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A65" s="25" t="b">
         <v>1</v>
       </c>
@@ -15575,19 +15574,19 @@
         <v>630</v>
       </c>
       <c r="C65" s="25" t="s">
-        <v>56</v>
+        <v>53</v>
       </c>
       <c r="E65" s="25" t="s">
         <v>117</v>
       </c>
       <c r="F65" s="25" t="s">
-        <v>144</v>
-      </c>
-      <c r="H65" s="25" t="s">
-        <v>923</v>
-      </c>
-    </row>
-    <row r="66" spans="1:11" s="25" customFormat="1" x14ac:dyDescent="0.2">
+        <v>139</v>
+      </c>
+      <c r="G65" s="25" t="s">
+        <v>700</v>
+      </c>
+    </row>
+    <row r="66" spans="1:10" s="25" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A66" s="25" t="b">
         <v>1</v>
       </c>
@@ -15595,144 +15594,149 @@
         <v>630</v>
       </c>
       <c r="C66" s="25" t="s">
-        <v>54</v>
+        <v>8</v>
       </c>
       <c r="E66" s="25" t="s">
         <v>117</v>
       </c>
       <c r="F66" s="25" t="s">
-        <v>143</v>
+        <v>77</v>
       </c>
       <c r="G66" s="25" t="s">
-        <v>701</v>
-      </c>
-    </row>
-    <row r="67" spans="1:11" s="25" customFormat="1" x14ac:dyDescent="0.2">
-      <c r="A67" s="25" t="b">
-        <v>1</v>
-      </c>
-      <c r="B67" s="25" t="s">
-        <v>630</v>
-      </c>
-      <c r="C67" s="25" t="s">
-        <v>7</v>
-      </c>
-      <c r="E67" s="25" t="s">
+        <v>694</v>
+      </c>
+    </row>
+    <row r="67" spans="1:10" s="25" customFormat="1" x14ac:dyDescent="0.2"/>
+    <row r="68" spans="1:10" s="17" customFormat="1" ht="17" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A68" s="17" t="b">
+        <v>0</v>
+      </c>
+      <c r="B68" s="17" t="s">
+        <v>630</v>
+      </c>
+      <c r="C68" s="26" t="s">
+        <v>44</v>
+      </c>
+      <c r="E68" s="17" t="s">
         <v>117</v>
       </c>
-      <c r="F67" s="25" t="s">
-        <v>713</v>
-      </c>
-      <c r="G67" s="25" t="s">
-        <v>693</v>
-      </c>
-      <c r="K67" s="17"/>
-    </row>
-    <row r="68" spans="1:11" s="25" customFormat="1" x14ac:dyDescent="0.2">
-      <c r="A68" s="25" t="b">
-        <v>1</v>
-      </c>
-      <c r="B68" s="25" t="s">
-        <v>630</v>
-      </c>
-      <c r="C68" s="25" t="s">
-        <v>53</v>
-      </c>
-      <c r="E68" s="25" t="s">
+      <c r="F68" s="17" t="s">
+        <v>137</v>
+      </c>
+      <c r="H68" s="27"/>
+      <c r="J68" s="17" t="s">
+        <v>138</v>
+      </c>
+    </row>
+    <row r="69" spans="1:10" s="17" customFormat="1" ht="16" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A69" s="17" t="b">
+        <v>0</v>
+      </c>
+      <c r="B69" s="17" t="s">
+        <v>630</v>
+      </c>
+      <c r="C69" s="17" t="s">
+        <v>45</v>
+      </c>
+      <c r="E69" s="17" t="s">
         <v>117</v>
       </c>
-      <c r="F68" s="25" t="s">
-        <v>139</v>
-      </c>
-      <c r="G68" s="25" t="s">
-        <v>700</v>
-      </c>
-    </row>
-    <row r="69" spans="1:11" s="25" customFormat="1" x14ac:dyDescent="0.2">
-      <c r="A69" s="25" t="b">
-        <v>1</v>
-      </c>
-      <c r="B69" s="25" t="s">
-        <v>630</v>
-      </c>
-      <c r="C69" s="25" t="s">
-        <v>8</v>
-      </c>
-      <c r="E69" s="25" t="s">
+      <c r="F69" s="17" t="s">
+        <v>137</v>
+      </c>
+      <c r="H69" s="27"/>
+      <c r="J69" s="17" t="s">
+        <v>138</v>
+      </c>
+    </row>
+    <row r="70" spans="1:10" s="17" customFormat="1" x14ac:dyDescent="0.2">
+      <c r="A70" s="17" t="b">
+        <v>0</v>
+      </c>
+      <c r="B70" s="17" t="s">
+        <v>630</v>
+      </c>
+      <c r="C70" s="17" t="s">
+        <v>46</v>
+      </c>
+      <c r="E70" s="17" t="s">
         <v>117</v>
       </c>
-      <c r="F69" s="25" t="s">
-        <v>77</v>
-      </c>
-      <c r="G69" s="25" t="s">
-        <v>694</v>
-      </c>
-    </row>
-    <row r="70" spans="1:11" s="25" customFormat="1" x14ac:dyDescent="0.2"/>
-    <row r="71" spans="1:11" s="17" customFormat="1" ht="17" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A71" s="17" t="b">
-        <v>0</v>
-      </c>
-      <c r="B71" s="17" t="s">
-        <v>630</v>
-      </c>
-      <c r="C71" s="27" t="s">
-        <v>44</v>
-      </c>
-      <c r="E71" s="17" t="s">
+      <c r="F70" s="17" t="s">
+        <v>137</v>
+      </c>
+      <c r="J70" s="17" t="s">
+        <v>138</v>
+      </c>
+    </row>
+    <row r="71" spans="1:10" s="25" customFormat="1" x14ac:dyDescent="0.2"/>
+    <row r="72" spans="1:10" s="25" customFormat="1" x14ac:dyDescent="0.2">
+      <c r="A72" s="25" t="b">
+        <v>1</v>
+      </c>
+      <c r="B72" s="25" t="s">
+        <v>630</v>
+      </c>
+      <c r="C72" s="25" t="s">
+        <v>772</v>
+      </c>
+      <c r="E72" s="25" t="s">
         <v>117</v>
       </c>
-      <c r="F71" s="17" t="s">
-        <v>137</v>
-      </c>
-      <c r="H71" s="28"/>
-      <c r="J71" s="17" t="s">
-        <v>138</v>
-      </c>
-    </row>
-    <row r="72" spans="1:11" s="17" customFormat="1" ht="16" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A72" s="17" t="b">
-        <v>0</v>
-      </c>
-      <c r="B72" s="17" t="s">
-        <v>630</v>
-      </c>
-      <c r="C72" s="17" t="s">
-        <v>45</v>
-      </c>
-      <c r="E72" s="17" t="s">
+      <c r="F72" s="25" t="s">
+        <v>725</v>
+      </c>
+      <c r="G72" s="25" t="s">
+        <v>875</v>
+      </c>
+    </row>
+    <row r="73" spans="1:10" s="25" customFormat="1" x14ac:dyDescent="0.2">
+      <c r="A73" s="25" t="b">
+        <v>1</v>
+      </c>
+      <c r="B73" s="25" t="s">
+        <v>630</v>
+      </c>
+      <c r="C73" s="25" t="s">
+        <v>24</v>
+      </c>
+      <c r="D73" s="33" t="s">
+        <v>121</v>
+      </c>
+      <c r="E73" s="25" t="s">
         <v>117</v>
       </c>
-      <c r="F72" s="17" t="s">
-        <v>137</v>
-      </c>
-      <c r="H72" s="28"/>
-      <c r="J72" s="17" t="s">
-        <v>138</v>
-      </c>
-    </row>
-    <row r="73" spans="1:11" s="17" customFormat="1" x14ac:dyDescent="0.2">
-      <c r="A73" s="17" t="b">
-        <v>0</v>
-      </c>
-      <c r="B73" s="17" t="s">
-        <v>630</v>
-      </c>
-      <c r="C73" s="17" t="s">
-        <v>46</v>
-      </c>
-      <c r="E73" s="17" t="s">
+      <c r="F73" s="25" t="s">
+        <v>129</v>
+      </c>
+      <c r="G73" s="25" t="s">
+        <v>136</v>
+      </c>
+    </row>
+    <row r="74" spans="1:10" s="25" customFormat="1" x14ac:dyDescent="0.2">
+      <c r="A74" s="25" t="b">
+        <v>1</v>
+      </c>
+      <c r="B74" s="25" t="s">
+        <v>630</v>
+      </c>
+      <c r="C74" s="25" t="s">
+        <v>24</v>
+      </c>
+      <c r="D74" s="32" t="s">
+        <v>122</v>
+      </c>
+      <c r="E74" s="25" t="s">
         <v>117</v>
       </c>
-      <c r="F73" s="17" t="s">
-        <v>137</v>
-      </c>
-      <c r="J73" s="17" t="s">
-        <v>138</v>
-      </c>
-    </row>
-    <row r="74" spans="1:11" s="25" customFormat="1" x14ac:dyDescent="0.2"/>
-    <row r="75" spans="1:11" s="25" customFormat="1" x14ac:dyDescent="0.2">
+      <c r="F74" s="25" t="s">
+        <v>129</v>
+      </c>
+      <c r="G74" s="25" t="s">
+        <v>134</v>
+      </c>
+    </row>
+    <row r="75" spans="1:10" s="25" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A75" s="25" t="b">
         <v>1</v>
       </c>
@@ -15740,19 +15744,22 @@
         <v>630</v>
       </c>
       <c r="C75" s="25" t="s">
-        <v>772</v>
+        <v>24</v>
+      </c>
+      <c r="D75" s="32" t="s">
+        <v>123</v>
       </c>
       <c r="E75" s="25" t="s">
         <v>117</v>
       </c>
       <c r="F75" s="25" t="s">
-        <v>725</v>
+        <v>129</v>
       </c>
       <c r="G75" s="25" t="s">
-        <v>876</v>
-      </c>
-    </row>
-    <row r="76" spans="1:11" s="25" customFormat="1" x14ac:dyDescent="0.2">
+        <v>130</v>
+      </c>
+    </row>
+    <row r="76" spans="1:10" s="25" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A76" s="25" t="b">
         <v>1</v>
       </c>
@@ -15762,8 +15769,8 @@
       <c r="C76" s="25" t="s">
         <v>24</v>
       </c>
-      <c r="D76" s="34" t="s">
-        <v>121</v>
+      <c r="D76" s="32" t="s">
+        <v>124</v>
       </c>
       <c r="E76" s="25" t="s">
         <v>117</v>
@@ -15772,10 +15779,10 @@
         <v>129</v>
       </c>
       <c r="G76" s="25" t="s">
-        <v>136</v>
-      </c>
-    </row>
-    <row r="77" spans="1:11" s="25" customFormat="1" x14ac:dyDescent="0.2">
+        <v>131</v>
+      </c>
+    </row>
+    <row r="77" spans="1:10" s="25" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A77" s="25" t="b">
         <v>1</v>
       </c>
@@ -15785,8 +15792,8 @@
       <c r="C77" s="25" t="s">
         <v>24</v>
       </c>
-      <c r="D77" s="33" t="s">
-        <v>122</v>
+      <c r="D77" s="32" t="s">
+        <v>125</v>
       </c>
       <c r="E77" s="25" t="s">
         <v>117</v>
@@ -15795,10 +15802,10 @@
         <v>129</v>
       </c>
       <c r="G77" s="25" t="s">
-        <v>134</v>
-      </c>
-    </row>
-    <row r="78" spans="1:11" s="25" customFormat="1" x14ac:dyDescent="0.2">
+        <v>132</v>
+      </c>
+    </row>
+    <row r="78" spans="1:10" s="25" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A78" s="25" t="b">
         <v>1</v>
       </c>
@@ -15808,8 +15815,8 @@
       <c r="C78" s="25" t="s">
         <v>24</v>
       </c>
-      <c r="D78" s="33" t="s">
-        <v>123</v>
+      <c r="D78" s="32" t="s">
+        <v>126</v>
       </c>
       <c r="E78" s="25" t="s">
         <v>117</v>
@@ -15818,10 +15825,10 @@
         <v>129</v>
       </c>
       <c r="G78" s="25" t="s">
-        <v>130</v>
-      </c>
-    </row>
-    <row r="79" spans="1:11" s="25" customFormat="1" x14ac:dyDescent="0.2">
+        <v>133</v>
+      </c>
+    </row>
+    <row r="79" spans="1:10" s="25" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A79" s="25" t="b">
         <v>1</v>
       </c>
@@ -15831,8 +15838,8 @@
       <c r="C79" s="25" t="s">
         <v>24</v>
       </c>
-      <c r="D79" s="33" t="s">
-        <v>124</v>
+      <c r="D79" s="32" t="s">
+        <v>127</v>
       </c>
       <c r="E79" s="25" t="s">
         <v>117</v>
@@ -15841,10 +15848,10 @@
         <v>129</v>
       </c>
       <c r="G79" s="25" t="s">
-        <v>131</v>
-      </c>
-    </row>
-    <row r="80" spans="1:11" s="25" customFormat="1" x14ac:dyDescent="0.2">
+        <v>127</v>
+      </c>
+    </row>
+    <row r="80" spans="1:10" s="25" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A80" s="25" t="b">
         <v>1</v>
       </c>
@@ -15854,8 +15861,8 @@
       <c r="C80" s="25" t="s">
         <v>24</v>
       </c>
-      <c r="D80" s="33" t="s">
-        <v>125</v>
+      <c r="D80" s="32" t="s">
+        <v>128</v>
       </c>
       <c r="E80" s="25" t="s">
         <v>117</v>
@@ -15864,31 +15871,11 @@
         <v>129</v>
       </c>
       <c r="G80" s="25" t="s">
-        <v>132</v>
+        <v>135</v>
       </c>
     </row>
     <row r="81" spans="1:10" s="25" customFormat="1" x14ac:dyDescent="0.2">
-      <c r="A81" s="25" t="b">
-        <v>1</v>
-      </c>
-      <c r="B81" s="25" t="s">
-        <v>630</v>
-      </c>
-      <c r="C81" s="25" t="s">
-        <v>24</v>
-      </c>
-      <c r="D81" s="33" t="s">
-        <v>126</v>
-      </c>
-      <c r="E81" s="25" t="s">
-        <v>117</v>
-      </c>
-      <c r="F81" s="25" t="s">
-        <v>129</v>
-      </c>
-      <c r="G81" s="25" t="s">
-        <v>133</v>
-      </c>
+      <c r="D81" s="32"/>
     </row>
     <row r="82" spans="1:10" s="25" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A82" s="25" t="b">
@@ -15898,19 +15885,16 @@
         <v>630</v>
       </c>
       <c r="C82" s="25" t="s">
-        <v>24</v>
-      </c>
-      <c r="D82" s="33" t="s">
-        <v>127</v>
-      </c>
-      <c r="E82" s="25" t="s">
-        <v>117</v>
-      </c>
-      <c r="F82" s="25" t="s">
-        <v>129</v>
-      </c>
-      <c r="G82" s="25" t="s">
-        <v>127</v>
+        <v>9</v>
+      </c>
+      <c r="E82" s="41" t="s">
+        <v>76</v>
+      </c>
+      <c r="F82" s="41" t="s">
+        <v>120</v>
+      </c>
+      <c r="H82" s="30" t="s">
+        <v>722</v>
       </c>
     </row>
     <row r="83" spans="1:10" s="25" customFormat="1" x14ac:dyDescent="0.2">
@@ -15921,23 +15905,37 @@
         <v>630</v>
       </c>
       <c r="C83" s="25" t="s">
-        <v>24</v>
-      </c>
-      <c r="D83" s="33" t="s">
-        <v>128</v>
+        <v>11</v>
       </c>
       <c r="E83" s="25" t="s">
-        <v>117</v>
+        <v>76</v>
       </c>
       <c r="F83" s="25" t="s">
-        <v>129</v>
+        <v>80</v>
       </c>
       <c r="G83" s="25" t="s">
-        <v>135</v>
+        <v>696</v>
       </c>
     </row>
     <row r="84" spans="1:10" s="25" customFormat="1" x14ac:dyDescent="0.2">
-      <c r="D84" s="33"/>
+      <c r="A84" s="25" t="b">
+        <v>1</v>
+      </c>
+      <c r="B84" s="25" t="s">
+        <v>630</v>
+      </c>
+      <c r="C84" s="25" t="s">
+        <v>8</v>
+      </c>
+      <c r="E84" s="25" t="s">
+        <v>76</v>
+      </c>
+      <c r="F84" s="25" t="s">
+        <v>77</v>
+      </c>
+      <c r="G84" s="25" t="s">
+        <v>694</v>
+      </c>
     </row>
     <row r="85" spans="1:10" s="25" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A85" s="25" t="b">
@@ -15947,16 +15945,16 @@
         <v>630</v>
       </c>
       <c r="C85" s="25" t="s">
-        <v>9</v>
-      </c>
-      <c r="E85" s="42" t="s">
+        <v>54</v>
+      </c>
+      <c r="E85" s="25" t="s">
         <v>76</v>
       </c>
-      <c r="F85" s="42" t="s">
-        <v>120</v>
-      </c>
-      <c r="H85" s="31" t="s">
-        <v>722</v>
+      <c r="F85" s="25" t="s">
+        <v>712</v>
+      </c>
+      <c r="G85" s="25" t="s">
+        <v>701</v>
       </c>
     </row>
     <row r="86" spans="1:10" s="25" customFormat="1" x14ac:dyDescent="0.2">
@@ -15967,19 +15965,19 @@
         <v>630</v>
       </c>
       <c r="C86" s="25" t="s">
-        <v>11</v>
+        <v>18</v>
       </c>
       <c r="E86" s="25" t="s">
         <v>76</v>
       </c>
       <c r="F86" s="25" t="s">
-        <v>80</v>
+        <v>115</v>
       </c>
       <c r="G86" s="25" t="s">
-        <v>696</v>
-      </c>
-    </row>
-    <row r="87" spans="1:10" s="25" customFormat="1" x14ac:dyDescent="0.2">
+        <v>697</v>
+      </c>
+    </row>
+    <row r="87" spans="1:10" s="25" customFormat="1" ht="17" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A87" s="25" t="b">
         <v>1</v>
       </c>
@@ -15987,16 +15985,17 @@
         <v>630</v>
       </c>
       <c r="C87" s="25" t="s">
-        <v>8</v>
-      </c>
+        <v>13</v>
+      </c>
+      <c r="D87" s="32"/>
       <c r="E87" s="25" t="s">
         <v>76</v>
       </c>
       <c r="F87" s="25" t="s">
-        <v>77</v>
-      </c>
-      <c r="G87" s="25" t="s">
-        <v>694</v>
+        <v>83</v>
+      </c>
+      <c r="H87" s="42" t="s">
+        <v>862</v>
       </c>
     </row>
     <row r="88" spans="1:10" s="25" customFormat="1" x14ac:dyDescent="0.2">
@@ -16007,19 +16006,19 @@
         <v>630</v>
       </c>
       <c r="C88" s="25" t="s">
-        <v>54</v>
+        <v>772</v>
       </c>
       <c r="E88" s="25" t="s">
         <v>76</v>
       </c>
       <c r="F88" s="25" t="s">
-        <v>712</v>
+        <v>725</v>
       </c>
       <c r="G88" s="25" t="s">
-        <v>701</v>
-      </c>
-    </row>
-    <row r="89" spans="1:10" s="25" customFormat="1" x14ac:dyDescent="0.2">
+        <v>875</v>
+      </c>
+    </row>
+    <row r="89" spans="1:10" s="17" customFormat="1" ht="17" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A89" s="25" t="b">
         <v>1</v>
       </c>
@@ -16027,19 +16026,25 @@
         <v>630</v>
       </c>
       <c r="C89" s="25" t="s">
-        <v>18</v>
+        <v>15</v>
+      </c>
+      <c r="D89" s="33" t="s">
+        <v>84</v>
       </c>
       <c r="E89" s="25" t="s">
         <v>76</v>
       </c>
       <c r="F89" s="25" t="s">
-        <v>115</v>
+        <v>100</v>
       </c>
       <c r="G89" s="25" t="s">
-        <v>697</v>
-      </c>
-    </row>
-    <row r="90" spans="1:10" s="25" customFormat="1" ht="17" customHeight="1" x14ac:dyDescent="0.2">
+        <v>75</v>
+      </c>
+      <c r="H89" s="25"/>
+      <c r="I89" s="25"/>
+      <c r="J89" s="25"/>
+    </row>
+    <row r="90" spans="1:10" s="25" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A90" s="25" t="b">
         <v>1</v>
       </c>
@@ -16047,17 +16052,19 @@
         <v>630</v>
       </c>
       <c r="C90" s="25" t="s">
-        <v>13</v>
-      </c>
-      <c r="D90" s="33"/>
+        <v>15</v>
+      </c>
+      <c r="D90" s="33" t="s">
+        <v>85</v>
+      </c>
       <c r="E90" s="25" t="s">
         <v>76</v>
       </c>
       <c r="F90" s="25" t="s">
-        <v>83</v>
-      </c>
-      <c r="H90" s="43" t="s">
-        <v>863</v>
+        <v>100</v>
+      </c>
+      <c r="G90" s="25" t="s">
+        <v>101</v>
       </c>
     </row>
     <row r="91" spans="1:10" s="25" customFormat="1" x14ac:dyDescent="0.2">
@@ -16068,19 +16075,22 @@
         <v>630</v>
       </c>
       <c r="C91" s="25" t="s">
-        <v>772</v>
+        <v>15</v>
+      </c>
+      <c r="D91" s="34" t="s">
+        <v>86</v>
       </c>
       <c r="E91" s="25" t="s">
         <v>76</v>
       </c>
       <c r="F91" s="25" t="s">
-        <v>725</v>
+        <v>100</v>
       </c>
       <c r="G91" s="25" t="s">
-        <v>876</v>
-      </c>
-    </row>
-    <row r="92" spans="1:10" s="17" customFormat="1" ht="17" customHeight="1" x14ac:dyDescent="0.2">
+        <v>102</v>
+      </c>
+    </row>
+    <row r="92" spans="1:10" s="25" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A92" s="25" t="b">
         <v>1</v>
       </c>
@@ -16091,7 +16101,7 @@
         <v>15</v>
       </c>
       <c r="D92" s="34" t="s">
-        <v>84</v>
+        <v>87</v>
       </c>
       <c r="E92" s="25" t="s">
         <v>76</v>
@@ -16100,11 +16110,8 @@
         <v>100</v>
       </c>
       <c r="G92" s="25" t="s">
-        <v>75</v>
-      </c>
-      <c r="H92" s="25"/>
-      <c r="I92" s="25"/>
-      <c r="J92" s="25"/>
+        <v>103</v>
+      </c>
     </row>
     <row r="93" spans="1:10" s="25" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A93" s="25" t="b">
@@ -16117,7 +16124,7 @@
         <v>15</v>
       </c>
       <c r="D93" s="34" t="s">
-        <v>85</v>
+        <v>88</v>
       </c>
       <c r="E93" s="25" t="s">
         <v>76</v>
@@ -16126,7 +16133,7 @@
         <v>100</v>
       </c>
       <c r="G93" s="25" t="s">
-        <v>101</v>
+        <v>104</v>
       </c>
     </row>
     <row r="94" spans="1:10" s="25" customFormat="1" x14ac:dyDescent="0.2">
@@ -16139,8 +16146,8 @@
       <c r="C94" s="25" t="s">
         <v>15</v>
       </c>
-      <c r="D94" s="35" t="s">
-        <v>86</v>
+      <c r="D94" s="32" t="s">
+        <v>89</v>
       </c>
       <c r="E94" s="25" t="s">
         <v>76</v>
@@ -16149,7 +16156,7 @@
         <v>100</v>
       </c>
       <c r="G94" s="25" t="s">
-        <v>102</v>
+        <v>113</v>
       </c>
     </row>
     <row r="95" spans="1:10" s="25" customFormat="1" x14ac:dyDescent="0.2">
@@ -16162,8 +16169,8 @@
       <c r="C95" s="25" t="s">
         <v>15</v>
       </c>
-      <c r="D95" s="35" t="s">
-        <v>87</v>
+      <c r="D95" s="32" t="s">
+        <v>90</v>
       </c>
       <c r="E95" s="25" t="s">
         <v>76</v>
@@ -16172,7 +16179,7 @@
         <v>100</v>
       </c>
       <c r="G95" s="25" t="s">
-        <v>103</v>
+        <v>112</v>
       </c>
     </row>
     <row r="96" spans="1:10" s="25" customFormat="1" x14ac:dyDescent="0.2">
@@ -16185,8 +16192,8 @@
       <c r="C96" s="25" t="s">
         <v>15</v>
       </c>
-      <c r="D96" s="35" t="s">
-        <v>88</v>
+      <c r="D96" s="33" t="s">
+        <v>91</v>
       </c>
       <c r="E96" s="25" t="s">
         <v>76</v>
@@ -16195,7 +16202,7 @@
         <v>100</v>
       </c>
       <c r="G96" s="25" t="s">
-        <v>104</v>
+        <v>109</v>
       </c>
     </row>
     <row r="97" spans="1:11" s="25" customFormat="1" x14ac:dyDescent="0.2">
@@ -16209,7 +16216,7 @@
         <v>15</v>
       </c>
       <c r="D97" s="33" t="s">
-        <v>89</v>
+        <v>92</v>
       </c>
       <c r="E97" s="25" t="s">
         <v>76</v>
@@ -16218,7 +16225,7 @@
         <v>100</v>
       </c>
       <c r="G97" s="25" t="s">
-        <v>113</v>
+        <v>108</v>
       </c>
     </row>
     <row r="98" spans="1:11" s="25" customFormat="1" x14ac:dyDescent="0.2">
@@ -16231,8 +16238,8 @@
       <c r="C98" s="25" t="s">
         <v>15</v>
       </c>
-      <c r="D98" s="33" t="s">
-        <v>90</v>
+      <c r="D98" s="32" t="s">
+        <v>93</v>
       </c>
       <c r="E98" s="25" t="s">
         <v>76</v>
@@ -16241,7 +16248,7 @@
         <v>100</v>
       </c>
       <c r="G98" s="25" t="s">
-        <v>112</v>
+        <v>107</v>
       </c>
     </row>
     <row r="99" spans="1:11" s="25" customFormat="1" x14ac:dyDescent="0.2">
@@ -16254,8 +16261,8 @@
       <c r="C99" s="25" t="s">
         <v>15</v>
       </c>
-      <c r="D99" s="34" t="s">
-        <v>91</v>
+      <c r="D99" s="32" t="s">
+        <v>94</v>
       </c>
       <c r="E99" s="25" t="s">
         <v>76</v>
@@ -16264,7 +16271,7 @@
         <v>100</v>
       </c>
       <c r="G99" s="25" t="s">
-        <v>109</v>
+        <v>106</v>
       </c>
     </row>
     <row r="100" spans="1:11" s="25" customFormat="1" x14ac:dyDescent="0.2">
@@ -16277,8 +16284,8 @@
       <c r="C100" s="25" t="s">
         <v>15</v>
       </c>
-      <c r="D100" s="34" t="s">
-        <v>92</v>
+      <c r="D100" s="32" t="s">
+        <v>95</v>
       </c>
       <c r="E100" s="25" t="s">
         <v>76</v>
@@ -16287,7 +16294,7 @@
         <v>100</v>
       </c>
       <c r="G100" s="25" t="s">
-        <v>108</v>
+        <v>105</v>
       </c>
     </row>
     <row r="101" spans="1:11" s="25" customFormat="1" x14ac:dyDescent="0.2">
@@ -16300,8 +16307,8 @@
       <c r="C101" s="25" t="s">
         <v>15</v>
       </c>
-      <c r="D101" s="33" t="s">
-        <v>93</v>
+      <c r="D101" s="32" t="s">
+        <v>96</v>
       </c>
       <c r="E101" s="25" t="s">
         <v>76</v>
@@ -16310,7 +16317,7 @@
         <v>100</v>
       </c>
       <c r="G101" s="25" t="s">
-        <v>107</v>
+        <v>110</v>
       </c>
     </row>
     <row r="102" spans="1:11" s="25" customFormat="1" x14ac:dyDescent="0.2">
@@ -16323,8 +16330,8 @@
       <c r="C102" s="25" t="s">
         <v>15</v>
       </c>
-      <c r="D102" s="33" t="s">
-        <v>94</v>
+      <c r="D102" s="32" t="s">
+        <v>97</v>
       </c>
       <c r="E102" s="25" t="s">
         <v>76</v>
@@ -16333,7 +16340,7 @@
         <v>100</v>
       </c>
       <c r="G102" s="25" t="s">
-        <v>106</v>
+        <v>97</v>
       </c>
     </row>
     <row r="103" spans="1:11" s="25" customFormat="1" x14ac:dyDescent="0.2">
@@ -16346,8 +16353,8 @@
       <c r="C103" s="25" t="s">
         <v>15</v>
       </c>
-      <c r="D103" s="33" t="s">
-        <v>95</v>
+      <c r="D103" s="32" t="s">
+        <v>98</v>
       </c>
       <c r="E103" s="25" t="s">
         <v>76</v>
@@ -16356,7 +16363,7 @@
         <v>100</v>
       </c>
       <c r="G103" s="25" t="s">
-        <v>105</v>
+        <v>111</v>
       </c>
     </row>
     <row r="104" spans="1:11" s="25" customFormat="1" x14ac:dyDescent="0.2">
@@ -16369,8 +16376,8 @@
       <c r="C104" s="25" t="s">
         <v>15</v>
       </c>
-      <c r="D104" s="33" t="s">
-        <v>96</v>
+      <c r="D104" s="32" t="s">
+        <v>99</v>
       </c>
       <c r="E104" s="25" t="s">
         <v>76</v>
@@ -16378,81 +16385,12 @@
       <c r="F104" s="25" t="s">
         <v>100</v>
       </c>
-      <c r="G104" s="25" t="s">
-        <v>110</v>
-      </c>
-    </row>
-    <row r="105" spans="1:11" s="25" customFormat="1" x14ac:dyDescent="0.2">
-      <c r="A105" s="25" t="b">
-        <v>1</v>
-      </c>
-      <c r="B105" s="25" t="s">
-        <v>630</v>
-      </c>
-      <c r="C105" s="25" t="s">
-        <v>15</v>
-      </c>
-      <c r="D105" s="33" t="s">
-        <v>97</v>
-      </c>
-      <c r="E105" s="25" t="s">
-        <v>76</v>
-      </c>
-      <c r="F105" s="25" t="s">
-        <v>100</v>
-      </c>
-      <c r="G105" s="25" t="s">
-        <v>97</v>
-      </c>
-    </row>
-    <row r="106" spans="1:11" s="25" customFormat="1" x14ac:dyDescent="0.2">
-      <c r="A106" s="25" t="b">
-        <v>1</v>
-      </c>
-      <c r="B106" s="25" t="s">
-        <v>630</v>
-      </c>
-      <c r="C106" s="25" t="s">
-        <v>15</v>
-      </c>
-      <c r="D106" s="33" t="s">
-        <v>98</v>
-      </c>
-      <c r="E106" s="25" t="s">
-        <v>76</v>
-      </c>
-      <c r="F106" s="25" t="s">
-        <v>100</v>
-      </c>
-      <c r="G106" s="25" t="s">
-        <v>111</v>
-      </c>
-    </row>
-    <row r="107" spans="1:11" s="25" customFormat="1" x14ac:dyDescent="0.2">
-      <c r="A107" s="25" t="b">
-        <v>1</v>
-      </c>
-      <c r="B107" s="25" t="s">
-        <v>630</v>
-      </c>
-      <c r="C107" s="25" t="s">
-        <v>15</v>
-      </c>
-      <c r="D107" s="33" t="s">
-        <v>99</v>
-      </c>
-      <c r="E107" s="25" t="s">
-        <v>76</v>
-      </c>
-      <c r="F107" s="25" t="s">
-        <v>100</v>
-      </c>
-      <c r="G107" s="42" t="s">
+      <c r="G104" s="41" t="s">
         <v>530</v>
       </c>
-      <c r="H107" s="30"/>
-      <c r="I107" s="30"/>
-      <c r="K107" s="42"/>
+      <c r="H104" s="29"/>
+      <c r="I104" s="29"/>
+      <c r="K104" s="41"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -16483,62 +16421,62 @@
     <col min="19" max="19" width="27.6640625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:19" s="40" customFormat="1" ht="19" x14ac:dyDescent="0.25">
-      <c r="A1" s="40" t="s">
+    <row r="1" spans="1:19" s="39" customFormat="1" ht="19" x14ac:dyDescent="0.25">
+      <c r="A1" s="39" t="s">
         <v>666</v>
       </c>
-      <c r="B1" s="40" t="s">
+      <c r="B1" s="39" t="s">
         <v>629</v>
       </c>
-      <c r="C1" s="40" t="s">
+      <c r="C1" s="39" t="s">
         <v>631</v>
       </c>
-      <c r="D1" s="40" t="s">
+      <c r="D1" s="39" t="s">
         <v>632</v>
       </c>
-      <c r="E1" s="40" t="s">
+      <c r="E1" s="39" t="s">
         <v>633</v>
       </c>
-      <c r="F1" s="40" t="s">
+      <c r="F1" s="39" t="s">
         <v>635</v>
       </c>
-      <c r="G1" s="40" t="s">
+      <c r="G1" s="39" t="s">
         <v>682</v>
       </c>
-      <c r="H1" s="40" t="s">
-        <v>808</v>
-      </c>
-      <c r="I1" s="40" t="s">
+      <c r="H1" s="39" t="s">
+        <v>807</v>
+      </c>
+      <c r="I1" s="39" t="s">
+        <v>864</v>
+      </c>
+      <c r="J1" s="40" t="s">
+        <v>799</v>
+      </c>
+      <c r="K1" s="40" t="s">
+        <v>800</v>
+      </c>
+      <c r="L1" s="40" t="s">
+        <v>802</v>
+      </c>
+      <c r="M1" s="40" t="s">
+        <v>847</v>
+      </c>
+      <c r="N1" s="40" t="s">
+        <v>803</v>
+      </c>
+      <c r="O1" s="40" t="s">
+        <v>804</v>
+      </c>
+      <c r="P1" s="39" t="s">
         <v>865</v>
       </c>
-      <c r="J1" s="41" t="s">
-        <v>800</v>
-      </c>
-      <c r="K1" s="41" t="s">
-        <v>801</v>
-      </c>
-      <c r="L1" s="41" t="s">
-        <v>803</v>
-      </c>
-      <c r="M1" s="41" t="s">
+      <c r="Q1" s="39" t="s">
+        <v>858</v>
+      </c>
+      <c r="R1" s="39" t="s">
         <v>848</v>
       </c>
-      <c r="N1" s="41" t="s">
-        <v>804</v>
-      </c>
-      <c r="O1" s="41" t="s">
-        <v>805</v>
-      </c>
-      <c r="P1" s="40" t="s">
-        <v>866</v>
-      </c>
-      <c r="Q1" s="40" t="s">
-        <v>859</v>
-      </c>
-      <c r="R1" s="40" t="s">
-        <v>849</v>
-      </c>
-      <c r="S1" s="41" t="s">
+      <c r="S1" s="40" t="s">
         <v>120</v>
       </c>
     </row>
@@ -16560,7 +16498,7 @@
       </c>
       <c r="G2"/>
       <c r="H2" s="25" t="s">
-        <v>809</v>
+        <v>808</v>
       </c>
       <c r="J2" s="25" t="s">
         <v>155</v>
@@ -16569,7 +16507,7 @@
         <v>160</v>
       </c>
       <c r="M2" s="25" t="s">
-        <v>889</v>
+        <v>888</v>
       </c>
       <c r="N2" s="25" t="s">
         <v>161</v>
@@ -16596,7 +16534,7 @@
       </c>
       <c r="G3"/>
       <c r="H3" s="25" t="s">
-        <v>810</v>
+        <v>809</v>
       </c>
       <c r="J3" s="25" t="s">
         <v>164</v>
@@ -16632,7 +16570,7 @@
       </c>
       <c r="G4"/>
       <c r="H4" s="25" t="s">
-        <v>811</v>
+        <v>810</v>
       </c>
       <c r="J4" s="25" t="s">
         <v>164</v>
@@ -16668,7 +16606,7 @@
       </c>
       <c r="G5"/>
       <c r="H5" s="25" t="s">
-        <v>812</v>
+        <v>811</v>
       </c>
       <c r="J5" s="25" t="s">
         <v>164</v>
@@ -16704,7 +16642,7 @@
       </c>
       <c r="G6"/>
       <c r="H6" s="25" t="s">
-        <v>813</v>
+        <v>812</v>
       </c>
       <c r="J6" s="25" t="s">
         <v>164</v>
@@ -16740,7 +16678,7 @@
       </c>
       <c r="G7"/>
       <c r="H7" s="25" t="s">
-        <v>814</v>
+        <v>813</v>
       </c>
       <c r="J7" s="25" t="s">
         <v>164</v>
@@ -16752,7 +16690,7 @@
         <v>661</v>
       </c>
       <c r="N7" s="25" t="s">
-        <v>870</v>
+        <v>869</v>
       </c>
       <c r="O7" s="25" t="s">
         <v>154</v>
@@ -16776,7 +16714,7 @@
       </c>
       <c r="G8"/>
       <c r="H8" s="25" t="s">
-        <v>815</v>
+        <v>814</v>
       </c>
       <c r="J8" s="25" t="s">
         <v>155</v>
@@ -16785,7 +16723,7 @@
         <v>170</v>
       </c>
       <c r="M8" s="25" t="s">
-        <v>888</v>
+        <v>887</v>
       </c>
       <c r="N8" s="25" t="s">
         <v>161</v>
@@ -16812,7 +16750,7 @@
       </c>
       <c r="G9"/>
       <c r="H9" s="25" t="s">
-        <v>816</v>
+        <v>815</v>
       </c>
       <c r="J9" s="25" t="s">
         <v>164</v>
@@ -16830,7 +16768,7 @@
         <v>158</v>
       </c>
       <c r="P9" s="25" t="s">
-        <v>854</v>
+        <v>853</v>
       </c>
     </row>
     <row r="10" spans="1:19" s="25" customFormat="1" x14ac:dyDescent="0.2">
@@ -16851,7 +16789,7 @@
       </c>
       <c r="G10"/>
       <c r="H10" s="25" t="s">
-        <v>817</v>
+        <v>816</v>
       </c>
       <c r="J10" s="25" t="s">
         <v>164</v>
@@ -16869,7 +16807,7 @@
         <v>158</v>
       </c>
       <c r="P10" s="25" t="s">
-        <v>855</v>
+        <v>854</v>
       </c>
     </row>
     <row r="11" spans="1:19" s="25" customFormat="1" x14ac:dyDescent="0.2">
@@ -16890,7 +16828,7 @@
       </c>
       <c r="G11"/>
       <c r="H11" s="25" t="s">
-        <v>818</v>
+        <v>817</v>
       </c>
       <c r="J11" s="25" t="s">
         <v>155</v>
@@ -16899,7 +16837,7 @@
         <v>162</v>
       </c>
       <c r="M11" s="25" t="s">
-        <v>887</v>
+        <v>886</v>
       </c>
       <c r="N11" s="25" t="s">
         <v>163</v>
@@ -16930,7 +16868,7 @@
       </c>
       <c r="G12"/>
       <c r="H12" s="25" t="s">
-        <v>819</v>
+        <v>818</v>
       </c>
       <c r="J12" s="25" t="s">
         <v>155</v>
@@ -16981,7 +16919,7 @@
         <v>114</v>
       </c>
       <c r="F14" s="25" t="s">
-        <v>885</v>
+        <v>884</v>
       </c>
       <c r="G14"/>
     </row>
@@ -17003,7 +16941,7 @@
       </c>
       <c r="G15"/>
       <c r="H15" s="25" t="s">
-        <v>820</v>
+        <v>819</v>
       </c>
       <c r="J15" s="25" t="s">
         <v>164</v>
@@ -17021,7 +16959,7 @@
         <v>158</v>
       </c>
       <c r="P15" s="25" t="s">
-        <v>856</v>
+        <v>855</v>
       </c>
     </row>
     <row r="16" spans="1:19" s="25" customFormat="1" x14ac:dyDescent="0.2">
@@ -17042,10 +16980,10 @@
       </c>
       <c r="G16"/>
       <c r="H16" s="25" t="s">
-        <v>821</v>
+        <v>820</v>
       </c>
       <c r="I16" s="25" t="s">
-        <v>853</v>
+        <v>852</v>
       </c>
       <c r="J16" s="25" t="s">
         <v>164</v>
@@ -17063,7 +17001,7 @@
         <v>158</v>
       </c>
       <c r="P16" s="25" t="s">
-        <v>857</v>
+        <v>856</v>
       </c>
     </row>
     <row r="17" spans="1:18" s="25" customFormat="1" x14ac:dyDescent="0.2">
@@ -17084,7 +17022,7 @@
       </c>
       <c r="G17"/>
       <c r="H17" s="25" t="s">
-        <v>852</v>
+        <v>851</v>
       </c>
       <c r="J17" s="25" t="s">
         <v>164</v>
@@ -17093,7 +17031,7 @@
         <v>637</v>
       </c>
       <c r="M17" s="25" t="s">
-        <v>919</v>
+        <v>918</v>
       </c>
       <c r="N17" t="s">
         <v>641</v>
@@ -17102,10 +17040,10 @@
         <v>158</v>
       </c>
       <c r="P17" s="25" t="s">
-        <v>858</v>
+        <v>857</v>
       </c>
       <c r="Q17" s="25" t="s">
-        <v>860</v>
+        <v>859</v>
       </c>
     </row>
     <row r="18" spans="1:18" s="25" customFormat="1" x14ac:dyDescent="0.2">
@@ -17126,7 +17064,7 @@
       </c>
       <c r="G18"/>
       <c r="H18" s="25" t="s">
-        <v>822</v>
+        <v>821</v>
       </c>
       <c r="J18" s="25" t="s">
         <v>164</v>
@@ -17135,7 +17073,7 @@
         <v>637</v>
       </c>
       <c r="M18" s="25" t="s">
-        <v>922</v>
+        <v>921</v>
       </c>
       <c r="N18" s="25" t="s">
         <v>641</v>
@@ -17144,7 +17082,7 @@
         <v>590</v>
       </c>
       <c r="P18" s="25" t="s">
-        <v>858</v>
+        <v>857</v>
       </c>
     </row>
     <row r="19" spans="1:18" s="25" customFormat="1" x14ac:dyDescent="0.2">
@@ -17165,7 +17103,7 @@
       </c>
       <c r="G19"/>
       <c r="H19" s="25" t="s">
-        <v>823</v>
+        <v>822</v>
       </c>
       <c r="J19" s="25" t="s">
         <v>164</v>
@@ -17174,7 +17112,7 @@
         <v>637</v>
       </c>
       <c r="M19" s="25" t="s">
-        <v>921</v>
+        <v>920</v>
       </c>
       <c r="N19" s="25" t="s">
         <v>641</v>
@@ -17183,7 +17121,7 @@
         <v>591</v>
       </c>
       <c r="P19" s="25" t="s">
-        <v>858</v>
+        <v>857</v>
       </c>
     </row>
     <row r="20" spans="1:18" s="25" customFormat="1" x14ac:dyDescent="0.2">
@@ -17204,7 +17142,7 @@
       </c>
       <c r="G20"/>
       <c r="H20" s="25" t="s">
-        <v>824</v>
+        <v>823</v>
       </c>
       <c r="J20" s="25" t="s">
         <v>164</v>
@@ -17213,7 +17151,7 @@
         <v>637</v>
       </c>
       <c r="M20" s="25" t="s">
-        <v>920</v>
+        <v>919</v>
       </c>
       <c r="N20" s="25" t="s">
         <v>641</v>
@@ -17222,7 +17160,7 @@
         <v>589</v>
       </c>
       <c r="P20" s="25" t="s">
-        <v>858</v>
+        <v>857</v>
       </c>
     </row>
     <row r="21" spans="1:18" s="25" customFormat="1" x14ac:dyDescent="0.2">
@@ -17243,7 +17181,7 @@
       </c>
       <c r="G21"/>
       <c r="H21" s="25" t="s">
-        <v>825</v>
+        <v>824</v>
       </c>
       <c r="J21" s="25" t="s">
         <v>164</v>
@@ -17279,7 +17217,7 @@
       </c>
       <c r="G22"/>
       <c r="H22" s="25" t="s">
-        <v>826</v>
+        <v>825</v>
       </c>
       <c r="J22" s="25" t="s">
         <v>164</v>
@@ -17291,7 +17229,7 @@
         <v>636</v>
       </c>
       <c r="R22" s="25" t="s">
-        <v>861</v>
+        <v>860</v>
       </c>
     </row>
     <row r="23" spans="1:18" s="25" customFormat="1" x14ac:dyDescent="0.2">
@@ -17312,7 +17250,7 @@
       </c>
       <c r="G23"/>
       <c r="H23" s="25" t="s">
-        <v>827</v>
+        <v>826</v>
       </c>
       <c r="J23" s="25" t="s">
         <v>164</v>
@@ -17321,7 +17259,7 @@
         <v>596</v>
       </c>
       <c r="M23" s="25" t="s">
-        <v>918</v>
+        <v>917</v>
       </c>
       <c r="N23" s="25" t="s">
         <v>163</v>
@@ -17348,7 +17286,7 @@
       </c>
       <c r="G24"/>
       <c r="H24" s="25" t="s">
-        <v>828</v>
+        <v>827</v>
       </c>
       <c r="J24" s="25" t="s">
         <v>164</v>
@@ -17384,22 +17322,22 @@
       </c>
       <c r="G25"/>
       <c r="H25" s="25" t="s">
-        <v>829</v>
-      </c>
-      <c r="J25" s="29" t="s">
+        <v>828</v>
+      </c>
+      <c r="J25" s="28" t="s">
         <v>155</v>
       </c>
-      <c r="K25" s="29" t="s">
+      <c r="K25" s="28" t="s">
         <v>159</v>
       </c>
-      <c r="L25" s="29"/>
-      <c r="M25" s="29" t="s">
-        <v>886</v>
-      </c>
-      <c r="N25" s="29" t="s">
+      <c r="L25" s="28"/>
+      <c r="M25" s="28" t="s">
+        <v>885</v>
+      </c>
+      <c r="N25" s="28" t="s">
         <v>157</v>
       </c>
-      <c r="O25" s="29" t="s">
+      <c r="O25" s="28" t="s">
         <v>158</v>
       </c>
     </row>
@@ -17421,7 +17359,7 @@
       </c>
       <c r="G26"/>
       <c r="H26" s="25" t="s">
-        <v>830</v>
+        <v>829</v>
       </c>
       <c r="J26" s="25" t="s">
         <v>164</v>
@@ -17471,44 +17409,44 @@
     <col min="12" max="12" width="35.1640625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:13" s="40" customFormat="1" ht="19" x14ac:dyDescent="0.25">
-      <c r="A1" s="40" t="s">
+    <row r="1" spans="1:13" s="39" customFormat="1" ht="19" x14ac:dyDescent="0.25">
+      <c r="A1" s="39" t="s">
         <v>666</v>
       </c>
-      <c r="B1" s="40" t="s">
+      <c r="B1" s="39" t="s">
         <v>629</v>
       </c>
-      <c r="C1" s="40" t="s">
+      <c r="C1" s="39" t="s">
         <v>631</v>
       </c>
-      <c r="D1" s="40" t="s">
+      <c r="D1" s="39" t="s">
         <v>632</v>
       </c>
-      <c r="E1" s="40" t="s">
+      <c r="E1" s="39" t="s">
         <v>633</v>
       </c>
-      <c r="F1" s="40" t="s">
+      <c r="F1" s="39" t="s">
         <v>635</v>
       </c>
-      <c r="G1" s="40" t="s">
+      <c r="G1" s="39" t="s">
         <v>682</v>
       </c>
-      <c r="H1" s="40" t="s">
-        <v>808</v>
-      </c>
-      <c r="I1" s="40" t="s">
+      <c r="H1" s="39" t="s">
+        <v>807</v>
+      </c>
+      <c r="I1" s="39" t="s">
+        <v>797</v>
+      </c>
+      <c r="J1" s="40" t="s">
         <v>798</v>
       </c>
-      <c r="J1" s="41" t="s">
-        <v>799</v>
-      </c>
-      <c r="K1" s="41" t="s">
-        <v>797</v>
-      </c>
-      <c r="L1" s="41" t="s">
-        <v>851</v>
-      </c>
-      <c r="M1" s="41" t="s">
+      <c r="K1" s="40" t="s">
+        <v>796</v>
+      </c>
+      <c r="L1" s="40" t="s">
+        <v>850</v>
+      </c>
+      <c r="M1" s="40" t="s">
         <v>120</v>
       </c>
     </row>
@@ -17526,21 +17464,21 @@
         <v>146</v>
       </c>
       <c r="H2" s="25" t="s">
-        <v>852</v>
+        <v>851</v>
       </c>
       <c r="I2" t="s">
         <v>787</v>
       </c>
-      <c r="K2" s="36" t="s">
-        <v>864</v>
-      </c>
-      <c r="L2" s="36" t="s">
-        <v>850</v>
+      <c r="K2" s="35" t="s">
+        <v>863</v>
+      </c>
+      <c r="L2" s="35" t="s">
+        <v>849</v>
       </c>
     </row>
     <row r="3" spans="1:13" ht="19" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="K3" s="36"/>
-      <c r="L3" s="36"/>
+      <c r="K3" s="35"/>
+      <c r="L3" s="35"/>
     </row>
     <row r="4" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A4" t="b">
@@ -17562,7 +17500,7 @@
         <v>597</v>
       </c>
       <c r="H4" s="25" t="s">
-        <v>852</v>
+        <v>851</v>
       </c>
       <c r="I4" t="s">
         <v>788</v>
@@ -17588,7 +17526,7 @@
         <v>146</v>
       </c>
       <c r="F5" t="s">
-        <v>831</v>
+        <v>830</v>
       </c>
     </row>
     <row r="7" spans="1:13" x14ac:dyDescent="0.2">
@@ -17611,7 +17549,7 @@
         <v>592</v>
       </c>
       <c r="H7" s="25" t="s">
-        <v>852</v>
+        <v>851</v>
       </c>
       <c r="I7" t="s">
         <v>790</v>
@@ -17637,7 +17575,7 @@
         <v>146</v>
       </c>
       <c r="F8" t="s">
-        <v>831</v>
+        <v>830</v>
       </c>
     </row>
     <row r="9" spans="1:13" x14ac:dyDescent="0.2">
@@ -17657,7 +17595,7 @@
         <v>146</v>
       </c>
       <c r="F9" t="s">
-        <v>831</v>
+        <v>830</v>
       </c>
     </row>
     <row r="11" spans="1:13" x14ac:dyDescent="0.2">
@@ -17680,7 +17618,7 @@
         <v>148</v>
       </c>
       <c r="H11" s="25" t="s">
-        <v>852</v>
+        <v>851</v>
       </c>
       <c r="I11" t="s">
         <v>792</v>
@@ -17749,7 +17687,7 @@
         <v>148</v>
       </c>
       <c r="H15" s="25" t="s">
-        <v>852</v>
+        <v>851</v>
       </c>
       <c r="I15" t="s">
         <v>793</v>
@@ -17826,50 +17764,50 @@
     <col min="15" max="15" width="96.33203125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:15" s="40" customFormat="1" ht="19" x14ac:dyDescent="0.25">
-      <c r="A1" s="40" t="s">
+    <row r="1" spans="1:15" s="39" customFormat="1" ht="19" x14ac:dyDescent="0.25">
+      <c r="A1" s="39" t="s">
         <v>666</v>
       </c>
-      <c r="B1" s="40" t="s">
+      <c r="B1" s="39" t="s">
         <v>629</v>
       </c>
-      <c r="C1" s="40" t="s">
+      <c r="C1" s="39" t="s">
         <v>631</v>
       </c>
-      <c r="D1" s="40" t="s">
+      <c r="D1" s="39" t="s">
         <v>632</v>
       </c>
-      <c r="E1" s="40" t="s">
+      <c r="E1" s="39" t="s">
         <v>633</v>
       </c>
-      <c r="F1" s="40" t="s">
+      <c r="F1" s="39" t="s">
         <v>635</v>
       </c>
-      <c r="G1" s="40" t="s">
+      <c r="G1" s="39" t="s">
         <v>682</v>
       </c>
-      <c r="H1" s="40" t="s">
-        <v>832</v>
-      </c>
-      <c r="I1" s="41" t="s">
+      <c r="H1" s="39" t="s">
+        <v>831</v>
+      </c>
+      <c r="I1" s="40" t="s">
+        <v>800</v>
+      </c>
+      <c r="J1" s="40" t="s">
         <v>801</v>
       </c>
-      <c r="J1" s="41" t="s">
+      <c r="K1" s="40" t="s">
         <v>802</v>
       </c>
-      <c r="K1" s="41" t="s">
+      <c r="L1" s="40" t="s">
         <v>803</v>
       </c>
-      <c r="L1" s="41" t="s">
+      <c r="M1" s="40" t="s">
         <v>804</v>
       </c>
-      <c r="M1" s="41" t="s">
-        <v>805</v>
-      </c>
-      <c r="N1" s="41" t="s">
-        <v>866</v>
-      </c>
-      <c r="O1" s="41" t="s">
+      <c r="N1" s="40" t="s">
+        <v>865</v>
+      </c>
+      <c r="O1" s="40" t="s">
         <v>120</v>
       </c>
     </row>
@@ -17889,8 +17827,8 @@
       <c r="F2" s="25" t="s">
         <v>645</v>
       </c>
-      <c r="H2" s="29" t="s">
-        <v>833</v>
+      <c r="H2" s="28" t="s">
+        <v>832</v>
       </c>
       <c r="I2" s="25" t="s">
         <v>645</v>
@@ -17915,8 +17853,8 @@
       <c r="E3" s="25" t="s">
         <v>151</v>
       </c>
-      <c r="H3" s="29" t="s">
-        <v>834</v>
+      <c r="H3" s="28" t="s">
+        <v>833</v>
       </c>
       <c r="I3" s="25" t="s">
         <v>645</v>
@@ -17950,8 +17888,8 @@
       <c r="F4" s="25" t="s">
         <v>645</v>
       </c>
-      <c r="H4" s="29" t="s">
-        <v>835</v>
+      <c r="H4" s="28" t="s">
+        <v>834</v>
       </c>
       <c r="I4" s="25" t="s">
         <v>645</v>
@@ -17979,8 +17917,8 @@
       <c r="F5" s="25" t="s">
         <v>645</v>
       </c>
-      <c r="H5" s="29" t="s">
-        <v>836</v>
+      <c r="H5" s="28" t="s">
+        <v>835</v>
       </c>
       <c r="I5" s="25" t="s">
         <v>477</v>
@@ -18014,8 +17952,8 @@
       <c r="F6" s="25" t="s">
         <v>645</v>
       </c>
-      <c r="H6" s="29" t="s">
-        <v>837</v>
+      <c r="H6" s="28" t="s">
+        <v>836</v>
       </c>
       <c r="I6" s="25" t="s">
         <v>476</v>
@@ -18049,8 +17987,8 @@
       <c r="F7" s="25" t="s">
         <v>645</v>
       </c>
-      <c r="H7" s="29" t="s">
-        <v>838</v>
+      <c r="H7" s="28" t="s">
+        <v>837</v>
       </c>
       <c r="I7" s="25" t="s">
         <v>479</v>
@@ -18084,8 +18022,8 @@
       <c r="F8" s="25" t="s">
         <v>645</v>
       </c>
-      <c r="H8" s="29" t="s">
-        <v>839</v>
+      <c r="H8" s="28" t="s">
+        <v>838</v>
       </c>
       <c r="I8" s="25" t="s">
         <v>478</v>
@@ -18119,8 +18057,8 @@
       <c r="F9" s="25" t="s">
         <v>645</v>
       </c>
-      <c r="H9" s="29" t="s">
-        <v>840</v>
+      <c r="H9" s="28" t="s">
+        <v>839</v>
       </c>
       <c r="I9" s="25" t="s">
         <v>645</v>
@@ -18149,7 +18087,7 @@
       <c r="C11" s="25" t="s">
         <v>29</v>
       </c>
-      <c r="D11" s="34" t="s">
+      <c r="D11" s="33" t="s">
         <v>181</v>
       </c>
       <c r="E11" s="25" t="s">
@@ -18159,7 +18097,7 @@
         <v>427</v>
       </c>
       <c r="H11" s="25" t="s">
-        <v>841</v>
+        <v>840</v>
       </c>
       <c r="I11" s="25" t="s">
         <v>645</v>
@@ -18181,7 +18119,7 @@
       <c r="C12" s="25" t="s">
         <v>29</v>
       </c>
-      <c r="D12" s="33" t="s">
+      <c r="D12" s="32" t="s">
         <v>182</v>
       </c>
       <c r="E12" s="25" t="s">
@@ -18210,7 +18148,7 @@
       <c r="C13" s="25" t="s">
         <v>29</v>
       </c>
-      <c r="D13" s="33" t="s">
+      <c r="D13" s="32" t="s">
         <v>183</v>
       </c>
       <c r="E13" s="25" t="s">
@@ -18239,7 +18177,7 @@
       <c r="C14" s="25" t="s">
         <v>29</v>
       </c>
-      <c r="D14" s="33" t="s">
+      <c r="D14" s="32" t="s">
         <v>184</v>
       </c>
       <c r="E14" s="25" t="s">
@@ -18268,7 +18206,7 @@
       <c r="C15" s="25" t="s">
         <v>29</v>
       </c>
-      <c r="D15" s="34" t="s">
+      <c r="D15" s="33" t="s">
         <v>185</v>
       </c>
       <c r="E15" s="25" t="s">
@@ -18294,7 +18232,7 @@
       <c r="C16" s="25" t="s">
         <v>29</v>
       </c>
-      <c r="D16" s="33" t="s">
+      <c r="D16" s="32" t="s">
         <v>186</v>
       </c>
       <c r="E16" s="25" t="s">
@@ -18323,7 +18261,7 @@
       <c r="C17" s="25" t="s">
         <v>29</v>
       </c>
-      <c r="D17" s="33" t="s">
+      <c r="D17" s="32" t="s">
         <v>187</v>
       </c>
       <c r="E17" s="25" t="s">
@@ -18352,7 +18290,7 @@
       <c r="C18" s="25" t="s">
         <v>29</v>
       </c>
-      <c r="D18" s="33" t="s">
+      <c r="D18" s="32" t="s">
         <v>188</v>
       </c>
       <c r="E18" s="25" t="s">
@@ -18381,7 +18319,7 @@
       <c r="C19" s="25" t="s">
         <v>29</v>
       </c>
-      <c r="D19" s="33" t="s">
+      <c r="D19" s="32" t="s">
         <v>189</v>
       </c>
       <c r="E19" s="25" t="s">
@@ -18410,7 +18348,7 @@
       <c r="C20" s="25" t="s">
         <v>29</v>
       </c>
-      <c r="D20" s="33" t="s">
+      <c r="D20" s="32" t="s">
         <v>190</v>
       </c>
       <c r="E20" s="25" t="s">
@@ -18439,7 +18377,7 @@
       <c r="C21" s="25" t="s">
         <v>29</v>
       </c>
-      <c r="D21" s="33" t="s">
+      <c r="D21" s="32" t="s">
         <v>191</v>
       </c>
       <c r="E21" s="25" t="s">
@@ -18468,7 +18406,7 @@
       <c r="C22" s="25" t="s">
         <v>29</v>
       </c>
-      <c r="D22" s="33" t="s">
+      <c r="D22" s="32" t="s">
         <v>192</v>
       </c>
       <c r="E22" s="25" t="s">
@@ -18497,7 +18435,7 @@
       <c r="C23" s="25" t="s">
         <v>29</v>
       </c>
-      <c r="D23" s="33" t="s">
+      <c r="D23" s="32" t="s">
         <v>193</v>
       </c>
       <c r="E23" s="25" t="s">
@@ -18526,7 +18464,7 @@
       <c r="C24" s="25" t="s">
         <v>29</v>
       </c>
-      <c r="D24" s="33" t="s">
+      <c r="D24" s="32" t="s">
         <v>194</v>
       </c>
       <c r="E24" s="25" t="s">
@@ -18555,7 +18493,7 @@
       <c r="C25" s="25" t="s">
         <v>29</v>
       </c>
-      <c r="D25" s="33" t="s">
+      <c r="D25" s="32" t="s">
         <v>195</v>
       </c>
       <c r="E25" s="25" t="s">
@@ -18584,7 +18522,7 @@
       <c r="C26" s="25" t="s">
         <v>29</v>
       </c>
-      <c r="D26" s="33" t="s">
+      <c r="D26" s="32" t="s">
         <v>196</v>
       </c>
       <c r="E26" s="25" t="s">
@@ -18613,7 +18551,7 @@
       <c r="C27" s="25" t="s">
         <v>29</v>
       </c>
-      <c r="D27" s="33" t="s">
+      <c r="D27" s="32" t="s">
         <v>197</v>
       </c>
       <c r="E27" s="25" t="s">
@@ -18671,7 +18609,7 @@
       <c r="C29" s="25" t="s">
         <v>29</v>
       </c>
-      <c r="D29" s="33" t="s">
+      <c r="D29" s="32" t="s">
         <v>199</v>
       </c>
       <c r="E29" s="25" t="s">
@@ -18700,7 +18638,7 @@
       <c r="C30" s="25" t="s">
         <v>29</v>
       </c>
-      <c r="D30" s="33" t="s">
+      <c r="D30" s="32" t="s">
         <v>200</v>
       </c>
       <c r="E30" s="25" t="s">
@@ -18729,7 +18667,7 @@
       <c r="C31" s="25" t="s">
         <v>29</v>
       </c>
-      <c r="D31" s="33" t="s">
+      <c r="D31" s="32" t="s">
         <v>201</v>
       </c>
       <c r="E31" s="25" t="s">
@@ -18758,7 +18696,7 @@
       <c r="C32" s="25" t="s">
         <v>29</v>
       </c>
-      <c r="D32" s="33" t="s">
+      <c r="D32" s="32" t="s">
         <v>202</v>
       </c>
       <c r="E32" s="25" t="s">
@@ -18787,7 +18725,7 @@
       <c r="C33" s="25" t="s">
         <v>29</v>
       </c>
-      <c r="D33" s="33" t="s">
+      <c r="D33" s="32" t="s">
         <v>203</v>
       </c>
       <c r="E33" s="25" t="s">
@@ -18816,7 +18754,7 @@
       <c r="C34" s="25" t="s">
         <v>29</v>
       </c>
-      <c r="D34" s="33" t="s">
+      <c r="D34" s="32" t="s">
         <v>180</v>
       </c>
       <c r="E34" s="25" t="s">
@@ -18836,7 +18774,7 @@
       </c>
     </row>
     <row r="35" spans="1:11" s="25" customFormat="1" x14ac:dyDescent="0.2">
-      <c r="D35" s="33"/>
+      <c r="D35" s="32"/>
     </row>
     <row r="36" spans="1:11" s="25" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A36" s="25" t="b">
@@ -18848,7 +18786,7 @@
       <c r="C36" s="25" t="s">
         <v>30</v>
       </c>
-      <c r="D36" s="29" t="s">
+      <c r="D36" s="28" t="s">
         <v>219</v>
       </c>
       <c r="E36" s="25" t="s">
@@ -18857,8 +18795,8 @@
       <c r="F36" s="25" t="s">
         <v>445</v>
       </c>
-      <c r="H36" s="29" t="s">
-        <v>842</v>
+      <c r="H36" s="28" t="s">
+        <v>841</v>
       </c>
       <c r="I36" s="25" t="s">
         <v>645</v>
@@ -18880,7 +18818,7 @@
       <c r="C37" s="25" t="s">
         <v>30</v>
       </c>
-      <c r="D37" s="33" t="s">
+      <c r="D37" s="32" t="s">
         <v>217</v>
       </c>
       <c r="E37" s="25" t="s">
@@ -18909,7 +18847,7 @@
       <c r="C38" s="25" t="s">
         <v>30</v>
       </c>
-      <c r="D38" s="33" t="s">
+      <c r="D38" s="32" t="s">
         <v>231</v>
       </c>
       <c r="E38" s="25" t="s">
@@ -18938,7 +18876,7 @@
       <c r="C39" s="25" t="s">
         <v>30</v>
       </c>
-      <c r="D39" s="33" t="s">
+      <c r="D39" s="32" t="s">
         <v>223</v>
       </c>
       <c r="E39" s="25" t="s">
@@ -18996,7 +18934,7 @@
       <c r="C41" s="25" t="s">
         <v>30</v>
       </c>
-      <c r="D41" s="37" t="s">
+      <c r="D41" s="36" t="s">
         <v>234</v>
       </c>
       <c r="E41" s="25" t="s">
@@ -19025,7 +18963,7 @@
       <c r="C42" s="25" t="s">
         <v>30</v>
       </c>
-      <c r="D42" s="33" t="s">
+      <c r="D42" s="32" t="s">
         <v>214</v>
       </c>
       <c r="E42" s="25" t="s">
@@ -19054,7 +18992,7 @@
       <c r="C43" s="25" t="s">
         <v>30</v>
       </c>
-      <c r="D43" s="33" t="s">
+      <c r="D43" s="32" t="s">
         <v>215</v>
       </c>
       <c r="E43" s="25" t="s">
@@ -19083,7 +19021,7 @@
       <c r="C44" s="25" t="s">
         <v>30</v>
       </c>
-      <c r="D44" s="33" t="s">
+      <c r="D44" s="32" t="s">
         <v>216</v>
       </c>
       <c r="E44" s="25" t="s">
@@ -19112,7 +19050,7 @@
       <c r="C45" s="25" t="s">
         <v>30</v>
       </c>
-      <c r="D45" s="33" t="s">
+      <c r="D45" s="32" t="s">
         <v>212</v>
       </c>
       <c r="E45" s="25" t="s">
@@ -19141,7 +19079,7 @@
       <c r="C46" s="25" t="s">
         <v>30</v>
       </c>
-      <c r="D46" s="33" t="s">
+      <c r="D46" s="32" t="s">
         <v>211</v>
       </c>
       <c r="E46" s="25" t="s">
@@ -19170,7 +19108,7 @@
       <c r="C47" s="25" t="s">
         <v>30</v>
       </c>
-      <c r="D47" s="33" t="s">
+      <c r="D47" s="32" t="s">
         <v>213</v>
       </c>
       <c r="E47" s="25" t="s">
@@ -19199,7 +19137,7 @@
       <c r="C48" s="25" t="s">
         <v>30</v>
       </c>
-      <c r="D48" s="33" t="s">
+      <c r="D48" s="32" t="s">
         <v>194</v>
       </c>
       <c r="E48" s="25" t="s">
@@ -19228,7 +19166,7 @@
       <c r="C49" s="25" t="s">
         <v>30</v>
       </c>
-      <c r="D49" s="33" t="s">
+      <c r="D49" s="32" t="s">
         <v>224</v>
       </c>
       <c r="E49" s="25" t="s">
@@ -19257,7 +19195,7 @@
       <c r="C50" s="25" t="s">
         <v>30</v>
       </c>
-      <c r="D50" s="33" t="s">
+      <c r="D50" s="32" t="s">
         <v>206</v>
       </c>
       <c r="E50" s="25" t="s">
@@ -19286,7 +19224,7 @@
       <c r="C51" s="25" t="s">
         <v>30</v>
       </c>
-      <c r="D51" s="33" t="s">
+      <c r="D51" s="32" t="s">
         <v>205</v>
       </c>
       <c r="E51" s="25" t="s">
@@ -19315,7 +19253,7 @@
       <c r="C52" s="25" t="s">
         <v>30</v>
       </c>
-      <c r="D52" s="34" t="s">
+      <c r="D52" s="33" t="s">
         <v>204</v>
       </c>
       <c r="E52" s="25" t="s">
@@ -19344,7 +19282,7 @@
       <c r="C53" s="25" t="s">
         <v>30</v>
       </c>
-      <c r="D53" s="33" t="s">
+      <c r="D53" s="32" t="s">
         <v>210</v>
       </c>
       <c r="E53" s="25" t="s">
@@ -19373,7 +19311,7 @@
       <c r="C54" s="25" t="s">
         <v>30</v>
       </c>
-      <c r="D54" s="33" t="s">
+      <c r="D54" s="32" t="s">
         <v>208</v>
       </c>
       <c r="E54" s="25" t="s">
@@ -19402,7 +19340,7 @@
       <c r="C55" s="25" t="s">
         <v>30</v>
       </c>
-      <c r="D55" s="33" t="s">
+      <c r="D55" s="32" t="s">
         <v>220</v>
       </c>
       <c r="E55" s="25" t="s">
@@ -19431,7 +19369,7 @@
       <c r="C56" s="25" t="s">
         <v>30</v>
       </c>
-      <c r="D56" s="33" t="s">
+      <c r="D56" s="32" t="s">
         <v>229</v>
       </c>
       <c r="E56" s="25" t="s">
@@ -19460,7 +19398,7 @@
       <c r="C57" s="25" t="s">
         <v>30</v>
       </c>
-      <c r="D57" s="33" t="s">
+      <c r="D57" s="32" t="s">
         <v>209</v>
       </c>
       <c r="E57" s="25" t="s">
@@ -19489,7 +19427,7 @@
       <c r="C58" s="25" t="s">
         <v>30</v>
       </c>
-      <c r="D58" s="33" t="s">
+      <c r="D58" s="32" t="s">
         <v>207</v>
       </c>
       <c r="E58" s="25" t="s">
@@ -19518,7 +19456,7 @@
       <c r="C59" s="25" t="s">
         <v>30</v>
       </c>
-      <c r="D59" s="33" t="s">
+      <c r="D59" s="32" t="s">
         <v>232</v>
       </c>
       <c r="E59" s="25" t="s">
@@ -19576,7 +19514,7 @@
       <c r="C61" s="25" t="s">
         <v>30</v>
       </c>
-      <c r="D61" s="33" t="s">
+      <c r="D61" s="32" t="s">
         <v>233</v>
       </c>
       <c r="E61" s="25" t="s">
@@ -19605,7 +19543,7 @@
       <c r="C62" s="25" t="s">
         <v>30</v>
       </c>
-      <c r="D62" s="37" t="s">
+      <c r="D62" s="36" t="s">
         <v>225</v>
       </c>
       <c r="E62" s="25" t="s">
@@ -19634,7 +19572,7 @@
       <c r="C63" s="25" t="s">
         <v>30</v>
       </c>
-      <c r="D63" s="37" t="s">
+      <c r="D63" s="36" t="s">
         <v>226</v>
       </c>
       <c r="E63" s="25" t="s">
@@ -19663,7 +19601,7 @@
       <c r="C64" s="25" t="s">
         <v>30</v>
       </c>
-      <c r="D64" s="33" t="s">
+      <c r="D64" s="32" t="s">
         <v>218</v>
       </c>
       <c r="E64" s="25" t="s">
@@ -19692,7 +19630,7 @@
       <c r="C65" s="25" t="s">
         <v>30</v>
       </c>
-      <c r="D65" s="33" t="s">
+      <c r="D65" s="32" t="s">
         <v>201</v>
       </c>
       <c r="E65" s="25" t="s">
@@ -19721,7 +19659,7 @@
       <c r="C66" s="25" t="s">
         <v>30</v>
       </c>
-      <c r="D66" s="33" t="s">
+      <c r="D66" s="32" t="s">
         <v>221</v>
       </c>
       <c r="E66" s="25" t="s">
@@ -19750,7 +19688,7 @@
       <c r="C67" s="25" t="s">
         <v>30</v>
       </c>
-      <c r="D67" s="38" t="s">
+      <c r="D67" s="37" t="s">
         <v>227</v>
       </c>
       <c r="E67" s="25" t="s">
@@ -19779,7 +19717,7 @@
       <c r="C68" s="25" t="s">
         <v>30</v>
       </c>
-      <c r="D68" s="38" t="s">
+      <c r="D68" s="37" t="s">
         <v>228</v>
       </c>
       <c r="E68" s="25" t="s">
@@ -19799,7 +19737,7 @@
       </c>
     </row>
     <row r="69" spans="1:14" s="25" customFormat="1" x14ac:dyDescent="0.2">
-      <c r="D69" s="38"/>
+      <c r="D69" s="37"/>
     </row>
     <row r="70" spans="1:14" s="25" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A70" s="25" t="b">
@@ -19811,7 +19749,7 @@
       <c r="C70" s="25" t="s">
         <v>41</v>
       </c>
-      <c r="D70" s="33" t="s">
+      <c r="D70" s="32" t="s">
         <v>387</v>
       </c>
       <c r="E70" s="25" t="s">
@@ -19820,8 +19758,8 @@
       <c r="F70" s="25" t="s">
         <v>387</v>
       </c>
-      <c r="H70" s="29" t="s">
-        <v>843</v>
+      <c r="H70" s="28" t="s">
+        <v>842</v>
       </c>
       <c r="I70" s="25" t="s">
         <v>645</v>
@@ -19843,7 +19781,7 @@
       <c r="C71" s="25" t="s">
         <v>41</v>
       </c>
-      <c r="D71" s="33" t="s">
+      <c r="D71" s="32" t="s">
         <v>388</v>
       </c>
       <c r="E71" s="25" t="s">
@@ -19872,7 +19810,7 @@
       <c r="C72" s="25" t="s">
         <v>41</v>
       </c>
-      <c r="D72" s="33" t="s">
+      <c r="D72" s="32" t="s">
         <v>389</v>
       </c>
       <c r="E72" s="25" t="s">
@@ -19901,7 +19839,7 @@
       <c r="C73" s="25" t="s">
         <v>41</v>
       </c>
-      <c r="D73" s="33" t="s">
+      <c r="D73" s="32" t="s">
         <v>390</v>
       </c>
       <c r="E73" s="25" t="s">
@@ -19930,7 +19868,7 @@
       <c r="C74" s="25" t="s">
         <v>41</v>
       </c>
-      <c r="D74" s="33" t="s">
+      <c r="D74" s="32" t="s">
         <v>391</v>
       </c>
       <c r="E74" s="25" t="s">
@@ -19959,7 +19897,7 @@
       <c r="C75" s="25" t="s">
         <v>41</v>
       </c>
-      <c r="D75" s="33" t="s">
+      <c r="D75" s="32" t="s">
         <v>392</v>
       </c>
       <c r="E75" s="25" t="s">
@@ -19988,7 +19926,7 @@
       <c r="C76" s="25" t="s">
         <v>41</v>
       </c>
-      <c r="D76" s="33" t="s">
+      <c r="D76" s="32" t="s">
         <v>393</v>
       </c>
       <c r="E76" s="25" t="s">
@@ -20008,7 +19946,7 @@
       </c>
     </row>
     <row r="77" spans="1:14" s="25" customFormat="1" x14ac:dyDescent="0.2">
-      <c r="D77" s="33"/>
+      <c r="D77" s="32"/>
     </row>
     <row r="78" spans="1:14" s="25" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A78" s="25" t="b">
@@ -20020,7 +19958,7 @@
       <c r="C78" s="25" t="s">
         <v>42</v>
       </c>
-      <c r="D78" s="33" t="s">
+      <c r="D78" s="32" t="s">
         <v>406</v>
       </c>
       <c r="E78" s="25" t="s">
@@ -20029,8 +19967,8 @@
       <c r="F78" s="25" t="s">
         <v>406</v>
       </c>
-      <c r="H78" s="29" t="s">
-        <v>844</v>
+      <c r="H78" s="28" t="s">
+        <v>843</v>
       </c>
       <c r="I78" s="25" t="s">
         <v>645</v>
@@ -20042,7 +19980,7 @@
         <v>676</v>
       </c>
       <c r="N78" s="25" t="s">
-        <v>862</v>
+        <v>861</v>
       </c>
     </row>
     <row r="79" spans="1:14" s="25" customFormat="1" x14ac:dyDescent="0.2">
@@ -20055,7 +19993,7 @@
       <c r="C79" s="25" t="s">
         <v>42</v>
       </c>
-      <c r="D79" s="33" t="s">
+      <c r="D79" s="32" t="s">
         <v>407</v>
       </c>
       <c r="E79" s="25" t="s">
@@ -20064,7 +20002,7 @@
       <c r="F79" s="25" t="s">
         <v>407</v>
       </c>
-      <c r="H79" s="29"/>
+      <c r="H79" s="28"/>
       <c r="I79" s="25" t="s">
         <v>645</v>
       </c>
@@ -20076,8 +20014,8 @@
       </c>
     </row>
     <row r="80" spans="1:14" s="25" customFormat="1" x14ac:dyDescent="0.2">
-      <c r="D80" s="33"/>
-      <c r="H80" s="29"/>
+      <c r="D80" s="32"/>
+      <c r="H80" s="28"/>
     </row>
     <row r="81" spans="1:11" s="25" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A81" s="25" t="b">
@@ -20089,14 +20027,14 @@
       <c r="C81" s="25" t="s">
         <v>38</v>
       </c>
-      <c r="D81" s="33" t="s">
+      <c r="D81" s="32" t="s">
         <v>795</v>
       </c>
       <c r="E81" s="25" t="s">
         <v>151</v>
       </c>
-      <c r="H81" s="29" t="s">
-        <v>845</v>
+      <c r="H81" s="28" t="s">
+        <v>844</v>
       </c>
       <c r="I81" s="25" t="s">
         <v>645</v>
@@ -20118,7 +20056,7 @@
       <c r="C82" s="25" t="s">
         <v>38</v>
       </c>
-      <c r="D82" s="33" t="s">
+      <c r="D82" s="32" t="s">
         <v>252</v>
       </c>
       <c r="E82" s="25" t="s">
@@ -20147,7 +20085,7 @@
       <c r="C83" s="25" t="s">
         <v>38</v>
       </c>
-      <c r="D83" s="33" t="s">
+      <c r="D83" s="32" t="s">
         <v>255</v>
       </c>
       <c r="E83" s="25" t="s">
@@ -20176,7 +20114,7 @@
       <c r="C84" s="25" t="s">
         <v>38</v>
       </c>
-      <c r="D84" s="33" t="s">
+      <c r="D84" s="32" t="s">
         <v>254</v>
       </c>
       <c r="E84" s="25" t="s">
@@ -20205,7 +20143,7 @@
       <c r="C85" s="25" t="s">
         <v>38</v>
       </c>
-      <c r="D85" s="33" t="s">
+      <c r="D85" s="32" t="s">
         <v>250</v>
       </c>
       <c r="E85" s="25" t="s">
@@ -20234,7 +20172,7 @@
       <c r="C86" s="25" t="s">
         <v>38</v>
       </c>
-      <c r="D86" s="33" t="s">
+      <c r="D86" s="32" t="s">
         <v>251</v>
       </c>
       <c r="E86" s="25" t="s">
@@ -20263,7 +20201,7 @@
       <c r="C87" s="25" t="s">
         <v>38</v>
       </c>
-      <c r="D87" s="33" t="s">
+      <c r="D87" s="32" t="s">
         <v>253</v>
       </c>
       <c r="E87" s="25" t="s">
@@ -20283,7 +20221,7 @@
       </c>
     </row>
     <row r="88" spans="1:11" s="25" customFormat="1" x14ac:dyDescent="0.2">
-      <c r="D88" s="33"/>
+      <c r="D88" s="32"/>
     </row>
     <row r="89" spans="1:11" s="25" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A89" s="25" t="b">
@@ -20295,14 +20233,14 @@
       <c r="C89" s="25" t="s">
         <v>37</v>
       </c>
-      <c r="D89" s="33" t="s">
+      <c r="D89" s="32" t="s">
         <v>795</v>
       </c>
       <c r="E89" s="25" t="s">
         <v>151</v>
       </c>
-      <c r="H89" s="29" t="s">
-        <v>846</v>
+      <c r="H89" s="28" t="s">
+        <v>845</v>
       </c>
       <c r="I89" s="25" t="s">
         <v>645</v>
@@ -20324,7 +20262,7 @@
       <c r="C90" s="25" t="s">
         <v>37</v>
       </c>
-      <c r="D90" s="33" t="s">
+      <c r="D90" s="32" t="s">
         <v>248</v>
       </c>
       <c r="E90" s="25" t="s">
@@ -20353,7 +20291,7 @@
       <c r="C91" s="25" t="s">
         <v>37</v>
       </c>
-      <c r="D91" s="33" t="s">
+      <c r="D91" s="32" t="s">
         <v>236</v>
       </c>
       <c r="E91" s="25" t="s">
@@ -20382,7 +20320,7 @@
       <c r="C92" s="25" t="s">
         <v>37</v>
       </c>
-      <c r="D92" s="33" t="s">
+      <c r="D92" s="32" t="s">
         <v>235</v>
       </c>
       <c r="E92" s="25" t="s">
@@ -20411,7 +20349,7 @@
       <c r="C93" s="25" t="s">
         <v>37</v>
       </c>
-      <c r="D93" s="33" t="s">
+      <c r="D93" s="32" t="s">
         <v>238</v>
       </c>
       <c r="E93" s="25" t="s">
@@ -20440,7 +20378,7 @@
       <c r="C94" s="25" t="s">
         <v>37</v>
       </c>
-      <c r="D94" s="33" t="s">
+      <c r="D94" s="32" t="s">
         <v>237</v>
       </c>
       <c r="E94" s="25" t="s">
@@ -20469,7 +20407,7 @@
       <c r="C95" s="25" t="s">
         <v>37</v>
       </c>
-      <c r="D95" s="33" t="s">
+      <c r="D95" s="32" t="s">
         <v>245</v>
       </c>
       <c r="E95" s="25" t="s">
@@ -20498,7 +20436,7 @@
       <c r="C96" s="25" t="s">
         <v>37</v>
       </c>
-      <c r="D96" s="33" t="s">
+      <c r="D96" s="32" t="s">
         <v>244</v>
       </c>
       <c r="E96" s="25" t="s">
@@ -20527,7 +20465,7 @@
       <c r="C97" s="25" t="s">
         <v>37</v>
       </c>
-      <c r="D97" s="33" t="s">
+      <c r="D97" s="32" t="s">
         <v>247</v>
       </c>
       <c r="E97" s="25" t="s">
@@ -20556,7 +20494,7 @@
       <c r="C98" s="25" t="s">
         <v>37</v>
       </c>
-      <c r="D98" s="33" t="s">
+      <c r="D98" s="32" t="s">
         <v>243</v>
       </c>
       <c r="E98" s="25" t="s">
@@ -20585,7 +20523,7 @@
       <c r="C99" s="25" t="s">
         <v>37</v>
       </c>
-      <c r="D99" s="33" t="s">
+      <c r="D99" s="32" t="s">
         <v>239</v>
       </c>
       <c r="E99" s="25" t="s">
@@ -20614,7 +20552,7 @@
       <c r="C100" s="25" t="s">
         <v>37</v>
       </c>
-      <c r="D100" s="33" t="s">
+      <c r="D100" s="32" t="s">
         <v>246</v>
       </c>
       <c r="E100" s="25" t="s">
@@ -20643,7 +20581,7 @@
       <c r="C101" s="25" t="s">
         <v>37</v>
       </c>
-      <c r="D101" s="33" t="s">
+      <c r="D101" s="32" t="s">
         <v>240</v>
       </c>
       <c r="E101" s="25" t="s">
@@ -20672,7 +20610,7 @@
       <c r="C102" s="25" t="s">
         <v>37</v>
       </c>
-      <c r="D102" s="33" t="s">
+      <c r="D102" s="32" t="s">
         <v>249</v>
       </c>
       <c r="E102" s="25" t="s">
@@ -20701,7 +20639,7 @@
       <c r="C103" s="25" t="s">
         <v>37</v>
       </c>
-      <c r="D103" s="33" t="s">
+      <c r="D103" s="32" t="s">
         <v>241</v>
       </c>
       <c r="E103" s="25" t="s">
@@ -20730,7 +20668,7 @@
       <c r="C104" s="25" t="s">
         <v>37</v>
       </c>
-      <c r="D104" s="33" t="s">
+      <c r="D104" s="32" t="s">
         <v>242</v>
       </c>
       <c r="E104" s="25" t="s">
@@ -20750,7 +20688,7 @@
       </c>
     </row>
     <row r="105" spans="1:11" s="25" customFormat="1" x14ac:dyDescent="0.2">
-      <c r="D105" s="33"/>
+      <c r="D105" s="32"/>
     </row>
     <row r="106" spans="1:11" s="25" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A106" s="25" t="b">
@@ -20762,7 +20700,7 @@
       <c r="C106" s="25" t="s">
         <v>28</v>
       </c>
-      <c r="D106" s="33" t="s">
+      <c r="D106" s="32" t="s">
         <v>177</v>
       </c>
       <c r="E106" s="25" t="s">
@@ -20772,7 +20710,7 @@
         <v>421</v>
       </c>
       <c r="H106" s="25" t="s">
-        <v>847</v>
+        <v>846</v>
       </c>
       <c r="I106" s="25" t="s">
         <v>645</v>
@@ -20794,7 +20732,7 @@
       <c r="C107" s="25" t="s">
         <v>28</v>
       </c>
-      <c r="D107" s="33" t="s">
+      <c r="D107" s="32" t="s">
         <v>178</v>
       </c>
       <c r="E107" s="25" t="s">
@@ -20823,7 +20761,7 @@
       <c r="C108" s="25" t="s">
         <v>28</v>
       </c>
-      <c r="D108" s="33" t="s">
+      <c r="D108" s="32" t="s">
         <v>179</v>
       </c>
       <c r="E108" s="25" t="s">
@@ -20852,7 +20790,7 @@
       <c r="C109" s="25" t="s">
         <v>28</v>
       </c>
-      <c r="D109" s="33" t="s">
+      <c r="D109" s="32" t="s">
         <v>180</v>
       </c>
       <c r="E109" s="25" t="s">
@@ -20881,7 +20819,7 @@
       <c r="C110" s="25" t="s">
         <v>28</v>
       </c>
-      <c r="D110" s="33" t="s">
+      <c r="D110" s="32" t="s">
         <v>795</v>
       </c>
       <c r="E110" s="25" t="s">
@@ -20924,54 +20862,54 @@
     <col min="16" max="16" width="12.5" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:16" s="40" customFormat="1" ht="19" x14ac:dyDescent="0.25">
-      <c r="A1" s="40" t="s">
+    <row r="1" spans="1:16" s="39" customFormat="1" ht="19" x14ac:dyDescent="0.25">
+      <c r="A1" s="39" t="s">
         <v>666</v>
       </c>
-      <c r="B1" s="40" t="s">
+      <c r="B1" s="39" t="s">
         <v>629</v>
       </c>
-      <c r="C1" s="40" t="s">
+      <c r="C1" s="39" t="s">
         <v>631</v>
       </c>
-      <c r="D1" s="40" t="s">
+      <c r="D1" s="39" t="s">
         <v>632</v>
       </c>
-      <c r="E1" s="40" t="s">
+      <c r="E1" s="39" t="s">
         <v>633</v>
       </c>
-      <c r="F1" s="40" t="s">
+      <c r="F1" s="39" t="s">
         <v>635</v>
       </c>
-      <c r="G1" s="40" t="s">
+      <c r="G1" s="39" t="s">
         <v>682</v>
       </c>
-      <c r="H1" s="40" t="s">
+      <c r="H1" s="39" t="s">
+        <v>889</v>
+      </c>
+      <c r="I1" s="40" t="s">
         <v>890</v>
       </c>
-      <c r="I1" s="41" t="s">
+      <c r="J1" s="40" t="s">
         <v>891</v>
       </c>
-      <c r="J1" s="41" t="s">
+      <c r="K1" s="40" t="s">
         <v>892</v>
       </c>
-      <c r="K1" s="41" t="s">
+      <c r="L1" s="40" t="s">
         <v>893</v>
       </c>
-      <c r="L1" s="41" t="s">
+      <c r="M1" s="40" t="s">
         <v>894</v>
       </c>
-      <c r="M1" s="41" t="s">
+      <c r="N1" s="40" t="s">
         <v>895</v>
       </c>
-      <c r="N1" s="41" t="s">
-        <v>896</v>
-      </c>
-      <c r="O1" s="41" t="s">
-        <v>902</v>
-      </c>
-      <c r="P1" s="40" t="s">
-        <v>849</v>
+      <c r="O1" s="40" t="s">
+        <v>901</v>
+      </c>
+      <c r="P1" s="39" t="s">
+        <v>848</v>
       </c>
     </row>
     <row r="2" spans="1:16" x14ac:dyDescent="0.2">
@@ -20988,7 +20926,7 @@
         <v>736</v>
       </c>
       <c r="H2" t="s">
-        <v>903</v>
+        <v>902</v>
       </c>
       <c r="I2" t="s">
         <v>703</v>
@@ -20997,13 +20935,13 @@
         <v>656</v>
       </c>
       <c r="L2" t="s">
-        <v>897</v>
+        <v>896</v>
       </c>
       <c r="N2" t="s">
         <v>670</v>
       </c>
       <c r="O2" t="s">
-        <v>898</v>
+        <v>897</v>
       </c>
     </row>
     <row r="3" spans="1:16" x14ac:dyDescent="0.2">
@@ -21020,7 +20958,7 @@
         <v>736</v>
       </c>
       <c r="H3" t="s">
-        <v>904</v>
+        <v>903</v>
       </c>
       <c r="I3" t="s">
         <v>703</v>
@@ -21029,13 +20967,13 @@
         <v>670</v>
       </c>
       <c r="L3" t="s">
-        <v>897</v>
+        <v>896</v>
       </c>
       <c r="N3" t="s">
         <v>649</v>
       </c>
       <c r="O3" t="s">
-        <v>898</v>
+        <v>897</v>
       </c>
     </row>
     <row r="4" spans="1:16" x14ac:dyDescent="0.2">
@@ -21052,7 +20990,7 @@
         <v>736</v>
       </c>
       <c r="H4" t="s">
-        <v>905</v>
+        <v>904</v>
       </c>
       <c r="I4" t="s">
         <v>703</v>
@@ -21061,13 +20999,13 @@
         <v>650</v>
       </c>
       <c r="L4" t="s">
-        <v>899</v>
+        <v>898</v>
       </c>
       <c r="N4" t="s">
         <v>649</v>
       </c>
       <c r="O4" t="s">
-        <v>898</v>
+        <v>897</v>
       </c>
     </row>
     <row r="5" spans="1:16" x14ac:dyDescent="0.2">
@@ -21084,7 +21022,7 @@
         <v>736</v>
       </c>
       <c r="H5" t="s">
-        <v>906</v>
+        <v>905</v>
       </c>
       <c r="I5" t="s">
         <v>703</v>
@@ -21093,13 +21031,13 @@
         <v>649</v>
       </c>
       <c r="L5" t="s">
-        <v>897</v>
+        <v>896</v>
       </c>
       <c r="N5" t="s">
         <v>671</v>
       </c>
       <c r="O5" t="s">
-        <v>898</v>
+        <v>897</v>
       </c>
     </row>
     <row r="6" spans="1:16" x14ac:dyDescent="0.2">
@@ -21116,7 +21054,7 @@
         <v>736</v>
       </c>
       <c r="H6" t="s">
-        <v>907</v>
+        <v>906</v>
       </c>
       <c r="I6" t="s">
         <v>703</v>
@@ -21125,13 +21063,13 @@
         <v>653</v>
       </c>
       <c r="L6" t="s">
-        <v>899</v>
+        <v>898</v>
       </c>
       <c r="N6" t="s">
         <v>671</v>
       </c>
       <c r="O6" t="s">
-        <v>898</v>
+        <v>897</v>
       </c>
     </row>
     <row r="7" spans="1:16" x14ac:dyDescent="0.2">
@@ -21148,7 +21086,7 @@
         <v>736</v>
       </c>
       <c r="H7" t="s">
-        <v>908</v>
+        <v>907</v>
       </c>
       <c r="I7" t="s">
         <v>703</v>
@@ -21157,13 +21095,13 @@
         <v>671</v>
       </c>
       <c r="L7" t="s">
-        <v>897</v>
+        <v>896</v>
       </c>
       <c r="N7" t="s">
         <v>651</v>
       </c>
       <c r="O7" t="s">
-        <v>898</v>
+        <v>897</v>
       </c>
     </row>
     <row r="8" spans="1:16" x14ac:dyDescent="0.2">
@@ -21180,7 +21118,7 @@
         <v>736</v>
       </c>
       <c r="H8" t="s">
-        <v>909</v>
+        <v>908</v>
       </c>
       <c r="I8" t="s">
         <v>703</v>
@@ -21189,13 +21127,13 @@
         <v>652</v>
       </c>
       <c r="L8" t="s">
-        <v>899</v>
+        <v>898</v>
       </c>
       <c r="N8" t="s">
         <v>651</v>
       </c>
       <c r="O8" t="s">
-        <v>898</v>
+        <v>897</v>
       </c>
     </row>
     <row r="9" spans="1:16" x14ac:dyDescent="0.2">
@@ -21212,7 +21150,7 @@
         <v>736</v>
       </c>
       <c r="H9" t="s">
-        <v>910</v>
+        <v>909</v>
       </c>
       <c r="I9" t="s">
         <v>703</v>
@@ -21221,13 +21159,13 @@
         <v>651</v>
       </c>
       <c r="L9" t="s">
-        <v>897</v>
+        <v>896</v>
       </c>
       <c r="N9" t="s">
         <v>672</v>
       </c>
       <c r="O9" t="s">
-        <v>898</v>
+        <v>897</v>
       </c>
     </row>
     <row r="10" spans="1:16" x14ac:dyDescent="0.2">
@@ -21244,7 +21182,7 @@
         <v>736</v>
       </c>
       <c r="H10" t="s">
-        <v>911</v>
+        <v>910</v>
       </c>
       <c r="I10" t="s">
         <v>703</v>
@@ -21253,13 +21191,13 @@
         <v>654</v>
       </c>
       <c r="L10" t="s">
-        <v>899</v>
+        <v>898</v>
       </c>
       <c r="N10" t="s">
         <v>672</v>
       </c>
       <c r="O10" t="s">
-        <v>898</v>
+        <v>897</v>
       </c>
     </row>
     <row r="11" spans="1:16" x14ac:dyDescent="0.2">
@@ -21276,7 +21214,7 @@
         <v>736</v>
       </c>
       <c r="H11" t="s">
-        <v>912</v>
+        <v>911</v>
       </c>
       <c r="I11" t="s">
         <v>703</v>
@@ -21285,13 +21223,13 @@
         <v>673</v>
       </c>
       <c r="L11" t="s">
-        <v>899</v>
+        <v>898</v>
       </c>
       <c r="N11" t="s">
         <v>654</v>
       </c>
       <c r="O11" t="s">
-        <v>898</v>
+        <v>897</v>
       </c>
     </row>
     <row r="12" spans="1:16" x14ac:dyDescent="0.2">
@@ -21308,7 +21246,7 @@
         <v>736</v>
       </c>
       <c r="H12" t="s">
-        <v>913</v>
+        <v>912</v>
       </c>
       <c r="I12" t="s">
         <v>703</v>
@@ -21317,13 +21255,13 @@
         <v>674</v>
       </c>
       <c r="L12" t="s">
-        <v>899</v>
+        <v>898</v>
       </c>
       <c r="N12" t="s">
         <v>654</v>
       </c>
       <c r="O12" t="s">
-        <v>898</v>
+        <v>897</v>
       </c>
     </row>
     <row r="13" spans="1:16" x14ac:dyDescent="0.2">
@@ -21340,7 +21278,7 @@
         <v>736</v>
       </c>
       <c r="H13" t="s">
-        <v>914</v>
+        <v>913</v>
       </c>
       <c r="I13" t="s">
         <v>703</v>
@@ -21349,13 +21287,13 @@
         <v>672</v>
       </c>
       <c r="L13" t="s">
-        <v>897</v>
+        <v>896</v>
       </c>
       <c r="N13" t="s">
         <v>675</v>
       </c>
       <c r="O13" t="s">
-        <v>898</v>
+        <v>897</v>
       </c>
     </row>
     <row r="14" spans="1:16" x14ac:dyDescent="0.2">
@@ -21372,7 +21310,7 @@
         <v>736</v>
       </c>
       <c r="H14" t="s">
-        <v>915</v>
+        <v>914</v>
       </c>
       <c r="I14" t="s">
         <v>703</v>
@@ -21381,13 +21319,13 @@
         <v>676</v>
       </c>
       <c r="L14" t="s">
-        <v>899</v>
+        <v>898</v>
       </c>
       <c r="N14" t="s">
         <v>675</v>
       </c>
       <c r="O14" t="s">
-        <v>898</v>
+        <v>897</v>
       </c>
     </row>
     <row r="15" spans="1:16" x14ac:dyDescent="0.2">
@@ -21398,28 +21336,28 @@
         <v>630</v>
       </c>
       <c r="C15" t="s">
-        <v>900</v>
+        <v>899</v>
       </c>
       <c r="E15" t="s">
         <v>736</v>
       </c>
       <c r="H15" t="s">
-        <v>916</v>
+        <v>915</v>
       </c>
       <c r="I15" t="s">
         <v>703</v>
       </c>
       <c r="K15" t="s">
-        <v>901</v>
+        <v>900</v>
       </c>
       <c r="L15" t="s">
-        <v>899</v>
+        <v>898</v>
       </c>
       <c r="N15" t="s">
         <v>675</v>
       </c>
       <c r="O15" t="s">
-        <v>898</v>
+        <v>897</v>
       </c>
     </row>
     <row r="16" spans="1:16" x14ac:dyDescent="0.2">
@@ -21436,7 +21374,7 @@
         <v>736</v>
       </c>
       <c r="H16" t="s">
-        <v>917</v>
+        <v>916</v>
       </c>
       <c r="I16" t="s">
         <v>703</v>
@@ -21445,13 +21383,13 @@
         <v>677</v>
       </c>
       <c r="L16" t="s">
-        <v>899</v>
+        <v>898</v>
       </c>
       <c r="N16" t="s">
         <v>675</v>
       </c>
       <c r="O16" t="s">
-        <v>898</v>
+        <v>897</v>
       </c>
     </row>
   </sheetData>
@@ -21476,35 +21414,35 @@
     <col min="10" max="10" width="62.1640625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:10" s="40" customFormat="1" ht="19" x14ac:dyDescent="0.25">
-      <c r="A1" s="40" t="s">
+    <row r="1" spans="1:10" s="39" customFormat="1" ht="19" x14ac:dyDescent="0.25">
+      <c r="A1" s="39" t="s">
         <v>666</v>
       </c>
-      <c r="B1" s="40" t="s">
+      <c r="B1" s="39" t="s">
         <v>629</v>
       </c>
-      <c r="C1" s="40" t="s">
+      <c r="C1" s="39" t="s">
         <v>631</v>
       </c>
-      <c r="D1" s="40" t="s">
+      <c r="D1" s="39" t="s">
         <v>680</v>
       </c>
-      <c r="E1" s="40" t="s">
+      <c r="E1" s="39" t="s">
         <v>632</v>
       </c>
-      <c r="F1" s="40" t="s">
+      <c r="F1" s="39" t="s">
         <v>633</v>
       </c>
-      <c r="G1" s="40" t="s">
+      <c r="G1" s="39" t="s">
         <v>634</v>
       </c>
-      <c r="H1" s="40" t="s">
+      <c r="H1" s="39" t="s">
         <v>681</v>
       </c>
-      <c r="I1" s="40" t="s">
+      <c r="I1" s="39" t="s">
         <v>635</v>
       </c>
-      <c r="J1" s="40" t="s">
+      <c r="J1" s="39" t="s">
         <v>120</v>
       </c>
     </row>
@@ -21578,7 +21516,7 @@
         <v>795</v>
       </c>
       <c r="I6" t="s">
-        <v>831</v>
+        <v>830</v>
       </c>
     </row>
     <row r="8" spans="1:10" x14ac:dyDescent="0.2">
@@ -21595,7 +21533,7 @@
         <v>502</v>
       </c>
       <c r="J8" t="s">
-        <v>807</v>
+        <v>806</v>
       </c>
     </row>
     <row r="9" spans="1:10" x14ac:dyDescent="0.2">
@@ -21679,7 +21617,7 @@
         <v>795</v>
       </c>
       <c r="I14" t="s">
-        <v>831</v>
+        <v>830</v>
       </c>
     </row>
     <row r="16" spans="1:10" x14ac:dyDescent="0.2">
@@ -22035,7 +21973,7 @@
         <v>795</v>
       </c>
       <c r="I41" t="s">
-        <v>831</v>
+        <v>830</v>
       </c>
     </row>
     <row r="43" spans="1:10" x14ac:dyDescent="0.2">
@@ -22192,7 +22130,7 @@
         <v>795</v>
       </c>
       <c r="I53" t="s">
-        <v>831</v>
+        <v>830</v>
       </c>
     </row>
     <row r="55" spans="1:10" x14ac:dyDescent="0.2">
@@ -22205,7 +22143,7 @@
       <c r="E55" t="s">
         <v>276</v>
       </c>
-      <c r="H55" s="39"/>
+      <c r="H55" s="38"/>
       <c r="I55" t="s">
         <v>505</v>
       </c>
@@ -24143,19 +24081,19 @@
         <v>753</v>
       </c>
       <c r="F1" s="17" t="s">
-        <v>936</v>
+        <v>935</v>
       </c>
       <c r="G1" s="17" t="s">
-        <v>930</v>
+        <v>929</v>
       </c>
       <c r="H1" s="17" t="s">
-        <v>938</v>
+        <v>937</v>
       </c>
       <c r="I1" s="17" t="s">
-        <v>935</v>
+        <v>934</v>
       </c>
       <c r="J1" s="17" t="s">
-        <v>924</v>
+        <v>923</v>
       </c>
     </row>
     <row r="2" spans="1:10" x14ac:dyDescent="0.2">
@@ -24175,16 +24113,16 @@
         <v>779</v>
       </c>
       <c r="G2" t="s">
-        <v>939</v>
+        <v>938</v>
       </c>
       <c r="H2" t="s">
-        <v>960</v>
+        <v>959</v>
       </c>
       <c r="I2" t="s">
         <v>778</v>
       </c>
       <c r="J2" t="s">
-        <v>931</v>
+        <v>930</v>
       </c>
     </row>
     <row r="3" spans="1:10" x14ac:dyDescent="0.2">
@@ -24198,10 +24136,10 @@
         <v>772</v>
       </c>
       <c r="G3" t="s">
-        <v>941</v>
+        <v>940</v>
       </c>
       <c r="H3" t="s">
-        <v>961</v>
+        <v>960</v>
       </c>
     </row>
     <row r="5" spans="1:10" x14ac:dyDescent="0.2">
@@ -24221,16 +24159,16 @@
         <v>759</v>
       </c>
       <c r="G5" t="s">
-        <v>940</v>
+        <v>939</v>
       </c>
       <c r="H5" t="s">
-        <v>962</v>
+        <v>961</v>
       </c>
       <c r="I5" t="s">
         <v>754</v>
       </c>
       <c r="J5" t="s">
-        <v>925</v>
+        <v>924</v>
       </c>
     </row>
     <row r="6" spans="1:10" x14ac:dyDescent="0.2">
@@ -24250,13 +24188,13 @@
         <v>703</v>
       </c>
       <c r="G6" t="s">
-        <v>942</v>
+        <v>941</v>
       </c>
       <c r="H6" t="s">
-        <v>963</v>
+        <v>962</v>
       </c>
       <c r="J6" t="s">
-        <v>965</v>
+        <v>964</v>
       </c>
     </row>
     <row r="7" spans="1:10" x14ac:dyDescent="0.2">
@@ -24273,13 +24211,13 @@
         <v>700</v>
       </c>
       <c r="G7" t="s">
-        <v>943</v>
+        <v>942</v>
       </c>
       <c r="H7" t="s">
-        <v>977</v>
+        <v>976</v>
       </c>
       <c r="J7" t="s">
-        <v>964</v>
+        <v>963</v>
       </c>
     </row>
     <row r="8" spans="1:10" x14ac:dyDescent="0.2">
@@ -24296,13 +24234,13 @@
         <v>771</v>
       </c>
       <c r="G8" t="s">
-        <v>944</v>
+        <v>943</v>
       </c>
       <c r="H8" t="s">
-        <v>967</v>
+        <v>966</v>
       </c>
       <c r="J8" t="s">
-        <v>966</v>
+        <v>965</v>
       </c>
     </row>
     <row r="9" spans="1:10" x14ac:dyDescent="0.2">
@@ -24319,10 +24257,10 @@
         <v>694</v>
       </c>
       <c r="G9" t="s">
-        <v>945</v>
+        <v>944</v>
       </c>
       <c r="H9" t="s">
-        <v>968</v>
+        <v>967</v>
       </c>
     </row>
     <row r="10" spans="1:10" x14ac:dyDescent="0.2">
@@ -24339,10 +24277,10 @@
         <v>772</v>
       </c>
       <c r="G10" t="s">
-        <v>941</v>
+        <v>940</v>
       </c>
       <c r="H10" t="s">
-        <v>961</v>
+        <v>960</v>
       </c>
     </row>
     <row r="11" spans="1:10" x14ac:dyDescent="0.2">
@@ -24359,10 +24297,10 @@
         <v>773</v>
       </c>
       <c r="G11" t="s">
-        <v>970</v>
+        <v>969</v>
       </c>
       <c r="H11" t="s">
-        <v>969</v>
+        <v>968</v>
       </c>
     </row>
     <row r="12" spans="1:10" x14ac:dyDescent="0.2">
@@ -24379,10 +24317,10 @@
         <v>701</v>
       </c>
       <c r="G12" t="s">
-        <v>946</v>
+        <v>945</v>
       </c>
       <c r="H12" t="s">
-        <v>971</v>
+        <v>970</v>
       </c>
     </row>
     <row r="13" spans="1:10" x14ac:dyDescent="0.2">
@@ -24402,10 +24340,10 @@
         <v>693</v>
       </c>
       <c r="G13" t="s">
-        <v>947</v>
+        <v>946</v>
       </c>
       <c r="H13" t="s">
-        <v>972</v>
+        <v>971</v>
       </c>
     </row>
     <row r="15" spans="1:10" x14ac:dyDescent="0.2">
@@ -24422,10 +24360,10 @@
         <v>733</v>
       </c>
       <c r="G15" t="s">
-        <v>934</v>
+        <v>933</v>
       </c>
       <c r="H15" t="s">
-        <v>934</v>
+        <v>933</v>
       </c>
     </row>
     <row r="16" spans="1:10" x14ac:dyDescent="0.2">
@@ -24448,16 +24386,16 @@
         <v>758</v>
       </c>
       <c r="G16" t="s">
-        <v>948</v>
+        <v>947</v>
       </c>
       <c r="H16" t="s">
-        <v>973</v>
+        <v>972</v>
       </c>
       <c r="I16" t="s">
         <v>757</v>
       </c>
       <c r="J16" t="s">
-        <v>933</v>
+        <v>932</v>
       </c>
     </row>
     <row r="17" spans="1:10" x14ac:dyDescent="0.2">
@@ -24474,10 +24412,10 @@
         <v>772</v>
       </c>
       <c r="G17" t="s">
-        <v>941</v>
+        <v>940</v>
       </c>
       <c r="H17" t="s">
-        <v>961</v>
+        <v>960</v>
       </c>
     </row>
     <row r="18" spans="1:10" x14ac:dyDescent="0.2">
@@ -24494,10 +24432,10 @@
         <v>701</v>
       </c>
       <c r="G18" t="s">
-        <v>946</v>
+        <v>945</v>
       </c>
       <c r="H18" t="s">
-        <v>971</v>
+        <v>970</v>
       </c>
     </row>
     <row r="19" spans="1:10" x14ac:dyDescent="0.2">
@@ -24514,10 +24452,10 @@
         <v>693</v>
       </c>
       <c r="G19" t="s">
-        <v>947</v>
+        <v>946</v>
       </c>
       <c r="H19" t="s">
-        <v>972</v>
+        <v>971</v>
       </c>
     </row>
     <row r="21" spans="1:10" x14ac:dyDescent="0.2">
@@ -24537,10 +24475,10 @@
         <v>783</v>
       </c>
       <c r="G21" t="s">
-        <v>959</v>
+        <v>958</v>
       </c>
       <c r="H21" t="s">
-        <v>974</v>
+        <v>973</v>
       </c>
       <c r="I21" t="s">
         <v>782</v>
@@ -24560,10 +24498,10 @@
         <v>701</v>
       </c>
       <c r="G22" t="s">
-        <v>946</v>
+        <v>945</v>
       </c>
       <c r="H22" t="s">
-        <v>971</v>
+        <v>970</v>
       </c>
     </row>
     <row r="23" spans="1:10" x14ac:dyDescent="0.2">
@@ -24580,13 +24518,13 @@
         <v>693</v>
       </c>
       <c r="G23" t="s">
-        <v>947</v>
+        <v>946</v>
       </c>
       <c r="H23" t="s">
-        <v>972</v>
+        <v>971</v>
       </c>
       <c r="I23" t="s">
-        <v>937</v>
+        <v>936</v>
       </c>
     </row>
     <row r="24" spans="1:10" x14ac:dyDescent="0.2">
@@ -24603,10 +24541,10 @@
         <v>775</v>
       </c>
       <c r="G24" t="s">
-        <v>949</v>
+        <v>948</v>
       </c>
       <c r="H24" t="s">
-        <v>975</v>
+        <v>974</v>
       </c>
     </row>
     <row r="26" spans="1:10" x14ac:dyDescent="0.2">
@@ -24626,7 +24564,7 @@
         <v>785</v>
       </c>
       <c r="H26" t="s">
-        <v>934</v>
+        <v>933</v>
       </c>
       <c r="I26" t="s">
         <v>784</v>
@@ -24646,10 +24584,10 @@
         <v>770</v>
       </c>
       <c r="G27" t="s">
-        <v>950</v>
+        <v>949</v>
       </c>
       <c r="H27" t="s">
-        <v>976</v>
+        <v>975</v>
       </c>
     </row>
     <row r="28" spans="1:10" x14ac:dyDescent="0.2">
@@ -24666,10 +24604,10 @@
         <v>700</v>
       </c>
       <c r="G28" t="s">
-        <v>943</v>
+        <v>942</v>
       </c>
       <c r="H28" t="s">
-        <v>977</v>
+        <v>976</v>
       </c>
     </row>
     <row r="29" spans="1:10" x14ac:dyDescent="0.2">
@@ -24686,10 +24624,10 @@
         <v>773</v>
       </c>
       <c r="G29" t="s">
-        <v>951</v>
+        <v>950</v>
       </c>
       <c r="H29" t="s">
-        <v>978</v>
+        <v>977</v>
       </c>
     </row>
     <row r="31" spans="1:10" x14ac:dyDescent="0.2">
@@ -24712,16 +24650,16 @@
         <v>760</v>
       </c>
       <c r="G31" t="s">
-        <v>952</v>
+        <v>951</v>
       </c>
       <c r="H31" t="s">
-        <v>986</v>
+        <v>985</v>
       </c>
       <c r="I31" t="s">
         <v>755</v>
       </c>
       <c r="J31" t="s">
-        <v>926</v>
+        <v>925</v>
       </c>
     </row>
     <row r="32" spans="1:10" x14ac:dyDescent="0.2">
@@ -24738,10 +24676,10 @@
         <v>703</v>
       </c>
       <c r="G32" t="s">
-        <v>942</v>
+        <v>941</v>
       </c>
       <c r="H32" t="s">
-        <v>963</v>
+        <v>962</v>
       </c>
     </row>
     <row r="33" spans="1:10" x14ac:dyDescent="0.2">
@@ -24761,10 +24699,10 @@
         <v>701</v>
       </c>
       <c r="G33" t="s">
-        <v>946</v>
+        <v>945</v>
       </c>
       <c r="H33" t="s">
-        <v>971</v>
+        <v>970</v>
       </c>
     </row>
     <row r="34" spans="1:10" x14ac:dyDescent="0.2">
@@ -24781,10 +24719,10 @@
         <v>693</v>
       </c>
       <c r="G34" t="s">
-        <v>947</v>
+        <v>946</v>
       </c>
       <c r="H34" t="s">
-        <v>972</v>
+        <v>971</v>
       </c>
     </row>
     <row r="35" spans="1:10" x14ac:dyDescent="0.2">
@@ -24801,10 +24739,10 @@
         <v>694</v>
       </c>
       <c r="G35" t="s">
-        <v>945</v>
+        <v>944</v>
       </c>
       <c r="H35" t="s">
-        <v>968</v>
+        <v>967</v>
       </c>
     </row>
     <row r="36" spans="1:10" x14ac:dyDescent="0.2">
@@ -24821,10 +24759,10 @@
         <v>772</v>
       </c>
       <c r="G36" t="s">
-        <v>941</v>
+        <v>940</v>
       </c>
       <c r="H36" t="s">
-        <v>961</v>
+        <v>960</v>
       </c>
     </row>
     <row r="38" spans="1:10" x14ac:dyDescent="0.2">
@@ -24838,10 +24776,10 @@
         <v>728</v>
       </c>
       <c r="G38" t="s">
-        <v>934</v>
+        <v>933</v>
       </c>
       <c r="H38" t="s">
-        <v>934</v>
+        <v>933</v>
       </c>
     </row>
     <row r="39" spans="1:10" x14ac:dyDescent="0.2">
@@ -24864,16 +24802,16 @@
         <v>761</v>
       </c>
       <c r="G39" t="s">
-        <v>957</v>
+        <v>956</v>
       </c>
       <c r="H39" t="s">
-        <v>979</v>
+        <v>978</v>
       </c>
       <c r="I39" t="s">
         <v>756</v>
       </c>
       <c r="J39" t="s">
-        <v>932</v>
+        <v>931</v>
       </c>
     </row>
     <row r="40" spans="1:10" x14ac:dyDescent="0.2">
@@ -24890,10 +24828,10 @@
         <v>772</v>
       </c>
       <c r="G40" t="s">
-        <v>941</v>
+        <v>940</v>
       </c>
       <c r="H40" t="s">
-        <v>961</v>
+        <v>960</v>
       </c>
     </row>
     <row r="41" spans="1:10" x14ac:dyDescent="0.2">
@@ -24910,10 +24848,10 @@
         <v>771</v>
       </c>
       <c r="G41" t="s">
-        <v>944</v>
+        <v>943</v>
       </c>
       <c r="H41" t="s">
-        <v>967</v>
+        <v>966</v>
       </c>
     </row>
     <row r="42" spans="1:10" x14ac:dyDescent="0.2">
@@ -24930,10 +24868,10 @@
         <v>777</v>
       </c>
       <c r="G42" t="s">
-        <v>953</v>
+        <v>952</v>
       </c>
       <c r="H42" t="s">
-        <v>980</v>
+        <v>979</v>
       </c>
     </row>
     <row r="43" spans="1:10" x14ac:dyDescent="0.2">
@@ -24950,10 +24888,10 @@
         <v>701</v>
       </c>
       <c r="G43" t="s">
-        <v>946</v>
+        <v>945</v>
       </c>
       <c r="H43" t="s">
-        <v>971</v>
+        <v>970</v>
       </c>
     </row>
     <row r="44" spans="1:10" x14ac:dyDescent="0.2">
@@ -24970,10 +24908,10 @@
         <v>693</v>
       </c>
       <c r="G44" t="s">
-        <v>947</v>
+        <v>946</v>
       </c>
       <c r="H44" t="s">
-        <v>972</v>
+        <v>971</v>
       </c>
     </row>
     <row r="45" spans="1:10" x14ac:dyDescent="0.2">
@@ -24987,7 +24925,7 @@
         <v>712</v>
       </c>
       <c r="H45" t="s">
-        <v>934</v>
+        <v>933</v>
       </c>
     </row>
     <row r="46" spans="1:10" x14ac:dyDescent="0.2">
@@ -25001,7 +24939,7 @@
         <v>730</v>
       </c>
       <c r="H46" t="s">
-        <v>934</v>
+        <v>933</v>
       </c>
     </row>
     <row r="48" spans="1:10" s="23" customFormat="1" x14ac:dyDescent="0.2">
@@ -25021,16 +24959,16 @@
         <v>768</v>
       </c>
       <c r="G48" s="23" t="s">
-        <v>954</v>
+        <v>953</v>
       </c>
       <c r="H48" s="23" t="s">
-        <v>984</v>
+        <v>983</v>
       </c>
       <c r="I48" s="23" t="s">
         <v>769</v>
       </c>
       <c r="J48" s="23" t="s">
-        <v>929</v>
+        <v>928</v>
       </c>
     </row>
     <row r="49" spans="1:10" s="23" customFormat="1" x14ac:dyDescent="0.2">
@@ -25041,10 +24979,10 @@
         <v>725</v>
       </c>
       <c r="G49" s="23" t="s">
-        <v>941</v>
+        <v>940</v>
       </c>
       <c r="H49" s="23" t="s">
-        <v>961</v>
+        <v>960</v>
       </c>
     </row>
     <row r="50" spans="1:10" s="23" customFormat="1" x14ac:dyDescent="0.2">
@@ -25055,10 +24993,10 @@
         <v>143</v>
       </c>
       <c r="G50" s="23" t="s">
-        <v>946</v>
+        <v>945</v>
       </c>
       <c r="H50" s="23" t="s">
-        <v>971</v>
+        <v>970</v>
       </c>
     </row>
     <row r="52" spans="1:10" s="23" customFormat="1" x14ac:dyDescent="0.2">
@@ -25080,7 +25018,7 @@
         <v>748</v>
       </c>
       <c r="H54" s="23" t="s">
-        <v>934</v>
+        <v>933</v>
       </c>
     </row>
     <row r="55" spans="1:10" s="23" customFormat="1" x14ac:dyDescent="0.2">
@@ -25094,16 +25032,16 @@
         <v>765</v>
       </c>
       <c r="G55" s="23" t="s">
-        <v>955</v>
+        <v>954</v>
       </c>
       <c r="H55" s="23" t="s">
-        <v>981</v>
+        <v>980</v>
       </c>
       <c r="I55" s="23" t="s">
         <v>764</v>
       </c>
       <c r="J55" s="23" t="s">
-        <v>928</v>
+        <v>927</v>
       </c>
     </row>
     <row r="56" spans="1:10" s="23" customFormat="1" x14ac:dyDescent="0.2">
@@ -25114,7 +25052,7 @@
         <v>751</v>
       </c>
       <c r="H56" s="23" t="s">
-        <v>934</v>
+        <v>933</v>
       </c>
     </row>
     <row r="57" spans="1:10" s="23" customFormat="1" x14ac:dyDescent="0.2">
@@ -25125,7 +25063,7 @@
         <v>752</v>
       </c>
       <c r="H57" s="23" t="s">
-        <v>934</v>
+        <v>933</v>
       </c>
     </row>
     <row r="58" spans="1:10" s="23" customFormat="1" x14ac:dyDescent="0.2">
@@ -25136,7 +25074,7 @@
         <v>749</v>
       </c>
       <c r="H58" s="23" t="s">
-        <v>934</v>
+        <v>933</v>
       </c>
     </row>
     <row r="59" spans="1:10" s="23" customFormat="1" x14ac:dyDescent="0.2">
@@ -25147,7 +25085,7 @@
         <v>750</v>
       </c>
       <c r="H59" s="23" t="s">
-        <v>934</v>
+        <v>933</v>
       </c>
     </row>
     <row r="61" spans="1:10" s="23" customFormat="1" x14ac:dyDescent="0.2">
@@ -25164,16 +25102,16 @@
         <v>781</v>
       </c>
       <c r="G61" s="23" t="s">
-        <v>958</v>
+        <v>957</v>
       </c>
       <c r="H61" s="23" t="s">
-        <v>982</v>
+        <v>981</v>
       </c>
       <c r="I61" s="23" t="s">
         <v>780</v>
       </c>
       <c r="J61" s="23" t="s">
-        <v>926</v>
+        <v>925</v>
       </c>
     </row>
     <row r="62" spans="1:10" s="23" customFormat="1" x14ac:dyDescent="0.2">
@@ -25184,10 +25122,10 @@
         <v>725</v>
       </c>
       <c r="G62" s="23" t="s">
-        <v>941</v>
+        <v>940</v>
       </c>
       <c r="H62" s="23" t="s">
-        <v>961</v>
+        <v>960</v>
       </c>
     </row>
     <row r="63" spans="1:10" s="23" customFormat="1" x14ac:dyDescent="0.2">
@@ -25198,10 +25136,10 @@
         <v>713</v>
       </c>
       <c r="G63" s="23" t="s">
-        <v>947</v>
+        <v>946</v>
       </c>
       <c r="H63" s="23" t="s">
-        <v>972</v>
+        <v>971</v>
       </c>
     </row>
     <row r="64" spans="1:10" s="23" customFormat="1" x14ac:dyDescent="0.2">
@@ -25212,10 +25150,10 @@
         <v>143</v>
       </c>
       <c r="G64" s="23" t="s">
-        <v>946</v>
+        <v>945</v>
       </c>
       <c r="H64" s="23" t="s">
-        <v>971</v>
+        <v>970</v>
       </c>
     </row>
     <row r="66" spans="1:10" s="23" customFormat="1" x14ac:dyDescent="0.2">
@@ -25239,8 +25177,8 @@
       <c r="F68" s="23" t="s">
         <v>767</v>
       </c>
-      <c r="H68" s="44" t="s">
-        <v>985</v>
+      <c r="H68" s="43" t="s">
+        <v>984</v>
       </c>
       <c r="I68" s="23" t="s">
         <v>766</v>
@@ -25254,10 +25192,10 @@
         <v>471</v>
       </c>
       <c r="G69" s="23" t="s">
-        <v>942</v>
+        <v>941</v>
       </c>
       <c r="H69" s="23" t="s">
-        <v>963</v>
+        <v>962</v>
       </c>
     </row>
     <row r="70" spans="1:10" s="23" customFormat="1" x14ac:dyDescent="0.2">
@@ -25268,10 +25206,10 @@
         <v>143</v>
       </c>
       <c r="G70" s="23" t="s">
-        <v>946</v>
+        <v>945</v>
       </c>
       <c r="H70" s="23" t="s">
-        <v>971</v>
+        <v>970</v>
       </c>
     </row>
     <row r="71" spans="1:10" s="23" customFormat="1" x14ac:dyDescent="0.2">
@@ -25282,10 +25220,10 @@
         <v>713</v>
       </c>
       <c r="G71" s="23" t="s">
-        <v>947</v>
+        <v>946</v>
       </c>
       <c r="H71" s="23" t="s">
-        <v>972</v>
+        <v>971</v>
       </c>
     </row>
     <row r="73" spans="1:10" s="23" customFormat="1" x14ac:dyDescent="0.2">
@@ -25305,16 +25243,16 @@
         <v>765</v>
       </c>
       <c r="G73" s="23" t="s">
-        <v>955</v>
+        <v>954</v>
       </c>
       <c r="H73" s="23" t="s">
-        <v>981</v>
+        <v>980</v>
       </c>
       <c r="I73" s="23" t="s">
+        <v>926</v>
+      </c>
+      <c r="J73" s="23" t="s">
         <v>927</v>
-      </c>
-      <c r="J73" s="23" t="s">
-        <v>928</v>
       </c>
     </row>
     <row r="74" spans="1:10" s="23" customFormat="1" x14ac:dyDescent="0.2">
@@ -25325,10 +25263,10 @@
         <v>729</v>
       </c>
       <c r="G74" s="23" t="s">
-        <v>953</v>
+        <v>952</v>
       </c>
       <c r="H74" s="23" t="s">
-        <v>980</v>
+        <v>979</v>
       </c>
     </row>
     <row r="75" spans="1:10" s="23" customFormat="1" x14ac:dyDescent="0.2">
@@ -25339,10 +25277,10 @@
         <v>725</v>
       </c>
       <c r="G75" s="23" t="s">
-        <v>941</v>
+        <v>940</v>
       </c>
       <c r="H75" s="23" t="s">
-        <v>961</v>
+        <v>960</v>
       </c>
     </row>
     <row r="77" spans="1:10" s="23" customFormat="1" x14ac:dyDescent="0.2">
@@ -25359,10 +25297,10 @@
         <v>763</v>
       </c>
       <c r="G77" s="23" t="s">
-        <v>956</v>
+        <v>955</v>
       </c>
       <c r="H77" s="23" t="s">
-        <v>983</v>
+        <v>982</v>
       </c>
       <c r="I77" s="23" t="s">
         <v>762</v>
@@ -25376,10 +25314,10 @@
         <v>725</v>
       </c>
       <c r="G78" s="23" t="s">
-        <v>941</v>
+        <v>940</v>
       </c>
       <c r="H78" s="23" t="s">
-        <v>961</v>
+        <v>960</v>
       </c>
     </row>
     <row r="79" spans="1:10" s="23" customFormat="1" x14ac:dyDescent="0.2">
@@ -25390,10 +25328,10 @@
         <v>143</v>
       </c>
       <c r="G79" s="23" t="s">
-        <v>946</v>
+        <v>945</v>
       </c>
       <c r="H79" s="23" t="s">
-        <v>971</v>
+        <v>970</v>
       </c>
     </row>
     <row r="80" spans="1:10" s="23" customFormat="1" x14ac:dyDescent="0.2">
@@ -25404,10 +25342,10 @@
         <v>713</v>
       </c>
       <c r="G80" s="23" t="s">
-        <v>947</v>
+        <v>946</v>
       </c>
       <c r="H80" s="23" t="s">
-        <v>972</v>
+        <v>971</v>
       </c>
     </row>
     <row r="82" spans="1:2" s="23" customFormat="1" x14ac:dyDescent="0.2">

</xml_diff>

<commit_message>
Addition of missing IDs to various classes
</commit_message>
<xml_diff>
--- a/data/mapping_config_files/nwss_to_odm_v2_mapping.xlsx
+++ b/data/mapping_config_files/nwss_to_odm_v2_mapping.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/martinwellman/Documents/Health/Wastewater/PHES-ODM-MapGenerator/PHES-ODM-MapGenerator/data/mapping_config_files/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C5389CD7-1A3A-0242-923B-0879027E46CC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{982605AD-774C-2D45-A0B2-4A681470F99A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="500" windowWidth="40960" windowHeight="20860" xr2:uid="{77810E24-F86B-BC44-A0D5-8790E6EC60B4}"/>
   </bookViews>
@@ -53,7 +53,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3228" uniqueCount="986">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3248" uniqueCount="985">
   <si>
     <t>Reporter</t>
   </si>
@@ -2725,9 +2725,6 @@
   </si>
   <si>
     <t>lastEdited</t>
-  </si>
-  <si>
-    <t>{{id:datasetID}}</t>
   </si>
   <si>
     <t>{{id:addressID}}</t>
@@ -3252,7 +3249,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="45">
+  <cellXfs count="44">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1"/>
@@ -3329,7 +3326,6 @@
       <alignment wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="6" fillId="6" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -14497,7 +14493,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{3154BFCE-06D9-9649-B340-B23DCF20DD83}">
-  <dimension ref="A1:K104"/>
+  <dimension ref="A1:K108"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="2" max="2" width="13" bestFit="1" customWidth="1"/>
@@ -14571,7 +14567,7 @@
         <v>630</v>
       </c>
       <c r="C3" s="25" t="s">
-        <v>772</v>
+        <v>54</v>
       </c>
       <c r="E3" s="25" t="s">
         <v>78</v>
@@ -14580,7 +14576,7 @@
         <v>725</v>
       </c>
       <c r="G3" s="25" t="s">
-        <v>875</v>
+        <v>701</v>
       </c>
     </row>
     <row r="4" spans="1:10" s="25" customFormat="1" x14ac:dyDescent="0.2">
@@ -14600,7 +14596,7 @@
         <v>729</v>
       </c>
       <c r="G4" s="25" t="s">
-        <v>876</v>
+        <v>875</v>
       </c>
     </row>
     <row r="5" spans="1:10" s="25" customFormat="1" x14ac:dyDescent="0.2"/>
@@ -14631,17 +14627,18 @@
       <c r="B7" s="25" t="s">
         <v>630</v>
       </c>
-      <c r="C7" s="25" t="s">
-        <v>772</v>
-      </c>
-      <c r="E7" s="25" t="s">
+      <c r="C7" s="28" t="s">
+        <v>54</v>
+      </c>
+      <c r="D7" s="28"/>
+      <c r="E7" s="28" t="s">
         <v>739</v>
       </c>
-      <c r="F7" s="25" t="s">
+      <c r="F7" s="28" t="s">
         <v>725</v>
       </c>
-      <c r="G7" s="25" t="s">
-        <v>875</v>
+      <c r="G7" s="28" t="s">
+        <v>701</v>
       </c>
     </row>
     <row r="8" spans="1:10" s="25" customFormat="1" x14ac:dyDescent="0.2">
@@ -14675,7 +14672,7 @@
         <v>739</v>
       </c>
       <c r="F9" s="25" t="s">
-        <v>879</v>
+        <v>878</v>
       </c>
     </row>
     <row r="10" spans="1:10" s="25" customFormat="1" x14ac:dyDescent="0.2">
@@ -14689,7 +14686,7 @@
         <v>739</v>
       </c>
       <c r="F10" s="25" t="s">
-        <v>880</v>
+        <v>879</v>
       </c>
     </row>
     <row r="11" spans="1:10" s="25" customFormat="1" x14ac:dyDescent="0.2">
@@ -14703,7 +14700,7 @@
         <v>739</v>
       </c>
       <c r="F11" s="25" t="s">
-        <v>881</v>
+        <v>880</v>
       </c>
     </row>
     <row r="12" spans="1:10" s="25" customFormat="1" x14ac:dyDescent="0.2">
@@ -14717,7 +14714,7 @@
         <v>739</v>
       </c>
       <c r="F12" s="25" t="s">
-        <v>882</v>
+        <v>881</v>
       </c>
     </row>
     <row r="13" spans="1:10" s="25" customFormat="1" x14ac:dyDescent="0.2">
@@ -14731,7 +14728,7 @@
         <v>739</v>
       </c>
       <c r="F13" s="25" t="s">
-        <v>883</v>
+        <v>882</v>
       </c>
     </row>
     <row r="14" spans="1:10" s="25" customFormat="1" x14ac:dyDescent="0.2">
@@ -14771,7 +14768,7 @@
         <v>630</v>
       </c>
       <c r="C17" s="25" t="s">
-        <v>772</v>
+        <v>54</v>
       </c>
       <c r="D17" s="25"/>
       <c r="E17" s="25" t="s">
@@ -14781,7 +14778,7 @@
         <v>725</v>
       </c>
       <c r="G17" s="25" t="s">
-        <v>875</v>
+        <v>701</v>
       </c>
     </row>
     <row r="18" spans="1:11" x14ac:dyDescent="0.2">
@@ -14800,18 +14797,18 @@
       <c r="B19" s="25" t="s">
         <v>630</v>
       </c>
-      <c r="C19" s="25" t="s">
-        <v>772</v>
-      </c>
-      <c r="D19" s="25"/>
-      <c r="E19" s="25" t="s">
+      <c r="C19" s="28" t="s">
+        <v>54</v>
+      </c>
+      <c r="D19" s="28"/>
+      <c r="E19" s="28" t="s">
         <v>740</v>
       </c>
-      <c r="F19" s="25" t="s">
+      <c r="F19" s="28" t="s">
         <v>725</v>
       </c>
-      <c r="G19" s="25" t="s">
-        <v>875</v>
+      <c r="G19" s="28" t="s">
+        <v>701</v>
       </c>
     </row>
     <row r="20" spans="1:11" s="25" customFormat="1" x14ac:dyDescent="0.2">
@@ -14851,7 +14848,7 @@
         <v>735</v>
       </c>
       <c r="G21" s="25" t="s">
-        <v>878</v>
+        <v>877</v>
       </c>
     </row>
     <row r="22" spans="1:11" s="25" customFormat="1" x14ac:dyDescent="0.2">
@@ -14882,17 +14879,18 @@
       <c r="B24" s="25" t="s">
         <v>630</v>
       </c>
-      <c r="C24" s="25" t="s">
-        <v>772</v>
-      </c>
-      <c r="E24" s="25" t="s">
+      <c r="C24" s="28" t="s">
+        <v>54</v>
+      </c>
+      <c r="D24" s="28"/>
+      <c r="E24" s="28" t="s">
         <v>114</v>
       </c>
-      <c r="F24" s="25" t="s">
+      <c r="F24" s="28" t="s">
         <v>725</v>
       </c>
-      <c r="G24" s="25" t="s">
-        <v>875</v>
+      <c r="G24" s="28" t="s">
+        <v>701</v>
       </c>
     </row>
     <row r="25" spans="1:11" s="25" customFormat="1" x14ac:dyDescent="0.2">
@@ -14912,7 +14910,7 @@
         <v>726</v>
       </c>
       <c r="G25" s="25" t="s">
-        <v>877</v>
+        <v>876</v>
       </c>
     </row>
     <row r="26" spans="1:11" s="25" customFormat="1" x14ac:dyDescent="0.2">
@@ -14995,7 +14993,6 @@
       <c r="G29" s="25" t="s">
         <v>700</v>
       </c>
-      <c r="K29" s="44"/>
     </row>
     <row r="30" spans="1:11" s="25" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A30" s="25" t="b">
@@ -15054,7 +15051,7 @@
         <v>726</v>
       </c>
       <c r="G33" s="25" t="s">
-        <v>877</v>
+        <v>876</v>
       </c>
       <c r="H33" s="30"/>
     </row>
@@ -15189,7 +15186,7 @@
         <v>729</v>
       </c>
       <c r="G41" s="25" t="s">
-        <v>876</v>
+        <v>875</v>
       </c>
     </row>
     <row r="42" spans="1:8" s="25" customFormat="1" x14ac:dyDescent="0.2">
@@ -15199,17 +15196,18 @@
       <c r="B42" s="25" t="s">
         <v>630</v>
       </c>
-      <c r="C42" s="25" t="s">
-        <v>772</v>
-      </c>
-      <c r="E42" s="25" t="s">
+      <c r="C42" s="28" t="s">
+        <v>54</v>
+      </c>
+      <c r="D42" s="28"/>
+      <c r="E42" s="28" t="s">
         <v>723</v>
       </c>
-      <c r="F42" s="25" t="s">
+      <c r="F42" s="28" t="s">
         <v>725</v>
       </c>
-      <c r="G42" s="25" t="s">
-        <v>875</v>
+      <c r="G42" s="28" t="s">
+        <v>701</v>
       </c>
     </row>
     <row r="43" spans="1:8" s="25" customFormat="1" x14ac:dyDescent="0.2">
@@ -15290,17 +15288,18 @@
       <c r="B49" s="25" t="s">
         <v>630</v>
       </c>
-      <c r="C49" s="25" t="s">
-        <v>772</v>
-      </c>
-      <c r="E49" s="25" t="s">
+      <c r="C49" s="28" t="s">
+        <v>54</v>
+      </c>
+      <c r="D49" s="28"/>
+      <c r="E49" s="28" t="s">
         <v>474</v>
       </c>
-      <c r="F49" s="25" t="s">
+      <c r="F49" s="28" t="s">
         <v>725</v>
       </c>
-      <c r="G49" s="25" t="s">
-        <v>875</v>
+      <c r="G49" s="28" t="s">
+        <v>701</v>
       </c>
     </row>
     <row r="50" spans="1:11" s="25" customFormat="1" x14ac:dyDescent="0.2">
@@ -15443,7 +15442,7 @@
         <v>735</v>
       </c>
       <c r="G57" s="25" t="s">
-        <v>878</v>
+        <v>877</v>
       </c>
     </row>
     <row r="58" spans="1:11" s="25" customFormat="1" x14ac:dyDescent="0.2"/>
@@ -15522,7 +15521,7 @@
         <v>144</v>
       </c>
       <c r="H62" s="25" t="s">
-        <v>922</v>
+        <v>921</v>
       </c>
     </row>
     <row r="63" spans="1:11" s="25" customFormat="1" x14ac:dyDescent="0.2">
@@ -15606,37 +15605,36 @@
         <v>694</v>
       </c>
     </row>
-    <row r="67" spans="1:10" s="25" customFormat="1" x14ac:dyDescent="0.2"/>
-    <row r="68" spans="1:10" s="17" customFormat="1" ht="17" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A68" s="17" t="b">
-        <v>0</v>
-      </c>
-      <c r="B68" s="17" t="s">
-        <v>630</v>
-      </c>
-      <c r="C68" s="26" t="s">
-        <v>44</v>
-      </c>
-      <c r="E68" s="17" t="s">
+    <row r="67" spans="1:10" s="25" customFormat="1" x14ac:dyDescent="0.2">
+      <c r="A67" s="25" t="b">
+        <v>1</v>
+      </c>
+      <c r="B67" s="25" t="s">
+        <v>630</v>
+      </c>
+      <c r="C67" s="25" t="s">
+        <v>73</v>
+      </c>
+      <c r="E67" s="25" t="s">
         <v>117</v>
       </c>
-      <c r="F68" s="17" t="s">
-        <v>137</v>
-      </c>
-      <c r="H68" s="27"/>
-      <c r="J68" s="17" t="s">
-        <v>138</v>
-      </c>
-    </row>
-    <row r="69" spans="1:10" s="17" customFormat="1" ht="16" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="F67" s="25" t="s">
+        <v>471</v>
+      </c>
+      <c r="G67" s="25" t="s">
+        <v>703</v>
+      </c>
+    </row>
+    <row r="68" spans="1:10" s="25" customFormat="1" x14ac:dyDescent="0.2"/>
+    <row r="69" spans="1:10" s="17" customFormat="1" ht="17" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A69" s="17" t="b">
         <v>0</v>
       </c>
       <c r="B69" s="17" t="s">
         <v>630</v>
       </c>
-      <c r="C69" s="17" t="s">
-        <v>45</v>
+      <c r="C69" s="26" t="s">
+        <v>44</v>
       </c>
       <c r="E69" s="17" t="s">
         <v>117</v>
@@ -15649,7 +15647,7 @@
         <v>138</v>
       </c>
     </row>
-    <row r="70" spans="1:10" s="17" customFormat="1" x14ac:dyDescent="0.2">
+    <row r="70" spans="1:10" s="17" customFormat="1" ht="16" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A70" s="17" t="b">
         <v>0</v>
       </c>
@@ -15657,7 +15655,7 @@
         <v>630</v>
       </c>
       <c r="C70" s="17" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="E70" s="17" t="s">
         <v>117</v>
@@ -15665,31 +15663,32 @@
       <c r="F70" s="17" t="s">
         <v>137</v>
       </c>
+      <c r="H70" s="27"/>
       <c r="J70" s="17" t="s">
         <v>138</v>
       </c>
     </row>
-    <row r="71" spans="1:10" s="25" customFormat="1" x14ac:dyDescent="0.2"/>
-    <row r="72" spans="1:10" s="25" customFormat="1" x14ac:dyDescent="0.2">
-      <c r="A72" s="25" t="b">
-        <v>1</v>
-      </c>
-      <c r="B72" s="25" t="s">
-        <v>630</v>
-      </c>
-      <c r="C72" s="25" t="s">
-        <v>772</v>
-      </c>
-      <c r="E72" s="25" t="s">
+    <row r="71" spans="1:10" s="17" customFormat="1" x14ac:dyDescent="0.2">
+      <c r="A71" s="17" t="b">
+        <v>0</v>
+      </c>
+      <c r="B71" s="17" t="s">
+        <v>630</v>
+      </c>
+      <c r="C71" s="17" t="s">
+        <v>46</v>
+      </c>
+      <c r="E71" s="17" t="s">
         <v>117</v>
       </c>
-      <c r="F72" s="25" t="s">
-        <v>725</v>
-      </c>
-      <c r="G72" s="25" t="s">
-        <v>875</v>
-      </c>
-    </row>
+      <c r="F71" s="17" t="s">
+        <v>137</v>
+      </c>
+      <c r="J71" s="17" t="s">
+        <v>138</v>
+      </c>
+    </row>
+    <row r="72" spans="1:10" s="25" customFormat="1" x14ac:dyDescent="0.2"/>
     <row r="73" spans="1:10" s="25" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A73" s="25" t="b">
         <v>1</v>
@@ -15697,20 +15696,18 @@
       <c r="B73" s="25" t="s">
         <v>630</v>
       </c>
-      <c r="C73" s="25" t="s">
-        <v>24</v>
-      </c>
-      <c r="D73" s="33" t="s">
-        <v>121</v>
-      </c>
-      <c r="E73" s="25" t="s">
+      <c r="C73" s="28" t="s">
+        <v>54</v>
+      </c>
+      <c r="D73" s="28"/>
+      <c r="E73" s="28" t="s">
         <v>117</v>
       </c>
-      <c r="F73" s="25" t="s">
-        <v>129</v>
-      </c>
-      <c r="G73" s="25" t="s">
-        <v>136</v>
+      <c r="F73" s="28" t="s">
+        <v>725</v>
+      </c>
+      <c r="G73" s="28" t="s">
+        <v>701</v>
       </c>
     </row>
     <row r="74" spans="1:10" s="25" customFormat="1" x14ac:dyDescent="0.2">
@@ -15723,8 +15720,8 @@
       <c r="C74" s="25" t="s">
         <v>24</v>
       </c>
-      <c r="D74" s="32" t="s">
-        <v>122</v>
+      <c r="D74" s="33" t="s">
+        <v>121</v>
       </c>
       <c r="E74" s="25" t="s">
         <v>117</v>
@@ -15733,7 +15730,7 @@
         <v>129</v>
       </c>
       <c r="G74" s="25" t="s">
-        <v>134</v>
+        <v>136</v>
       </c>
     </row>
     <row r="75" spans="1:10" s="25" customFormat="1" x14ac:dyDescent="0.2">
@@ -15747,7 +15744,7 @@
         <v>24</v>
       </c>
       <c r="D75" s="32" t="s">
-        <v>123</v>
+        <v>122</v>
       </c>
       <c r="E75" s="25" t="s">
         <v>117</v>
@@ -15756,7 +15753,7 @@
         <v>129</v>
       </c>
       <c r="G75" s="25" t="s">
-        <v>130</v>
+        <v>134</v>
       </c>
     </row>
     <row r="76" spans="1:10" s="25" customFormat="1" x14ac:dyDescent="0.2">
@@ -15770,7 +15767,7 @@
         <v>24</v>
       </c>
       <c r="D76" s="32" t="s">
-        <v>124</v>
+        <v>123</v>
       </c>
       <c r="E76" s="25" t="s">
         <v>117</v>
@@ -15779,7 +15776,7 @@
         <v>129</v>
       </c>
       <c r="G76" s="25" t="s">
-        <v>131</v>
+        <v>130</v>
       </c>
     </row>
     <row r="77" spans="1:10" s="25" customFormat="1" x14ac:dyDescent="0.2">
@@ -15793,7 +15790,7 @@
         <v>24</v>
       </c>
       <c r="D77" s="32" t="s">
-        <v>125</v>
+        <v>124</v>
       </c>
       <c r="E77" s="25" t="s">
         <v>117</v>
@@ -15802,7 +15799,7 @@
         <v>129</v>
       </c>
       <c r="G77" s="25" t="s">
-        <v>132</v>
+        <v>131</v>
       </c>
     </row>
     <row r="78" spans="1:10" s="25" customFormat="1" x14ac:dyDescent="0.2">
@@ -15816,7 +15813,7 @@
         <v>24</v>
       </c>
       <c r="D78" s="32" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
       <c r="E78" s="25" t="s">
         <v>117</v>
@@ -15825,7 +15822,7 @@
         <v>129</v>
       </c>
       <c r="G78" s="25" t="s">
-        <v>133</v>
+        <v>132</v>
       </c>
     </row>
     <row r="79" spans="1:10" s="25" customFormat="1" x14ac:dyDescent="0.2">
@@ -15839,7 +15836,7 @@
         <v>24</v>
       </c>
       <c r="D79" s="32" t="s">
-        <v>127</v>
+        <v>126</v>
       </c>
       <c r="E79" s="25" t="s">
         <v>117</v>
@@ -15848,7 +15845,7 @@
         <v>129</v>
       </c>
       <c r="G79" s="25" t="s">
-        <v>127</v>
+        <v>133</v>
       </c>
     </row>
     <row r="80" spans="1:10" s="25" customFormat="1" x14ac:dyDescent="0.2">
@@ -15862,7 +15859,7 @@
         <v>24</v>
       </c>
       <c r="D80" s="32" t="s">
-        <v>128</v>
+        <v>127</v>
       </c>
       <c r="E80" s="25" t="s">
         <v>117</v>
@@ -15871,31 +15868,34 @@
         <v>129</v>
       </c>
       <c r="G80" s="25" t="s">
+        <v>127</v>
+      </c>
+    </row>
+    <row r="81" spans="1:10" s="25" customFormat="1" x14ac:dyDescent="0.2">
+      <c r="A81" s="25" t="b">
+        <v>1</v>
+      </c>
+      <c r="B81" s="25" t="s">
+        <v>630</v>
+      </c>
+      <c r="C81" s="25" t="s">
+        <v>24</v>
+      </c>
+      <c r="D81" s="32" t="s">
+        <v>128</v>
+      </c>
+      <c r="E81" s="25" t="s">
+        <v>117</v>
+      </c>
+      <c r="F81" s="25" t="s">
+        <v>129</v>
+      </c>
+      <c r="G81" s="25" t="s">
         <v>135</v>
       </c>
     </row>
-    <row r="81" spans="1:10" s="25" customFormat="1" x14ac:dyDescent="0.2">
-      <c r="D81" s="32"/>
-    </row>
     <row r="82" spans="1:10" s="25" customFormat="1" x14ac:dyDescent="0.2">
-      <c r="A82" s="25" t="b">
-        <v>1</v>
-      </c>
-      <c r="B82" s="25" t="s">
-        <v>630</v>
-      </c>
-      <c r="C82" s="25" t="s">
-        <v>9</v>
-      </c>
-      <c r="E82" s="41" t="s">
-        <v>76</v>
-      </c>
-      <c r="F82" s="41" t="s">
-        <v>120</v>
-      </c>
-      <c r="H82" s="30" t="s">
-        <v>722</v>
-      </c>
+      <c r="D82" s="32"/>
     </row>
     <row r="83" spans="1:10" s="25" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A83" s="25" t="b">
@@ -15905,16 +15905,16 @@
         <v>630</v>
       </c>
       <c r="C83" s="25" t="s">
-        <v>11</v>
-      </c>
-      <c r="E83" s="25" t="s">
+        <v>9</v>
+      </c>
+      <c r="E83" s="41" t="s">
         <v>76</v>
       </c>
-      <c r="F83" s="25" t="s">
-        <v>80</v>
-      </c>
-      <c r="G83" s="25" t="s">
-        <v>696</v>
+      <c r="F83" s="41" t="s">
+        <v>120</v>
+      </c>
+      <c r="H83" s="30" t="s">
+        <v>722</v>
       </c>
     </row>
     <row r="84" spans="1:10" s="25" customFormat="1" x14ac:dyDescent="0.2">
@@ -15925,16 +15925,16 @@
         <v>630</v>
       </c>
       <c r="C84" s="25" t="s">
-        <v>8</v>
+        <v>11</v>
       </c>
       <c r="E84" s="25" t="s">
         <v>76</v>
       </c>
       <c r="F84" s="25" t="s">
-        <v>77</v>
+        <v>80</v>
       </c>
       <c r="G84" s="25" t="s">
-        <v>694</v>
+        <v>696</v>
       </c>
     </row>
     <row r="85" spans="1:10" s="25" customFormat="1" x14ac:dyDescent="0.2">
@@ -15945,16 +15945,16 @@
         <v>630</v>
       </c>
       <c r="C85" s="25" t="s">
-        <v>54</v>
+        <v>8</v>
       </c>
       <c r="E85" s="25" t="s">
         <v>76</v>
       </c>
       <c r="F85" s="25" t="s">
-        <v>712</v>
+        <v>77</v>
       </c>
       <c r="G85" s="25" t="s">
-        <v>701</v>
+        <v>694</v>
       </c>
     </row>
     <row r="86" spans="1:10" s="25" customFormat="1" x14ac:dyDescent="0.2">
@@ -15965,19 +15965,19 @@
         <v>630</v>
       </c>
       <c r="C86" s="25" t="s">
-        <v>18</v>
+        <v>54</v>
       </c>
       <c r="E86" s="25" t="s">
         <v>76</v>
       </c>
       <c r="F86" s="25" t="s">
-        <v>115</v>
+        <v>712</v>
       </c>
       <c r="G86" s="25" t="s">
-        <v>697</v>
-      </c>
-    </row>
-    <row r="87" spans="1:10" s="25" customFormat="1" ht="17" customHeight="1" x14ac:dyDescent="0.2">
+        <v>701</v>
+      </c>
+    </row>
+    <row r="87" spans="1:10" s="25" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A87" s="25" t="b">
         <v>1</v>
       </c>
@@ -15985,20 +15985,19 @@
         <v>630</v>
       </c>
       <c r="C87" s="25" t="s">
-        <v>13</v>
-      </c>
-      <c r="D87" s="32"/>
+        <v>18</v>
+      </c>
       <c r="E87" s="25" t="s">
         <v>76</v>
       </c>
       <c r="F87" s="25" t="s">
-        <v>83</v>
-      </c>
-      <c r="H87" s="42" t="s">
-        <v>862</v>
-      </c>
-    </row>
-    <row r="88" spans="1:10" s="25" customFormat="1" x14ac:dyDescent="0.2">
+        <v>115</v>
+      </c>
+      <c r="G87" s="25" t="s">
+        <v>697</v>
+      </c>
+    </row>
+    <row r="88" spans="1:10" s="25" customFormat="1" ht="17" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A88" s="25" t="b">
         <v>1</v>
       </c>
@@ -16006,43 +16005,39 @@
         <v>630</v>
       </c>
       <c r="C88" s="25" t="s">
-        <v>772</v>
-      </c>
+        <v>13</v>
+      </c>
+      <c r="D88" s="32"/>
       <c r="E88" s="25" t="s">
         <v>76</v>
       </c>
       <c r="F88" s="25" t="s">
+        <v>83</v>
+      </c>
+      <c r="H88" s="42" t="s">
+        <v>862</v>
+      </c>
+    </row>
+    <row r="89" spans="1:10" s="25" customFormat="1" x14ac:dyDescent="0.2">
+      <c r="A89" s="25" t="b">
+        <v>1</v>
+      </c>
+      <c r="B89" s="25" t="s">
+        <v>630</v>
+      </c>
+      <c r="C89" s="28" t="s">
+        <v>54</v>
+      </c>
+      <c r="D89" s="28"/>
+      <c r="E89" s="28" t="s">
+        <v>76</v>
+      </c>
+      <c r="F89" s="28" t="s">
         <v>725</v>
       </c>
-      <c r="G88" s="25" t="s">
-        <v>875</v>
-      </c>
-    </row>
-    <row r="89" spans="1:10" s="17" customFormat="1" ht="17" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A89" s="25" t="b">
-        <v>1</v>
-      </c>
-      <c r="B89" s="25" t="s">
-        <v>630</v>
-      </c>
-      <c r="C89" s="25" t="s">
-        <v>15</v>
-      </c>
-      <c r="D89" s="33" t="s">
-        <v>84</v>
-      </c>
-      <c r="E89" s="25" t="s">
-        <v>76</v>
-      </c>
-      <c r="F89" s="25" t="s">
-        <v>100</v>
-      </c>
-      <c r="G89" s="25" t="s">
-        <v>75</v>
-      </c>
-      <c r="H89" s="25"/>
-      <c r="I89" s="25"/>
-      <c r="J89" s="25"/>
+      <c r="G89" s="28" t="s">
+        <v>701</v>
+      </c>
     </row>
     <row r="90" spans="1:10" s="25" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A90" s="25" t="b">
@@ -16052,19 +16047,16 @@
         <v>630</v>
       </c>
       <c r="C90" s="25" t="s">
-        <v>15</v>
-      </c>
-      <c r="D90" s="33" t="s">
-        <v>85</v>
+        <v>777</v>
       </c>
       <c r="E90" s="25" t="s">
         <v>76</v>
       </c>
       <c r="F90" s="25" t="s">
-        <v>100</v>
+        <v>729</v>
       </c>
       <c r="G90" s="25" t="s">
-        <v>101</v>
+        <v>875</v>
       </c>
     </row>
     <row r="91" spans="1:10" s="25" customFormat="1" x14ac:dyDescent="0.2">
@@ -16075,19 +16067,16 @@
         <v>630</v>
       </c>
       <c r="C91" s="25" t="s">
-        <v>15</v>
-      </c>
-      <c r="D91" s="34" t="s">
-        <v>86</v>
+        <v>54</v>
       </c>
       <c r="E91" s="25" t="s">
         <v>76</v>
       </c>
       <c r="F91" s="25" t="s">
-        <v>100</v>
+        <v>143</v>
       </c>
       <c r="G91" s="25" t="s">
-        <v>102</v>
+        <v>701</v>
       </c>
     </row>
     <row r="92" spans="1:10" s="25" customFormat="1" x14ac:dyDescent="0.2">
@@ -16098,22 +16087,19 @@
         <v>630</v>
       </c>
       <c r="C92" s="25" t="s">
-        <v>15</v>
-      </c>
-      <c r="D92" s="34" t="s">
-        <v>87</v>
+        <v>7</v>
       </c>
       <c r="E92" s="25" t="s">
         <v>76</v>
       </c>
       <c r="F92" s="25" t="s">
-        <v>100</v>
+        <v>713</v>
       </c>
       <c r="G92" s="25" t="s">
-        <v>103</v>
-      </c>
-    </row>
-    <row r="93" spans="1:10" s="25" customFormat="1" x14ac:dyDescent="0.2">
+        <v>693</v>
+      </c>
+    </row>
+    <row r="93" spans="1:10" s="17" customFormat="1" ht="17" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A93" s="25" t="b">
         <v>1</v>
       </c>
@@ -16123,8 +16109,8 @@
       <c r="C93" s="25" t="s">
         <v>15</v>
       </c>
-      <c r="D93" s="34" t="s">
-        <v>88</v>
+      <c r="D93" s="33" t="s">
+        <v>84</v>
       </c>
       <c r="E93" s="25" t="s">
         <v>76</v>
@@ -16133,8 +16119,11 @@
         <v>100</v>
       </c>
       <c r="G93" s="25" t="s">
-        <v>104</v>
-      </c>
+        <v>75</v>
+      </c>
+      <c r="H93" s="25"/>
+      <c r="I93" s="25"/>
+      <c r="J93" s="25"/>
     </row>
     <row r="94" spans="1:10" s="25" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A94" s="25" t="b">
@@ -16146,8 +16135,8 @@
       <c r="C94" s="25" t="s">
         <v>15</v>
       </c>
-      <c r="D94" s="32" t="s">
-        <v>89</v>
+      <c r="D94" s="33" t="s">
+        <v>85</v>
       </c>
       <c r="E94" s="25" t="s">
         <v>76</v>
@@ -16156,7 +16145,7 @@
         <v>100</v>
       </c>
       <c r="G94" s="25" t="s">
-        <v>113</v>
+        <v>101</v>
       </c>
     </row>
     <row r="95" spans="1:10" s="25" customFormat="1" x14ac:dyDescent="0.2">
@@ -16169,8 +16158,8 @@
       <c r="C95" s="25" t="s">
         <v>15</v>
       </c>
-      <c r="D95" s="32" t="s">
-        <v>90</v>
+      <c r="D95" s="34" t="s">
+        <v>86</v>
       </c>
       <c r="E95" s="25" t="s">
         <v>76</v>
@@ -16179,7 +16168,7 @@
         <v>100</v>
       </c>
       <c r="G95" s="25" t="s">
-        <v>112</v>
+        <v>102</v>
       </c>
     </row>
     <row r="96" spans="1:10" s="25" customFormat="1" x14ac:dyDescent="0.2">
@@ -16192,8 +16181,8 @@
       <c r="C96" s="25" t="s">
         <v>15</v>
       </c>
-      <c r="D96" s="33" t="s">
-        <v>91</v>
+      <c r="D96" s="34" t="s">
+        <v>87</v>
       </c>
       <c r="E96" s="25" t="s">
         <v>76</v>
@@ -16202,7 +16191,7 @@
         <v>100</v>
       </c>
       <c r="G96" s="25" t="s">
-        <v>109</v>
+        <v>103</v>
       </c>
     </row>
     <row r="97" spans="1:11" s="25" customFormat="1" x14ac:dyDescent="0.2">
@@ -16215,8 +16204,8 @@
       <c r="C97" s="25" t="s">
         <v>15</v>
       </c>
-      <c r="D97" s="33" t="s">
-        <v>92</v>
+      <c r="D97" s="34" t="s">
+        <v>88</v>
       </c>
       <c r="E97" s="25" t="s">
         <v>76</v>
@@ -16225,7 +16214,7 @@
         <v>100</v>
       </c>
       <c r="G97" s="25" t="s">
-        <v>108</v>
+        <v>104</v>
       </c>
     </row>
     <row r="98" spans="1:11" s="25" customFormat="1" x14ac:dyDescent="0.2">
@@ -16239,7 +16228,7 @@
         <v>15</v>
       </c>
       <c r="D98" s="32" t="s">
-        <v>93</v>
+        <v>89</v>
       </c>
       <c r="E98" s="25" t="s">
         <v>76</v>
@@ -16248,7 +16237,7 @@
         <v>100</v>
       </c>
       <c r="G98" s="25" t="s">
-        <v>107</v>
+        <v>113</v>
       </c>
     </row>
     <row r="99" spans="1:11" s="25" customFormat="1" x14ac:dyDescent="0.2">
@@ -16262,7 +16251,7 @@
         <v>15</v>
       </c>
       <c r="D99" s="32" t="s">
-        <v>94</v>
+        <v>90</v>
       </c>
       <c r="E99" s="25" t="s">
         <v>76</v>
@@ -16271,7 +16260,7 @@
         <v>100</v>
       </c>
       <c r="G99" s="25" t="s">
-        <v>106</v>
+        <v>112</v>
       </c>
     </row>
     <row r="100" spans="1:11" s="25" customFormat="1" x14ac:dyDescent="0.2">
@@ -16284,8 +16273,8 @@
       <c r="C100" s="25" t="s">
         <v>15</v>
       </c>
-      <c r="D100" s="32" t="s">
-        <v>95</v>
+      <c r="D100" s="33" t="s">
+        <v>91</v>
       </c>
       <c r="E100" s="25" t="s">
         <v>76</v>
@@ -16294,7 +16283,7 @@
         <v>100</v>
       </c>
       <c r="G100" s="25" t="s">
-        <v>105</v>
+        <v>109</v>
       </c>
     </row>
     <row r="101" spans="1:11" s="25" customFormat="1" x14ac:dyDescent="0.2">
@@ -16307,8 +16296,8 @@
       <c r="C101" s="25" t="s">
         <v>15</v>
       </c>
-      <c r="D101" s="32" t="s">
-        <v>96</v>
+      <c r="D101" s="33" t="s">
+        <v>92</v>
       </c>
       <c r="E101" s="25" t="s">
         <v>76</v>
@@ -16317,7 +16306,7 @@
         <v>100</v>
       </c>
       <c r="G101" s="25" t="s">
-        <v>110</v>
+        <v>108</v>
       </c>
     </row>
     <row r="102" spans="1:11" s="25" customFormat="1" x14ac:dyDescent="0.2">
@@ -16331,7 +16320,7 @@
         <v>15</v>
       </c>
       <c r="D102" s="32" t="s">
-        <v>97</v>
+        <v>93</v>
       </c>
       <c r="E102" s="25" t="s">
         <v>76</v>
@@ -16340,7 +16329,7 @@
         <v>100</v>
       </c>
       <c r="G102" s="25" t="s">
-        <v>97</v>
+        <v>107</v>
       </c>
     </row>
     <row r="103" spans="1:11" s="25" customFormat="1" x14ac:dyDescent="0.2">
@@ -16354,7 +16343,7 @@
         <v>15</v>
       </c>
       <c r="D103" s="32" t="s">
-        <v>98</v>
+        <v>94</v>
       </c>
       <c r="E103" s="25" t="s">
         <v>76</v>
@@ -16363,7 +16352,7 @@
         <v>100</v>
       </c>
       <c r="G103" s="25" t="s">
-        <v>111</v>
+        <v>106</v>
       </c>
     </row>
     <row r="104" spans="1:11" s="25" customFormat="1" x14ac:dyDescent="0.2">
@@ -16377,7 +16366,7 @@
         <v>15</v>
       </c>
       <c r="D104" s="32" t="s">
-        <v>99</v>
+        <v>95</v>
       </c>
       <c r="E104" s="25" t="s">
         <v>76</v>
@@ -16385,12 +16374,104 @@
       <c r="F104" s="25" t="s">
         <v>100</v>
       </c>
-      <c r="G104" s="41" t="s">
+      <c r="G104" s="25" t="s">
+        <v>105</v>
+      </c>
+    </row>
+    <row r="105" spans="1:11" s="25" customFormat="1" x14ac:dyDescent="0.2">
+      <c r="A105" s="25" t="b">
+        <v>1</v>
+      </c>
+      <c r="B105" s="25" t="s">
+        <v>630</v>
+      </c>
+      <c r="C105" s="25" t="s">
+        <v>15</v>
+      </c>
+      <c r="D105" s="32" t="s">
+        <v>96</v>
+      </c>
+      <c r="E105" s="25" t="s">
+        <v>76</v>
+      </c>
+      <c r="F105" s="25" t="s">
+        <v>100</v>
+      </c>
+      <c r="G105" s="25" t="s">
+        <v>110</v>
+      </c>
+    </row>
+    <row r="106" spans="1:11" s="25" customFormat="1" x14ac:dyDescent="0.2">
+      <c r="A106" s="25" t="b">
+        <v>1</v>
+      </c>
+      <c r="B106" s="25" t="s">
+        <v>630</v>
+      </c>
+      <c r="C106" s="25" t="s">
+        <v>15</v>
+      </c>
+      <c r="D106" s="32" t="s">
+        <v>97</v>
+      </c>
+      <c r="E106" s="25" t="s">
+        <v>76</v>
+      </c>
+      <c r="F106" s="25" t="s">
+        <v>100</v>
+      </c>
+      <c r="G106" s="25" t="s">
+        <v>97</v>
+      </c>
+    </row>
+    <row r="107" spans="1:11" s="25" customFormat="1" x14ac:dyDescent="0.2">
+      <c r="A107" s="25" t="b">
+        <v>1</v>
+      </c>
+      <c r="B107" s="25" t="s">
+        <v>630</v>
+      </c>
+      <c r="C107" s="25" t="s">
+        <v>15</v>
+      </c>
+      <c r="D107" s="32" t="s">
+        <v>98</v>
+      </c>
+      <c r="E107" s="25" t="s">
+        <v>76</v>
+      </c>
+      <c r="F107" s="25" t="s">
+        <v>100</v>
+      </c>
+      <c r="G107" s="25" t="s">
+        <v>111</v>
+      </c>
+    </row>
+    <row r="108" spans="1:11" s="25" customFormat="1" x14ac:dyDescent="0.2">
+      <c r="A108" s="25" t="b">
+        <v>1</v>
+      </c>
+      <c r="B108" s="25" t="s">
+        <v>630</v>
+      </c>
+      <c r="C108" s="25" t="s">
+        <v>15</v>
+      </c>
+      <c r="D108" s="32" t="s">
+        <v>99</v>
+      </c>
+      <c r="E108" s="25" t="s">
+        <v>76</v>
+      </c>
+      <c r="F108" s="25" t="s">
+        <v>100</v>
+      </c>
+      <c r="G108" s="41" t="s">
         <v>530</v>
       </c>
-      <c r="H104" s="29"/>
-      <c r="I104" s="29"/>
-      <c r="K104" s="41"/>
+      <c r="H108" s="29"/>
+      <c r="I108" s="29"/>
+      <c r="K108" s="41"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -16507,7 +16588,7 @@
         <v>160</v>
       </c>
       <c r="M2" s="25" t="s">
-        <v>888</v>
+        <v>887</v>
       </c>
       <c r="N2" s="25" t="s">
         <v>161</v>
@@ -16723,7 +16804,7 @@
         <v>170</v>
       </c>
       <c r="M8" s="25" t="s">
-        <v>887</v>
+        <v>886</v>
       </c>
       <c r="N8" s="25" t="s">
         <v>161</v>
@@ -16837,7 +16918,7 @@
         <v>162</v>
       </c>
       <c r="M11" s="25" t="s">
-        <v>886</v>
+        <v>885</v>
       </c>
       <c r="N11" s="25" t="s">
         <v>163</v>
@@ -16919,7 +17000,7 @@
         <v>114</v>
       </c>
       <c r="F14" s="25" t="s">
-        <v>884</v>
+        <v>883</v>
       </c>
       <c r="G14"/>
     </row>
@@ -17031,7 +17112,7 @@
         <v>637</v>
       </c>
       <c r="M17" s="25" t="s">
-        <v>918</v>
+        <v>917</v>
       </c>
       <c r="N17" t="s">
         <v>641</v>
@@ -17073,7 +17154,7 @@
         <v>637</v>
       </c>
       <c r="M18" s="25" t="s">
-        <v>921</v>
+        <v>920</v>
       </c>
       <c r="N18" s="25" t="s">
         <v>641</v>
@@ -17112,7 +17193,7 @@
         <v>637</v>
       </c>
       <c r="M19" s="25" t="s">
-        <v>920</v>
+        <v>919</v>
       </c>
       <c r="N19" s="25" t="s">
         <v>641</v>
@@ -17151,7 +17232,7 @@
         <v>637</v>
       </c>
       <c r="M20" s="25" t="s">
-        <v>919</v>
+        <v>918</v>
       </c>
       <c r="N20" s="25" t="s">
         <v>641</v>
@@ -17259,7 +17340,7 @@
         <v>596</v>
       </c>
       <c r="M23" s="25" t="s">
-        <v>917</v>
+        <v>916</v>
       </c>
       <c r="N23" s="25" t="s">
         <v>163</v>
@@ -17332,7 +17413,7 @@
       </c>
       <c r="L25" s="28"/>
       <c r="M25" s="28" t="s">
-        <v>885</v>
+        <v>884</v>
       </c>
       <c r="N25" s="28" t="s">
         <v>157</v>
@@ -20885,28 +20966,28 @@
         <v>682</v>
       </c>
       <c r="H1" s="39" t="s">
+        <v>888</v>
+      </c>
+      <c r="I1" s="40" t="s">
         <v>889</v>
       </c>
-      <c r="I1" s="40" t="s">
+      <c r="J1" s="40" t="s">
         <v>890</v>
       </c>
-      <c r="J1" s="40" t="s">
+      <c r="K1" s="40" t="s">
         <v>891</v>
       </c>
-      <c r="K1" s="40" t="s">
+      <c r="L1" s="40" t="s">
         <v>892</v>
       </c>
-      <c r="L1" s="40" t="s">
+      <c r="M1" s="40" t="s">
         <v>893</v>
       </c>
-      <c r="M1" s="40" t="s">
+      <c r="N1" s="40" t="s">
         <v>894</v>
       </c>
-      <c r="N1" s="40" t="s">
-        <v>895</v>
-      </c>
       <c r="O1" s="40" t="s">
-        <v>901</v>
+        <v>900</v>
       </c>
       <c r="P1" s="39" t="s">
         <v>848</v>
@@ -20926,7 +21007,7 @@
         <v>736</v>
       </c>
       <c r="H2" t="s">
-        <v>902</v>
+        <v>901</v>
       </c>
       <c r="I2" t="s">
         <v>703</v>
@@ -20935,13 +21016,13 @@
         <v>656</v>
       </c>
       <c r="L2" t="s">
-        <v>896</v>
+        <v>895</v>
       </c>
       <c r="N2" t="s">
         <v>670</v>
       </c>
       <c r="O2" t="s">
-        <v>897</v>
+        <v>896</v>
       </c>
     </row>
     <row r="3" spans="1:16" x14ac:dyDescent="0.2">
@@ -20958,7 +21039,7 @@
         <v>736</v>
       </c>
       <c r="H3" t="s">
-        <v>903</v>
+        <v>902</v>
       </c>
       <c r="I3" t="s">
         <v>703</v>
@@ -20967,13 +21048,13 @@
         <v>670</v>
       </c>
       <c r="L3" t="s">
-        <v>896</v>
+        <v>895</v>
       </c>
       <c r="N3" t="s">
         <v>649</v>
       </c>
       <c r="O3" t="s">
-        <v>897</v>
+        <v>896</v>
       </c>
     </row>
     <row r="4" spans="1:16" x14ac:dyDescent="0.2">
@@ -20990,7 +21071,7 @@
         <v>736</v>
       </c>
       <c r="H4" t="s">
-        <v>904</v>
+        <v>903</v>
       </c>
       <c r="I4" t="s">
         <v>703</v>
@@ -20999,13 +21080,13 @@
         <v>650</v>
       </c>
       <c r="L4" t="s">
-        <v>898</v>
+        <v>897</v>
       </c>
       <c r="N4" t="s">
         <v>649</v>
       </c>
       <c r="O4" t="s">
-        <v>897</v>
+        <v>896</v>
       </c>
     </row>
     <row r="5" spans="1:16" x14ac:dyDescent="0.2">
@@ -21022,7 +21103,7 @@
         <v>736</v>
       </c>
       <c r="H5" t="s">
-        <v>905</v>
+        <v>904</v>
       </c>
       <c r="I5" t="s">
         <v>703</v>
@@ -21031,13 +21112,13 @@
         <v>649</v>
       </c>
       <c r="L5" t="s">
-        <v>896</v>
+        <v>895</v>
       </c>
       <c r="N5" t="s">
         <v>671</v>
       </c>
       <c r="O5" t="s">
-        <v>897</v>
+        <v>896</v>
       </c>
     </row>
     <row r="6" spans="1:16" x14ac:dyDescent="0.2">
@@ -21054,7 +21135,7 @@
         <v>736</v>
       </c>
       <c r="H6" t="s">
-        <v>906</v>
+        <v>905</v>
       </c>
       <c r="I6" t="s">
         <v>703</v>
@@ -21063,13 +21144,13 @@
         <v>653</v>
       </c>
       <c r="L6" t="s">
-        <v>898</v>
+        <v>897</v>
       </c>
       <c r="N6" t="s">
         <v>671</v>
       </c>
       <c r="O6" t="s">
-        <v>897</v>
+        <v>896</v>
       </c>
     </row>
     <row r="7" spans="1:16" x14ac:dyDescent="0.2">
@@ -21086,7 +21167,7 @@
         <v>736</v>
       </c>
       <c r="H7" t="s">
-        <v>907</v>
+        <v>906</v>
       </c>
       <c r="I7" t="s">
         <v>703</v>
@@ -21095,13 +21176,13 @@
         <v>671</v>
       </c>
       <c r="L7" t="s">
-        <v>896</v>
+        <v>895</v>
       </c>
       <c r="N7" t="s">
         <v>651</v>
       </c>
       <c r="O7" t="s">
-        <v>897</v>
+        <v>896</v>
       </c>
     </row>
     <row r="8" spans="1:16" x14ac:dyDescent="0.2">
@@ -21118,7 +21199,7 @@
         <v>736</v>
       </c>
       <c r="H8" t="s">
-        <v>908</v>
+        <v>907</v>
       </c>
       <c r="I8" t="s">
         <v>703</v>
@@ -21127,13 +21208,13 @@
         <v>652</v>
       </c>
       <c r="L8" t="s">
-        <v>898</v>
+        <v>897</v>
       </c>
       <c r="N8" t="s">
         <v>651</v>
       </c>
       <c r="O8" t="s">
-        <v>897</v>
+        <v>896</v>
       </c>
     </row>
     <row r="9" spans="1:16" x14ac:dyDescent="0.2">
@@ -21150,7 +21231,7 @@
         <v>736</v>
       </c>
       <c r="H9" t="s">
-        <v>909</v>
+        <v>908</v>
       </c>
       <c r="I9" t="s">
         <v>703</v>
@@ -21159,13 +21240,13 @@
         <v>651</v>
       </c>
       <c r="L9" t="s">
-        <v>896</v>
+        <v>895</v>
       </c>
       <c r="N9" t="s">
         <v>672</v>
       </c>
       <c r="O9" t="s">
-        <v>897</v>
+        <v>896</v>
       </c>
     </row>
     <row r="10" spans="1:16" x14ac:dyDescent="0.2">
@@ -21182,7 +21263,7 @@
         <v>736</v>
       </c>
       <c r="H10" t="s">
-        <v>910</v>
+        <v>909</v>
       </c>
       <c r="I10" t="s">
         <v>703</v>
@@ -21191,13 +21272,13 @@
         <v>654</v>
       </c>
       <c r="L10" t="s">
-        <v>898</v>
+        <v>897</v>
       </c>
       <c r="N10" t="s">
         <v>672</v>
       </c>
       <c r="O10" t="s">
-        <v>897</v>
+        <v>896</v>
       </c>
     </row>
     <row r="11" spans="1:16" x14ac:dyDescent="0.2">
@@ -21214,7 +21295,7 @@
         <v>736</v>
       </c>
       <c r="H11" t="s">
-        <v>911</v>
+        <v>910</v>
       </c>
       <c r="I11" t="s">
         <v>703</v>
@@ -21223,13 +21304,13 @@
         <v>673</v>
       </c>
       <c r="L11" t="s">
-        <v>898</v>
+        <v>897</v>
       </c>
       <c r="N11" t="s">
         <v>654</v>
       </c>
       <c r="O11" t="s">
-        <v>897</v>
+        <v>896</v>
       </c>
     </row>
     <row r="12" spans="1:16" x14ac:dyDescent="0.2">
@@ -21246,7 +21327,7 @@
         <v>736</v>
       </c>
       <c r="H12" t="s">
-        <v>912</v>
+        <v>911</v>
       </c>
       <c r="I12" t="s">
         <v>703</v>
@@ -21255,13 +21336,13 @@
         <v>674</v>
       </c>
       <c r="L12" t="s">
-        <v>898</v>
+        <v>897</v>
       </c>
       <c r="N12" t="s">
         <v>654</v>
       </c>
       <c r="O12" t="s">
-        <v>897</v>
+        <v>896</v>
       </c>
     </row>
     <row r="13" spans="1:16" x14ac:dyDescent="0.2">
@@ -21278,7 +21359,7 @@
         <v>736</v>
       </c>
       <c r="H13" t="s">
-        <v>913</v>
+        <v>912</v>
       </c>
       <c r="I13" t="s">
         <v>703</v>
@@ -21287,13 +21368,13 @@
         <v>672</v>
       </c>
       <c r="L13" t="s">
-        <v>896</v>
+        <v>895</v>
       </c>
       <c r="N13" t="s">
         <v>675</v>
       </c>
       <c r="O13" t="s">
-        <v>897</v>
+        <v>896</v>
       </c>
     </row>
     <row r="14" spans="1:16" x14ac:dyDescent="0.2">
@@ -21310,7 +21391,7 @@
         <v>736</v>
       </c>
       <c r="H14" t="s">
-        <v>914</v>
+        <v>913</v>
       </c>
       <c r="I14" t="s">
         <v>703</v>
@@ -21319,13 +21400,13 @@
         <v>676</v>
       </c>
       <c r="L14" t="s">
-        <v>898</v>
+        <v>897</v>
       </c>
       <c r="N14" t="s">
         <v>675</v>
       </c>
       <c r="O14" t="s">
-        <v>897</v>
+        <v>896</v>
       </c>
     </row>
     <row r="15" spans="1:16" x14ac:dyDescent="0.2">
@@ -21336,28 +21417,28 @@
         <v>630</v>
       </c>
       <c r="C15" t="s">
-        <v>899</v>
+        <v>898</v>
       </c>
       <c r="E15" t="s">
         <v>736</v>
       </c>
       <c r="H15" t="s">
-        <v>915</v>
+        <v>914</v>
       </c>
       <c r="I15" t="s">
         <v>703</v>
       </c>
       <c r="K15" t="s">
-        <v>900</v>
+        <v>899</v>
       </c>
       <c r="L15" t="s">
-        <v>898</v>
+        <v>897</v>
       </c>
       <c r="N15" t="s">
         <v>675</v>
       </c>
       <c r="O15" t="s">
-        <v>897</v>
+        <v>896</v>
       </c>
     </row>
     <row r="16" spans="1:16" x14ac:dyDescent="0.2">
@@ -21374,7 +21455,7 @@
         <v>736</v>
       </c>
       <c r="H16" t="s">
-        <v>916</v>
+        <v>915</v>
       </c>
       <c r="I16" t="s">
         <v>703</v>
@@ -21383,13 +21464,13 @@
         <v>677</v>
       </c>
       <c r="L16" t="s">
-        <v>898</v>
+        <v>897</v>
       </c>
       <c r="N16" t="s">
         <v>675</v>
       </c>
       <c r="O16" t="s">
-        <v>897</v>
+        <v>896</v>
       </c>
     </row>
   </sheetData>
@@ -24081,19 +24162,19 @@
         <v>753</v>
       </c>
       <c r="F1" s="17" t="s">
-        <v>935</v>
+        <v>934</v>
       </c>
       <c r="G1" s="17" t="s">
-        <v>929</v>
+        <v>928</v>
       </c>
       <c r="H1" s="17" t="s">
-        <v>937</v>
+        <v>936</v>
       </c>
       <c r="I1" s="17" t="s">
-        <v>934</v>
+        <v>933</v>
       </c>
       <c r="J1" s="17" t="s">
-        <v>923</v>
+        <v>922</v>
       </c>
     </row>
     <row r="2" spans="1:10" x14ac:dyDescent="0.2">
@@ -24113,16 +24194,16 @@
         <v>779</v>
       </c>
       <c r="G2" t="s">
-        <v>938</v>
+        <v>937</v>
       </c>
       <c r="H2" t="s">
-        <v>959</v>
+        <v>958</v>
       </c>
       <c r="I2" t="s">
         <v>778</v>
       </c>
       <c r="J2" t="s">
-        <v>930</v>
+        <v>929</v>
       </c>
     </row>
     <row r="3" spans="1:10" x14ac:dyDescent="0.2">
@@ -24136,10 +24217,10 @@
         <v>772</v>
       </c>
       <c r="G3" t="s">
-        <v>940</v>
+        <v>939</v>
       </c>
       <c r="H3" t="s">
-        <v>960</v>
+        <v>959</v>
       </c>
     </row>
     <row r="5" spans="1:10" x14ac:dyDescent="0.2">
@@ -24159,16 +24240,16 @@
         <v>759</v>
       </c>
       <c r="G5" t="s">
-        <v>939</v>
+        <v>938</v>
       </c>
       <c r="H5" t="s">
-        <v>961</v>
+        <v>960</v>
       </c>
       <c r="I5" t="s">
         <v>754</v>
       </c>
       <c r="J5" t="s">
-        <v>924</v>
+        <v>923</v>
       </c>
     </row>
     <row r="6" spans="1:10" x14ac:dyDescent="0.2">
@@ -24188,13 +24269,13 @@
         <v>703</v>
       </c>
       <c r="G6" t="s">
-        <v>941</v>
+        <v>940</v>
       </c>
       <c r="H6" t="s">
-        <v>962</v>
+        <v>961</v>
       </c>
       <c r="J6" t="s">
-        <v>964</v>
+        <v>963</v>
       </c>
     </row>
     <row r="7" spans="1:10" x14ac:dyDescent="0.2">
@@ -24211,13 +24292,13 @@
         <v>700</v>
       </c>
       <c r="G7" t="s">
-        <v>942</v>
+        <v>941</v>
       </c>
       <c r="H7" t="s">
-        <v>976</v>
+        <v>975</v>
       </c>
       <c r="J7" t="s">
-        <v>963</v>
+        <v>962</v>
       </c>
     </row>
     <row r="8" spans="1:10" x14ac:dyDescent="0.2">
@@ -24234,13 +24315,13 @@
         <v>771</v>
       </c>
       <c r="G8" t="s">
-        <v>943</v>
+        <v>942</v>
       </c>
       <c r="H8" t="s">
-        <v>966</v>
+        <v>965</v>
       </c>
       <c r="J8" t="s">
-        <v>965</v>
+        <v>964</v>
       </c>
     </row>
     <row r="9" spans="1:10" x14ac:dyDescent="0.2">
@@ -24257,10 +24338,10 @@
         <v>694</v>
       </c>
       <c r="G9" t="s">
-        <v>944</v>
+        <v>943</v>
       </c>
       <c r="H9" t="s">
-        <v>967</v>
+        <v>966</v>
       </c>
     </row>
     <row r="10" spans="1:10" x14ac:dyDescent="0.2">
@@ -24277,10 +24358,10 @@
         <v>772</v>
       </c>
       <c r="G10" t="s">
-        <v>940</v>
+        <v>939</v>
       </c>
       <c r="H10" t="s">
-        <v>960</v>
+        <v>959</v>
       </c>
     </row>
     <row r="11" spans="1:10" x14ac:dyDescent="0.2">
@@ -24297,10 +24378,10 @@
         <v>773</v>
       </c>
       <c r="G11" t="s">
-        <v>969</v>
+        <v>968</v>
       </c>
       <c r="H11" t="s">
-        <v>968</v>
+        <v>967</v>
       </c>
     </row>
     <row r="12" spans="1:10" x14ac:dyDescent="0.2">
@@ -24317,10 +24398,10 @@
         <v>701</v>
       </c>
       <c r="G12" t="s">
-        <v>945</v>
+        <v>944</v>
       </c>
       <c r="H12" t="s">
-        <v>970</v>
+        <v>969</v>
       </c>
     </row>
     <row r="13" spans="1:10" x14ac:dyDescent="0.2">
@@ -24340,10 +24421,10 @@
         <v>693</v>
       </c>
       <c r="G13" t="s">
-        <v>946</v>
+        <v>945</v>
       </c>
       <c r="H13" t="s">
-        <v>971</v>
+        <v>970</v>
       </c>
     </row>
     <row r="15" spans="1:10" x14ac:dyDescent="0.2">
@@ -24360,10 +24441,10 @@
         <v>733</v>
       </c>
       <c r="G15" t="s">
-        <v>933</v>
+        <v>932</v>
       </c>
       <c r="H15" t="s">
-        <v>933</v>
+        <v>932</v>
       </c>
     </row>
     <row r="16" spans="1:10" x14ac:dyDescent="0.2">
@@ -24386,16 +24467,16 @@
         <v>758</v>
       </c>
       <c r="G16" t="s">
-        <v>947</v>
+        <v>946</v>
       </c>
       <c r="H16" t="s">
-        <v>972</v>
+        <v>971</v>
       </c>
       <c r="I16" t="s">
         <v>757</v>
       </c>
       <c r="J16" t="s">
-        <v>932</v>
+        <v>931</v>
       </c>
     </row>
     <row r="17" spans="1:10" x14ac:dyDescent="0.2">
@@ -24412,10 +24493,10 @@
         <v>772</v>
       </c>
       <c r="G17" t="s">
-        <v>940</v>
+        <v>939</v>
       </c>
       <c r="H17" t="s">
-        <v>960</v>
+        <v>959</v>
       </c>
     </row>
     <row r="18" spans="1:10" x14ac:dyDescent="0.2">
@@ -24432,10 +24513,10 @@
         <v>701</v>
       </c>
       <c r="G18" t="s">
-        <v>945</v>
+        <v>944</v>
       </c>
       <c r="H18" t="s">
-        <v>970</v>
+        <v>969</v>
       </c>
     </row>
     <row r="19" spans="1:10" x14ac:dyDescent="0.2">
@@ -24452,10 +24533,10 @@
         <v>693</v>
       </c>
       <c r="G19" t="s">
-        <v>946</v>
+        <v>945</v>
       </c>
       <c r="H19" t="s">
-        <v>971</v>
+        <v>970</v>
       </c>
     </row>
     <row r="21" spans="1:10" x14ac:dyDescent="0.2">
@@ -24475,10 +24556,10 @@
         <v>783</v>
       </c>
       <c r="G21" t="s">
-        <v>958</v>
+        <v>957</v>
       </c>
       <c r="H21" t="s">
-        <v>973</v>
+        <v>972</v>
       </c>
       <c r="I21" t="s">
         <v>782</v>
@@ -24498,10 +24579,10 @@
         <v>701</v>
       </c>
       <c r="G22" t="s">
-        <v>945</v>
+        <v>944</v>
       </c>
       <c r="H22" t="s">
-        <v>970</v>
+        <v>969</v>
       </c>
     </row>
     <row r="23" spans="1:10" x14ac:dyDescent="0.2">
@@ -24518,13 +24599,13 @@
         <v>693</v>
       </c>
       <c r="G23" t="s">
-        <v>946</v>
+        <v>945</v>
       </c>
       <c r="H23" t="s">
-        <v>971</v>
+        <v>970</v>
       </c>
       <c r="I23" t="s">
-        <v>936</v>
+        <v>935</v>
       </c>
     </row>
     <row r="24" spans="1:10" x14ac:dyDescent="0.2">
@@ -24541,10 +24622,10 @@
         <v>775</v>
       </c>
       <c r="G24" t="s">
-        <v>948</v>
+        <v>947</v>
       </c>
       <c r="H24" t="s">
-        <v>974</v>
+        <v>973</v>
       </c>
     </row>
     <row r="26" spans="1:10" x14ac:dyDescent="0.2">
@@ -24564,7 +24645,7 @@
         <v>785</v>
       </c>
       <c r="H26" t="s">
-        <v>933</v>
+        <v>932</v>
       </c>
       <c r="I26" t="s">
         <v>784</v>
@@ -24584,10 +24665,10 @@
         <v>770</v>
       </c>
       <c r="G27" t="s">
-        <v>949</v>
+        <v>948</v>
       </c>
       <c r="H27" t="s">
-        <v>975</v>
+        <v>974</v>
       </c>
     </row>
     <row r="28" spans="1:10" x14ac:dyDescent="0.2">
@@ -24604,10 +24685,10 @@
         <v>700</v>
       </c>
       <c r="G28" t="s">
-        <v>942</v>
+        <v>941</v>
       </c>
       <c r="H28" t="s">
-        <v>976</v>
+        <v>975</v>
       </c>
     </row>
     <row r="29" spans="1:10" x14ac:dyDescent="0.2">
@@ -24624,10 +24705,10 @@
         <v>773</v>
       </c>
       <c r="G29" t="s">
-        <v>950</v>
+        <v>949</v>
       </c>
       <c r="H29" t="s">
-        <v>977</v>
+        <v>976</v>
       </c>
     </row>
     <row r="31" spans="1:10" x14ac:dyDescent="0.2">
@@ -24650,16 +24731,16 @@
         <v>760</v>
       </c>
       <c r="G31" t="s">
-        <v>951</v>
+        <v>950</v>
       </c>
       <c r="H31" t="s">
-        <v>985</v>
+        <v>984</v>
       </c>
       <c r="I31" t="s">
         <v>755</v>
       </c>
       <c r="J31" t="s">
-        <v>925</v>
+        <v>924</v>
       </c>
     </row>
     <row r="32" spans="1:10" x14ac:dyDescent="0.2">
@@ -24676,10 +24757,10 @@
         <v>703</v>
       </c>
       <c r="G32" t="s">
-        <v>941</v>
+        <v>940</v>
       </c>
       <c r="H32" t="s">
-        <v>962</v>
+        <v>961</v>
       </c>
     </row>
     <row r="33" spans="1:10" x14ac:dyDescent="0.2">
@@ -24699,10 +24780,10 @@
         <v>701</v>
       </c>
       <c r="G33" t="s">
-        <v>945</v>
+        <v>944</v>
       </c>
       <c r="H33" t="s">
-        <v>970</v>
+        <v>969</v>
       </c>
     </row>
     <row r="34" spans="1:10" x14ac:dyDescent="0.2">
@@ -24719,10 +24800,10 @@
         <v>693</v>
       </c>
       <c r="G34" t="s">
-        <v>946</v>
+        <v>945</v>
       </c>
       <c r="H34" t="s">
-        <v>971</v>
+        <v>970</v>
       </c>
     </row>
     <row r="35" spans="1:10" x14ac:dyDescent="0.2">
@@ -24739,10 +24820,10 @@
         <v>694</v>
       </c>
       <c r="G35" t="s">
-        <v>944</v>
+        <v>943</v>
       </c>
       <c r="H35" t="s">
-        <v>967</v>
+        <v>966</v>
       </c>
     </row>
     <row r="36" spans="1:10" x14ac:dyDescent="0.2">
@@ -24759,10 +24840,10 @@
         <v>772</v>
       </c>
       <c r="G36" t="s">
-        <v>940</v>
+        <v>939</v>
       </c>
       <c r="H36" t="s">
-        <v>960</v>
+        <v>959</v>
       </c>
     </row>
     <row r="38" spans="1:10" x14ac:dyDescent="0.2">
@@ -24776,10 +24857,10 @@
         <v>728</v>
       </c>
       <c r="G38" t="s">
-        <v>933</v>
+        <v>932</v>
       </c>
       <c r="H38" t="s">
-        <v>933</v>
+        <v>932</v>
       </c>
     </row>
     <row r="39" spans="1:10" x14ac:dyDescent="0.2">
@@ -24802,16 +24883,16 @@
         <v>761</v>
       </c>
       <c r="G39" t="s">
-        <v>956</v>
+        <v>955</v>
       </c>
       <c r="H39" t="s">
-        <v>978</v>
+        <v>977</v>
       </c>
       <c r="I39" t="s">
         <v>756</v>
       </c>
       <c r="J39" t="s">
-        <v>931</v>
+        <v>930</v>
       </c>
     </row>
     <row r="40" spans="1:10" x14ac:dyDescent="0.2">
@@ -24828,10 +24909,10 @@
         <v>772</v>
       </c>
       <c r="G40" t="s">
-        <v>940</v>
+        <v>939</v>
       </c>
       <c r="H40" t="s">
-        <v>960</v>
+        <v>959</v>
       </c>
     </row>
     <row r="41" spans="1:10" x14ac:dyDescent="0.2">
@@ -24848,10 +24929,10 @@
         <v>771</v>
       </c>
       <c r="G41" t="s">
-        <v>943</v>
+        <v>942</v>
       </c>
       <c r="H41" t="s">
-        <v>966</v>
+        <v>965</v>
       </c>
     </row>
     <row r="42" spans="1:10" x14ac:dyDescent="0.2">
@@ -24868,10 +24949,10 @@
         <v>777</v>
       </c>
       <c r="G42" t="s">
-        <v>952</v>
+        <v>951</v>
       </c>
       <c r="H42" t="s">
-        <v>979</v>
+        <v>978</v>
       </c>
     </row>
     <row r="43" spans="1:10" x14ac:dyDescent="0.2">
@@ -24888,10 +24969,10 @@
         <v>701</v>
       </c>
       <c r="G43" t="s">
-        <v>945</v>
+        <v>944</v>
       </c>
       <c r="H43" t="s">
-        <v>970</v>
+        <v>969</v>
       </c>
     </row>
     <row r="44" spans="1:10" x14ac:dyDescent="0.2">
@@ -24908,10 +24989,10 @@
         <v>693</v>
       </c>
       <c r="G44" t="s">
-        <v>946</v>
+        <v>945</v>
       </c>
       <c r="H44" t="s">
-        <v>971</v>
+        <v>970</v>
       </c>
     </row>
     <row r="45" spans="1:10" x14ac:dyDescent="0.2">
@@ -24925,7 +25006,7 @@
         <v>712</v>
       </c>
       <c r="H45" t="s">
-        <v>933</v>
+        <v>932</v>
       </c>
     </row>
     <row r="46" spans="1:10" x14ac:dyDescent="0.2">
@@ -24939,7 +25020,7 @@
         <v>730</v>
       </c>
       <c r="H46" t="s">
-        <v>933</v>
+        <v>932</v>
       </c>
     </row>
     <row r="48" spans="1:10" s="23" customFormat="1" x14ac:dyDescent="0.2">
@@ -24959,16 +25040,16 @@
         <v>768</v>
       </c>
       <c r="G48" s="23" t="s">
-        <v>953</v>
+        <v>952</v>
       </c>
       <c r="H48" s="23" t="s">
-        <v>983</v>
+        <v>982</v>
       </c>
       <c r="I48" s="23" t="s">
         <v>769</v>
       </c>
       <c r="J48" s="23" t="s">
-        <v>928</v>
+        <v>927</v>
       </c>
     </row>
     <row r="49" spans="1:10" s="23" customFormat="1" x14ac:dyDescent="0.2">
@@ -24979,10 +25060,10 @@
         <v>725</v>
       </c>
       <c r="G49" s="23" t="s">
-        <v>940</v>
+        <v>939</v>
       </c>
       <c r="H49" s="23" t="s">
-        <v>960</v>
+        <v>959</v>
       </c>
     </row>
     <row r="50" spans="1:10" s="23" customFormat="1" x14ac:dyDescent="0.2">
@@ -24993,10 +25074,10 @@
         <v>143</v>
       </c>
       <c r="G50" s="23" t="s">
-        <v>945</v>
+        <v>944</v>
       </c>
       <c r="H50" s="23" t="s">
-        <v>970</v>
+        <v>969</v>
       </c>
     </row>
     <row r="52" spans="1:10" s="23" customFormat="1" x14ac:dyDescent="0.2">
@@ -25018,7 +25099,7 @@
         <v>748</v>
       </c>
       <c r="H54" s="23" t="s">
-        <v>933</v>
+        <v>932</v>
       </c>
     </row>
     <row r="55" spans="1:10" s="23" customFormat="1" x14ac:dyDescent="0.2">
@@ -25032,16 +25113,16 @@
         <v>765</v>
       </c>
       <c r="G55" s="23" t="s">
-        <v>954</v>
+        <v>953</v>
       </c>
       <c r="H55" s="23" t="s">
-        <v>980</v>
+        <v>979</v>
       </c>
       <c r="I55" s="23" t="s">
         <v>764</v>
       </c>
       <c r="J55" s="23" t="s">
-        <v>927</v>
+        <v>926</v>
       </c>
     </row>
     <row r="56" spans="1:10" s="23" customFormat="1" x14ac:dyDescent="0.2">
@@ -25052,7 +25133,7 @@
         <v>751</v>
       </c>
       <c r="H56" s="23" t="s">
-        <v>933</v>
+        <v>932</v>
       </c>
     </row>
     <row r="57" spans="1:10" s="23" customFormat="1" x14ac:dyDescent="0.2">
@@ -25063,7 +25144,7 @@
         <v>752</v>
       </c>
       <c r="H57" s="23" t="s">
-        <v>933</v>
+        <v>932</v>
       </c>
     </row>
     <row r="58" spans="1:10" s="23" customFormat="1" x14ac:dyDescent="0.2">
@@ -25074,7 +25155,7 @@
         <v>749</v>
       </c>
       <c r="H58" s="23" t="s">
-        <v>933</v>
+        <v>932</v>
       </c>
     </row>
     <row r="59" spans="1:10" s="23" customFormat="1" x14ac:dyDescent="0.2">
@@ -25085,7 +25166,7 @@
         <v>750</v>
       </c>
       <c r="H59" s="23" t="s">
-        <v>933</v>
+        <v>932</v>
       </c>
     </row>
     <row r="61" spans="1:10" s="23" customFormat="1" x14ac:dyDescent="0.2">
@@ -25102,16 +25183,16 @@
         <v>781</v>
       </c>
       <c r="G61" s="23" t="s">
-        <v>957</v>
+        <v>956</v>
       </c>
       <c r="H61" s="23" t="s">
-        <v>981</v>
+        <v>980</v>
       </c>
       <c r="I61" s="23" t="s">
         <v>780</v>
       </c>
       <c r="J61" s="23" t="s">
-        <v>925</v>
+        <v>924</v>
       </c>
     </row>
     <row r="62" spans="1:10" s="23" customFormat="1" x14ac:dyDescent="0.2">
@@ -25122,10 +25203,10 @@
         <v>725</v>
       </c>
       <c r="G62" s="23" t="s">
-        <v>940</v>
+        <v>939</v>
       </c>
       <c r="H62" s="23" t="s">
-        <v>960</v>
+        <v>959</v>
       </c>
     </row>
     <row r="63" spans="1:10" s="23" customFormat="1" x14ac:dyDescent="0.2">
@@ -25136,10 +25217,10 @@
         <v>713</v>
       </c>
       <c r="G63" s="23" t="s">
-        <v>946</v>
+        <v>945</v>
       </c>
       <c r="H63" s="23" t="s">
-        <v>971</v>
+        <v>970</v>
       </c>
     </row>
     <row r="64" spans="1:10" s="23" customFormat="1" x14ac:dyDescent="0.2">
@@ -25150,10 +25231,10 @@
         <v>143</v>
       </c>
       <c r="G64" s="23" t="s">
-        <v>945</v>
+        <v>944</v>
       </c>
       <c r="H64" s="23" t="s">
-        <v>970</v>
+        <v>969</v>
       </c>
     </row>
     <row r="66" spans="1:10" s="23" customFormat="1" x14ac:dyDescent="0.2">
@@ -25178,7 +25259,7 @@
         <v>767</v>
       </c>
       <c r="H68" s="43" t="s">
-        <v>984</v>
+        <v>983</v>
       </c>
       <c r="I68" s="23" t="s">
         <v>766</v>
@@ -25192,10 +25273,10 @@
         <v>471</v>
       </c>
       <c r="G69" s="23" t="s">
-        <v>941</v>
+        <v>940</v>
       </c>
       <c r="H69" s="23" t="s">
-        <v>962</v>
+        <v>961</v>
       </c>
     </row>
     <row r="70" spans="1:10" s="23" customFormat="1" x14ac:dyDescent="0.2">
@@ -25206,10 +25287,10 @@
         <v>143</v>
       </c>
       <c r="G70" s="23" t="s">
-        <v>945</v>
+        <v>944</v>
       </c>
       <c r="H70" s="23" t="s">
-        <v>970</v>
+        <v>969</v>
       </c>
     </row>
     <row r="71" spans="1:10" s="23" customFormat="1" x14ac:dyDescent="0.2">
@@ -25220,10 +25301,10 @@
         <v>713</v>
       </c>
       <c r="G71" s="23" t="s">
-        <v>946</v>
+        <v>945</v>
       </c>
       <c r="H71" s="23" t="s">
-        <v>971</v>
+        <v>970</v>
       </c>
     </row>
     <row r="73" spans="1:10" s="23" customFormat="1" x14ac:dyDescent="0.2">
@@ -25243,16 +25324,16 @@
         <v>765</v>
       </c>
       <c r="G73" s="23" t="s">
-        <v>954</v>
+        <v>953</v>
       </c>
       <c r="H73" s="23" t="s">
-        <v>980</v>
+        <v>979</v>
       </c>
       <c r="I73" s="23" t="s">
+        <v>925</v>
+      </c>
+      <c r="J73" s="23" t="s">
         <v>926</v>
-      </c>
-      <c r="J73" s="23" t="s">
-        <v>927</v>
       </c>
     </row>
     <row r="74" spans="1:10" s="23" customFormat="1" x14ac:dyDescent="0.2">
@@ -25263,10 +25344,10 @@
         <v>729</v>
       </c>
       <c r="G74" s="23" t="s">
-        <v>952</v>
+        <v>951</v>
       </c>
       <c r="H74" s="23" t="s">
-        <v>979</v>
+        <v>978</v>
       </c>
     </row>
     <row r="75" spans="1:10" s="23" customFormat="1" x14ac:dyDescent="0.2">
@@ -25277,10 +25358,10 @@
         <v>725</v>
       </c>
       <c r="G75" s="23" t="s">
-        <v>940</v>
+        <v>939</v>
       </c>
       <c r="H75" s="23" t="s">
-        <v>960</v>
+        <v>959</v>
       </c>
     </row>
     <row r="77" spans="1:10" s="23" customFormat="1" x14ac:dyDescent="0.2">
@@ -25297,10 +25378,10 @@
         <v>763</v>
       </c>
       <c r="G77" s="23" t="s">
-        <v>955</v>
+        <v>954</v>
       </c>
       <c r="H77" s="23" t="s">
-        <v>982</v>
+        <v>981</v>
       </c>
       <c r="I77" s="23" t="s">
         <v>762</v>
@@ -25314,10 +25395,10 @@
         <v>725</v>
       </c>
       <c r="G78" s="23" t="s">
-        <v>940</v>
+        <v>939</v>
       </c>
       <c r="H78" s="23" t="s">
-        <v>960</v>
+        <v>959</v>
       </c>
     </row>
     <row r="79" spans="1:10" s="23" customFormat="1" x14ac:dyDescent="0.2">
@@ -25328,10 +25409,10 @@
         <v>143</v>
       </c>
       <c r="G79" s="23" t="s">
-        <v>945</v>
+        <v>944</v>
       </c>
       <c r="H79" s="23" t="s">
-        <v>970</v>
+        <v>969</v>
       </c>
     </row>
     <row r="80" spans="1:10" s="23" customFormat="1" x14ac:dyDescent="0.2">
@@ -25342,10 +25423,10 @@
         <v>713</v>
       </c>
       <c r="G80" s="23" t="s">
-        <v>946</v>
+        <v>945</v>
       </c>
       <c r="H80" s="23" t="s">
-        <v>971</v>
+        <v>970</v>
       </c>
     </row>
     <row r="82" spans="1:2" s="23" customFormat="1" x14ac:dyDescent="0.2">

</xml_diff>

<commit_message>
Added polygons table and polygonID fields in other tables
</commit_message>
<xml_diff>
--- a/data/mapping_config_files/nwss_to_odm_v2_mapping.xlsx
+++ b/data/mapping_config_files/nwss_to_odm_v2_mapping.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/martinwellman/Documents/Health/Wastewater/PHES-ODM-MapGenerator/PHES-ODM-MapGenerator/data/mapping_config_files/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{982605AD-774C-2D45-A0B2-4A681470F99A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{38902763-A490-C344-9B72-443A878B1074}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="500" windowWidth="40960" windowHeight="20860" xr2:uid="{77810E24-F86B-BC44-A0D5-8790E6EC60B4}"/>
   </bookViews>
@@ -27,7 +27,7 @@
   </externalReferences>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">enums!$A$1:$J$41</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">maps!$A$1:$K$52</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">maps!$A$1:$K$58</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="7" hidden="1">'maps original'!$A$1:$L$87</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">wide_measures!$A$1:$S$26</definedName>
     <definedName name="partID">[1]parts!$A:$A</definedName>
@@ -53,7 +53,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3248" uniqueCount="985">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3278" uniqueCount="986">
   <si>
     <t>Reporter</t>
   </si>
@@ -3055,6 +3055,9 @@
   </si>
   <si>
     <t>makeid(samples.siteID, case((samples.collDT, date(samples.collDT), (True, date(samples.collDTEnd)), rowNum)</t>
+  </si>
+  <si>
+    <t>{{id:polygonID}}</t>
   </si>
 </sst>
 </file>
@@ -14493,7 +14496,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{3154BFCE-06D9-9649-B340-B23DCF20DD83}">
-  <dimension ref="A1:K108"/>
+  <dimension ref="A1:K115"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="2" max="2" width="13" bestFit="1" customWidth="1"/>
@@ -15032,27 +15035,26 @@
       </c>
     </row>
     <row r="32" spans="1:11" s="25" customFormat="1" x14ac:dyDescent="0.2">
-      <c r="H32" s="30"/>
+      <c r="A32" s="25" t="b">
+        <v>1</v>
+      </c>
+      <c r="B32" s="25" t="s">
+        <v>630</v>
+      </c>
+      <c r="C32" s="25" t="s">
+        <v>771</v>
+      </c>
+      <c r="E32" s="25" t="s">
+        <v>114</v>
+      </c>
+      <c r="F32" s="25" t="s">
+        <v>727</v>
+      </c>
+      <c r="G32" s="25" t="s">
+        <v>985</v>
+      </c>
     </row>
     <row r="33" spans="1:8" s="25" customFormat="1" x14ac:dyDescent="0.2">
-      <c r="A33" s="25" t="b">
-        <v>1</v>
-      </c>
-      <c r="B33" s="25" t="s">
-        <v>630</v>
-      </c>
-      <c r="C33" s="25" t="s">
-        <v>773</v>
-      </c>
-      <c r="E33" s="25" t="s">
-        <v>737</v>
-      </c>
-      <c r="F33" s="25" t="s">
-        <v>726</v>
-      </c>
-      <c r="G33" s="25" t="s">
-        <v>876</v>
-      </c>
       <c r="H33" s="30"/>
     </row>
     <row r="34" spans="1:8" s="25" customFormat="1" x14ac:dyDescent="0.2">
@@ -15063,16 +15065,16 @@
         <v>630</v>
       </c>
       <c r="C34" s="25" t="s">
-        <v>73</v>
+        <v>773</v>
       </c>
       <c r="E34" s="25" t="s">
         <v>737</v>
       </c>
       <c r="F34" s="25" t="s">
-        <v>471</v>
+        <v>726</v>
       </c>
       <c r="G34" s="25" t="s">
-        <v>703</v>
+        <v>876</v>
       </c>
       <c r="H34" s="30"/>
     </row>
@@ -15084,16 +15086,16 @@
         <v>630</v>
       </c>
       <c r="C35" s="25" t="s">
-        <v>54</v>
+        <v>73</v>
       </c>
       <c r="E35" s="25" t="s">
         <v>737</v>
       </c>
       <c r="F35" s="25" t="s">
-        <v>143</v>
+        <v>471</v>
       </c>
       <c r="G35" s="25" t="s">
-        <v>701</v>
+        <v>703</v>
       </c>
       <c r="H35" s="30"/>
     </row>
@@ -15105,54 +15107,61 @@
         <v>630</v>
       </c>
       <c r="C36" s="25" t="s">
-        <v>7</v>
+        <v>54</v>
       </c>
       <c r="E36" s="25" t="s">
         <v>737</v>
       </c>
       <c r="F36" s="25" t="s">
+        <v>143</v>
+      </c>
+      <c r="G36" s="25" t="s">
+        <v>701</v>
+      </c>
+      <c r="H36" s="30"/>
+    </row>
+    <row r="37" spans="1:8" s="25" customFormat="1" x14ac:dyDescent="0.2">
+      <c r="A37" s="25" t="b">
+        <v>1</v>
+      </c>
+      <c r="B37" s="25" t="s">
+        <v>630</v>
+      </c>
+      <c r="C37" s="25" t="s">
+        <v>7</v>
+      </c>
+      <c r="E37" s="25" t="s">
+        <v>737</v>
+      </c>
+      <c r="F37" s="25" t="s">
         <v>713</v>
       </c>
-      <c r="G36" s="25" t="s">
+      <c r="G37" s="25" t="s">
         <v>693</v>
       </c>
-      <c r="H36" s="30"/>
-    </row>
-    <row r="37" spans="1:8" s="25" customFormat="1" x14ac:dyDescent="0.2">
       <c r="H37" s="30"/>
     </row>
     <row r="38" spans="1:8" s="25" customFormat="1" x14ac:dyDescent="0.2">
-      <c r="A38" s="25" t="b">
-        <v>1</v>
-      </c>
-      <c r="B38" s="25" t="s">
-        <v>630</v>
-      </c>
-      <c r="C38" s="25" t="s">
-        <v>54</v>
-      </c>
-      <c r="E38" s="25" t="s">
-        <v>723</v>
-      </c>
-      <c r="F38" s="25" t="s">
-        <v>143</v>
-      </c>
-      <c r="G38" s="25" t="s">
-        <v>701</v>
-      </c>
+      <c r="H38" s="30"/>
     </row>
     <row r="39" spans="1:8" s="25" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A39" s="25" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="B39" s="25" t="s">
         <v>630</v>
+      </c>
+      <c r="C39" s="25" t="s">
+        <v>54</v>
       </c>
       <c r="E39" s="25" t="s">
         <v>723</v>
       </c>
       <c r="F39" s="25" t="s">
-        <v>115</v>
+        <v>143</v>
+      </c>
+      <c r="G39" s="25" t="s">
+        <v>701</v>
       </c>
     </row>
     <row r="40" spans="1:8" s="25" customFormat="1" x14ac:dyDescent="0.2">
@@ -15166,27 +15175,21 @@
         <v>723</v>
       </c>
       <c r="F40" s="25" t="s">
-        <v>870</v>
+        <v>115</v>
       </c>
     </row>
     <row r="41" spans="1:8" s="25" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A41" s="25" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="B41" s="25" t="s">
         <v>630</v>
-      </c>
-      <c r="C41" s="25" t="s">
-        <v>777</v>
       </c>
       <c r="E41" s="25" t="s">
         <v>723</v>
       </c>
       <c r="F41" s="25" t="s">
-        <v>729</v>
-      </c>
-      <c r="G41" s="25" t="s">
-        <v>875</v>
+        <v>870</v>
       </c>
     </row>
     <row r="42" spans="1:8" s="25" customFormat="1" x14ac:dyDescent="0.2">
@@ -15196,32 +15199,38 @@
       <c r="B42" s="25" t="s">
         <v>630</v>
       </c>
-      <c r="C42" s="28" t="s">
-        <v>54</v>
-      </c>
-      <c r="D42" s="28"/>
-      <c r="E42" s="28" t="s">
+      <c r="C42" s="25" t="s">
+        <v>777</v>
+      </c>
+      <c r="E42" s="25" t="s">
         <v>723</v>
       </c>
-      <c r="F42" s="28" t="s">
-        <v>725</v>
-      </c>
-      <c r="G42" s="28" t="s">
-        <v>701</v>
+      <c r="F42" s="25" t="s">
+        <v>729</v>
+      </c>
+      <c r="G42" s="25" t="s">
+        <v>875</v>
       </c>
     </row>
     <row r="43" spans="1:8" s="25" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A43" s="25" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="B43" s="25" t="s">
         <v>630</v>
       </c>
-      <c r="E43" s="25" t="s">
+      <c r="C43" s="28" t="s">
+        <v>54</v>
+      </c>
+      <c r="D43" s="28"/>
+      <c r="E43" s="28" t="s">
         <v>723</v>
       </c>
-      <c r="F43" s="25" t="s">
-        <v>871</v>
+      <c r="F43" s="28" t="s">
+        <v>725</v>
+      </c>
+      <c r="G43" s="28" t="s">
+        <v>701</v>
       </c>
     </row>
     <row r="44" spans="1:8" s="25" customFormat="1" x14ac:dyDescent="0.2">
@@ -15235,7 +15244,7 @@
         <v>723</v>
       </c>
       <c r="F44" s="25" t="s">
-        <v>872</v>
+        <v>871</v>
       </c>
     </row>
     <row r="45" spans="1:8" s="25" customFormat="1" x14ac:dyDescent="0.2">
@@ -15249,7 +15258,7 @@
         <v>723</v>
       </c>
       <c r="F45" s="25" t="s">
-        <v>873</v>
+        <v>872</v>
       </c>
     </row>
     <row r="46" spans="1:8" s="25" customFormat="1" x14ac:dyDescent="0.2">
@@ -15263,7 +15272,7 @@
         <v>723</v>
       </c>
       <c r="F46" s="25" t="s">
-        <v>874</v>
+        <v>873</v>
       </c>
     </row>
     <row r="47" spans="1:8" s="25" customFormat="1" x14ac:dyDescent="0.2">
@@ -15277,31 +15286,24 @@
         <v>723</v>
       </c>
       <c r="F47" s="25" t="s">
+        <v>874</v>
+      </c>
+    </row>
+    <row r="48" spans="1:8" s="25" customFormat="1" x14ac:dyDescent="0.2">
+      <c r="A48" s="25" t="b">
+        <v>0</v>
+      </c>
+      <c r="B48" s="25" t="s">
+        <v>630</v>
+      </c>
+      <c r="E48" s="25" t="s">
+        <v>723</v>
+      </c>
+      <c r="F48" s="25" t="s">
         <v>120</v>
       </c>
     </row>
-    <row r="48" spans="1:8" s="25" customFormat="1" x14ac:dyDescent="0.2"/>
-    <row r="49" spans="1:11" s="25" customFormat="1" x14ac:dyDescent="0.2">
-      <c r="A49" s="25" t="b">
-        <v>1</v>
-      </c>
-      <c r="B49" s="25" t="s">
-        <v>630</v>
-      </c>
-      <c r="C49" s="28" t="s">
-        <v>54</v>
-      </c>
-      <c r="D49" s="28"/>
-      <c r="E49" s="28" t="s">
-        <v>474</v>
-      </c>
-      <c r="F49" s="28" t="s">
-        <v>725</v>
-      </c>
-      <c r="G49" s="28" t="s">
-        <v>701</v>
-      </c>
-    </row>
+    <row r="49" spans="1:11" s="25" customFormat="1" x14ac:dyDescent="0.2"/>
     <row r="50" spans="1:11" s="25" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A50" s="25" t="b">
         <v>1</v>
@@ -15310,16 +15312,16 @@
         <v>630</v>
       </c>
       <c r="C50" s="25" t="s">
-        <v>54</v>
+        <v>771</v>
       </c>
       <c r="E50" s="25" t="s">
-        <v>474</v>
+        <v>741</v>
       </c>
       <c r="F50" s="25" t="s">
-        <v>143</v>
+        <v>727</v>
       </c>
       <c r="G50" s="25" t="s">
-        <v>701</v>
+        <v>985</v>
       </c>
     </row>
     <row r="51" spans="1:11" s="25" customFormat="1" x14ac:dyDescent="0.2">
@@ -15329,17 +15331,18 @@
       <c r="B51" s="25" t="s">
         <v>630</v>
       </c>
-      <c r="C51" s="25" t="s">
-        <v>73</v>
-      </c>
-      <c r="E51" s="25" t="s">
-        <v>474</v>
-      </c>
-      <c r="F51" s="25" t="s">
-        <v>471</v>
-      </c>
-      <c r="G51" s="25" t="s">
-        <v>703</v>
+      <c r="C51" s="28" t="s">
+        <v>54</v>
+      </c>
+      <c r="D51" s="28"/>
+      <c r="E51" s="28" t="s">
+        <v>741</v>
+      </c>
+      <c r="F51" s="28" t="s">
+        <v>725</v>
+      </c>
+      <c r="G51" s="28" t="s">
+        <v>701</v>
       </c>
     </row>
     <row r="52" spans="1:11" s="25" customFormat="1" x14ac:dyDescent="0.2">
@@ -15350,18 +15353,17 @@
         <v>630</v>
       </c>
       <c r="C52" s="25" t="s">
-        <v>74</v>
-      </c>
-      <c r="E52" s="25" t="s">
-        <v>474</v>
+        <v>54</v>
+      </c>
+      <c r="E52" s="28" t="s">
+        <v>741</v>
       </c>
       <c r="F52" s="25" t="s">
-        <v>868</v>
+        <v>143</v>
       </c>
       <c r="G52" s="25" t="s">
-        <v>704</v>
-      </c>
-      <c r="K52" s="17"/>
+        <v>701</v>
+      </c>
     </row>
     <row r="53" spans="1:11" s="25" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A53" s="25" t="b">
@@ -15373,8 +15375,8 @@
       <c r="C53" s="25" t="s">
         <v>7</v>
       </c>
-      <c r="E53" s="25" t="s">
-        <v>474</v>
+      <c r="E53" s="28" t="s">
+        <v>741</v>
       </c>
       <c r="F53" s="25" t="s">
         <v>713</v>
@@ -15382,7 +15384,6 @@
       <c r="G53" s="25" t="s">
         <v>693</v>
       </c>
-      <c r="K53" s="17"/>
     </row>
     <row r="54" spans="1:11" s="25" customFormat="1" x14ac:dyDescent="0.2"/>
     <row r="55" spans="1:11" s="25" customFormat="1" x14ac:dyDescent="0.2">
@@ -15392,17 +15393,18 @@
       <c r="B55" s="25" t="s">
         <v>630</v>
       </c>
-      <c r="C55" s="25" t="s">
-        <v>7</v>
-      </c>
-      <c r="E55" s="25" t="s">
-        <v>151</v>
-      </c>
-      <c r="F55" s="25" t="s">
-        <v>713</v>
-      </c>
-      <c r="G55" s="25" t="s">
-        <v>693</v>
+      <c r="C55" s="28" t="s">
+        <v>54</v>
+      </c>
+      <c r="D55" s="28"/>
+      <c r="E55" s="28" t="s">
+        <v>474</v>
+      </c>
+      <c r="F55" s="28" t="s">
+        <v>725</v>
+      </c>
+      <c r="G55" s="28" t="s">
+        <v>701</v>
       </c>
     </row>
     <row r="56" spans="1:11" s="25" customFormat="1" x14ac:dyDescent="0.2">
@@ -15416,7 +15418,7 @@
         <v>54</v>
       </c>
       <c r="E56" s="25" t="s">
-        <v>151</v>
+        <v>474</v>
       </c>
       <c r="F56" s="25" t="s">
         <v>143</v>
@@ -15433,56 +15435,61 @@
         <v>630</v>
       </c>
       <c r="C57" s="25" t="s">
-        <v>775</v>
+        <v>73</v>
       </c>
       <c r="E57" s="25" t="s">
-        <v>151</v>
+        <v>474</v>
       </c>
       <c r="F57" s="25" t="s">
-        <v>735</v>
+        <v>471</v>
       </c>
       <c r="G57" s="25" t="s">
-        <v>877</v>
-      </c>
-    </row>
-    <row r="58" spans="1:11" s="25" customFormat="1" x14ac:dyDescent="0.2"/>
-    <row r="59" spans="1:11" s="25" customFormat="1" ht="16" customHeight="1" x14ac:dyDescent="0.2">
+        <v>703</v>
+      </c>
+    </row>
+    <row r="58" spans="1:11" s="25" customFormat="1" x14ac:dyDescent="0.2">
+      <c r="A58" s="25" t="b">
+        <v>1</v>
+      </c>
+      <c r="B58" s="25" t="s">
+        <v>630</v>
+      </c>
+      <c r="C58" s="25" t="s">
+        <v>74</v>
+      </c>
+      <c r="E58" s="25" t="s">
+        <v>474</v>
+      </c>
+      <c r="F58" s="25" t="s">
+        <v>868</v>
+      </c>
+      <c r="G58" s="25" t="s">
+        <v>704</v>
+      </c>
+      <c r="K58" s="17"/>
+    </row>
+    <row r="59" spans="1:11" s="25" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A59" s="25" t="b">
         <v>1</v>
       </c>
       <c r="B59" s="25" t="s">
         <v>630</v>
       </c>
+      <c r="C59" s="25" t="s">
+        <v>7</v>
+      </c>
       <c r="E59" s="25" t="s">
-        <v>117</v>
+        <v>474</v>
       </c>
       <c r="F59" s="25" t="s">
-        <v>669</v>
-      </c>
-      <c r="G59" s="29"/>
-      <c r="H59" s="31" t="s">
-        <v>691</v>
-      </c>
-    </row>
-    <row r="60" spans="1:11" s="25" customFormat="1" ht="16" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A60" s="25" t="b">
-        <v>1</v>
-      </c>
-      <c r="B60" s="25" t="s">
-        <v>630</v>
-      </c>
-      <c r="C60" s="30"/>
-      <c r="D60" s="32"/>
-      <c r="E60" s="25" t="s">
-        <v>117</v>
-      </c>
-      <c r="F60" s="25" t="s">
-        <v>118</v>
-      </c>
-      <c r="H60" s="31" t="s">
-        <v>692</v>
-      </c>
-    </row>
+        <v>713</v>
+      </c>
+      <c r="G59" s="25" t="s">
+        <v>693</v>
+      </c>
+      <c r="K59" s="17"/>
+    </row>
+    <row r="60" spans="1:11" s="25" customFormat="1" x14ac:dyDescent="0.2"/>
     <row r="61" spans="1:11" s="25" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A61" s="25" t="b">
         <v>1</v>
@@ -15491,17 +15498,16 @@
         <v>630</v>
       </c>
       <c r="C61" s="25" t="s">
-        <v>23</v>
-      </c>
-      <c r="D61" s="32"/>
+        <v>7</v>
+      </c>
       <c r="E61" s="25" t="s">
-        <v>117</v>
+        <v>151</v>
       </c>
       <c r="F61" s="25" t="s">
-        <v>119</v>
+        <v>713</v>
       </c>
       <c r="G61" s="25" t="s">
-        <v>699</v>
+        <v>693</v>
       </c>
     </row>
     <row r="62" spans="1:11" s="25" customFormat="1" x14ac:dyDescent="0.2">
@@ -15512,16 +15518,16 @@
         <v>630</v>
       </c>
       <c r="C62" s="25" t="s">
-        <v>56</v>
+        <v>54</v>
       </c>
       <c r="E62" s="25" t="s">
-        <v>117</v>
+        <v>151</v>
       </c>
       <c r="F62" s="25" t="s">
-        <v>144</v>
-      </c>
-      <c r="H62" s="25" t="s">
-        <v>921</v>
+        <v>143</v>
+      </c>
+      <c r="G62" s="25" t="s">
+        <v>701</v>
       </c>
     </row>
     <row r="63" spans="1:11" s="25" customFormat="1" x14ac:dyDescent="0.2">
@@ -15532,80 +15538,57 @@
         <v>630</v>
       </c>
       <c r="C63" s="25" t="s">
-        <v>54</v>
+        <v>775</v>
       </c>
       <c r="E63" s="25" t="s">
-        <v>117</v>
+        <v>151</v>
       </c>
       <c r="F63" s="25" t="s">
-        <v>143</v>
+        <v>735</v>
       </c>
       <c r="G63" s="25" t="s">
-        <v>701</v>
-      </c>
-    </row>
-    <row r="64" spans="1:11" s="25" customFormat="1" x14ac:dyDescent="0.2">
-      <c r="A64" s="25" t="b">
-        <v>1</v>
-      </c>
-      <c r="B64" s="25" t="s">
-        <v>630</v>
-      </c>
-      <c r="C64" s="25" t="s">
-        <v>7</v>
-      </c>
-      <c r="E64" s="25" t="s">
-        <v>117</v>
-      </c>
-      <c r="F64" s="25" t="s">
-        <v>713</v>
-      </c>
-      <c r="G64" s="25" t="s">
-        <v>693</v>
-      </c>
-      <c r="K64" s="17"/>
-    </row>
-    <row r="65" spans="1:10" s="25" customFormat="1" x14ac:dyDescent="0.2">
+        <v>877</v>
+      </c>
+    </row>
+    <row r="64" spans="1:11" s="25" customFormat="1" x14ac:dyDescent="0.2"/>
+    <row r="65" spans="1:11" s="25" customFormat="1" ht="16" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A65" s="25" t="b">
         <v>1</v>
       </c>
       <c r="B65" s="25" t="s">
         <v>630</v>
-      </c>
-      <c r="C65" s="25" t="s">
-        <v>53</v>
       </c>
       <c r="E65" s="25" t="s">
         <v>117</v>
       </c>
       <c r="F65" s="25" t="s">
-        <v>139</v>
-      </c>
-      <c r="G65" s="25" t="s">
-        <v>700</v>
-      </c>
-    </row>
-    <row r="66" spans="1:10" s="25" customFormat="1" x14ac:dyDescent="0.2">
+        <v>669</v>
+      </c>
+      <c r="G65" s="29"/>
+      <c r="H65" s="31" t="s">
+        <v>691</v>
+      </c>
+    </row>
+    <row r="66" spans="1:11" s="25" customFormat="1" ht="16" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A66" s="25" t="b">
         <v>1</v>
       </c>
       <c r="B66" s="25" t="s">
         <v>630</v>
       </c>
-      <c r="C66" s="25" t="s">
-        <v>8</v>
-      </c>
+      <c r="C66" s="30"/>
+      <c r="D66" s="32"/>
       <c r="E66" s="25" t="s">
         <v>117</v>
       </c>
       <c r="F66" s="25" t="s">
-        <v>77</v>
-      </c>
-      <c r="G66" s="25" t="s">
-        <v>694</v>
-      </c>
-    </row>
-    <row r="67" spans="1:10" s="25" customFormat="1" x14ac:dyDescent="0.2">
+        <v>118</v>
+      </c>
+      <c r="H66" s="31" t="s">
+        <v>692</v>
+      </c>
+    </row>
+    <row r="67" spans="1:11" s="25" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A67" s="25" t="b">
         <v>1</v>
       </c>
@@ -15613,242 +15596,226 @@
         <v>630</v>
       </c>
       <c r="C67" s="25" t="s">
-        <v>73</v>
-      </c>
+        <v>23</v>
+      </c>
+      <c r="D67" s="32"/>
       <c r="E67" s="25" t="s">
         <v>117</v>
       </c>
       <c r="F67" s="25" t="s">
+        <v>119</v>
+      </c>
+      <c r="G67" s="25" t="s">
+        <v>699</v>
+      </c>
+    </row>
+    <row r="68" spans="1:11" s="25" customFormat="1" x14ac:dyDescent="0.2">
+      <c r="A68" s="25" t="b">
+        <v>1</v>
+      </c>
+      <c r="B68" s="25" t="s">
+        <v>630</v>
+      </c>
+      <c r="C68" s="25" t="s">
+        <v>56</v>
+      </c>
+      <c r="E68" s="25" t="s">
+        <v>117</v>
+      </c>
+      <c r="F68" s="25" t="s">
+        <v>144</v>
+      </c>
+      <c r="H68" s="25" t="s">
+        <v>921</v>
+      </c>
+    </row>
+    <row r="69" spans="1:11" s="25" customFormat="1" x14ac:dyDescent="0.2">
+      <c r="A69" s="25" t="b">
+        <v>1</v>
+      </c>
+      <c r="B69" s="25" t="s">
+        <v>630</v>
+      </c>
+      <c r="C69" s="25" t="s">
+        <v>54</v>
+      </c>
+      <c r="E69" s="25" t="s">
+        <v>117</v>
+      </c>
+      <c r="F69" s="25" t="s">
+        <v>143</v>
+      </c>
+      <c r="G69" s="25" t="s">
+        <v>701</v>
+      </c>
+    </row>
+    <row r="70" spans="1:11" s="25" customFormat="1" x14ac:dyDescent="0.2">
+      <c r="A70" s="25" t="b">
+        <v>1</v>
+      </c>
+      <c r="B70" s="25" t="s">
+        <v>630</v>
+      </c>
+      <c r="C70" s="25" t="s">
+        <v>7</v>
+      </c>
+      <c r="E70" s="25" t="s">
+        <v>117</v>
+      </c>
+      <c r="F70" s="25" t="s">
+        <v>713</v>
+      </c>
+      <c r="G70" s="25" t="s">
+        <v>693</v>
+      </c>
+      <c r="K70" s="17"/>
+    </row>
+    <row r="71" spans="1:11" s="25" customFormat="1" x14ac:dyDescent="0.2">
+      <c r="A71" s="25" t="b">
+        <v>1</v>
+      </c>
+      <c r="B71" s="25" t="s">
+        <v>630</v>
+      </c>
+      <c r="C71" s="25" t="s">
+        <v>53</v>
+      </c>
+      <c r="E71" s="25" t="s">
+        <v>117</v>
+      </c>
+      <c r="F71" s="25" t="s">
+        <v>139</v>
+      </c>
+      <c r="G71" s="25" t="s">
+        <v>700</v>
+      </c>
+    </row>
+    <row r="72" spans="1:11" s="25" customFormat="1" x14ac:dyDescent="0.2">
+      <c r="A72" s="25" t="b">
+        <v>1</v>
+      </c>
+      <c r="B72" s="25" t="s">
+        <v>630</v>
+      </c>
+      <c r="C72" s="25" t="s">
+        <v>8</v>
+      </c>
+      <c r="E72" s="25" t="s">
+        <v>117</v>
+      </c>
+      <c r="F72" s="25" t="s">
+        <v>77</v>
+      </c>
+      <c r="G72" s="25" t="s">
+        <v>694</v>
+      </c>
+    </row>
+    <row r="73" spans="1:11" s="25" customFormat="1" x14ac:dyDescent="0.2">
+      <c r="A73" s="25" t="b">
+        <v>1</v>
+      </c>
+      <c r="B73" s="25" t="s">
+        <v>630</v>
+      </c>
+      <c r="C73" s="25" t="s">
+        <v>73</v>
+      </c>
+      <c r="E73" s="25" t="s">
+        <v>117</v>
+      </c>
+      <c r="F73" s="25" t="s">
         <v>471</v>
       </c>
-      <c r="G67" s="25" t="s">
+      <c r="G73" s="25" t="s">
         <v>703</v>
       </c>
     </row>
-    <row r="68" spans="1:10" s="25" customFormat="1" x14ac:dyDescent="0.2"/>
-    <row r="69" spans="1:10" s="17" customFormat="1" ht="17" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A69" s="17" t="b">
+    <row r="74" spans="1:11" s="25" customFormat="1" x14ac:dyDescent="0.2"/>
+    <row r="75" spans="1:11" s="17" customFormat="1" ht="17" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A75" s="17" t="b">
         <v>0</v>
       </c>
-      <c r="B69" s="17" t="s">
-        <v>630</v>
-      </c>
-      <c r="C69" s="26" t="s">
+      <c r="B75" s="17" t="s">
+        <v>630</v>
+      </c>
+      <c r="C75" s="26" t="s">
         <v>44</v>
       </c>
-      <c r="E69" s="17" t="s">
+      <c r="E75" s="17" t="s">
         <v>117</v>
       </c>
-      <c r="F69" s="17" t="s">
+      <c r="F75" s="17" t="s">
         <v>137</v>
       </c>
-      <c r="H69" s="27"/>
-      <c r="J69" s="17" t="s">
+      <c r="H75" s="27"/>
+      <c r="J75" s="17" t="s">
         <v>138</v>
       </c>
     </row>
-    <row r="70" spans="1:10" s="17" customFormat="1" ht="16" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A70" s="17" t="b">
+    <row r="76" spans="1:11" s="17" customFormat="1" ht="16" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A76" s="17" t="b">
         <v>0</v>
       </c>
-      <c r="B70" s="17" t="s">
-        <v>630</v>
-      </c>
-      <c r="C70" s="17" t="s">
+      <c r="B76" s="17" t="s">
+        <v>630</v>
+      </c>
+      <c r="C76" s="17" t="s">
         <v>45</v>
       </c>
-      <c r="E70" s="17" t="s">
+      <c r="E76" s="17" t="s">
         <v>117</v>
       </c>
-      <c r="F70" s="17" t="s">
+      <c r="F76" s="17" t="s">
         <v>137</v>
       </c>
-      <c r="H70" s="27"/>
-      <c r="J70" s="17" t="s">
+      <c r="H76" s="27"/>
+      <c r="J76" s="17" t="s">
         <v>138</v>
       </c>
     </row>
-    <row r="71" spans="1:10" s="17" customFormat="1" x14ac:dyDescent="0.2">
-      <c r="A71" s="17" t="b">
+    <row r="77" spans="1:11" s="17" customFormat="1" x14ac:dyDescent="0.2">
+      <c r="A77" s="17" t="b">
         <v>0</v>
       </c>
-      <c r="B71" s="17" t="s">
-        <v>630</v>
-      </c>
-      <c r="C71" s="17" t="s">
+      <c r="B77" s="17" t="s">
+        <v>630</v>
+      </c>
+      <c r="C77" s="17" t="s">
         <v>46</v>
       </c>
-      <c r="E71" s="17" t="s">
+      <c r="E77" s="17" t="s">
         <v>117</v>
       </c>
-      <c r="F71" s="17" t="s">
+      <c r="F77" s="17" t="s">
         <v>137</v>
       </c>
-      <c r="J71" s="17" t="s">
+      <c r="J77" s="17" t="s">
         <v>138</v>
       </c>
     </row>
-    <row r="72" spans="1:10" s="25" customFormat="1" x14ac:dyDescent="0.2"/>
-    <row r="73" spans="1:10" s="25" customFormat="1" x14ac:dyDescent="0.2">
-      <c r="A73" s="25" t="b">
-        <v>1</v>
-      </c>
-      <c r="B73" s="25" t="s">
-        <v>630</v>
-      </c>
-      <c r="C73" s="28" t="s">
+    <row r="78" spans="1:11" s="25" customFormat="1" x14ac:dyDescent="0.2"/>
+    <row r="79" spans="1:11" s="25" customFormat="1" x14ac:dyDescent="0.2">
+      <c r="A79" s="25" t="b">
+        <v>1</v>
+      </c>
+      <c r="B79" s="25" t="s">
+        <v>630</v>
+      </c>
+      <c r="C79" s="28" t="s">
         <v>54</v>
       </c>
-      <c r="D73" s="28"/>
-      <c r="E73" s="28" t="s">
+      <c r="D79" s="28"/>
+      <c r="E79" s="28" t="s">
         <v>117</v>
       </c>
-      <c r="F73" s="28" t="s">
+      <c r="F79" s="28" t="s">
         <v>725</v>
       </c>
-      <c r="G73" s="28" t="s">
+      <c r="G79" s="28" t="s">
         <v>701</v>
       </c>
     </row>
-    <row r="74" spans="1:10" s="25" customFormat="1" x14ac:dyDescent="0.2">
-      <c r="A74" s="25" t="b">
-        <v>1</v>
-      </c>
-      <c r="B74" s="25" t="s">
-        <v>630</v>
-      </c>
-      <c r="C74" s="25" t="s">
-        <v>24</v>
-      </c>
-      <c r="D74" s="33" t="s">
-        <v>121</v>
-      </c>
-      <c r="E74" s="25" t="s">
-        <v>117</v>
-      </c>
-      <c r="F74" s="25" t="s">
-        <v>129</v>
-      </c>
-      <c r="G74" s="25" t="s">
-        <v>136</v>
-      </c>
-    </row>
-    <row r="75" spans="1:10" s="25" customFormat="1" x14ac:dyDescent="0.2">
-      <c r="A75" s="25" t="b">
-        <v>1</v>
-      </c>
-      <c r="B75" s="25" t="s">
-        <v>630</v>
-      </c>
-      <c r="C75" s="25" t="s">
-        <v>24</v>
-      </c>
-      <c r="D75" s="32" t="s">
-        <v>122</v>
-      </c>
-      <c r="E75" s="25" t="s">
-        <v>117</v>
-      </c>
-      <c r="F75" s="25" t="s">
-        <v>129</v>
-      </c>
-      <c r="G75" s="25" t="s">
-        <v>134</v>
-      </c>
-    </row>
-    <row r="76" spans="1:10" s="25" customFormat="1" x14ac:dyDescent="0.2">
-      <c r="A76" s="25" t="b">
-        <v>1</v>
-      </c>
-      <c r="B76" s="25" t="s">
-        <v>630</v>
-      </c>
-      <c r="C76" s="25" t="s">
-        <v>24</v>
-      </c>
-      <c r="D76" s="32" t="s">
-        <v>123</v>
-      </c>
-      <c r="E76" s="25" t="s">
-        <v>117</v>
-      </c>
-      <c r="F76" s="25" t="s">
-        <v>129</v>
-      </c>
-      <c r="G76" s="25" t="s">
-        <v>130</v>
-      </c>
-    </row>
-    <row r="77" spans="1:10" s="25" customFormat="1" x14ac:dyDescent="0.2">
-      <c r="A77" s="25" t="b">
-        <v>1</v>
-      </c>
-      <c r="B77" s="25" t="s">
-        <v>630</v>
-      </c>
-      <c r="C77" s="25" t="s">
-        <v>24</v>
-      </c>
-      <c r="D77" s="32" t="s">
-        <v>124</v>
-      </c>
-      <c r="E77" s="25" t="s">
-        <v>117</v>
-      </c>
-      <c r="F77" s="25" t="s">
-        <v>129</v>
-      </c>
-      <c r="G77" s="25" t="s">
-        <v>131</v>
-      </c>
-    </row>
-    <row r="78" spans="1:10" s="25" customFormat="1" x14ac:dyDescent="0.2">
-      <c r="A78" s="25" t="b">
-        <v>1</v>
-      </c>
-      <c r="B78" s="25" t="s">
-        <v>630</v>
-      </c>
-      <c r="C78" s="25" t="s">
-        <v>24</v>
-      </c>
-      <c r="D78" s="32" t="s">
-        <v>125</v>
-      </c>
-      <c r="E78" s="25" t="s">
-        <v>117</v>
-      </c>
-      <c r="F78" s="25" t="s">
-        <v>129</v>
-      </c>
-      <c r="G78" s="25" t="s">
-        <v>132</v>
-      </c>
-    </row>
-    <row r="79" spans="1:10" s="25" customFormat="1" x14ac:dyDescent="0.2">
-      <c r="A79" s="25" t="b">
-        <v>1</v>
-      </c>
-      <c r="B79" s="25" t="s">
-        <v>630</v>
-      </c>
-      <c r="C79" s="25" t="s">
-        <v>24</v>
-      </c>
-      <c r="D79" s="32" t="s">
-        <v>126</v>
-      </c>
-      <c r="E79" s="25" t="s">
-        <v>117</v>
-      </c>
-      <c r="F79" s="25" t="s">
-        <v>129</v>
-      </c>
-      <c r="G79" s="25" t="s">
-        <v>133</v>
-      </c>
-    </row>
-    <row r="80" spans="1:10" s="25" customFormat="1" x14ac:dyDescent="0.2">
+    <row r="80" spans="1:11" s="25" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A80" s="25" t="b">
         <v>1</v>
       </c>
@@ -15858,8 +15825,8 @@
       <c r="C80" s="25" t="s">
         <v>24</v>
       </c>
-      <c r="D80" s="32" t="s">
-        <v>127</v>
+      <c r="D80" s="33" t="s">
+        <v>121</v>
       </c>
       <c r="E80" s="25" t="s">
         <v>117</v>
@@ -15868,10 +15835,10 @@
         <v>129</v>
       </c>
       <c r="G80" s="25" t="s">
-        <v>127</v>
-      </c>
-    </row>
-    <row r="81" spans="1:10" s="25" customFormat="1" x14ac:dyDescent="0.2">
+        <v>136</v>
+      </c>
+    </row>
+    <row r="81" spans="1:8" s="25" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A81" s="25" t="b">
         <v>1</v>
       </c>
@@ -15882,7 +15849,7 @@
         <v>24</v>
       </c>
       <c r="D81" s="32" t="s">
-        <v>128</v>
+        <v>122</v>
       </c>
       <c r="E81" s="25" t="s">
         <v>117</v>
@@ -15891,175 +15858,191 @@
         <v>129</v>
       </c>
       <c r="G81" s="25" t="s">
+        <v>134</v>
+      </c>
+    </row>
+    <row r="82" spans="1:8" s="25" customFormat="1" x14ac:dyDescent="0.2">
+      <c r="A82" s="25" t="b">
+        <v>1</v>
+      </c>
+      <c r="B82" s="25" t="s">
+        <v>630</v>
+      </c>
+      <c r="C82" s="25" t="s">
+        <v>24</v>
+      </c>
+      <c r="D82" s="32" t="s">
+        <v>123</v>
+      </c>
+      <c r="E82" s="25" t="s">
+        <v>117</v>
+      </c>
+      <c r="F82" s="25" t="s">
+        <v>129</v>
+      </c>
+      <c r="G82" s="25" t="s">
+        <v>130</v>
+      </c>
+    </row>
+    <row r="83" spans="1:8" s="25" customFormat="1" x14ac:dyDescent="0.2">
+      <c r="A83" s="25" t="b">
+        <v>1</v>
+      </c>
+      <c r="B83" s="25" t="s">
+        <v>630</v>
+      </c>
+      <c r="C83" s="25" t="s">
+        <v>24</v>
+      </c>
+      <c r="D83" s="32" t="s">
+        <v>124</v>
+      </c>
+      <c r="E83" s="25" t="s">
+        <v>117</v>
+      </c>
+      <c r="F83" s="25" t="s">
+        <v>129</v>
+      </c>
+      <c r="G83" s="25" t="s">
+        <v>131</v>
+      </c>
+    </row>
+    <row r="84" spans="1:8" s="25" customFormat="1" x14ac:dyDescent="0.2">
+      <c r="A84" s="25" t="b">
+        <v>1</v>
+      </c>
+      <c r="B84" s="25" t="s">
+        <v>630</v>
+      </c>
+      <c r="C84" s="25" t="s">
+        <v>24</v>
+      </c>
+      <c r="D84" s="32" t="s">
+        <v>125</v>
+      </c>
+      <c r="E84" s="25" t="s">
+        <v>117</v>
+      </c>
+      <c r="F84" s="25" t="s">
+        <v>129</v>
+      </c>
+      <c r="G84" s="25" t="s">
+        <v>132</v>
+      </c>
+    </row>
+    <row r="85" spans="1:8" s="25" customFormat="1" x14ac:dyDescent="0.2">
+      <c r="A85" s="25" t="b">
+        <v>1</v>
+      </c>
+      <c r="B85" s="25" t="s">
+        <v>630</v>
+      </c>
+      <c r="C85" s="25" t="s">
+        <v>24</v>
+      </c>
+      <c r="D85" s="32" t="s">
+        <v>126</v>
+      </c>
+      <c r="E85" s="25" t="s">
+        <v>117</v>
+      </c>
+      <c r="F85" s="25" t="s">
+        <v>129</v>
+      </c>
+      <c r="G85" s="25" t="s">
+        <v>133</v>
+      </c>
+    </row>
+    <row r="86" spans="1:8" s="25" customFormat="1" x14ac:dyDescent="0.2">
+      <c r="A86" s="25" t="b">
+        <v>1</v>
+      </c>
+      <c r="B86" s="25" t="s">
+        <v>630</v>
+      </c>
+      <c r="C86" s="25" t="s">
+        <v>24</v>
+      </c>
+      <c r="D86" s="32" t="s">
+        <v>127</v>
+      </c>
+      <c r="E86" s="25" t="s">
+        <v>117</v>
+      </c>
+      <c r="F86" s="25" t="s">
+        <v>129</v>
+      </c>
+      <c r="G86" s="25" t="s">
+        <v>127</v>
+      </c>
+    </row>
+    <row r="87" spans="1:8" s="25" customFormat="1" x14ac:dyDescent="0.2">
+      <c r="A87" s="25" t="b">
+        <v>1</v>
+      </c>
+      <c r="B87" s="25" t="s">
+        <v>630</v>
+      </c>
+      <c r="C87" s="25" t="s">
+        <v>24</v>
+      </c>
+      <c r="D87" s="32" t="s">
+        <v>128</v>
+      </c>
+      <c r="E87" s="25" t="s">
+        <v>117</v>
+      </c>
+      <c r="F87" s="25" t="s">
+        <v>129</v>
+      </c>
+      <c r="G87" s="25" t="s">
         <v>135</v>
       </c>
     </row>
-    <row r="82" spans="1:10" s="25" customFormat="1" x14ac:dyDescent="0.2">
-      <c r="D82" s="32"/>
-    </row>
-    <row r="83" spans="1:10" s="25" customFormat="1" x14ac:dyDescent="0.2">
-      <c r="A83" s="25" t="b">
-        <v>1</v>
-      </c>
-      <c r="B83" s="25" t="s">
-        <v>630</v>
-      </c>
-      <c r="C83" s="25" t="s">
+    <row r="88" spans="1:8" s="25" customFormat="1" x14ac:dyDescent="0.2">
+      <c r="D88" s="32"/>
+    </row>
+    <row r="89" spans="1:8" s="25" customFormat="1" x14ac:dyDescent="0.2">
+      <c r="A89" s="25" t="b">
+        <v>1</v>
+      </c>
+      <c r="B89" s="25" t="s">
+        <v>630</v>
+      </c>
+      <c r="C89" s="25" t="s">
         <v>9</v>
       </c>
-      <c r="E83" s="41" t="s">
+      <c r="E89" s="41" t="s">
         <v>76</v>
       </c>
-      <c r="F83" s="41" t="s">
+      <c r="F89" s="41" t="s">
         <v>120</v>
       </c>
-      <c r="H83" s="30" t="s">
+      <c r="H89" s="30" t="s">
         <v>722</v>
       </c>
     </row>
-    <row r="84" spans="1:10" s="25" customFormat="1" x14ac:dyDescent="0.2">
-      <c r="A84" s="25" t="b">
-        <v>1</v>
-      </c>
-      <c r="B84" s="25" t="s">
-        <v>630</v>
-      </c>
-      <c r="C84" s="25" t="s">
+    <row r="90" spans="1:8" s="25" customFormat="1" x14ac:dyDescent="0.2">
+      <c r="A90" s="25" t="b">
+        <v>1</v>
+      </c>
+      <c r="B90" s="25" t="s">
+        <v>630</v>
+      </c>
+      <c r="C90" s="25" t="s">
         <v>11</v>
-      </c>
-      <c r="E84" s="25" t="s">
-        <v>76</v>
-      </c>
-      <c r="F84" s="25" t="s">
-        <v>80</v>
-      </c>
-      <c r="G84" s="25" t="s">
-        <v>696</v>
-      </c>
-    </row>
-    <row r="85" spans="1:10" s="25" customFormat="1" x14ac:dyDescent="0.2">
-      <c r="A85" s="25" t="b">
-        <v>1</v>
-      </c>
-      <c r="B85" s="25" t="s">
-        <v>630</v>
-      </c>
-      <c r="C85" s="25" t="s">
-        <v>8</v>
-      </c>
-      <c r="E85" s="25" t="s">
-        <v>76</v>
-      </c>
-      <c r="F85" s="25" t="s">
-        <v>77</v>
-      </c>
-      <c r="G85" s="25" t="s">
-        <v>694</v>
-      </c>
-    </row>
-    <row r="86" spans="1:10" s="25" customFormat="1" x14ac:dyDescent="0.2">
-      <c r="A86" s="25" t="b">
-        <v>1</v>
-      </c>
-      <c r="B86" s="25" t="s">
-        <v>630</v>
-      </c>
-      <c r="C86" s="25" t="s">
-        <v>54</v>
-      </c>
-      <c r="E86" s="25" t="s">
-        <v>76</v>
-      </c>
-      <c r="F86" s="25" t="s">
-        <v>712</v>
-      </c>
-      <c r="G86" s="25" t="s">
-        <v>701</v>
-      </c>
-    </row>
-    <row r="87" spans="1:10" s="25" customFormat="1" x14ac:dyDescent="0.2">
-      <c r="A87" s="25" t="b">
-        <v>1</v>
-      </c>
-      <c r="B87" s="25" t="s">
-        <v>630</v>
-      </c>
-      <c r="C87" s="25" t="s">
-        <v>18</v>
-      </c>
-      <c r="E87" s="25" t="s">
-        <v>76</v>
-      </c>
-      <c r="F87" s="25" t="s">
-        <v>115</v>
-      </c>
-      <c r="G87" s="25" t="s">
-        <v>697</v>
-      </c>
-    </row>
-    <row r="88" spans="1:10" s="25" customFormat="1" ht="17" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A88" s="25" t="b">
-        <v>1</v>
-      </c>
-      <c r="B88" s="25" t="s">
-        <v>630</v>
-      </c>
-      <c r="C88" s="25" t="s">
-        <v>13</v>
-      </c>
-      <c r="D88" s="32"/>
-      <c r="E88" s="25" t="s">
-        <v>76</v>
-      </c>
-      <c r="F88" s="25" t="s">
-        <v>83</v>
-      </c>
-      <c r="H88" s="42" t="s">
-        <v>862</v>
-      </c>
-    </row>
-    <row r="89" spans="1:10" s="25" customFormat="1" x14ac:dyDescent="0.2">
-      <c r="A89" s="25" t="b">
-        <v>1</v>
-      </c>
-      <c r="B89" s="25" t="s">
-        <v>630</v>
-      </c>
-      <c r="C89" s="28" t="s">
-        <v>54</v>
-      </c>
-      <c r="D89" s="28"/>
-      <c r="E89" s="28" t="s">
-        <v>76</v>
-      </c>
-      <c r="F89" s="28" t="s">
-        <v>725</v>
-      </c>
-      <c r="G89" s="28" t="s">
-        <v>701</v>
-      </c>
-    </row>
-    <row r="90" spans="1:10" s="25" customFormat="1" x14ac:dyDescent="0.2">
-      <c r="A90" s="25" t="b">
-        <v>1</v>
-      </c>
-      <c r="B90" s="25" t="s">
-        <v>630</v>
-      </c>
-      <c r="C90" s="25" t="s">
-        <v>777</v>
       </c>
       <c r="E90" s="25" t="s">
         <v>76</v>
       </c>
       <c r="F90" s="25" t="s">
-        <v>729</v>
+        <v>80</v>
       </c>
       <c r="G90" s="25" t="s">
-        <v>875</v>
-      </c>
-    </row>
-    <row r="91" spans="1:10" s="25" customFormat="1" x14ac:dyDescent="0.2">
+        <v>696</v>
+      </c>
+    </row>
+    <row r="91" spans="1:8" s="25" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A91" s="25" t="b">
         <v>1</v>
       </c>
@@ -16067,19 +16050,19 @@
         <v>630</v>
       </c>
       <c r="C91" s="25" t="s">
-        <v>54</v>
+        <v>8</v>
       </c>
       <c r="E91" s="25" t="s">
         <v>76</v>
       </c>
       <c r="F91" s="25" t="s">
-        <v>143</v>
+        <v>77</v>
       </c>
       <c r="G91" s="25" t="s">
-        <v>701</v>
-      </c>
-    </row>
-    <row r="92" spans="1:10" s="25" customFormat="1" x14ac:dyDescent="0.2">
+        <v>694</v>
+      </c>
+    </row>
+    <row r="92" spans="1:8" s="25" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A92" s="25" t="b">
         <v>1</v>
       </c>
@@ -16087,19 +16070,19 @@
         <v>630</v>
       </c>
       <c r="C92" s="25" t="s">
-        <v>7</v>
+        <v>54</v>
       </c>
       <c r="E92" s="25" t="s">
         <v>76</v>
       </c>
       <c r="F92" s="25" t="s">
-        <v>713</v>
+        <v>712</v>
       </c>
       <c r="G92" s="25" t="s">
-        <v>693</v>
-      </c>
-    </row>
-    <row r="93" spans="1:10" s="17" customFormat="1" ht="17" customHeight="1" x14ac:dyDescent="0.2">
+        <v>701</v>
+      </c>
+    </row>
+    <row r="93" spans="1:8" s="25" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A93" s="25" t="b">
         <v>1</v>
       </c>
@@ -16107,25 +16090,19 @@
         <v>630</v>
       </c>
       <c r="C93" s="25" t="s">
-        <v>15</v>
-      </c>
-      <c r="D93" s="33" t="s">
-        <v>84</v>
+        <v>18</v>
       </c>
       <c r="E93" s="25" t="s">
         <v>76</v>
       </c>
       <c r="F93" s="25" t="s">
-        <v>100</v>
+        <v>115</v>
       </c>
       <c r="G93" s="25" t="s">
-        <v>75</v>
-      </c>
-      <c r="H93" s="25"/>
-      <c r="I93" s="25"/>
-      <c r="J93" s="25"/>
-    </row>
-    <row r="94" spans="1:10" s="25" customFormat="1" x14ac:dyDescent="0.2">
+        <v>697</v>
+      </c>
+    </row>
+    <row r="94" spans="1:8" s="25" customFormat="1" ht="17" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A94" s="25" t="b">
         <v>1</v>
       </c>
@@ -16133,45 +16110,41 @@
         <v>630</v>
       </c>
       <c r="C94" s="25" t="s">
-        <v>15</v>
-      </c>
-      <c r="D94" s="33" t="s">
-        <v>85</v>
-      </c>
+        <v>13</v>
+      </c>
+      <c r="D94" s="32"/>
       <c r="E94" s="25" t="s">
         <v>76</v>
       </c>
       <c r="F94" s="25" t="s">
-        <v>100</v>
-      </c>
-      <c r="G94" s="25" t="s">
-        <v>101</v>
-      </c>
-    </row>
-    <row r="95" spans="1:10" s="25" customFormat="1" x14ac:dyDescent="0.2">
+        <v>83</v>
+      </c>
+      <c r="H94" s="42" t="s">
+        <v>862</v>
+      </c>
+    </row>
+    <row r="95" spans="1:8" s="25" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A95" s="25" t="b">
         <v>1</v>
       </c>
       <c r="B95" s="25" t="s">
         <v>630</v>
       </c>
-      <c r="C95" s="25" t="s">
-        <v>15</v>
-      </c>
-      <c r="D95" s="34" t="s">
-        <v>86</v>
-      </c>
-      <c r="E95" s="25" t="s">
+      <c r="C95" s="28" t="s">
+        <v>54</v>
+      </c>
+      <c r="D95" s="28"/>
+      <c r="E95" s="28" t="s">
         <v>76</v>
       </c>
-      <c r="F95" s="25" t="s">
-        <v>100</v>
-      </c>
-      <c r="G95" s="25" t="s">
-        <v>102</v>
-      </c>
-    </row>
-    <row r="96" spans="1:10" s="25" customFormat="1" x14ac:dyDescent="0.2">
+      <c r="F95" s="28" t="s">
+        <v>725</v>
+      </c>
+      <c r="G95" s="28" t="s">
+        <v>701</v>
+      </c>
+    </row>
+    <row r="96" spans="1:8" s="25" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A96" s="25" t="b">
         <v>1</v>
       </c>
@@ -16179,22 +16152,19 @@
         <v>630</v>
       </c>
       <c r="C96" s="25" t="s">
-        <v>15</v>
-      </c>
-      <c r="D96" s="34" t="s">
-        <v>87</v>
+        <v>777</v>
       </c>
       <c r="E96" s="25" t="s">
         <v>76</v>
       </c>
       <c r="F96" s="25" t="s">
-        <v>100</v>
+        <v>729</v>
       </c>
       <c r="G96" s="25" t="s">
-        <v>103</v>
-      </c>
-    </row>
-    <row r="97" spans="1:11" s="25" customFormat="1" x14ac:dyDescent="0.2">
+        <v>875</v>
+      </c>
+    </row>
+    <row r="97" spans="1:10" s="25" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A97" s="25" t="b">
         <v>1</v>
       </c>
@@ -16202,22 +16172,19 @@
         <v>630</v>
       </c>
       <c r="C97" s="25" t="s">
-        <v>15</v>
-      </c>
-      <c r="D97" s="34" t="s">
-        <v>88</v>
+        <v>54</v>
       </c>
       <c r="E97" s="25" t="s">
         <v>76</v>
       </c>
       <c r="F97" s="25" t="s">
-        <v>100</v>
+        <v>143</v>
       </c>
       <c r="G97" s="25" t="s">
-        <v>104</v>
-      </c>
-    </row>
-    <row r="98" spans="1:11" s="25" customFormat="1" x14ac:dyDescent="0.2">
+        <v>701</v>
+      </c>
+    </row>
+    <row r="98" spans="1:10" s="25" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A98" s="25" t="b">
         <v>1</v>
       </c>
@@ -16225,22 +16192,19 @@
         <v>630</v>
       </c>
       <c r="C98" s="25" t="s">
-        <v>15</v>
-      </c>
-      <c r="D98" s="32" t="s">
-        <v>89</v>
+        <v>7</v>
       </c>
       <c r="E98" s="25" t="s">
         <v>76</v>
       </c>
       <c r="F98" s="25" t="s">
-        <v>100</v>
+        <v>713</v>
       </c>
       <c r="G98" s="25" t="s">
-        <v>113</v>
-      </c>
-    </row>
-    <row r="99" spans="1:11" s="25" customFormat="1" x14ac:dyDescent="0.2">
+        <v>693</v>
+      </c>
+    </row>
+    <row r="99" spans="1:10" s="25" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A99" s="25" t="b">
         <v>1</v>
       </c>
@@ -16248,22 +16212,19 @@
         <v>630</v>
       </c>
       <c r="C99" s="25" t="s">
-        <v>15</v>
-      </c>
-      <c r="D99" s="32" t="s">
-        <v>90</v>
+        <v>771</v>
       </c>
       <c r="E99" s="25" t="s">
         <v>76</v>
       </c>
       <c r="F99" s="25" t="s">
-        <v>100</v>
+        <v>727</v>
       </c>
       <c r="G99" s="25" t="s">
-        <v>112</v>
-      </c>
-    </row>
-    <row r="100" spans="1:11" s="25" customFormat="1" x14ac:dyDescent="0.2">
+        <v>985</v>
+      </c>
+    </row>
+    <row r="100" spans="1:10" s="17" customFormat="1" ht="17" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A100" s="25" t="b">
         <v>1</v>
       </c>
@@ -16274,7 +16235,7 @@
         <v>15</v>
       </c>
       <c r="D100" s="33" t="s">
-        <v>91</v>
+        <v>84</v>
       </c>
       <c r="E100" s="25" t="s">
         <v>76</v>
@@ -16283,10 +16244,13 @@
         <v>100</v>
       </c>
       <c r="G100" s="25" t="s">
-        <v>109</v>
-      </c>
-    </row>
-    <row r="101" spans="1:11" s="25" customFormat="1" x14ac:dyDescent="0.2">
+        <v>75</v>
+      </c>
+      <c r="H100" s="25"/>
+      <c r="I100" s="25"/>
+      <c r="J100" s="25"/>
+    </row>
+    <row r="101" spans="1:10" s="25" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A101" s="25" t="b">
         <v>1</v>
       </c>
@@ -16297,7 +16261,7 @@
         <v>15</v>
       </c>
       <c r="D101" s="33" t="s">
-        <v>92</v>
+        <v>85</v>
       </c>
       <c r="E101" s="25" t="s">
         <v>76</v>
@@ -16306,10 +16270,10 @@
         <v>100</v>
       </c>
       <c r="G101" s="25" t="s">
-        <v>108</v>
-      </c>
-    </row>
-    <row r="102" spans="1:11" s="25" customFormat="1" x14ac:dyDescent="0.2">
+        <v>101</v>
+      </c>
+    </row>
+    <row r="102" spans="1:10" s="25" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A102" s="25" t="b">
         <v>1</v>
       </c>
@@ -16319,8 +16283,8 @@
       <c r="C102" s="25" t="s">
         <v>15</v>
       </c>
-      <c r="D102" s="32" t="s">
-        <v>93</v>
+      <c r="D102" s="34" t="s">
+        <v>86</v>
       </c>
       <c r="E102" s="25" t="s">
         <v>76</v>
@@ -16329,10 +16293,10 @@
         <v>100</v>
       </c>
       <c r="G102" s="25" t="s">
-        <v>107</v>
-      </c>
-    </row>
-    <row r="103" spans="1:11" s="25" customFormat="1" x14ac:dyDescent="0.2">
+        <v>102</v>
+      </c>
+    </row>
+    <row r="103" spans="1:10" s="25" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A103" s="25" t="b">
         <v>1</v>
       </c>
@@ -16342,8 +16306,8 @@
       <c r="C103" s="25" t="s">
         <v>15</v>
       </c>
-      <c r="D103" s="32" t="s">
-        <v>94</v>
+      <c r="D103" s="34" t="s">
+        <v>87</v>
       </c>
       <c r="E103" s="25" t="s">
         <v>76</v>
@@ -16352,10 +16316,10 @@
         <v>100</v>
       </c>
       <c r="G103" s="25" t="s">
-        <v>106</v>
-      </c>
-    </row>
-    <row r="104" spans="1:11" s="25" customFormat="1" x14ac:dyDescent="0.2">
+        <v>103</v>
+      </c>
+    </row>
+    <row r="104" spans="1:10" s="25" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A104" s="25" t="b">
         <v>1</v>
       </c>
@@ -16365,8 +16329,8 @@
       <c r="C104" s="25" t="s">
         <v>15</v>
       </c>
-      <c r="D104" s="32" t="s">
-        <v>95</v>
+      <c r="D104" s="34" t="s">
+        <v>88</v>
       </c>
       <c r="E104" s="25" t="s">
         <v>76</v>
@@ -16375,10 +16339,10 @@
         <v>100</v>
       </c>
       <c r="G104" s="25" t="s">
-        <v>105</v>
-      </c>
-    </row>
-    <row r="105" spans="1:11" s="25" customFormat="1" x14ac:dyDescent="0.2">
+        <v>104</v>
+      </c>
+    </row>
+    <row r="105" spans="1:10" s="25" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A105" s="25" t="b">
         <v>1</v>
       </c>
@@ -16389,7 +16353,7 @@
         <v>15</v>
       </c>
       <c r="D105" s="32" t="s">
-        <v>96</v>
+        <v>89</v>
       </c>
       <c r="E105" s="25" t="s">
         <v>76</v>
@@ -16398,10 +16362,10 @@
         <v>100</v>
       </c>
       <c r="G105" s="25" t="s">
-        <v>110</v>
-      </c>
-    </row>
-    <row r="106" spans="1:11" s="25" customFormat="1" x14ac:dyDescent="0.2">
+        <v>113</v>
+      </c>
+    </row>
+    <row r="106" spans="1:10" s="25" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A106" s="25" t="b">
         <v>1</v>
       </c>
@@ -16412,7 +16376,7 @@
         <v>15</v>
       </c>
       <c r="D106" s="32" t="s">
-        <v>97</v>
+        <v>90</v>
       </c>
       <c r="E106" s="25" t="s">
         <v>76</v>
@@ -16421,10 +16385,10 @@
         <v>100</v>
       </c>
       <c r="G106" s="25" t="s">
-        <v>97</v>
-      </c>
-    </row>
-    <row r="107" spans="1:11" s="25" customFormat="1" x14ac:dyDescent="0.2">
+        <v>112</v>
+      </c>
+    </row>
+    <row r="107" spans="1:10" s="25" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A107" s="25" t="b">
         <v>1</v>
       </c>
@@ -16434,8 +16398,8 @@
       <c r="C107" s="25" t="s">
         <v>15</v>
       </c>
-      <c r="D107" s="32" t="s">
-        <v>98</v>
+      <c r="D107" s="33" t="s">
+        <v>91</v>
       </c>
       <c r="E107" s="25" t="s">
         <v>76</v>
@@ -16444,10 +16408,10 @@
         <v>100</v>
       </c>
       <c r="G107" s="25" t="s">
-        <v>111</v>
-      </c>
-    </row>
-    <row r="108" spans="1:11" s="25" customFormat="1" x14ac:dyDescent="0.2">
+        <v>109</v>
+      </c>
+    </row>
+    <row r="108" spans="1:10" s="25" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A108" s="25" t="b">
         <v>1</v>
       </c>
@@ -16457,8 +16421,8 @@
       <c r="C108" s="25" t="s">
         <v>15</v>
       </c>
-      <c r="D108" s="32" t="s">
-        <v>99</v>
+      <c r="D108" s="33" t="s">
+        <v>92</v>
       </c>
       <c r="E108" s="25" t="s">
         <v>76</v>
@@ -16466,12 +16430,173 @@
       <c r="F108" s="25" t="s">
         <v>100</v>
       </c>
-      <c r="G108" s="41" t="s">
+      <c r="G108" s="25" t="s">
+        <v>108</v>
+      </c>
+    </row>
+    <row r="109" spans="1:10" s="25" customFormat="1" x14ac:dyDescent="0.2">
+      <c r="A109" s="25" t="b">
+        <v>1</v>
+      </c>
+      <c r="B109" s="25" t="s">
+        <v>630</v>
+      </c>
+      <c r="C109" s="25" t="s">
+        <v>15</v>
+      </c>
+      <c r="D109" s="32" t="s">
+        <v>93</v>
+      </c>
+      <c r="E109" s="25" t="s">
+        <v>76</v>
+      </c>
+      <c r="F109" s="25" t="s">
+        <v>100</v>
+      </c>
+      <c r="G109" s="25" t="s">
+        <v>107</v>
+      </c>
+    </row>
+    <row r="110" spans="1:10" s="25" customFormat="1" x14ac:dyDescent="0.2">
+      <c r="A110" s="25" t="b">
+        <v>1</v>
+      </c>
+      <c r="B110" s="25" t="s">
+        <v>630</v>
+      </c>
+      <c r="C110" s="25" t="s">
+        <v>15</v>
+      </c>
+      <c r="D110" s="32" t="s">
+        <v>94</v>
+      </c>
+      <c r="E110" s="25" t="s">
+        <v>76</v>
+      </c>
+      <c r="F110" s="25" t="s">
+        <v>100</v>
+      </c>
+      <c r="G110" s="25" t="s">
+        <v>106</v>
+      </c>
+    </row>
+    <row r="111" spans="1:10" s="25" customFormat="1" x14ac:dyDescent="0.2">
+      <c r="A111" s="25" t="b">
+        <v>1</v>
+      </c>
+      <c r="B111" s="25" t="s">
+        <v>630</v>
+      </c>
+      <c r="C111" s="25" t="s">
+        <v>15</v>
+      </c>
+      <c r="D111" s="32" t="s">
+        <v>95</v>
+      </c>
+      <c r="E111" s="25" t="s">
+        <v>76</v>
+      </c>
+      <c r="F111" s="25" t="s">
+        <v>100</v>
+      </c>
+      <c r="G111" s="25" t="s">
+        <v>105</v>
+      </c>
+    </row>
+    <row r="112" spans="1:10" s="25" customFormat="1" x14ac:dyDescent="0.2">
+      <c r="A112" s="25" t="b">
+        <v>1</v>
+      </c>
+      <c r="B112" s="25" t="s">
+        <v>630</v>
+      </c>
+      <c r="C112" s="25" t="s">
+        <v>15</v>
+      </c>
+      <c r="D112" s="32" t="s">
+        <v>96</v>
+      </c>
+      <c r="E112" s="25" t="s">
+        <v>76</v>
+      </c>
+      <c r="F112" s="25" t="s">
+        <v>100</v>
+      </c>
+      <c r="G112" s="25" t="s">
+        <v>110</v>
+      </c>
+    </row>
+    <row r="113" spans="1:11" s="25" customFormat="1" x14ac:dyDescent="0.2">
+      <c r="A113" s="25" t="b">
+        <v>1</v>
+      </c>
+      <c r="B113" s="25" t="s">
+        <v>630</v>
+      </c>
+      <c r="C113" s="25" t="s">
+        <v>15</v>
+      </c>
+      <c r="D113" s="32" t="s">
+        <v>97</v>
+      </c>
+      <c r="E113" s="25" t="s">
+        <v>76</v>
+      </c>
+      <c r="F113" s="25" t="s">
+        <v>100</v>
+      </c>
+      <c r="G113" s="25" t="s">
+        <v>97</v>
+      </c>
+    </row>
+    <row r="114" spans="1:11" s="25" customFormat="1" x14ac:dyDescent="0.2">
+      <c r="A114" s="25" t="b">
+        <v>1</v>
+      </c>
+      <c r="B114" s="25" t="s">
+        <v>630</v>
+      </c>
+      <c r="C114" s="25" t="s">
+        <v>15</v>
+      </c>
+      <c r="D114" s="32" t="s">
+        <v>98</v>
+      </c>
+      <c r="E114" s="25" t="s">
+        <v>76</v>
+      </c>
+      <c r="F114" s="25" t="s">
+        <v>100</v>
+      </c>
+      <c r="G114" s="25" t="s">
+        <v>111</v>
+      </c>
+    </row>
+    <row r="115" spans="1:11" s="25" customFormat="1" x14ac:dyDescent="0.2">
+      <c r="A115" s="25" t="b">
+        <v>1</v>
+      </c>
+      <c r="B115" s="25" t="s">
+        <v>630</v>
+      </c>
+      <c r="C115" s="25" t="s">
+        <v>15</v>
+      </c>
+      <c r="D115" s="32" t="s">
+        <v>99</v>
+      </c>
+      <c r="E115" s="25" t="s">
+        <v>76</v>
+      </c>
+      <c r="F115" s="25" t="s">
+        <v>100</v>
+      </c>
+      <c r="G115" s="41" t="s">
         <v>530</v>
       </c>
-      <c r="H108" s="29"/>
-      <c r="I108" s="29"/>
-      <c r="K108" s="41"/>
+      <c r="H115" s="29"/>
+      <c r="I115" s="29"/>
+      <c r="K115" s="41"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>

<commit_message>
Rename data binding variables (dat0->dat, dat->datEmpty)
</commit_message>
<xml_diff>
--- a/data/mapping_config_files/nwss_to_odm_v2_mapping.xlsx
+++ b/data/mapping_config_files/nwss_to_odm_v2_mapping.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/martinwellman/Documents/Health/Wastewater/PHES-ODM-MapGenerator/PHES-ODM-MapGenerator/data/mapping_config_files/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{38902763-A490-C344-9B72-443A878B1074}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7088432A-D37C-B44E-A1BD-206B19DDDC14}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="500" windowWidth="40960" windowHeight="20860" xr2:uid="{77810E24-F86B-BC44-A0D5-8790E6EC60B4}"/>
   </bookViews>
@@ -29,7 +29,7 @@
     <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">enums!$A$1:$J$41</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">maps!$A$1:$K$58</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="7" hidden="1">'maps original'!$A$1:$L$87</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">wide_measures!$A$1:$S$26</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">wide_measures!$A$1:$T$26</definedName>
     <definedName name="partID">[1]parts!$A:$A</definedName>
     <definedName name="partLabel">[1]parts!$B:$B</definedName>
   </definedNames>
@@ -53,7 +53,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3278" uniqueCount="986">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3283" uniqueCount="990">
   <si>
     <t>Reporter</t>
   </si>
@@ -3058,6 +3058,18 @@
   </si>
   <si>
     <t>{{id:polygonID}}</t>
+  </si>
+  <si>
+    <t>old measureRepID</t>
+  </si>
+  <si>
+    <t>old qualityReportID</t>
+  </si>
+  <si>
+    <t>old stepID</t>
+  </si>
+  <si>
+    <t>old protocolRelationshipsID</t>
   </si>
 </sst>
 </file>
@@ -14584,7 +14596,7 @@
     </row>
     <row r="4" spans="1:10" s="25" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A4" s="25" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="B4" s="25" t="s">
         <v>630</v>
@@ -14598,7 +14610,7 @@
       <c r="F4" s="25" t="s">
         <v>729</v>
       </c>
-      <c r="G4" s="25" t="s">
+      <c r="J4" s="25" t="s">
         <v>875</v>
       </c>
     </row>
@@ -14836,7 +14848,7 @@
     </row>
     <row r="21" spans="1:11" s="25" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A21" s="25" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="B21" s="25" t="s">
         <v>630</v>
@@ -14850,7 +14862,7 @@
       <c r="F21" s="25" t="s">
         <v>735</v>
       </c>
-      <c r="G21" s="25" t="s">
+      <c r="J21" s="25" t="s">
         <v>877</v>
       </c>
     </row>
@@ -15036,7 +15048,7 @@
     </row>
     <row r="32" spans="1:11" s="25" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A32" s="25" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="B32" s="25" t="s">
         <v>630</v>
@@ -15050,14 +15062,14 @@
       <c r="F32" s="25" t="s">
         <v>727</v>
       </c>
-      <c r="G32" s="25" t="s">
+      <c r="J32" s="25" t="s">
         <v>985</v>
       </c>
     </row>
-    <row r="33" spans="1:8" s="25" customFormat="1" x14ac:dyDescent="0.2">
+    <row r="33" spans="1:10" s="25" customFormat="1" x14ac:dyDescent="0.2">
       <c r="H33" s="30"/>
     </row>
-    <row r="34" spans="1:8" s="25" customFormat="1" x14ac:dyDescent="0.2">
+    <row r="34" spans="1:10" s="25" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A34" s="25" t="b">
         <v>1</v>
       </c>
@@ -15078,7 +15090,7 @@
       </c>
       <c r="H34" s="30"/>
     </row>
-    <row r="35" spans="1:8" s="25" customFormat="1" x14ac:dyDescent="0.2">
+    <row r="35" spans="1:10" s="25" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A35" s="25" t="b">
         <v>1</v>
       </c>
@@ -15099,7 +15111,7 @@
       </c>
       <c r="H35" s="30"/>
     </row>
-    <row r="36" spans="1:8" s="25" customFormat="1" x14ac:dyDescent="0.2">
+    <row r="36" spans="1:10" s="25" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A36" s="25" t="b">
         <v>1</v>
       </c>
@@ -15120,7 +15132,7 @@
       </c>
       <c r="H36" s="30"/>
     </row>
-    <row r="37" spans="1:8" s="25" customFormat="1" x14ac:dyDescent="0.2">
+    <row r="37" spans="1:10" s="25" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A37" s="25" t="b">
         <v>1</v>
       </c>
@@ -15141,10 +15153,10 @@
       </c>
       <c r="H37" s="30"/>
     </row>
-    <row r="38" spans="1:8" s="25" customFormat="1" x14ac:dyDescent="0.2">
+    <row r="38" spans="1:10" s="25" customFormat="1" x14ac:dyDescent="0.2">
       <c r="H38" s="30"/>
     </row>
-    <row r="39" spans="1:8" s="25" customFormat="1" x14ac:dyDescent="0.2">
+    <row r="39" spans="1:10" s="25" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A39" s="25" t="b">
         <v>1</v>
       </c>
@@ -15164,7 +15176,7 @@
         <v>701</v>
       </c>
     </row>
-    <row r="40" spans="1:8" s="25" customFormat="1" x14ac:dyDescent="0.2">
+    <row r="40" spans="1:10" s="25" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A40" s="25" t="b">
         <v>0</v>
       </c>
@@ -15178,7 +15190,7 @@
         <v>115</v>
       </c>
     </row>
-    <row r="41" spans="1:8" s="25" customFormat="1" x14ac:dyDescent="0.2">
+    <row r="41" spans="1:10" s="25" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A41" s="25" t="b">
         <v>0</v>
       </c>
@@ -15192,9 +15204,9 @@
         <v>870</v>
       </c>
     </row>
-    <row r="42" spans="1:8" s="25" customFormat="1" x14ac:dyDescent="0.2">
+    <row r="42" spans="1:10" s="25" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A42" s="25" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="B42" s="25" t="s">
         <v>630</v>
@@ -15208,11 +15220,11 @@
       <c r="F42" s="25" t="s">
         <v>729</v>
       </c>
-      <c r="G42" s="25" t="s">
+      <c r="J42" s="25" t="s">
         <v>875</v>
       </c>
     </row>
-    <row r="43" spans="1:8" s="25" customFormat="1" x14ac:dyDescent="0.2">
+    <row r="43" spans="1:10" s="25" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A43" s="25" t="b">
         <v>1</v>
       </c>
@@ -15233,7 +15245,7 @@
         <v>701</v>
       </c>
     </row>
-    <row r="44" spans="1:8" s="25" customFormat="1" x14ac:dyDescent="0.2">
+    <row r="44" spans="1:10" s="25" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A44" s="25" t="b">
         <v>0</v>
       </c>
@@ -15247,7 +15259,7 @@
         <v>871</v>
       </c>
     </row>
-    <row r="45" spans="1:8" s="25" customFormat="1" x14ac:dyDescent="0.2">
+    <row r="45" spans="1:10" s="25" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A45" s="25" t="b">
         <v>0</v>
       </c>
@@ -15261,7 +15273,7 @@
         <v>872</v>
       </c>
     </row>
-    <row r="46" spans="1:8" s="25" customFormat="1" x14ac:dyDescent="0.2">
+    <row r="46" spans="1:10" s="25" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A46" s="25" t="b">
         <v>0</v>
       </c>
@@ -15275,7 +15287,7 @@
         <v>873</v>
       </c>
     </row>
-    <row r="47" spans="1:8" s="25" customFormat="1" x14ac:dyDescent="0.2">
+    <row r="47" spans="1:10" s="25" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A47" s="25" t="b">
         <v>0</v>
       </c>
@@ -15289,7 +15301,7 @@
         <v>874</v>
       </c>
     </row>
-    <row r="48" spans="1:8" s="25" customFormat="1" x14ac:dyDescent="0.2">
+    <row r="48" spans="1:10" s="25" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A48" s="25" t="b">
         <v>0</v>
       </c>
@@ -15306,7 +15318,7 @@
     <row r="49" spans="1:11" s="25" customFormat="1" x14ac:dyDescent="0.2"/>
     <row r="50" spans="1:11" s="25" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A50" s="25" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="B50" s="25" t="s">
         <v>630</v>
@@ -15320,7 +15332,7 @@
       <c r="F50" s="25" t="s">
         <v>727</v>
       </c>
-      <c r="G50" s="25" t="s">
+      <c r="J50" s="25" t="s">
         <v>985</v>
       </c>
     </row>
@@ -15532,7 +15544,7 @@
     </row>
     <row r="63" spans="1:11" s="25" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A63" s="25" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="B63" s="25" t="s">
         <v>630</v>
@@ -15546,7 +15558,7 @@
       <c r="F63" s="25" t="s">
         <v>735</v>
       </c>
-      <c r="G63" s="25" t="s">
+      <c r="J63" s="25" t="s">
         <v>877</v>
       </c>
     </row>
@@ -15838,7 +15850,7 @@
         <v>136</v>
       </c>
     </row>
-    <row r="81" spans="1:8" s="25" customFormat="1" x14ac:dyDescent="0.2">
+    <row r="81" spans="1:10" s="25" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A81" s="25" t="b">
         <v>1</v>
       </c>
@@ -15861,7 +15873,7 @@
         <v>134</v>
       </c>
     </row>
-    <row r="82" spans="1:8" s="25" customFormat="1" x14ac:dyDescent="0.2">
+    <row r="82" spans="1:10" s="25" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A82" s="25" t="b">
         <v>1</v>
       </c>
@@ -15884,7 +15896,7 @@
         <v>130</v>
       </c>
     </row>
-    <row r="83" spans="1:8" s="25" customFormat="1" x14ac:dyDescent="0.2">
+    <row r="83" spans="1:10" s="25" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A83" s="25" t="b">
         <v>1</v>
       </c>
@@ -15907,7 +15919,7 @@
         <v>131</v>
       </c>
     </row>
-    <row r="84" spans="1:8" s="25" customFormat="1" x14ac:dyDescent="0.2">
+    <row r="84" spans="1:10" s="25" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A84" s="25" t="b">
         <v>1</v>
       </c>
@@ -15930,7 +15942,7 @@
         <v>132</v>
       </c>
     </row>
-    <row r="85" spans="1:8" s="25" customFormat="1" x14ac:dyDescent="0.2">
+    <row r="85" spans="1:10" s="25" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A85" s="25" t="b">
         <v>1</v>
       </c>
@@ -15953,7 +15965,7 @@
         <v>133</v>
       </c>
     </row>
-    <row r="86" spans="1:8" s="25" customFormat="1" x14ac:dyDescent="0.2">
+    <row r="86" spans="1:10" s="25" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A86" s="25" t="b">
         <v>1</v>
       </c>
@@ -15976,7 +15988,7 @@
         <v>127</v>
       </c>
     </row>
-    <row r="87" spans="1:8" s="25" customFormat="1" x14ac:dyDescent="0.2">
+    <row r="87" spans="1:10" s="25" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A87" s="25" t="b">
         <v>1</v>
       </c>
@@ -15999,10 +16011,10 @@
         <v>135</v>
       </c>
     </row>
-    <row r="88" spans="1:8" s="25" customFormat="1" x14ac:dyDescent="0.2">
+    <row r="88" spans="1:10" s="25" customFormat="1" x14ac:dyDescent="0.2">
       <c r="D88" s="32"/>
     </row>
-    <row r="89" spans="1:8" s="25" customFormat="1" x14ac:dyDescent="0.2">
+    <row r="89" spans="1:10" s="25" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A89" s="25" t="b">
         <v>1</v>
       </c>
@@ -16022,9 +16034,9 @@
         <v>722</v>
       </c>
     </row>
-    <row r="90" spans="1:8" s="25" customFormat="1" x14ac:dyDescent="0.2">
+    <row r="90" spans="1:10" s="25" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A90" s="25" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="B90" s="25" t="s">
         <v>630</v>
@@ -16042,7 +16054,7 @@
         <v>696</v>
       </c>
     </row>
-    <row r="91" spans="1:8" s="25" customFormat="1" x14ac:dyDescent="0.2">
+    <row r="91" spans="1:10" s="25" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A91" s="25" t="b">
         <v>1</v>
       </c>
@@ -16062,7 +16074,7 @@
         <v>694</v>
       </c>
     </row>
-    <row r="92" spans="1:8" s="25" customFormat="1" x14ac:dyDescent="0.2">
+    <row r="92" spans="1:10" s="25" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A92" s="25" t="b">
         <v>1</v>
       </c>
@@ -16082,7 +16094,7 @@
         <v>701</v>
       </c>
     </row>
-    <row r="93" spans="1:8" s="25" customFormat="1" x14ac:dyDescent="0.2">
+    <row r="93" spans="1:10" s="25" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A93" s="25" t="b">
         <v>1</v>
       </c>
@@ -16102,7 +16114,7 @@
         <v>697</v>
       </c>
     </row>
-    <row r="94" spans="1:8" s="25" customFormat="1" ht="17" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="94" spans="1:10" s="25" customFormat="1" ht="17" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A94" s="25" t="b">
         <v>1</v>
       </c>
@@ -16123,7 +16135,7 @@
         <v>862</v>
       </c>
     </row>
-    <row r="95" spans="1:8" s="25" customFormat="1" x14ac:dyDescent="0.2">
+    <row r="95" spans="1:10" s="25" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A95" s="25" t="b">
         <v>1</v>
       </c>
@@ -16144,9 +16156,9 @@
         <v>701</v>
       </c>
     </row>
-    <row r="96" spans="1:8" s="25" customFormat="1" x14ac:dyDescent="0.2">
+    <row r="96" spans="1:10" s="25" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A96" s="25" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="B96" s="25" t="s">
         <v>630</v>
@@ -16160,7 +16172,7 @@
       <c r="F96" s="25" t="s">
         <v>729</v>
       </c>
-      <c r="G96" s="25" t="s">
+      <c r="J96" s="25" t="s">
         <v>875</v>
       </c>
     </row>
@@ -16206,7 +16218,7 @@
     </row>
     <row r="99" spans="1:10" s="25" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A99" s="25" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="B99" s="25" t="s">
         <v>630</v>
@@ -16220,7 +16232,7 @@
       <c r="F99" s="25" t="s">
         <v>727</v>
       </c>
-      <c r="G99" s="25" t="s">
+      <c r="J99" s="25" t="s">
         <v>985</v>
       </c>
     </row>
@@ -16606,7 +16618,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B39AC7DD-3F73-2C47-925D-21E5B4EBE6FC}">
-  <dimension ref="A1:S28"/>
+  <dimension ref="A1:T28"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="2" max="2" width="13" bestFit="1" customWidth="1"/>
@@ -16615,19 +16627,20 @@
     <col min="5" max="5" width="12" bestFit="1" customWidth="1"/>
     <col min="6" max="6" width="12.1640625" bestFit="1" customWidth="1"/>
     <col min="7" max="7" width="15.83203125" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="35.33203125" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="21.83203125" customWidth="1"/>
-    <col min="10" max="10" width="16.83203125" bestFit="1" customWidth="1"/>
-    <col min="11" max="11" width="22" bestFit="1" customWidth="1"/>
-    <col min="12" max="12" width="23.5" bestFit="1" customWidth="1"/>
-    <col min="13" max="13" width="83.6640625" bestFit="1" customWidth="1"/>
-    <col min="14" max="14" width="20.1640625" bestFit="1" customWidth="1"/>
-    <col min="15" max="15" width="18.5" bestFit="1" customWidth="1"/>
-    <col min="16" max="18" width="21.83203125" customWidth="1"/>
-    <col min="19" max="19" width="27.6640625" customWidth="1"/>
+    <col min="8" max="8" width="15.83203125" customWidth="1"/>
+    <col min="9" max="9" width="35.33203125" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="21.83203125" customWidth="1"/>
+    <col min="11" max="11" width="16.83203125" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="22" bestFit="1" customWidth="1"/>
+    <col min="13" max="13" width="23.5" bestFit="1" customWidth="1"/>
+    <col min="14" max="14" width="83.6640625" bestFit="1" customWidth="1"/>
+    <col min="15" max="15" width="20.1640625" bestFit="1" customWidth="1"/>
+    <col min="16" max="16" width="18.5" bestFit="1" customWidth="1"/>
+    <col min="17" max="19" width="21.83203125" customWidth="1"/>
+    <col min="20" max="20" width="27.6640625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:19" s="39" customFormat="1" ht="19" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:20" s="39" customFormat="1" ht="19" x14ac:dyDescent="0.25">
       <c r="A1" s="39" t="s">
         <v>666</v>
       </c>
@@ -16650,43 +16663,46 @@
         <v>682</v>
       </c>
       <c r="H1" s="39" t="s">
+        <v>986</v>
+      </c>
+      <c r="I1" s="39" t="s">
         <v>807</v>
       </c>
-      <c r="I1" s="39" t="s">
+      <c r="J1" s="39" t="s">
         <v>864</v>
       </c>
-      <c r="J1" s="40" t="s">
+      <c r="K1" s="40" t="s">
         <v>799</v>
       </c>
-      <c r="K1" s="40" t="s">
+      <c r="L1" s="40" t="s">
         <v>800</v>
       </c>
-      <c r="L1" s="40" t="s">
+      <c r="M1" s="40" t="s">
         <v>802</v>
       </c>
-      <c r="M1" s="40" t="s">
+      <c r="N1" s="40" t="s">
         <v>847</v>
       </c>
-      <c r="N1" s="40" t="s">
+      <c r="O1" s="40" t="s">
         <v>803</v>
       </c>
-      <c r="O1" s="40" t="s">
+      <c r="P1" s="40" t="s">
         <v>804</v>
       </c>
-      <c r="P1" s="39" t="s">
+      <c r="Q1" s="39" t="s">
         <v>865</v>
       </c>
-      <c r="Q1" s="39" t="s">
+      <c r="R1" s="39" t="s">
         <v>858</v>
       </c>
-      <c r="R1" s="39" t="s">
+      <c r="S1" s="39" t="s">
         <v>848</v>
       </c>
-      <c r="S1" s="40" t="s">
+      <c r="T1" s="40" t="s">
         <v>120</v>
       </c>
     </row>
-    <row r="2" spans="1:19" s="25" customFormat="1" x14ac:dyDescent="0.2">
+    <row r="2" spans="1:20" s="25" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A2" s="25" t="b">
         <v>1</v>
       </c>
@@ -16706,23 +16722,23 @@
       <c r="H2" s="25" t="s">
         <v>808</v>
       </c>
-      <c r="J2" s="25" t="s">
+      <c r="K2" s="25" t="s">
         <v>155</v>
       </c>
-      <c r="K2" s="25" t="s">
+      <c r="L2" s="25" t="s">
         <v>160</v>
       </c>
-      <c r="M2" s="25" t="s">
+      <c r="N2" s="25" t="s">
         <v>887</v>
       </c>
-      <c r="N2" s="25" t="s">
+      <c r="O2" s="25" t="s">
         <v>161</v>
       </c>
-      <c r="O2" s="25" t="s">
+      <c r="P2" s="25" t="s">
         <v>154</v>
       </c>
     </row>
-    <row r="3" spans="1:19" s="25" customFormat="1" x14ac:dyDescent="0.2">
+    <row r="3" spans="1:20" s="25" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A3" s="25" t="b">
         <v>1</v>
       </c>
@@ -16742,23 +16758,23 @@
       <c r="H3" s="25" t="s">
         <v>809</v>
       </c>
-      <c r="J3" s="25" t="s">
+      <c r="K3" s="25" t="s">
         <v>164</v>
       </c>
-      <c r="K3" s="25" t="s">
+      <c r="L3" s="25" t="s">
         <v>167</v>
       </c>
-      <c r="L3" s="25" t="s">
+      <c r="M3" s="25" t="s">
         <v>648</v>
       </c>
-      <c r="N3" s="25" t="s">
+      <c r="O3" s="25" t="s">
         <v>168</v>
       </c>
-      <c r="O3" s="25" t="s">
+      <c r="P3" s="25" t="s">
         <v>154</v>
       </c>
     </row>
-    <row r="4" spans="1:19" s="25" customFormat="1" x14ac:dyDescent="0.2">
+    <row r="4" spans="1:20" s="25" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A4" s="25" t="b">
         <v>1</v>
       </c>
@@ -16778,23 +16794,23 @@
       <c r="H4" s="25" t="s">
         <v>810</v>
       </c>
-      <c r="J4" s="25" t="s">
+      <c r="K4" s="25" t="s">
         <v>164</v>
       </c>
-      <c r="K4" s="25" t="s">
+      <c r="L4" s="25" t="s">
         <v>166</v>
       </c>
-      <c r="L4" s="25" t="s">
+      <c r="M4" s="25" t="s">
         <v>647</v>
       </c>
-      <c r="N4" s="25" t="s">
+      <c r="O4" s="25" t="s">
         <v>157</v>
       </c>
-      <c r="O4" s="25" t="s">
+      <c r="P4" s="25" t="s">
         <v>154</v>
       </c>
     </row>
-    <row r="5" spans="1:19" s="25" customFormat="1" x14ac:dyDescent="0.2">
+    <row r="5" spans="1:20" s="25" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A5" s="25" t="b">
         <v>1</v>
       </c>
@@ -16814,23 +16830,23 @@
       <c r="H5" s="25" t="s">
         <v>811</v>
       </c>
-      <c r="J5" s="25" t="s">
+      <c r="K5" s="25" t="s">
         <v>164</v>
       </c>
-      <c r="K5" s="25" t="s">
+      <c r="L5" s="25" t="s">
         <v>175</v>
       </c>
-      <c r="L5" s="25" t="s">
+      <c r="M5" s="25" t="s">
         <v>660</v>
       </c>
-      <c r="N5" s="25" t="s">
+      <c r="O5" s="25" t="s">
         <v>168</v>
       </c>
-      <c r="O5" s="25" t="s">
+      <c r="P5" s="25" t="s">
         <v>154</v>
       </c>
     </row>
-    <row r="6" spans="1:19" s="25" customFormat="1" x14ac:dyDescent="0.2">
+    <row r="6" spans="1:20" s="25" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A6" s="25" t="b">
         <v>1</v>
       </c>
@@ -16850,23 +16866,23 @@
       <c r="H6" s="25" t="s">
         <v>812</v>
       </c>
-      <c r="J6" s="25" t="s">
+      <c r="K6" s="25" t="s">
         <v>164</v>
       </c>
-      <c r="K6" s="25" t="s">
+      <c r="L6" s="25" t="s">
         <v>172</v>
       </c>
-      <c r="L6" s="25" t="s">
+      <c r="M6" s="25" t="s">
         <v>658</v>
       </c>
-      <c r="N6" s="25" t="s">
+      <c r="O6" s="25" t="s">
         <v>173</v>
       </c>
-      <c r="O6" s="25" t="s">
+      <c r="P6" s="25" t="s">
         <v>154</v>
       </c>
     </row>
-    <row r="7" spans="1:19" s="25" customFormat="1" x14ac:dyDescent="0.2">
+    <row r="7" spans="1:20" s="25" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A7" s="25" t="b">
         <v>1</v>
       </c>
@@ -16886,23 +16902,23 @@
       <c r="H7" s="25" t="s">
         <v>813</v>
       </c>
-      <c r="J7" s="25" t="s">
+      <c r="K7" s="25" t="s">
         <v>164</v>
       </c>
-      <c r="K7" s="25" t="s">
+      <c r="L7" s="25" t="s">
         <v>176</v>
       </c>
-      <c r="L7" s="25" t="s">
+      <c r="M7" s="25" t="s">
         <v>661</v>
       </c>
-      <c r="N7" s="25" t="s">
+      <c r="O7" s="25" t="s">
         <v>869</v>
       </c>
-      <c r="O7" s="25" t="s">
+      <c r="P7" s="25" t="s">
         <v>154</v>
       </c>
     </row>
-    <row r="8" spans="1:19" s="25" customFormat="1" x14ac:dyDescent="0.2">
+    <row r="8" spans="1:20" s="25" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A8" s="25" t="b">
         <v>1</v>
       </c>
@@ -16922,23 +16938,23 @@
       <c r="H8" s="25" t="s">
         <v>814</v>
       </c>
-      <c r="J8" s="25" t="s">
+      <c r="K8" s="25" t="s">
         <v>155</v>
       </c>
-      <c r="K8" s="25" t="s">
+      <c r="L8" s="25" t="s">
         <v>170</v>
       </c>
-      <c r="M8" s="25" t="s">
+      <c r="N8" s="25" t="s">
         <v>886</v>
       </c>
-      <c r="N8" s="25" t="s">
+      <c r="O8" s="25" t="s">
         <v>161</v>
       </c>
-      <c r="O8" s="25" t="s">
+      <c r="P8" s="25" t="s">
         <v>158</v>
       </c>
     </row>
-    <row r="9" spans="1:19" s="25" customFormat="1" x14ac:dyDescent="0.2">
+    <row r="9" spans="1:20" s="25" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A9" s="25" t="b">
         <v>1</v>
       </c>
@@ -16958,26 +16974,26 @@
       <c r="H9" s="25" t="s">
         <v>815</v>
       </c>
-      <c r="J9" s="25" t="s">
+      <c r="K9" s="25" t="s">
         <v>164</v>
       </c>
-      <c r="K9" s="25" t="s">
+      <c r="L9" s="25" t="s">
         <v>639</v>
       </c>
-      <c r="L9" s="25" t="s">
+      <c r="M9" s="25" t="s">
         <v>664</v>
       </c>
-      <c r="N9" s="25" t="s">
+      <c r="O9" s="25" t="s">
         <v>643</v>
       </c>
-      <c r="O9" s="25" t="s">
+      <c r="P9" s="25" t="s">
         <v>158</v>
       </c>
-      <c r="P9" s="25" t="s">
+      <c r="Q9" s="25" t="s">
         <v>853</v>
       </c>
     </row>
-    <row r="10" spans="1:19" s="25" customFormat="1" x14ac:dyDescent="0.2">
+    <row r="10" spans="1:20" s="25" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A10" s="25" t="b">
         <v>1</v>
       </c>
@@ -16997,26 +17013,26 @@
       <c r="H10" s="25" t="s">
         <v>816</v>
       </c>
-      <c r="J10" s="25" t="s">
+      <c r="K10" s="25" t="s">
         <v>164</v>
       </c>
-      <c r="K10" s="25" t="s">
+      <c r="L10" s="25" t="s">
         <v>638</v>
       </c>
-      <c r="L10" s="25" t="s">
+      <c r="M10" s="25" t="s">
         <v>663</v>
       </c>
-      <c r="N10" s="25" t="s">
+      <c r="O10" s="25" t="s">
         <v>642</v>
       </c>
-      <c r="O10" s="25" t="s">
+      <c r="P10" s="25" t="s">
         <v>158</v>
       </c>
-      <c r="P10" s="25" t="s">
+      <c r="Q10" s="25" t="s">
         <v>854</v>
       </c>
     </row>
-    <row r="11" spans="1:19" s="25" customFormat="1" x14ac:dyDescent="0.2">
+    <row r="11" spans="1:20" s="25" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A11" s="25" t="b">
         <v>1</v>
       </c>
@@ -17036,23 +17052,23 @@
       <c r="H11" s="25" t="s">
         <v>817</v>
       </c>
-      <c r="J11" s="25" t="s">
+      <c r="K11" s="25" t="s">
         <v>155</v>
       </c>
-      <c r="K11" s="25" t="s">
+      <c r="L11" s="25" t="s">
         <v>162</v>
       </c>
-      <c r="M11" s="25" t="s">
+      <c r="N11" s="25" t="s">
         <v>885</v>
       </c>
-      <c r="N11" s="25" t="s">
+      <c r="O11" s="25" t="s">
         <v>163</v>
       </c>
-      <c r="O11" s="25" t="s">
+      <c r="P11" s="25" t="s">
         <v>158</v>
       </c>
     </row>
-    <row r="12" spans="1:19" s="25" customFormat="1" x14ac:dyDescent="0.2">
+    <row r="12" spans="1:20" s="25" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A12" s="25" t="b">
         <v>1</v>
       </c>
@@ -17076,17 +17092,17 @@
       <c r="H12" s="25" t="s">
         <v>818</v>
       </c>
-      <c r="J12" s="25" t="s">
+      <c r="K12" s="25" t="s">
         <v>155</v>
       </c>
-      <c r="K12" s="25" t="s">
+      <c r="L12" s="25" t="s">
         <v>165</v>
       </c>
-      <c r="L12" s="25" t="s">
+      <c r="M12" s="25" t="s">
         <v>646</v>
       </c>
     </row>
-    <row r="13" spans="1:19" s="25" customFormat="1" x14ac:dyDescent="0.2">
+    <row r="13" spans="1:20" s="25" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A13" s="25" t="b">
         <v>1</v>
       </c>
@@ -17108,7 +17124,7 @@
       </c>
       <c r="G13"/>
     </row>
-    <row r="14" spans="1:19" s="25" customFormat="1" x14ac:dyDescent="0.2">
+    <row r="14" spans="1:20" s="25" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A14" s="25" t="b">
         <v>1</v>
       </c>
@@ -17129,7 +17145,7 @@
       </c>
       <c r="G14"/>
     </row>
-    <row r="15" spans="1:19" s="25" customFormat="1" x14ac:dyDescent="0.2">
+    <row r="15" spans="1:20" s="25" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A15" s="25" t="b">
         <v>1</v>
       </c>
@@ -17149,26 +17165,26 @@
       <c r="H15" s="25" t="s">
         <v>819</v>
       </c>
-      <c r="J15" s="25" t="s">
+      <c r="K15" s="25" t="s">
         <v>164</v>
       </c>
-      <c r="K15" s="25" t="s">
+      <c r="L15" s="25" t="s">
         <v>595</v>
       </c>
-      <c r="L15" s="25" t="s">
+      <c r="M15" s="25" t="s">
         <v>662</v>
       </c>
-      <c r="N15" s="25" t="s">
+      <c r="O15" s="25" t="s">
         <v>641</v>
       </c>
-      <c r="O15" s="25" t="s">
+      <c r="P15" s="25" t="s">
         <v>158</v>
       </c>
-      <c r="P15" s="25" t="s">
+      <c r="Q15" s="25" t="s">
         <v>855</v>
       </c>
     </row>
-    <row r="16" spans="1:19" s="25" customFormat="1" x14ac:dyDescent="0.2">
+    <row r="16" spans="1:20" s="25" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A16" s="25" t="b">
         <v>1</v>
       </c>
@@ -17188,29 +17204,29 @@
       <c r="H16" s="25" t="s">
         <v>820</v>
       </c>
-      <c r="I16" s="25" t="s">
+      <c r="J16" s="25" t="s">
         <v>852</v>
       </c>
-      <c r="J16" s="25" t="s">
+      <c r="K16" s="25" t="s">
         <v>164</v>
       </c>
-      <c r="K16" s="25" t="s">
+      <c r="L16" s="25" t="s">
         <v>640</v>
       </c>
-      <c r="L16" s="25" t="s">
+      <c r="M16" s="25" t="s">
         <v>665</v>
       </c>
-      <c r="N16" s="25" t="s">
+      <c r="O16" s="25" t="s">
         <v>644</v>
       </c>
-      <c r="O16" s="25" t="s">
+      <c r="P16" s="25" t="s">
         <v>158</v>
       </c>
-      <c r="P16" s="25" t="s">
+      <c r="Q16" s="25" t="s">
         <v>856</v>
       </c>
     </row>
-    <row r="17" spans="1:18" s="25" customFormat="1" x14ac:dyDescent="0.2">
+    <row r="17" spans="1:19" s="25" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A17" s="25" t="b">
         <v>1</v>
       </c>
@@ -17230,29 +17246,29 @@
       <c r="H17" s="25" t="s">
         <v>851</v>
       </c>
-      <c r="J17" s="25" t="s">
+      <c r="K17" s="25" t="s">
         <v>164</v>
       </c>
-      <c r="K17" s="25" t="s">
+      <c r="L17" s="25" t="s">
         <v>637</v>
       </c>
-      <c r="M17" s="25" t="s">
+      <c r="N17" s="25" t="s">
         <v>917</v>
       </c>
-      <c r="N17" t="s">
+      <c r="O17" t="s">
         <v>641</v>
       </c>
-      <c r="O17" s="25" t="s">
+      <c r="P17" s="25" t="s">
         <v>158</v>
       </c>
-      <c r="P17" s="25" t="s">
+      <c r="Q17" s="25" t="s">
         <v>857</v>
       </c>
-      <c r="Q17" s="25" t="s">
+      <c r="R17" s="25" t="s">
         <v>859</v>
       </c>
     </row>
-    <row r="18" spans="1:18" s="25" customFormat="1" x14ac:dyDescent="0.2">
+    <row r="18" spans="1:19" s="25" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A18" s="25" t="b">
         <v>1</v>
       </c>
@@ -17272,26 +17288,26 @@
       <c r="H18" s="25" t="s">
         <v>821</v>
       </c>
-      <c r="J18" s="25" t="s">
+      <c r="K18" s="25" t="s">
         <v>164</v>
       </c>
-      <c r="K18" s="25" t="s">
+      <c r="L18" s="25" t="s">
         <v>637</v>
       </c>
-      <c r="M18" s="25" t="s">
+      <c r="N18" s="25" t="s">
         <v>920</v>
       </c>
-      <c r="N18" s="25" t="s">
+      <c r="O18" s="25" t="s">
         <v>641</v>
       </c>
-      <c r="O18" s="25" t="s">
+      <c r="P18" s="25" t="s">
         <v>590</v>
       </c>
-      <c r="P18" s="25" t="s">
+      <c r="Q18" s="25" t="s">
         <v>857</v>
       </c>
     </row>
-    <row r="19" spans="1:18" s="25" customFormat="1" x14ac:dyDescent="0.2">
+    <row r="19" spans="1:19" s="25" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A19" s="25" t="b">
         <v>1</v>
       </c>
@@ -17311,26 +17327,26 @@
       <c r="H19" s="25" t="s">
         <v>822</v>
       </c>
-      <c r="J19" s="25" t="s">
+      <c r="K19" s="25" t="s">
         <v>164</v>
       </c>
-      <c r="K19" s="25" t="s">
+      <c r="L19" s="25" t="s">
         <v>637</v>
       </c>
-      <c r="M19" s="25" t="s">
+      <c r="N19" s="25" t="s">
         <v>919</v>
       </c>
-      <c r="N19" s="25" t="s">
+      <c r="O19" s="25" t="s">
         <v>641</v>
       </c>
-      <c r="O19" s="25" t="s">
+      <c r="P19" s="25" t="s">
         <v>591</v>
       </c>
-      <c r="P19" s="25" t="s">
+      <c r="Q19" s="25" t="s">
         <v>857</v>
       </c>
     </row>
-    <row r="20" spans="1:18" s="25" customFormat="1" x14ac:dyDescent="0.2">
+    <row r="20" spans="1:19" s="25" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A20" s="25" t="b">
         <v>1</v>
       </c>
@@ -17350,26 +17366,26 @@
       <c r="H20" s="25" t="s">
         <v>823</v>
       </c>
-      <c r="J20" s="25" t="s">
+      <c r="K20" s="25" t="s">
         <v>164</v>
       </c>
-      <c r="K20" s="25" t="s">
+      <c r="L20" s="25" t="s">
         <v>637</v>
       </c>
-      <c r="M20" s="25" t="s">
+      <c r="N20" s="25" t="s">
         <v>918</v>
       </c>
-      <c r="N20" s="25" t="s">
+      <c r="O20" s="25" t="s">
         <v>641</v>
       </c>
-      <c r="O20" s="25" t="s">
+      <c r="P20" s="25" t="s">
         <v>589</v>
       </c>
-      <c r="P20" s="25" t="s">
+      <c r="Q20" s="25" t="s">
         <v>857</v>
       </c>
     </row>
-    <row r="21" spans="1:18" s="25" customFormat="1" x14ac:dyDescent="0.2">
+    <row r="21" spans="1:19" s="25" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A21" s="25" t="b">
         <v>1</v>
       </c>
@@ -17389,23 +17405,23 @@
       <c r="H21" s="25" t="s">
         <v>824</v>
       </c>
-      <c r="J21" s="25" t="s">
+      <c r="K21" s="25" t="s">
         <v>164</v>
       </c>
-      <c r="K21" s="25" t="s">
+      <c r="L21" s="25" t="s">
         <v>48</v>
       </c>
-      <c r="L21" s="25" t="s">
+      <c r="M21" s="25" t="s">
         <v>657</v>
       </c>
-      <c r="N21" s="25" t="s">
+      <c r="O21" s="25" t="s">
         <v>171</v>
       </c>
-      <c r="O21" s="25" t="s">
+      <c r="P21" s="25" t="s">
         <v>154</v>
       </c>
     </row>
-    <row r="22" spans="1:18" s="25" customFormat="1" x14ac:dyDescent="0.2">
+    <row r="22" spans="1:19" s="25" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A22" s="25" t="b">
         <v>1</v>
       </c>
@@ -17425,20 +17441,20 @@
       <c r="H22" s="25" t="s">
         <v>825</v>
       </c>
-      <c r="J22" s="25" t="s">
+      <c r="K22" s="25" t="s">
         <v>164</v>
       </c>
-      <c r="K22" s="25" t="s">
+      <c r="L22" s="25" t="s">
         <v>169</v>
       </c>
-      <c r="L22" s="25" t="s">
+      <c r="M22" s="25" t="s">
         <v>636</v>
       </c>
-      <c r="R22" s="25" t="s">
+      <c r="S22" s="25" t="s">
         <v>860</v>
       </c>
     </row>
-    <row r="23" spans="1:18" s="25" customFormat="1" x14ac:dyDescent="0.2">
+    <row r="23" spans="1:19" s="25" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A23" s="25" t="b">
         <v>1</v>
       </c>
@@ -17458,23 +17474,23 @@
       <c r="H23" s="25" t="s">
         <v>826</v>
       </c>
-      <c r="J23" s="25" t="s">
+      <c r="K23" s="25" t="s">
         <v>164</v>
       </c>
-      <c r="K23" s="25" t="s">
+      <c r="L23" s="25" t="s">
         <v>596</v>
       </c>
-      <c r="M23" s="25" t="s">
+      <c r="N23" s="25" t="s">
         <v>916</v>
       </c>
-      <c r="N23" s="25" t="s">
+      <c r="O23" s="25" t="s">
         <v>163</v>
       </c>
-      <c r="O23" s="25" t="s">
+      <c r="P23" s="25" t="s">
         <v>158</v>
       </c>
     </row>
-    <row r="24" spans="1:18" s="25" customFormat="1" x14ac:dyDescent="0.2">
+    <row r="24" spans="1:19" s="25" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A24" s="25" t="b">
         <v>1</v>
       </c>
@@ -17494,23 +17510,23 @@
       <c r="H24" s="25" t="s">
         <v>827</v>
       </c>
-      <c r="J24" s="25" t="s">
+      <c r="K24" s="25" t="s">
         <v>164</v>
       </c>
-      <c r="K24" s="25" t="s">
+      <c r="L24" s="25" t="s">
         <v>578</v>
       </c>
-      <c r="L24" s="25" t="s">
+      <c r="M24" s="25" t="s">
         <v>655</v>
       </c>
-      <c r="N24" s="25" t="s">
+      <c r="O24" s="25" t="s">
         <v>579</v>
       </c>
-      <c r="O24" s="25" t="s">
+      <c r="P24" s="25" t="s">
         <v>154</v>
       </c>
     </row>
-    <row r="25" spans="1:18" s="25" customFormat="1" x14ac:dyDescent="0.2">
+    <row r="25" spans="1:19" s="25" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A25" s="25" t="b">
         <v>1</v>
       </c>
@@ -17530,24 +17546,24 @@
       <c r="H25" s="25" t="s">
         <v>828</v>
       </c>
-      <c r="J25" s="28" t="s">
+      <c r="K25" s="28" t="s">
         <v>155</v>
       </c>
-      <c r="K25" s="28" t="s">
+      <c r="L25" s="28" t="s">
         <v>159</v>
       </c>
-      <c r="L25" s="28"/>
-      <c r="M25" s="28" t="s">
+      <c r="M25" s="28"/>
+      <c r="N25" s="28" t="s">
         <v>884</v>
       </c>
-      <c r="N25" s="28" t="s">
+      <c r="O25" s="28" t="s">
         <v>157</v>
       </c>
-      <c r="O25" s="28" t="s">
+      <c r="P25" s="28" t="s">
         <v>158</v>
       </c>
     </row>
-    <row r="26" spans="1:18" s="25" customFormat="1" x14ac:dyDescent="0.2">
+    <row r="26" spans="1:19" s="25" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A26" s="25" t="b">
         <v>1</v>
       </c>
@@ -17567,30 +17583,32 @@
       <c r="H26" s="25" t="s">
         <v>829</v>
       </c>
-      <c r="J26" s="25" t="s">
+      <c r="K26" s="25" t="s">
         <v>164</v>
       </c>
-      <c r="K26" s="25" t="s">
+      <c r="L26" s="25" t="s">
         <v>50</v>
       </c>
-      <c r="L26" s="25" t="s">
+      <c r="M26" s="25" t="s">
         <v>659</v>
       </c>
-      <c r="N26" s="25" t="s">
+      <c r="O26" s="25" t="s">
         <v>174</v>
       </c>
-      <c r="O26" s="25" t="s">
+      <c r="P26" s="25" t="s">
         <v>154</v>
       </c>
     </row>
-    <row r="27" spans="1:18" s="25" customFormat="1" x14ac:dyDescent="0.2">
+    <row r="27" spans="1:19" s="25" customFormat="1" x14ac:dyDescent="0.2">
       <c r="G27"/>
-    </row>
-    <row r="28" spans="1:18" s="25" customFormat="1" x14ac:dyDescent="0.2">
+      <c r="H27"/>
+    </row>
+    <row r="28" spans="1:19" s="25" customFormat="1" x14ac:dyDescent="0.2">
       <c r="G28"/>
+      <c r="H28"/>
     </row>
   </sheetData>
-  <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:S28">
+  <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:T28">
     <sortCondition ref="C1:C28"/>
   </sortState>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -17600,7 +17618,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{6B4CA3B6-4765-0A43-8534-6DA7BF8A336D}">
-  <dimension ref="A1:M17"/>
+  <dimension ref="A1:O17"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="2" max="2" width="13" bestFit="1" customWidth="1"/>
@@ -17611,11 +17629,13 @@
     <col min="7" max="7" width="15.83203125" bestFit="1" customWidth="1"/>
     <col min="8" max="8" width="35.33203125" bestFit="1" customWidth="1"/>
     <col min="9" max="9" width="23" customWidth="1"/>
-    <col min="10" max="11" width="22.33203125" customWidth="1"/>
-    <col min="12" max="12" width="35.1640625" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="35.33203125" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="23" customWidth="1"/>
+    <col min="12" max="13" width="22.33203125" customWidth="1"/>
+    <col min="14" max="14" width="35.1640625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:13" s="39" customFormat="1" ht="19" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:15" s="39" customFormat="1" ht="19" x14ac:dyDescent="0.25">
       <c r="A1" s="39" t="s">
         <v>666</v>
       </c>
@@ -17638,25 +17658,31 @@
         <v>682</v>
       </c>
       <c r="H1" s="39" t="s">
+        <v>986</v>
+      </c>
+      <c r="I1" s="39" t="s">
+        <v>987</v>
+      </c>
+      <c r="J1" s="39" t="s">
         <v>807</v>
       </c>
-      <c r="I1" s="39" t="s">
+      <c r="K1" s="39" t="s">
         <v>797</v>
       </c>
-      <c r="J1" s="40" t="s">
+      <c r="L1" s="40" t="s">
         <v>798</v>
       </c>
-      <c r="K1" s="40" t="s">
+      <c r="M1" s="40" t="s">
         <v>796</v>
       </c>
-      <c r="L1" s="40" t="s">
+      <c r="N1" s="40" t="s">
         <v>850</v>
       </c>
-      <c r="M1" s="40" t="s">
+      <c r="O1" s="40" t="s">
         <v>120</v>
       </c>
     </row>
-    <row r="2" spans="1:13" ht="17" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="2" spans="1:15" ht="17" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A2" t="b">
         <v>1</v>
       </c>
@@ -17675,18 +17701,19 @@
       <c r="I2" t="s">
         <v>787</v>
       </c>
-      <c r="K2" s="35" t="s">
+      <c r="J2" s="25"/>
+      <c r="M2" s="35" t="s">
         <v>863</v>
       </c>
-      <c r="L2" s="35" t="s">
+      <c r="N2" s="35" t="s">
         <v>849</v>
       </c>
     </row>
-    <row r="3" spans="1:13" ht="19" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="K3" s="35"/>
-      <c r="L3" s="35"/>
-    </row>
-    <row r="4" spans="1:13" x14ac:dyDescent="0.2">
+    <row r="3" spans="1:15" ht="19" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="M3" s="35"/>
+      <c r="N3" s="35"/>
+    </row>
+    <row r="4" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A4" t="b">
         <v>1</v>
       </c>
@@ -17711,11 +17738,12 @@
       <c r="I4" t="s">
         <v>788</v>
       </c>
-      <c r="J4" t="s">
+      <c r="J4" s="25"/>
+      <c r="L4" t="s">
         <v>791</v>
       </c>
     </row>
-    <row r="5" spans="1:13" x14ac:dyDescent="0.2">
+    <row r="5" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A5" t="b">
         <v>1</v>
       </c>
@@ -17735,7 +17763,7 @@
         <v>830</v>
       </c>
     </row>
-    <row r="7" spans="1:13" x14ac:dyDescent="0.2">
+    <row r="7" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A7" t="b">
         <v>1</v>
       </c>
@@ -17760,11 +17788,12 @@
       <c r="I7" t="s">
         <v>790</v>
       </c>
-      <c r="J7" t="s">
+      <c r="J7" s="25"/>
+      <c r="L7" t="s">
         <v>789</v>
       </c>
     </row>
-    <row r="8" spans="1:13" x14ac:dyDescent="0.2">
+    <row r="8" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A8" t="b">
         <v>1</v>
       </c>
@@ -17784,7 +17813,7 @@
         <v>830</v>
       </c>
     </row>
-    <row r="9" spans="1:13" x14ac:dyDescent="0.2">
+    <row r="9" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A9" t="b">
         <v>1</v>
       </c>
@@ -17804,7 +17833,7 @@
         <v>830</v>
       </c>
     </row>
-    <row r="11" spans="1:13" x14ac:dyDescent="0.2">
+    <row r="11" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A11" t="b">
         <v>1</v>
       </c>
@@ -17829,11 +17858,12 @@
       <c r="I11" t="s">
         <v>792</v>
       </c>
-      <c r="J11" t="s">
+      <c r="J11" s="25"/>
+      <c r="L11" t="s">
         <v>786</v>
       </c>
     </row>
-    <row r="12" spans="1:13" x14ac:dyDescent="0.2">
+    <row r="12" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A12" t="b">
         <v>1</v>
       </c>
@@ -17853,7 +17883,7 @@
         <v>149</v>
       </c>
     </row>
-    <row r="13" spans="1:13" x14ac:dyDescent="0.2">
+    <row r="13" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A13" t="b">
         <v>1</v>
       </c>
@@ -17873,7 +17903,7 @@
         <v>149</v>
       </c>
     </row>
-    <row r="15" spans="1:13" x14ac:dyDescent="0.2">
+    <row r="15" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A15" t="b">
         <v>1</v>
       </c>
@@ -17898,11 +17928,12 @@
       <c r="I15" t="s">
         <v>793</v>
       </c>
-      <c r="J15" t="s">
+      <c r="J15" s="25"/>
+      <c r="L15" t="s">
         <v>794</v>
       </c>
     </row>
-    <row r="16" spans="1:13" x14ac:dyDescent="0.2">
+    <row r="16" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A16" t="b">
         <v>1</v>
       </c>
@@ -17950,7 +17981,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{FDC6A21B-0669-0743-9D12-F41DCA15CA4A}">
-  <dimension ref="A1:O110"/>
+  <dimension ref="A1:P110"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="10.5" bestFit="1" customWidth="1"/>
@@ -17960,17 +17991,17 @@
     <col min="5" max="5" width="12.6640625" bestFit="1" customWidth="1"/>
     <col min="6" max="6" width="14.83203125" bestFit="1" customWidth="1"/>
     <col min="7" max="7" width="15.83203125" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="13.5" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="15.6640625" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="14.5" bestFit="1" customWidth="1"/>
-    <col min="11" max="11" width="22.83203125" bestFit="1" customWidth="1"/>
-    <col min="12" max="12" width="11" bestFit="1" customWidth="1"/>
-    <col min="13" max="13" width="18.5" bestFit="1" customWidth="1"/>
-    <col min="14" max="14" width="18.5" customWidth="1"/>
-    <col min="15" max="15" width="96.33203125" bestFit="1" customWidth="1"/>
+    <col min="8" max="9" width="13.5" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="15.6640625" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="14.5" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="22.83203125" bestFit="1" customWidth="1"/>
+    <col min="13" max="13" width="11" bestFit="1" customWidth="1"/>
+    <col min="14" max="14" width="18.5" bestFit="1" customWidth="1"/>
+    <col min="15" max="15" width="18.5" customWidth="1"/>
+    <col min="16" max="16" width="96.33203125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:15" s="39" customFormat="1" ht="19" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:16" s="39" customFormat="1" ht="19" x14ac:dyDescent="0.25">
       <c r="A1" s="39" t="s">
         <v>666</v>
       </c>
@@ -17993,31 +18024,34 @@
         <v>682</v>
       </c>
       <c r="H1" s="39" t="s">
+        <v>988</v>
+      </c>
+      <c r="I1" s="39" t="s">
         <v>831</v>
       </c>
-      <c r="I1" s="40" t="s">
+      <c r="J1" s="40" t="s">
         <v>800</v>
       </c>
-      <c r="J1" s="40" t="s">
+      <c r="K1" s="40" t="s">
         <v>801</v>
       </c>
-      <c r="K1" s="40" t="s">
+      <c r="L1" s="40" t="s">
         <v>802</v>
       </c>
-      <c r="L1" s="40" t="s">
+      <c r="M1" s="40" t="s">
         <v>803</v>
       </c>
-      <c r="M1" s="40" t="s">
+      <c r="N1" s="40" t="s">
         <v>804</v>
       </c>
-      <c r="N1" s="40" t="s">
+      <c r="O1" s="40" t="s">
         <v>865</v>
       </c>
-      <c r="O1" s="40" t="s">
+      <c r="P1" s="40" t="s">
         <v>120</v>
       </c>
     </row>
-    <row r="2" spans="1:15" s="25" customFormat="1" x14ac:dyDescent="0.2">
+    <row r="2" spans="1:16" s="25" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A2" s="25" t="b">
         <v>1</v>
       </c>
@@ -18036,17 +18070,18 @@
       <c r="H2" s="28" t="s">
         <v>832</v>
       </c>
-      <c r="I2" s="25" t="s">
-        <v>645</v>
-      </c>
+      <c r="I2" s="28"/>
       <c r="J2" s="25" t="s">
+        <v>645</v>
+      </c>
+      <c r="K2" s="25" t="s">
         <v>481</v>
       </c>
-      <c r="K2" s="25" t="s">
+      <c r="L2" s="25" t="s">
         <v>654</v>
       </c>
     </row>
-    <row r="3" spans="1:15" s="25" customFormat="1" x14ac:dyDescent="0.2">
+    <row r="3" spans="1:16" s="25" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A3" s="25" t="b">
         <v>1</v>
       </c>
@@ -18062,23 +18097,24 @@
       <c r="H3" s="28" t="s">
         <v>833</v>
       </c>
-      <c r="I3" s="25" t="s">
-        <v>645</v>
-      </c>
+      <c r="I3" s="28"/>
       <c r="J3" s="25" t="s">
+        <v>645</v>
+      </c>
+      <c r="K3" s="25" t="s">
         <v>580</v>
       </c>
-      <c r="K3" s="25" t="s">
+      <c r="L3" s="25" t="s">
         <v>677</v>
       </c>
-      <c r="L3" s="25" t="s">
+      <c r="M3" s="25" t="s">
         <v>171</v>
       </c>
-      <c r="M3" s="25" t="s">
+      <c r="N3" s="25" t="s">
         <v>158</v>
       </c>
     </row>
-    <row r="4" spans="1:15" s="25" customFormat="1" x14ac:dyDescent="0.2">
+    <row r="4" spans="1:16" s="25" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A4" s="25" t="b">
         <v>1</v>
       </c>
@@ -18097,17 +18133,18 @@
       <c r="H4" s="28" t="s">
         <v>834</v>
       </c>
-      <c r="I4" s="25" t="s">
-        <v>645</v>
-      </c>
+      <c r="I4" s="28"/>
       <c r="J4" s="25" t="s">
+        <v>645</v>
+      </c>
+      <c r="K4" s="25" t="s">
         <v>501</v>
       </c>
-      <c r="K4" s="25" t="s">
+      <c r="L4" s="25" t="s">
         <v>656</v>
       </c>
     </row>
-    <row r="5" spans="1:15" s="25" customFormat="1" x14ac:dyDescent="0.2">
+    <row r="5" spans="1:16" s="25" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A5" s="25" t="b">
         <v>1</v>
       </c>
@@ -18126,23 +18163,24 @@
       <c r="H5" s="28" t="s">
         <v>835</v>
       </c>
-      <c r="I5" s="25" t="s">
+      <c r="I5" s="28"/>
+      <c r="J5" s="25" t="s">
         <v>477</v>
       </c>
-      <c r="J5" s="25" t="s">
-        <v>645</v>
-      </c>
       <c r="K5" s="25" t="s">
+        <v>645</v>
+      </c>
+      <c r="L5" s="25" t="s">
         <v>650</v>
       </c>
-      <c r="L5" s="25" t="s">
+      <c r="M5" s="25" t="s">
         <v>168</v>
       </c>
-      <c r="M5" s="25" t="s">
+      <c r="N5" s="25" t="s">
         <v>154</v>
       </c>
     </row>
-    <row r="6" spans="1:15" s="25" customFormat="1" x14ac:dyDescent="0.2">
+    <row r="6" spans="1:16" s="25" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A6" s="25" t="b">
         <v>1</v>
       </c>
@@ -18161,23 +18199,24 @@
       <c r="H6" s="28" t="s">
         <v>836</v>
       </c>
-      <c r="I6" s="25" t="s">
+      <c r="I6" s="28"/>
+      <c r="J6" s="25" t="s">
         <v>476</v>
       </c>
-      <c r="J6" s="25" t="s">
-        <v>645</v>
-      </c>
       <c r="K6" s="25" t="s">
+        <v>645</v>
+      </c>
+      <c r="L6" s="25" t="s">
         <v>649</v>
       </c>
-      <c r="L6" s="25" t="s">
+      <c r="M6" s="25" t="s">
         <v>157</v>
       </c>
-      <c r="M6" s="25" t="s">
+      <c r="N6" s="25" t="s">
         <v>154</v>
       </c>
     </row>
-    <row r="7" spans="1:15" s="25" customFormat="1" x14ac:dyDescent="0.2">
+    <row r="7" spans="1:16" s="25" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A7" s="25" t="b">
         <v>1</v>
       </c>
@@ -18196,23 +18235,24 @@
       <c r="H7" s="28" t="s">
         <v>837</v>
       </c>
-      <c r="I7" s="25" t="s">
+      <c r="I7" s="28"/>
+      <c r="J7" s="25" t="s">
         <v>479</v>
       </c>
-      <c r="J7" s="25" t="s">
-        <v>645</v>
-      </c>
       <c r="K7" s="25" t="s">
+        <v>645</v>
+      </c>
+      <c r="L7" s="25" t="s">
         <v>652</v>
       </c>
-      <c r="L7" s="25" t="s">
+      <c r="M7" s="25" t="s">
         <v>168</v>
       </c>
-      <c r="M7" s="25" t="s">
+      <c r="N7" s="25" t="s">
         <v>154</v>
       </c>
     </row>
-    <row r="8" spans="1:15" s="25" customFormat="1" x14ac:dyDescent="0.2">
+    <row r="8" spans="1:16" s="25" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A8" s="25" t="b">
         <v>1</v>
       </c>
@@ -18231,23 +18271,24 @@
       <c r="H8" s="28" t="s">
         <v>838</v>
       </c>
-      <c r="I8" s="25" t="s">
+      <c r="I8" s="28"/>
+      <c r="J8" s="25" t="s">
         <v>478</v>
       </c>
-      <c r="J8" s="25" t="s">
-        <v>645</v>
-      </c>
       <c r="K8" s="25" t="s">
+        <v>645</v>
+      </c>
+      <c r="L8" s="25" t="s">
         <v>651</v>
       </c>
-      <c r="L8" s="25" t="s">
+      <c r="M8" s="25" t="s">
         <v>157</v>
       </c>
-      <c r="M8" s="25" t="s">
+      <c r="N8" s="25" t="s">
         <v>154</v>
       </c>
     </row>
-    <row r="9" spans="1:15" s="25" customFormat="1" x14ac:dyDescent="0.2">
+    <row r="9" spans="1:16" s="25" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A9" s="25" t="b">
         <v>1</v>
       </c>
@@ -18266,24 +18307,25 @@
       <c r="H9" s="28" t="s">
         <v>839</v>
       </c>
-      <c r="I9" s="25" t="s">
-        <v>645</v>
-      </c>
+      <c r="I9" s="28"/>
       <c r="J9" s="25" t="s">
+        <v>645</v>
+      </c>
+      <c r="K9" s="25" t="s">
         <v>480</v>
       </c>
-      <c r="K9" s="25" t="s">
+      <c r="L9" s="25" t="s">
         <v>653</v>
       </c>
-      <c r="L9" s="25" t="s">
+      <c r="M9" s="25" t="s">
         <v>153</v>
       </c>
-      <c r="M9" s="25" t="s">
+      <c r="N9" s="25" t="s">
         <v>154</v>
       </c>
     </row>
-    <row r="10" spans="1:15" s="25" customFormat="1" x14ac:dyDescent="0.2"/>
-    <row r="11" spans="1:15" s="25" customFormat="1" x14ac:dyDescent="0.2">
+    <row r="10" spans="1:16" s="25" customFormat="1" x14ac:dyDescent="0.2"/>
+    <row r="11" spans="1:16" s="25" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A11" s="25" t="b">
         <v>1</v>
       </c>
@@ -18305,17 +18347,17 @@
       <c r="H11" s="25" t="s">
         <v>840</v>
       </c>
-      <c r="I11" s="25" t="s">
-        <v>645</v>
-      </c>
       <c r="J11" s="25" t="s">
+        <v>645</v>
+      </c>
+      <c r="K11" s="25" t="s">
         <v>425</v>
       </c>
-      <c r="K11" s="25" t="s">
+      <c r="L11" s="25" t="s">
         <v>671</v>
       </c>
     </row>
-    <row r="12" spans="1:15" s="25" customFormat="1" x14ac:dyDescent="0.2">
+    <row r="12" spans="1:16" s="25" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A12" s="25" t="b">
         <v>1</v>
       </c>
@@ -18334,17 +18376,17 @@
       <c r="F12" s="25" t="s">
         <v>426</v>
       </c>
-      <c r="I12" s="25" t="s">
-        <v>645</v>
-      </c>
       <c r="J12" s="25" t="s">
         <v>645</v>
       </c>
       <c r="K12" s="25" t="s">
         <v>645</v>
       </c>
-    </row>
-    <row r="13" spans="1:15" s="25" customFormat="1" x14ac:dyDescent="0.2">
+      <c r="L12" s="25" t="s">
+        <v>645</v>
+      </c>
+    </row>
+    <row r="13" spans="1:16" s="25" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A13" s="25" t="b">
         <v>1</v>
       </c>
@@ -18363,17 +18405,17 @@
       <c r="F13" s="25" t="s">
         <v>428</v>
       </c>
-      <c r="I13" s="25" t="s">
-        <v>645</v>
-      </c>
       <c r="J13" s="25" t="s">
         <v>645</v>
       </c>
       <c r="K13" s="25" t="s">
         <v>645</v>
       </c>
-    </row>
-    <row r="14" spans="1:15" s="25" customFormat="1" x14ac:dyDescent="0.2">
+      <c r="L13" s="25" t="s">
+        <v>645</v>
+      </c>
+    </row>
+    <row r="14" spans="1:16" s="25" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A14" s="25" t="b">
         <v>1</v>
       </c>
@@ -18392,17 +18434,17 @@
       <c r="F14" s="25" t="s">
         <v>429</v>
       </c>
-      <c r="I14" s="25" t="s">
-        <v>645</v>
-      </c>
       <c r="J14" s="25" t="s">
         <v>645</v>
       </c>
       <c r="K14" s="25" t="s">
         <v>645</v>
       </c>
-    </row>
-    <row r="15" spans="1:15" s="25" customFormat="1" x14ac:dyDescent="0.2">
+      <c r="L14" s="25" t="s">
+        <v>645</v>
+      </c>
+    </row>
+    <row r="15" spans="1:16" s="25" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A15" s="25" t="b">
         <v>1</v>
       </c>
@@ -18421,14 +18463,14 @@
       <c r="F15" s="25" t="s">
         <v>430</v>
       </c>
-      <c r="I15" s="25" t="s">
-        <v>645</v>
-      </c>
       <c r="J15" s="25" t="s">
         <v>645</v>
       </c>
-    </row>
-    <row r="16" spans="1:15" s="25" customFormat="1" x14ac:dyDescent="0.2">
+      <c r="K15" s="25" t="s">
+        <v>645</v>
+      </c>
+    </row>
+    <row r="16" spans="1:16" s="25" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A16" s="25" t="b">
         <v>1</v>
       </c>
@@ -18447,17 +18489,17 @@
       <c r="F16" s="25" t="s">
         <v>431</v>
       </c>
-      <c r="I16" s="25" t="s">
-        <v>645</v>
-      </c>
       <c r="J16" s="25" t="s">
         <v>645</v>
       </c>
       <c r="K16" s="25" t="s">
         <v>645</v>
       </c>
-    </row>
-    <row r="17" spans="1:11" s="25" customFormat="1" x14ac:dyDescent="0.2">
+      <c r="L16" s="25" t="s">
+        <v>645</v>
+      </c>
+    </row>
+    <row r="17" spans="1:12" s="25" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A17" s="25" t="b">
         <v>1</v>
       </c>
@@ -18476,17 +18518,17 @@
       <c r="F17" s="25" t="s">
         <v>430</v>
       </c>
-      <c r="I17" s="25" t="s">
-        <v>645</v>
-      </c>
       <c r="J17" s="25" t="s">
         <v>645</v>
       </c>
       <c r="K17" s="25" t="s">
         <v>645</v>
       </c>
-    </row>
-    <row r="18" spans="1:11" s="25" customFormat="1" x14ac:dyDescent="0.2">
+      <c r="L17" s="25" t="s">
+        <v>645</v>
+      </c>
+    </row>
+    <row r="18" spans="1:12" s="25" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A18" s="25" t="b">
         <v>1</v>
       </c>
@@ -18505,17 +18547,17 @@
       <c r="F18" s="25" t="s">
         <v>432</v>
       </c>
-      <c r="I18" s="25" t="s">
-        <v>645</v>
-      </c>
       <c r="J18" s="25" t="s">
         <v>645</v>
       </c>
       <c r="K18" s="25" t="s">
         <v>645</v>
       </c>
-    </row>
-    <row r="19" spans="1:11" s="25" customFormat="1" x14ac:dyDescent="0.2">
+      <c r="L18" s="25" t="s">
+        <v>645</v>
+      </c>
+    </row>
+    <row r="19" spans="1:12" s="25" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A19" s="25" t="b">
         <v>1</v>
       </c>
@@ -18534,17 +18576,17 @@
       <c r="F19" s="25" t="s">
         <v>433</v>
       </c>
-      <c r="I19" s="25" t="s">
-        <v>645</v>
-      </c>
       <c r="J19" s="25" t="s">
         <v>645</v>
       </c>
       <c r="K19" s="25" t="s">
         <v>645</v>
       </c>
-    </row>
-    <row r="20" spans="1:11" s="25" customFormat="1" x14ac:dyDescent="0.2">
+      <c r="L19" s="25" t="s">
+        <v>645</v>
+      </c>
+    </row>
+    <row r="20" spans="1:12" s="25" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A20" s="25" t="b">
         <v>1</v>
       </c>
@@ -18563,17 +18605,17 @@
       <c r="F20" s="25" t="s">
         <v>434</v>
       </c>
-      <c r="I20" s="25" t="s">
-        <v>645</v>
-      </c>
       <c r="J20" s="25" t="s">
         <v>645</v>
       </c>
       <c r="K20" s="25" t="s">
         <v>645</v>
       </c>
-    </row>
-    <row r="21" spans="1:11" s="25" customFormat="1" x14ac:dyDescent="0.2">
+      <c r="L20" s="25" t="s">
+        <v>645</v>
+      </c>
+    </row>
+    <row r="21" spans="1:12" s="25" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A21" s="25" t="b">
         <v>1</v>
       </c>
@@ -18592,17 +18634,17 @@
       <c r="F21" s="25" t="s">
         <v>436</v>
       </c>
-      <c r="I21" s="25" t="s">
-        <v>645</v>
-      </c>
       <c r="J21" s="25" t="s">
         <v>645</v>
       </c>
       <c r="K21" s="25" t="s">
         <v>645</v>
       </c>
-    </row>
-    <row r="22" spans="1:11" s="25" customFormat="1" x14ac:dyDescent="0.2">
+      <c r="L21" s="25" t="s">
+        <v>645</v>
+      </c>
+    </row>
+    <row r="22" spans="1:12" s="25" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A22" s="25" t="b">
         <v>1</v>
       </c>
@@ -18621,17 +18663,17 @@
       <c r="F22" s="25" t="s">
         <v>435</v>
       </c>
-      <c r="I22" s="25" t="s">
-        <v>645</v>
-      </c>
       <c r="J22" s="25" t="s">
         <v>645</v>
       </c>
       <c r="K22" s="25" t="s">
         <v>645</v>
       </c>
-    </row>
-    <row r="23" spans="1:11" s="25" customFormat="1" x14ac:dyDescent="0.2">
+      <c r="L22" s="25" t="s">
+        <v>645</v>
+      </c>
+    </row>
+    <row r="23" spans="1:12" s="25" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A23" s="25" t="b">
         <v>1</v>
       </c>
@@ -18650,17 +18692,17 @@
       <c r="F23" s="25" t="s">
         <v>437</v>
       </c>
-      <c r="I23" s="25" t="s">
-        <v>645</v>
-      </c>
       <c r="J23" s="25" t="s">
         <v>645</v>
       </c>
       <c r="K23" s="25" t="s">
         <v>645</v>
       </c>
-    </row>
-    <row r="24" spans="1:11" s="25" customFormat="1" x14ac:dyDescent="0.2">
+      <c r="L23" s="25" t="s">
+        <v>645</v>
+      </c>
+    </row>
+    <row r="24" spans="1:12" s="25" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A24" s="25" t="b">
         <v>1</v>
       </c>
@@ -18679,17 +18721,17 @@
       <c r="F24" s="25" t="s">
         <v>610</v>
       </c>
-      <c r="I24" s="25" t="s">
-        <v>645</v>
-      </c>
       <c r="J24" s="25" t="s">
         <v>645</v>
       </c>
       <c r="K24" s="25" t="s">
         <v>645</v>
       </c>
-    </row>
-    <row r="25" spans="1:11" s="25" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="L24" s="25" t="s">
+        <v>645</v>
+      </c>
+    </row>
+    <row r="25" spans="1:12" s="25" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A25" s="25" t="b">
         <v>1</v>
       </c>
@@ -18708,17 +18750,17 @@
       <c r="F25" s="25" t="s">
         <v>438</v>
       </c>
-      <c r="I25" s="25" t="s">
-        <v>645</v>
-      </c>
       <c r="J25" s="25" t="s">
         <v>645</v>
       </c>
       <c r="K25" s="25" t="s">
         <v>645</v>
       </c>
-    </row>
-    <row r="26" spans="1:11" s="25" customFormat="1" x14ac:dyDescent="0.2">
+      <c r="L25" s="25" t="s">
+        <v>645</v>
+      </c>
+    </row>
+    <row r="26" spans="1:12" s="25" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A26" s="25" t="b">
         <v>1</v>
       </c>
@@ -18737,17 +18779,17 @@
       <c r="F26" s="25" t="s">
         <v>439</v>
       </c>
-      <c r="I26" s="25" t="s">
-        <v>645</v>
-      </c>
       <c r="J26" s="25" t="s">
         <v>645</v>
       </c>
       <c r="K26" s="25" t="s">
         <v>645</v>
       </c>
-    </row>
-    <row r="27" spans="1:11" s="25" customFormat="1" x14ac:dyDescent="0.2">
+      <c r="L26" s="25" t="s">
+        <v>645</v>
+      </c>
+    </row>
+    <row r="27" spans="1:12" s="25" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A27" s="25" t="b">
         <v>1</v>
       </c>
@@ -18766,17 +18808,17 @@
       <c r="F27" s="25" t="s">
         <v>440</v>
       </c>
-      <c r="I27" s="25" t="s">
-        <v>645</v>
-      </c>
       <c r="J27" s="25" t="s">
         <v>645</v>
       </c>
       <c r="K27" s="25" t="s">
         <v>645</v>
       </c>
-    </row>
-    <row r="28" spans="1:11" s="25" customFormat="1" x14ac:dyDescent="0.2">
+      <c r="L27" s="25" t="s">
+        <v>645</v>
+      </c>
+    </row>
+    <row r="28" spans="1:12" s="25" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A28" s="25" t="b">
         <v>1</v>
       </c>
@@ -18795,17 +18837,17 @@
       <c r="F28" s="25" t="s">
         <v>441</v>
       </c>
-      <c r="I28" s="25" t="s">
-        <v>645</v>
-      </c>
       <c r="J28" s="25" t="s">
         <v>645</v>
       </c>
       <c r="K28" s="25" t="s">
         <v>645</v>
       </c>
-    </row>
-    <row r="29" spans="1:11" s="25" customFormat="1" x14ac:dyDescent="0.2">
+      <c r="L28" s="25" t="s">
+        <v>645</v>
+      </c>
+    </row>
+    <row r="29" spans="1:12" s="25" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A29" s="25" t="b">
         <v>1</v>
       </c>
@@ -18824,17 +18866,17 @@
       <c r="F29" s="25" t="s">
         <v>443</v>
       </c>
-      <c r="I29" s="25" t="s">
-        <v>645</v>
-      </c>
       <c r="J29" s="25" t="s">
         <v>645</v>
       </c>
       <c r="K29" s="25" t="s">
         <v>645</v>
       </c>
-    </row>
-    <row r="30" spans="1:11" s="25" customFormat="1" x14ac:dyDescent="0.2">
+      <c r="L29" s="25" t="s">
+        <v>645</v>
+      </c>
+    </row>
+    <row r="30" spans="1:12" s="25" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A30" s="25" t="b">
         <v>1</v>
       </c>
@@ -18853,17 +18895,17 @@
       <c r="F30" s="25" t="s">
         <v>442</v>
       </c>
-      <c r="I30" s="25" t="s">
-        <v>645</v>
-      </c>
       <c r="J30" s="25" t="s">
         <v>645</v>
       </c>
       <c r="K30" s="25" t="s">
         <v>645</v>
       </c>
-    </row>
-    <row r="31" spans="1:11" s="25" customFormat="1" x14ac:dyDescent="0.2">
+      <c r="L30" s="25" t="s">
+        <v>645</v>
+      </c>
+    </row>
+    <row r="31" spans="1:12" s="25" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A31" s="25" t="b">
         <v>1</v>
       </c>
@@ -18882,17 +18924,17 @@
       <c r="F31" s="25" t="s">
         <v>611</v>
       </c>
-      <c r="I31" s="25" t="s">
-        <v>645</v>
-      </c>
       <c r="J31" s="25" t="s">
         <v>645</v>
       </c>
       <c r="K31" s="25" t="s">
         <v>645</v>
       </c>
-    </row>
-    <row r="32" spans="1:11" s="25" customFormat="1" x14ac:dyDescent="0.2">
+      <c r="L31" s="25" t="s">
+        <v>645</v>
+      </c>
+    </row>
+    <row r="32" spans="1:12" s="25" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A32" s="25" t="b">
         <v>1</v>
       </c>
@@ -18911,17 +18953,17 @@
       <c r="F32" s="25" t="s">
         <v>612</v>
       </c>
-      <c r="I32" s="25" t="s">
-        <v>645</v>
-      </c>
       <c r="J32" s="25" t="s">
         <v>645</v>
       </c>
       <c r="K32" s="25" t="s">
         <v>645</v>
       </c>
-    </row>
-    <row r="33" spans="1:11" s="25" customFormat="1" x14ac:dyDescent="0.2">
+      <c r="L32" s="25" t="s">
+        <v>645</v>
+      </c>
+    </row>
+    <row r="33" spans="1:12" s="25" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A33" s="25" t="b">
         <v>1</v>
       </c>
@@ -18940,17 +18982,17 @@
       <c r="F33" s="25" t="s">
         <v>613</v>
       </c>
-      <c r="I33" s="25" t="s">
-        <v>645</v>
-      </c>
       <c r="J33" s="25" t="s">
         <v>645</v>
       </c>
       <c r="K33" s="25" t="s">
         <v>645</v>
       </c>
-    </row>
-    <row r="34" spans="1:11" s="25" customFormat="1" x14ac:dyDescent="0.2">
+      <c r="L33" s="25" t="s">
+        <v>645</v>
+      </c>
+    </row>
+    <row r="34" spans="1:12" s="25" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A34" s="25" t="b">
         <v>1</v>
       </c>
@@ -18969,20 +19011,20 @@
       <c r="F34" s="25" t="s">
         <v>424</v>
       </c>
-      <c r="I34" s="25" t="s">
-        <v>645</v>
-      </c>
       <c r="J34" s="25" t="s">
         <v>645</v>
       </c>
       <c r="K34" s="25" t="s">
         <v>645</v>
       </c>
-    </row>
-    <row r="35" spans="1:11" s="25" customFormat="1" x14ac:dyDescent="0.2">
+      <c r="L34" s="25" t="s">
+        <v>645</v>
+      </c>
+    </row>
+    <row r="35" spans="1:12" s="25" customFormat="1" x14ac:dyDescent="0.2">
       <c r="D35" s="32"/>
     </row>
-    <row r="36" spans="1:11" s="25" customFormat="1" x14ac:dyDescent="0.2">
+    <row r="36" spans="1:12" s="25" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A36" s="25" t="b">
         <v>1</v>
       </c>
@@ -19004,17 +19046,18 @@
       <c r="H36" s="28" t="s">
         <v>841</v>
       </c>
-      <c r="I36" s="25" t="s">
-        <v>645</v>
-      </c>
+      <c r="I36" s="28"/>
       <c r="J36" s="25" t="s">
+        <v>645</v>
+      </c>
+      <c r="K36" s="25" t="s">
         <v>444</v>
       </c>
-      <c r="K36" s="25" t="s">
+      <c r="L36" s="25" t="s">
         <v>672</v>
       </c>
     </row>
-    <row r="37" spans="1:11" s="25" customFormat="1" x14ac:dyDescent="0.2">
+    <row r="37" spans="1:12" s="25" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A37" s="25" t="b">
         <v>1</v>
       </c>
@@ -19033,17 +19076,17 @@
       <c r="F37" s="25" t="s">
         <v>446</v>
       </c>
-      <c r="I37" s="25" t="s">
-        <v>645</v>
-      </c>
       <c r="J37" s="25" t="s">
         <v>645</v>
       </c>
       <c r="K37" s="25" t="s">
         <v>645</v>
       </c>
-    </row>
-    <row r="38" spans="1:11" s="25" customFormat="1" x14ac:dyDescent="0.2">
+      <c r="L37" s="25" t="s">
+        <v>645</v>
+      </c>
+    </row>
+    <row r="38" spans="1:12" s="25" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A38" s="25" t="b">
         <v>1</v>
       </c>
@@ -19062,17 +19105,17 @@
       <c r="F38" s="25" t="s">
         <v>614</v>
       </c>
-      <c r="I38" s="25" t="s">
-        <v>645</v>
-      </c>
       <c r="J38" s="25" t="s">
         <v>645</v>
       </c>
       <c r="K38" s="25" t="s">
         <v>645</v>
       </c>
-    </row>
-    <row r="39" spans="1:11" s="25" customFormat="1" x14ac:dyDescent="0.2">
+      <c r="L38" s="25" t="s">
+        <v>645</v>
+      </c>
+    </row>
+    <row r="39" spans="1:12" s="25" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A39" s="25" t="b">
         <v>1</v>
       </c>
@@ -19091,17 +19134,17 @@
       <c r="F39" s="25" t="s">
         <v>615</v>
       </c>
-      <c r="I39" s="25" t="s">
-        <v>645</v>
-      </c>
       <c r="J39" s="25" t="s">
         <v>645</v>
       </c>
       <c r="K39" s="25" t="s">
         <v>645</v>
       </c>
-    </row>
-    <row r="40" spans="1:11" s="25" customFormat="1" x14ac:dyDescent="0.2">
+      <c r="L39" s="25" t="s">
+        <v>645</v>
+      </c>
+    </row>
+    <row r="40" spans="1:12" s="25" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A40" s="25" t="b">
         <v>1</v>
       </c>
@@ -19120,17 +19163,17 @@
       <c r="F40" s="25" t="s">
         <v>616</v>
       </c>
-      <c r="I40" s="25" t="s">
-        <v>645</v>
-      </c>
       <c r="J40" s="25" t="s">
         <v>645</v>
       </c>
       <c r="K40" s="25" t="s">
         <v>645</v>
       </c>
-    </row>
-    <row r="41" spans="1:11" s="25" customFormat="1" x14ac:dyDescent="0.2">
+      <c r="L40" s="25" t="s">
+        <v>645</v>
+      </c>
+    </row>
+    <row r="41" spans="1:12" s="25" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A41" s="25" t="b">
         <v>1</v>
       </c>
@@ -19149,17 +19192,17 @@
       <c r="F41" s="25" t="s">
         <v>617</v>
       </c>
-      <c r="I41" s="25" t="s">
-        <v>645</v>
-      </c>
       <c r="J41" s="25" t="s">
         <v>645</v>
       </c>
       <c r="K41" s="25" t="s">
         <v>645</v>
       </c>
-    </row>
-    <row r="42" spans="1:11" s="25" customFormat="1" x14ac:dyDescent="0.2">
+      <c r="L41" s="25" t="s">
+        <v>645</v>
+      </c>
+    </row>
+    <row r="42" spans="1:12" s="25" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A42" s="25" t="b">
         <v>1</v>
       </c>
@@ -19178,17 +19221,17 @@
       <c r="F42" s="25" t="s">
         <v>447</v>
       </c>
-      <c r="I42" s="25" t="s">
-        <v>645</v>
-      </c>
       <c r="J42" s="25" t="s">
         <v>645</v>
       </c>
       <c r="K42" s="25" t="s">
         <v>645</v>
       </c>
-    </row>
-    <row r="43" spans="1:11" s="25" customFormat="1" x14ac:dyDescent="0.2">
+      <c r="L42" s="25" t="s">
+        <v>645</v>
+      </c>
+    </row>
+    <row r="43" spans="1:12" s="25" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A43" s="25" t="b">
         <v>1</v>
       </c>
@@ -19207,17 +19250,17 @@
       <c r="F43" s="25" t="s">
         <v>448</v>
       </c>
-      <c r="I43" s="25" t="s">
-        <v>645</v>
-      </c>
       <c r="J43" s="25" t="s">
         <v>645</v>
       </c>
       <c r="K43" s="25" t="s">
         <v>645</v>
       </c>
-    </row>
-    <row r="44" spans="1:11" s="25" customFormat="1" x14ac:dyDescent="0.2">
+      <c r="L43" s="25" t="s">
+        <v>645</v>
+      </c>
+    </row>
+    <row r="44" spans="1:12" s="25" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A44" s="25" t="b">
         <v>1</v>
       </c>
@@ -19236,17 +19279,17 @@
       <c r="F44" s="25" t="s">
         <v>449</v>
       </c>
-      <c r="I44" s="25" t="s">
-        <v>645</v>
-      </c>
       <c r="J44" s="25" t="s">
         <v>645</v>
       </c>
       <c r="K44" s="25" t="s">
         <v>645</v>
       </c>
-    </row>
-    <row r="45" spans="1:11" s="25" customFormat="1" x14ac:dyDescent="0.2">
+      <c r="L44" s="25" t="s">
+        <v>645</v>
+      </c>
+    </row>
+    <row r="45" spans="1:12" s="25" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A45" s="25" t="b">
         <v>1</v>
       </c>
@@ -19265,17 +19308,17 @@
       <c r="F45" s="25" t="s">
         <v>450</v>
       </c>
-      <c r="I45" s="25" t="s">
-        <v>645</v>
-      </c>
       <c r="J45" s="25" t="s">
         <v>645</v>
       </c>
       <c r="K45" s="25" t="s">
         <v>645</v>
       </c>
-    </row>
-    <row r="46" spans="1:11" s="25" customFormat="1" x14ac:dyDescent="0.2">
+      <c r="L45" s="25" t="s">
+        <v>645</v>
+      </c>
+    </row>
+    <row r="46" spans="1:12" s="25" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A46" s="25" t="b">
         <v>1</v>
       </c>
@@ -19294,17 +19337,17 @@
       <c r="F46" s="25" t="s">
         <v>451</v>
       </c>
-      <c r="I46" s="25" t="s">
-        <v>645</v>
-      </c>
       <c r="J46" s="25" t="s">
         <v>645</v>
       </c>
       <c r="K46" s="25" t="s">
         <v>645</v>
       </c>
-    </row>
-    <row r="47" spans="1:11" s="25" customFormat="1" x14ac:dyDescent="0.2">
+      <c r="L46" s="25" t="s">
+        <v>645</v>
+      </c>
+    </row>
+    <row r="47" spans="1:12" s="25" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A47" s="25" t="b">
         <v>1</v>
       </c>
@@ -19323,17 +19366,17 @@
       <c r="F47" s="25" t="s">
         <v>452</v>
       </c>
-      <c r="I47" s="25" t="s">
-        <v>645</v>
-      </c>
       <c r="J47" s="25" t="s">
         <v>645</v>
       </c>
       <c r="K47" s="25" t="s">
         <v>645</v>
       </c>
-    </row>
-    <row r="48" spans="1:11" s="25" customFormat="1" x14ac:dyDescent="0.2">
+      <c r="L47" s="25" t="s">
+        <v>645</v>
+      </c>
+    </row>
+    <row r="48" spans="1:12" s="25" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A48" s="25" t="b">
         <v>1</v>
       </c>
@@ -19352,17 +19395,17 @@
       <c r="F48" s="25" t="s">
         <v>453</v>
       </c>
-      <c r="I48" s="25" t="s">
-        <v>645</v>
-      </c>
       <c r="J48" s="25" t="s">
         <v>645</v>
       </c>
       <c r="K48" s="25" t="s">
         <v>645</v>
       </c>
-    </row>
-    <row r="49" spans="1:11" s="25" customFormat="1" x14ac:dyDescent="0.2">
+      <c r="L48" s="25" t="s">
+        <v>645</v>
+      </c>
+    </row>
+    <row r="49" spans="1:12" s="25" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A49" s="25" t="b">
         <v>1</v>
       </c>
@@ -19381,17 +19424,17 @@
       <c r="F49" s="25" t="s">
         <v>454</v>
       </c>
-      <c r="I49" s="25" t="s">
-        <v>645</v>
-      </c>
       <c r="J49" s="25" t="s">
         <v>645</v>
       </c>
       <c r="K49" s="25" t="s">
         <v>645</v>
       </c>
-    </row>
-    <row r="50" spans="1:11" s="25" customFormat="1" x14ac:dyDescent="0.2">
+      <c r="L49" s="25" t="s">
+        <v>645</v>
+      </c>
+    </row>
+    <row r="50" spans="1:12" s="25" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A50" s="25" t="b">
         <v>1</v>
       </c>
@@ -19410,17 +19453,17 @@
       <c r="F50" s="25" t="s">
         <v>618</v>
       </c>
-      <c r="I50" s="25" t="s">
-        <v>645</v>
-      </c>
       <c r="J50" s="25" t="s">
         <v>645</v>
       </c>
       <c r="K50" s="25" t="s">
         <v>645</v>
       </c>
-    </row>
-    <row r="51" spans="1:11" s="25" customFormat="1" x14ac:dyDescent="0.2">
+      <c r="L50" s="25" t="s">
+        <v>645</v>
+      </c>
+    </row>
+    <row r="51" spans="1:12" s="25" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A51" s="25" t="b">
         <v>1</v>
       </c>
@@ -19439,17 +19482,17 @@
       <c r="F51" s="25" t="s">
         <v>456</v>
       </c>
-      <c r="I51" s="25" t="s">
-        <v>645</v>
-      </c>
       <c r="J51" s="25" t="s">
         <v>645</v>
       </c>
       <c r="K51" s="25" t="s">
         <v>645</v>
       </c>
-    </row>
-    <row r="52" spans="1:11" s="25" customFormat="1" x14ac:dyDescent="0.2">
+      <c r="L51" s="25" t="s">
+        <v>645</v>
+      </c>
+    </row>
+    <row r="52" spans="1:12" s="25" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A52" s="25" t="b">
         <v>1</v>
       </c>
@@ -19468,17 +19511,17 @@
       <c r="F52" s="25" t="s">
         <v>457</v>
       </c>
-      <c r="I52" s="25" t="s">
-        <v>645</v>
-      </c>
       <c r="J52" s="25" t="s">
         <v>645</v>
       </c>
       <c r="K52" s="25" t="s">
         <v>645</v>
       </c>
-    </row>
-    <row r="53" spans="1:11" s="25" customFormat="1" x14ac:dyDescent="0.2">
+      <c r="L52" s="25" t="s">
+        <v>645</v>
+      </c>
+    </row>
+    <row r="53" spans="1:12" s="25" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A53" s="25" t="b">
         <v>1</v>
       </c>
@@ -19497,17 +19540,17 @@
       <c r="F53" s="25" t="s">
         <v>455</v>
       </c>
-      <c r="I53" s="25" t="s">
-        <v>645</v>
-      </c>
       <c r="J53" s="25" t="s">
         <v>645</v>
       </c>
       <c r="K53" s="25" t="s">
         <v>645</v>
       </c>
-    </row>
-    <row r="54" spans="1:11" s="25" customFormat="1" x14ac:dyDescent="0.2">
+      <c r="L53" s="25" t="s">
+        <v>645</v>
+      </c>
+    </row>
+    <row r="54" spans="1:12" s="25" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A54" s="25" t="b">
         <v>1</v>
       </c>
@@ -19526,17 +19569,17 @@
       <c r="F54" s="25" t="s">
         <v>458</v>
       </c>
-      <c r="I54" s="25" t="s">
-        <v>645</v>
-      </c>
       <c r="J54" s="25" t="s">
         <v>645</v>
       </c>
       <c r="K54" s="25" t="s">
         <v>645</v>
       </c>
-    </row>
-    <row r="55" spans="1:11" s="25" customFormat="1" x14ac:dyDescent="0.2">
+      <c r="L54" s="25" t="s">
+        <v>645</v>
+      </c>
+    </row>
+    <row r="55" spans="1:12" s="25" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A55" s="25" t="b">
         <v>1</v>
       </c>
@@ -19555,17 +19598,17 @@
       <c r="F55" s="25" t="s">
         <v>459</v>
       </c>
-      <c r="I55" s="25" t="s">
-        <v>645</v>
-      </c>
       <c r="J55" s="25" t="s">
         <v>645</v>
       </c>
       <c r="K55" s="25" t="s">
         <v>645</v>
       </c>
-    </row>
-    <row r="56" spans="1:11" s="25" customFormat="1" x14ac:dyDescent="0.2">
+      <c r="L55" s="25" t="s">
+        <v>645</v>
+      </c>
+    </row>
+    <row r="56" spans="1:12" s="25" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A56" s="25" t="b">
         <v>1</v>
       </c>
@@ -19584,17 +19627,17 @@
       <c r="F56" s="25" t="s">
         <v>619</v>
       </c>
-      <c r="I56" s="25" t="s">
-        <v>645</v>
-      </c>
       <c r="J56" s="25" t="s">
         <v>645</v>
       </c>
       <c r="K56" s="25" t="s">
         <v>645</v>
       </c>
-    </row>
-    <row r="57" spans="1:11" s="25" customFormat="1" x14ac:dyDescent="0.2">
+      <c r="L56" s="25" t="s">
+        <v>645</v>
+      </c>
+    </row>
+    <row r="57" spans="1:12" s="25" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A57" s="25" t="b">
         <v>1</v>
       </c>
@@ -19613,17 +19656,17 @@
       <c r="F57" s="25" t="s">
         <v>460</v>
       </c>
-      <c r="I57" s="25" t="s">
-        <v>645</v>
-      </c>
       <c r="J57" s="25" t="s">
         <v>645</v>
       </c>
       <c r="K57" s="25" t="s">
         <v>645</v>
       </c>
-    </row>
-    <row r="58" spans="1:11" s="25" customFormat="1" x14ac:dyDescent="0.2">
+      <c r="L57" s="25" t="s">
+        <v>645</v>
+      </c>
+    </row>
+    <row r="58" spans="1:12" s="25" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A58" s="25" t="b">
         <v>1</v>
       </c>
@@ -19642,17 +19685,17 @@
       <c r="F58" s="25" t="s">
         <v>461</v>
       </c>
-      <c r="I58" s="25" t="s">
-        <v>645</v>
-      </c>
       <c r="J58" s="25" t="s">
         <v>645</v>
       </c>
       <c r="K58" s="25" t="s">
         <v>645</v>
       </c>
-    </row>
-    <row r="59" spans="1:11" s="25" customFormat="1" x14ac:dyDescent="0.2">
+      <c r="L58" s="25" t="s">
+        <v>645</v>
+      </c>
+    </row>
+    <row r="59" spans="1:12" s="25" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A59" s="25" t="b">
         <v>1</v>
       </c>
@@ -19671,17 +19714,17 @@
       <c r="F59" s="25" t="s">
         <v>620</v>
       </c>
-      <c r="I59" s="25" t="s">
-        <v>645</v>
-      </c>
       <c r="J59" s="25" t="s">
         <v>645</v>
       </c>
       <c r="K59" s="25" t="s">
         <v>645</v>
       </c>
-    </row>
-    <row r="60" spans="1:11" s="25" customFormat="1" x14ac:dyDescent="0.2">
+      <c r="L59" s="25" t="s">
+        <v>645</v>
+      </c>
+    </row>
+    <row r="60" spans="1:12" s="25" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A60" s="25" t="b">
         <v>1</v>
       </c>
@@ -19700,17 +19743,17 @@
       <c r="F60" s="25" t="s">
         <v>462</v>
       </c>
-      <c r="I60" s="25" t="s">
-        <v>645</v>
-      </c>
       <c r="J60" s="25" t="s">
         <v>645</v>
       </c>
       <c r="K60" s="25" t="s">
         <v>645</v>
       </c>
-    </row>
-    <row r="61" spans="1:11" s="25" customFormat="1" x14ac:dyDescent="0.2">
+      <c r="L60" s="25" t="s">
+        <v>645</v>
+      </c>
+    </row>
+    <row r="61" spans="1:12" s="25" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A61" s="25" t="b">
         <v>1</v>
       </c>
@@ -19729,17 +19772,17 @@
       <c r="F61" s="25" t="s">
         <v>621</v>
       </c>
-      <c r="I61" s="25" t="s">
-        <v>645</v>
-      </c>
       <c r="J61" s="25" t="s">
         <v>645</v>
       </c>
       <c r="K61" s="25" t="s">
         <v>645</v>
       </c>
-    </row>
-    <row r="62" spans="1:11" s="25" customFormat="1" x14ac:dyDescent="0.2">
+      <c r="L61" s="25" t="s">
+        <v>645</v>
+      </c>
+    </row>
+    <row r="62" spans="1:12" s="25" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A62" s="25" t="b">
         <v>1</v>
       </c>
@@ -19758,17 +19801,17 @@
       <c r="F62" s="25" t="s">
         <v>622</v>
       </c>
-      <c r="I62" s="25" t="s">
-        <v>645</v>
-      </c>
       <c r="J62" s="25" t="s">
         <v>645</v>
       </c>
       <c r="K62" s="25" t="s">
         <v>645</v>
       </c>
-    </row>
-    <row r="63" spans="1:11" s="25" customFormat="1" x14ac:dyDescent="0.2">
+      <c r="L62" s="25" t="s">
+        <v>645</v>
+      </c>
+    </row>
+    <row r="63" spans="1:12" s="25" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A63" s="25" t="b">
         <v>1</v>
       </c>
@@ -19787,17 +19830,17 @@
       <c r="F63" s="25" t="s">
         <v>623</v>
       </c>
-      <c r="I63" s="25" t="s">
-        <v>645</v>
-      </c>
       <c r="J63" s="25" t="s">
         <v>645</v>
       </c>
       <c r="K63" s="25" t="s">
         <v>645</v>
       </c>
-    </row>
-    <row r="64" spans="1:11" s="25" customFormat="1" x14ac:dyDescent="0.2">
+      <c r="L63" s="25" t="s">
+        <v>645</v>
+      </c>
+    </row>
+    <row r="64" spans="1:12" s="25" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A64" s="25" t="b">
         <v>1</v>
       </c>
@@ -19816,17 +19859,17 @@
       <c r="F64" s="25" t="s">
         <v>463</v>
       </c>
-      <c r="I64" s="25" t="s">
-        <v>645</v>
-      </c>
       <c r="J64" s="25" t="s">
         <v>645</v>
       </c>
       <c r="K64" s="25" t="s">
         <v>645</v>
       </c>
-    </row>
-    <row r="65" spans="1:14" s="25" customFormat="1" x14ac:dyDescent="0.2">
+      <c r="L64" s="25" t="s">
+        <v>645</v>
+      </c>
+    </row>
+    <row r="65" spans="1:15" s="25" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A65" s="25" t="b">
         <v>1</v>
       </c>
@@ -19845,17 +19888,17 @@
       <c r="F65" s="25" t="s">
         <v>464</v>
       </c>
-      <c r="I65" s="25" t="s">
-        <v>645</v>
-      </c>
       <c r="J65" s="25" t="s">
         <v>645</v>
       </c>
       <c r="K65" s="25" t="s">
         <v>645</v>
       </c>
-    </row>
-    <row r="66" spans="1:14" s="25" customFormat="1" x14ac:dyDescent="0.2">
+      <c r="L65" s="25" t="s">
+        <v>645</v>
+      </c>
+    </row>
+    <row r="66" spans="1:15" s="25" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A66" s="25" t="b">
         <v>1</v>
       </c>
@@ -19874,17 +19917,17 @@
       <c r="F66" s="25" t="s">
         <v>465</v>
       </c>
-      <c r="I66" s="25" t="s">
-        <v>645</v>
-      </c>
       <c r="J66" s="25" t="s">
         <v>645</v>
       </c>
       <c r="K66" s="25" t="s">
         <v>645</v>
       </c>
-    </row>
-    <row r="67" spans="1:14" s="25" customFormat="1" x14ac:dyDescent="0.2">
+      <c r="L66" s="25" t="s">
+        <v>645</v>
+      </c>
+    </row>
+    <row r="67" spans="1:15" s="25" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A67" s="25" t="b">
         <v>1</v>
       </c>
@@ -19903,17 +19946,17 @@
       <c r="F67" s="25" t="s">
         <v>624</v>
       </c>
-      <c r="I67" s="25" t="s">
-        <v>645</v>
-      </c>
       <c r="J67" s="25" t="s">
         <v>645</v>
       </c>
       <c r="K67" s="25" t="s">
         <v>645</v>
       </c>
-    </row>
-    <row r="68" spans="1:14" s="25" customFormat="1" x14ac:dyDescent="0.2">
+      <c r="L67" s="25" t="s">
+        <v>645</v>
+      </c>
+    </row>
+    <row r="68" spans="1:15" s="25" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A68" s="25" t="b">
         <v>1</v>
       </c>
@@ -19932,20 +19975,20 @@
       <c r="F68" s="25" t="s">
         <v>625</v>
       </c>
-      <c r="I68" s="25" t="s">
-        <v>645</v>
-      </c>
       <c r="J68" s="25" t="s">
         <v>645</v>
       </c>
       <c r="K68" s="25" t="s">
         <v>645</v>
       </c>
-    </row>
-    <row r="69" spans="1:14" s="25" customFormat="1" x14ac:dyDescent="0.2">
+      <c r="L68" s="25" t="s">
+        <v>645</v>
+      </c>
+    </row>
+    <row r="69" spans="1:15" s="25" customFormat="1" x14ac:dyDescent="0.2">
       <c r="D69" s="37"/>
     </row>
-    <row r="70" spans="1:14" s="25" customFormat="1" x14ac:dyDescent="0.2">
+    <row r="70" spans="1:15" s="25" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A70" s="25" t="b">
         <v>1</v>
       </c>
@@ -19967,17 +20010,18 @@
       <c r="H70" s="28" t="s">
         <v>842</v>
       </c>
-      <c r="I70" s="25" t="s">
-        <v>645</v>
-      </c>
+      <c r="I70" s="28"/>
       <c r="J70" s="25" t="s">
+        <v>645</v>
+      </c>
+      <c r="K70" s="25" t="s">
         <v>466</v>
       </c>
-      <c r="K70" s="25" t="s">
+      <c r="L70" s="25" t="s">
         <v>675</v>
       </c>
     </row>
-    <row r="71" spans="1:14" s="25" customFormat="1" x14ac:dyDescent="0.2">
+    <row r="71" spans="1:15" s="25" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A71" s="25" t="b">
         <v>1</v>
       </c>
@@ -19996,17 +20040,17 @@
       <c r="F71" s="25" t="s">
         <v>388</v>
       </c>
-      <c r="I71" s="25" t="s">
-        <v>645</v>
-      </c>
       <c r="J71" s="25" t="s">
         <v>645</v>
       </c>
       <c r="K71" s="25" t="s">
         <v>645</v>
       </c>
-    </row>
-    <row r="72" spans="1:14" s="25" customFormat="1" x14ac:dyDescent="0.2">
+      <c r="L71" s="25" t="s">
+        <v>645</v>
+      </c>
+    </row>
+    <row r="72" spans="1:15" s="25" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A72" s="25" t="b">
         <v>1</v>
       </c>
@@ -20025,17 +20069,17 @@
       <c r="F72" s="25" t="s">
         <v>470</v>
       </c>
-      <c r="I72" s="25" t="s">
-        <v>645</v>
-      </c>
       <c r="J72" s="25" t="s">
         <v>645</v>
       </c>
       <c r="K72" s="25" t="s">
         <v>645</v>
       </c>
-    </row>
-    <row r="73" spans="1:14" s="25" customFormat="1" x14ac:dyDescent="0.2">
+      <c r="L72" s="25" t="s">
+        <v>645</v>
+      </c>
+    </row>
+    <row r="73" spans="1:15" s="25" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A73" s="25" t="b">
         <v>1</v>
       </c>
@@ -20054,17 +20098,17 @@
       <c r="F73" s="25" t="s">
         <v>467</v>
       </c>
-      <c r="I73" s="25" t="s">
-        <v>645</v>
-      </c>
       <c r="J73" s="25" t="s">
         <v>645</v>
       </c>
       <c r="K73" s="25" t="s">
         <v>645</v>
       </c>
-    </row>
-    <row r="74" spans="1:14" s="25" customFormat="1" x14ac:dyDescent="0.2">
+      <c r="L73" s="25" t="s">
+        <v>645</v>
+      </c>
+    </row>
+    <row r="74" spans="1:15" s="25" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A74" s="25" t="b">
         <v>1</v>
       </c>
@@ -20083,17 +20127,17 @@
       <c r="F74" s="25" t="s">
         <v>468</v>
       </c>
-      <c r="I74" s="25" t="s">
-        <v>645</v>
-      </c>
       <c r="J74" s="25" t="s">
         <v>645</v>
       </c>
       <c r="K74" s="25" t="s">
         <v>645</v>
       </c>
-    </row>
-    <row r="75" spans="1:14" s="25" customFormat="1" x14ac:dyDescent="0.2">
+      <c r="L74" s="25" t="s">
+        <v>645</v>
+      </c>
+    </row>
+    <row r="75" spans="1:15" s="25" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A75" s="25" t="b">
         <v>1</v>
       </c>
@@ -20112,17 +20156,17 @@
       <c r="F75" s="25" t="s">
         <v>469</v>
       </c>
-      <c r="I75" s="25" t="s">
-        <v>645</v>
-      </c>
       <c r="J75" s="25" t="s">
         <v>645</v>
       </c>
       <c r="K75" s="25" t="s">
         <v>645</v>
       </c>
-    </row>
-    <row r="76" spans="1:14" s="25" customFormat="1" x14ac:dyDescent="0.2">
+      <c r="L75" s="25" t="s">
+        <v>645</v>
+      </c>
+    </row>
+    <row r="76" spans="1:15" s="25" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A76" s="25" t="b">
         <v>1</v>
       </c>
@@ -20141,20 +20185,20 @@
       <c r="F76" s="25" t="s">
         <v>388</v>
       </c>
-      <c r="I76" s="25" t="s">
-        <v>645</v>
-      </c>
       <c r="J76" s="25" t="s">
         <v>645</v>
       </c>
       <c r="K76" s="25" t="s">
         <v>645</v>
       </c>
-    </row>
-    <row r="77" spans="1:14" s="25" customFormat="1" x14ac:dyDescent="0.2">
+      <c r="L76" s="25" t="s">
+        <v>645</v>
+      </c>
+    </row>
+    <row r="77" spans="1:15" s="25" customFormat="1" x14ac:dyDescent="0.2">
       <c r="D77" s="32"/>
     </row>
-    <row r="78" spans="1:14" s="25" customFormat="1" x14ac:dyDescent="0.2">
+    <row r="78" spans="1:15" s="25" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A78" s="25" t="b">
         <v>1</v>
       </c>
@@ -20176,20 +20220,21 @@
       <c r="H78" s="28" t="s">
         <v>843</v>
       </c>
-      <c r="I78" s="25" t="s">
-        <v>645</v>
-      </c>
+      <c r="I78" s="28"/>
       <c r="J78" s="25" t="s">
+        <v>645</v>
+      </c>
+      <c r="K78" s="25" t="s">
         <v>504</v>
       </c>
-      <c r="K78" s="25" t="s">
+      <c r="L78" s="25" t="s">
         <v>676</v>
       </c>
-      <c r="N78" s="25" t="s">
+      <c r="O78" s="25" t="s">
         <v>861</v>
       </c>
     </row>
-    <row r="79" spans="1:14" s="25" customFormat="1" x14ac:dyDescent="0.2">
+    <row r="79" spans="1:15" s="25" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A79" s="25" t="b">
         <v>1</v>
       </c>
@@ -20209,21 +20254,23 @@
         <v>407</v>
       </c>
       <c r="H79" s="28"/>
-      <c r="I79" s="25" t="s">
-        <v>645</v>
-      </c>
+      <c r="I79" s="28"/>
       <c r="J79" s="25" t="s">
         <v>645</v>
       </c>
       <c r="K79" s="25" t="s">
         <v>645</v>
       </c>
-    </row>
-    <row r="80" spans="1:14" s="25" customFormat="1" x14ac:dyDescent="0.2">
+      <c r="L79" s="25" t="s">
+        <v>645</v>
+      </c>
+    </row>
+    <row r="80" spans="1:15" s="25" customFormat="1" x14ac:dyDescent="0.2">
       <c r="D80" s="32"/>
       <c r="H80" s="28"/>
-    </row>
-    <row r="81" spans="1:11" s="25" customFormat="1" x14ac:dyDescent="0.2">
+      <c r="I80" s="28"/>
+    </row>
+    <row r="81" spans="1:12" s="25" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A81" s="25" t="b">
         <v>1</v>
       </c>
@@ -20242,17 +20289,18 @@
       <c r="H81" s="28" t="s">
         <v>844</v>
       </c>
-      <c r="I81" s="25" t="s">
-        <v>645</v>
-      </c>
+      <c r="I81" s="28"/>
       <c r="J81" s="25" t="s">
+        <v>645</v>
+      </c>
+      <c r="K81" s="25" t="s">
         <v>483</v>
       </c>
-      <c r="K81" s="25" t="s">
+      <c r="L81" s="25" t="s">
         <v>674</v>
       </c>
     </row>
-    <row r="82" spans="1:11" s="25" customFormat="1" x14ac:dyDescent="0.2">
+    <row r="82" spans="1:12" s="25" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A82" s="25" t="b">
         <v>1</v>
       </c>
@@ -20271,17 +20319,17 @@
       <c r="F82" s="25" t="s">
         <v>495</v>
       </c>
-      <c r="I82" s="25" t="s">
-        <v>645</v>
-      </c>
       <c r="J82" s="25" t="s">
         <v>645</v>
       </c>
       <c r="K82" s="25" t="s">
         <v>645</v>
       </c>
-    </row>
-    <row r="83" spans="1:11" s="25" customFormat="1" x14ac:dyDescent="0.2">
+      <c r="L82" s="25" t="s">
+        <v>645</v>
+      </c>
+    </row>
+    <row r="83" spans="1:12" s="25" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A83" s="25" t="b">
         <v>1</v>
       </c>
@@ -20300,17 +20348,17 @@
       <c r="F83" s="25" t="s">
         <v>497</v>
       </c>
-      <c r="I83" s="25" t="s">
-        <v>645</v>
-      </c>
       <c r="J83" s="25" t="s">
         <v>645</v>
       </c>
       <c r="K83" s="25" t="s">
         <v>645</v>
       </c>
-    </row>
-    <row r="84" spans="1:11" s="25" customFormat="1" x14ac:dyDescent="0.2">
+      <c r="L83" s="25" t="s">
+        <v>645</v>
+      </c>
+    </row>
+    <row r="84" spans="1:12" s="25" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A84" s="25" t="b">
         <v>1</v>
       </c>
@@ -20329,17 +20377,17 @@
       <c r="F84" s="25" t="s">
         <v>498</v>
       </c>
-      <c r="I84" s="25" t="s">
-        <v>645</v>
-      </c>
       <c r="J84" s="25" t="s">
         <v>645</v>
       </c>
       <c r="K84" s="25" t="s">
         <v>645</v>
       </c>
-    </row>
-    <row r="85" spans="1:11" s="25" customFormat="1" x14ac:dyDescent="0.2">
+      <c r="L84" s="25" t="s">
+        <v>645</v>
+      </c>
+    </row>
+    <row r="85" spans="1:12" s="25" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A85" s="25" t="b">
         <v>1</v>
       </c>
@@ -20358,17 +20406,17 @@
       <c r="F85" s="25" t="s">
         <v>499</v>
       </c>
-      <c r="I85" s="25" t="s">
-        <v>645</v>
-      </c>
       <c r="J85" s="25" t="s">
         <v>645</v>
       </c>
       <c r="K85" s="25" t="s">
         <v>645</v>
       </c>
-    </row>
-    <row r="86" spans="1:11" s="25" customFormat="1" x14ac:dyDescent="0.2">
+      <c r="L85" s="25" t="s">
+        <v>645</v>
+      </c>
+    </row>
+    <row r="86" spans="1:12" s="25" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A86" s="25" t="b">
         <v>1</v>
       </c>
@@ -20387,17 +20435,17 @@
       <c r="F86" s="25" t="s">
         <v>500</v>
       </c>
-      <c r="I86" s="25" t="s">
-        <v>645</v>
-      </c>
       <c r="J86" s="25" t="s">
         <v>645</v>
       </c>
       <c r="K86" s="25" t="s">
         <v>645</v>
       </c>
-    </row>
-    <row r="87" spans="1:11" s="25" customFormat="1" x14ac:dyDescent="0.2">
+      <c r="L86" s="25" t="s">
+        <v>645</v>
+      </c>
+    </row>
+    <row r="87" spans="1:12" s="25" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A87" s="25" t="b">
         <v>1</v>
       </c>
@@ -20416,20 +20464,20 @@
       <c r="F87" s="25" t="s">
         <v>496</v>
       </c>
-      <c r="I87" s="25" t="s">
-        <v>645</v>
-      </c>
       <c r="J87" s="25" t="s">
         <v>645</v>
       </c>
       <c r="K87" s="25" t="s">
         <v>645</v>
       </c>
-    </row>
-    <row r="88" spans="1:11" s="25" customFormat="1" x14ac:dyDescent="0.2">
+      <c r="L87" s="25" t="s">
+        <v>645</v>
+      </c>
+    </row>
+    <row r="88" spans="1:12" s="25" customFormat="1" x14ac:dyDescent="0.2">
       <c r="D88" s="32"/>
     </row>
-    <row r="89" spans="1:11" s="25" customFormat="1" x14ac:dyDescent="0.2">
+    <row r="89" spans="1:12" s="25" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A89" s="25" t="b">
         <v>1</v>
       </c>
@@ -20448,17 +20496,18 @@
       <c r="H89" s="28" t="s">
         <v>845</v>
       </c>
-      <c r="I89" s="25" t="s">
-        <v>645</v>
-      </c>
+      <c r="I89" s="28"/>
       <c r="J89" s="25" t="s">
+        <v>645</v>
+      </c>
+      <c r="K89" s="25" t="s">
         <v>482</v>
       </c>
-      <c r="K89" s="25" t="s">
+      <c r="L89" s="25" t="s">
         <v>673</v>
       </c>
     </row>
-    <row r="90" spans="1:11" s="25" customFormat="1" x14ac:dyDescent="0.2">
+    <row r="90" spans="1:12" s="25" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A90" s="25" t="b">
         <v>1</v>
       </c>
@@ -20477,17 +20526,17 @@
       <c r="F90" s="25" t="s">
         <v>626</v>
       </c>
-      <c r="I90" s="25" t="s">
-        <v>645</v>
-      </c>
       <c r="J90" s="25" t="s">
         <v>645</v>
       </c>
       <c r="K90" s="25" t="s">
         <v>645</v>
       </c>
-    </row>
-    <row r="91" spans="1:11" s="25" customFormat="1" x14ac:dyDescent="0.2">
+      <c r="L90" s="25" t="s">
+        <v>645</v>
+      </c>
+    </row>
+    <row r="91" spans="1:12" s="25" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A91" s="25" t="b">
         <v>1</v>
       </c>
@@ -20506,17 +20555,17 @@
       <c r="F91" s="25" t="s">
         <v>484</v>
       </c>
-      <c r="I91" s="25" t="s">
-        <v>645</v>
-      </c>
       <c r="J91" s="25" t="s">
         <v>645</v>
       </c>
       <c r="K91" s="25" t="s">
         <v>645</v>
       </c>
-    </row>
-    <row r="92" spans="1:11" s="25" customFormat="1" x14ac:dyDescent="0.2">
+      <c r="L91" s="25" t="s">
+        <v>645</v>
+      </c>
+    </row>
+    <row r="92" spans="1:12" s="25" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A92" s="25" t="b">
         <v>1</v>
       </c>
@@ -20535,17 +20584,17 @@
       <c r="F92" s="25" t="s">
         <v>485</v>
       </c>
-      <c r="I92" s="25" t="s">
-        <v>645</v>
-      </c>
       <c r="J92" s="25" t="s">
         <v>645</v>
       </c>
       <c r="K92" s="25" t="s">
         <v>645</v>
       </c>
-    </row>
-    <row r="93" spans="1:11" s="25" customFormat="1" x14ac:dyDescent="0.2">
+      <c r="L92" s="25" t="s">
+        <v>645</v>
+      </c>
+    </row>
+    <row r="93" spans="1:12" s="25" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A93" s="25" t="b">
         <v>1</v>
       </c>
@@ -20564,17 +20613,17 @@
       <c r="F93" s="25" t="s">
         <v>486</v>
       </c>
-      <c r="I93" s="25" t="s">
-        <v>645</v>
-      </c>
       <c r="J93" s="25" t="s">
         <v>645</v>
       </c>
       <c r="K93" s="25" t="s">
         <v>645</v>
       </c>
-    </row>
-    <row r="94" spans="1:11" s="25" customFormat="1" x14ac:dyDescent="0.2">
+      <c r="L93" s="25" t="s">
+        <v>645</v>
+      </c>
+    </row>
+    <row r="94" spans="1:12" s="25" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A94" s="25" t="b">
         <v>1</v>
       </c>
@@ -20593,17 +20642,17 @@
       <c r="F94" s="25" t="s">
         <v>487</v>
       </c>
-      <c r="I94" s="25" t="s">
-        <v>645</v>
-      </c>
       <c r="J94" s="25" t="s">
         <v>645</v>
       </c>
       <c r="K94" s="25" t="s">
         <v>645</v>
       </c>
-    </row>
-    <row r="95" spans="1:11" s="25" customFormat="1" x14ac:dyDescent="0.2">
+      <c r="L94" s="25" t="s">
+        <v>645</v>
+      </c>
+    </row>
+    <row r="95" spans="1:12" s="25" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A95" s="25" t="b">
         <v>1</v>
       </c>
@@ -20622,17 +20671,17 @@
       <c r="F95" s="25" t="s">
         <v>488</v>
       </c>
-      <c r="I95" s="25" t="s">
-        <v>645</v>
-      </c>
       <c r="J95" s="25" t="s">
         <v>645</v>
       </c>
       <c r="K95" s="25" t="s">
         <v>645</v>
       </c>
-    </row>
-    <row r="96" spans="1:11" s="25" customFormat="1" x14ac:dyDescent="0.2">
+      <c r="L95" s="25" t="s">
+        <v>645</v>
+      </c>
+    </row>
+    <row r="96" spans="1:12" s="25" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A96" s="25" t="b">
         <v>1</v>
       </c>
@@ -20651,17 +20700,17 @@
       <c r="F96" s="25" t="s">
         <v>489</v>
       </c>
-      <c r="I96" s="25" t="s">
-        <v>645</v>
-      </c>
       <c r="J96" s="25" t="s">
         <v>645</v>
       </c>
       <c r="K96" s="25" t="s">
         <v>645</v>
       </c>
-    </row>
-    <row r="97" spans="1:11" s="25" customFormat="1" x14ac:dyDescent="0.2">
+      <c r="L96" s="25" t="s">
+        <v>645</v>
+      </c>
+    </row>
+    <row r="97" spans="1:12" s="25" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A97" s="25" t="b">
         <v>1</v>
       </c>
@@ -20680,17 +20729,17 @@
       <c r="F97" s="25" t="s">
         <v>490</v>
       </c>
-      <c r="I97" s="25" t="s">
-        <v>645</v>
-      </c>
       <c r="J97" s="25" t="s">
         <v>645</v>
       </c>
       <c r="K97" s="25" t="s">
         <v>645</v>
       </c>
-    </row>
-    <row r="98" spans="1:11" s="25" customFormat="1" x14ac:dyDescent="0.2">
+      <c r="L97" s="25" t="s">
+        <v>645</v>
+      </c>
+    </row>
+    <row r="98" spans="1:12" s="25" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A98" s="25" t="b">
         <v>1</v>
       </c>
@@ -20709,17 +20758,17 @@
       <c r="F98" s="25" t="s">
         <v>491</v>
       </c>
-      <c r="I98" s="25" t="s">
-        <v>645</v>
-      </c>
       <c r="J98" s="25" t="s">
         <v>645</v>
       </c>
       <c r="K98" s="25" t="s">
         <v>645</v>
       </c>
-    </row>
-    <row r="99" spans="1:11" s="25" customFormat="1" x14ac:dyDescent="0.2">
+      <c r="L98" s="25" t="s">
+        <v>645</v>
+      </c>
+    </row>
+    <row r="99" spans="1:12" s="25" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A99" s="25" t="b">
         <v>1</v>
       </c>
@@ -20738,17 +20787,17 @@
       <c r="F99" s="25" t="s">
         <v>492</v>
       </c>
-      <c r="I99" s="25" t="s">
-        <v>645</v>
-      </c>
       <c r="J99" s="25" t="s">
         <v>645</v>
       </c>
       <c r="K99" s="25" t="s">
         <v>645</v>
       </c>
-    </row>
-    <row r="100" spans="1:11" s="25" customFormat="1" x14ac:dyDescent="0.2">
+      <c r="L99" s="25" t="s">
+        <v>645</v>
+      </c>
+    </row>
+    <row r="100" spans="1:12" s="25" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A100" s="25" t="b">
         <v>1</v>
       </c>
@@ -20767,17 +20816,17 @@
       <c r="F100" s="25" t="s">
         <v>627</v>
       </c>
-      <c r="I100" s="25" t="s">
-        <v>645</v>
-      </c>
       <c r="J100" s="25" t="s">
         <v>645</v>
       </c>
       <c r="K100" s="25" t="s">
         <v>645</v>
       </c>
-    </row>
-    <row r="101" spans="1:11" s="25" customFormat="1" x14ac:dyDescent="0.2">
+      <c r="L100" s="25" t="s">
+        <v>645</v>
+      </c>
+    </row>
+    <row r="101" spans="1:12" s="25" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A101" s="25" t="b">
         <v>1</v>
       </c>
@@ -20796,17 +20845,17 @@
       <c r="F101" s="25" t="s">
         <v>492</v>
       </c>
-      <c r="I101" s="25" t="s">
-        <v>645</v>
-      </c>
       <c r="J101" s="25" t="s">
         <v>645</v>
       </c>
       <c r="K101" s="25" t="s">
         <v>645</v>
       </c>
-    </row>
-    <row r="102" spans="1:11" s="25" customFormat="1" x14ac:dyDescent="0.2">
+      <c r="L101" s="25" t="s">
+        <v>645</v>
+      </c>
+    </row>
+    <row r="102" spans="1:12" s="25" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A102" s="25" t="b">
         <v>1</v>
       </c>
@@ -20825,17 +20874,17 @@
       <c r="F102" s="25" t="s">
         <v>628</v>
       </c>
-      <c r="I102" s="25" t="s">
-        <v>645</v>
-      </c>
       <c r="J102" s="25" t="s">
         <v>645</v>
       </c>
       <c r="K102" s="25" t="s">
         <v>645</v>
       </c>
-    </row>
-    <row r="103" spans="1:11" s="25" customFormat="1" x14ac:dyDescent="0.2">
+      <c r="L102" s="25" t="s">
+        <v>645</v>
+      </c>
+    </row>
+    <row r="103" spans="1:12" s="25" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A103" s="25" t="b">
         <v>1</v>
       </c>
@@ -20854,17 +20903,17 @@
       <c r="F103" s="25" t="s">
         <v>493</v>
       </c>
-      <c r="I103" s="25" t="s">
-        <v>645</v>
-      </c>
       <c r="J103" s="25" t="s">
         <v>645</v>
       </c>
       <c r="K103" s="25" t="s">
         <v>645</v>
       </c>
-    </row>
-    <row r="104" spans="1:11" s="25" customFormat="1" x14ac:dyDescent="0.2">
+      <c r="L103" s="25" t="s">
+        <v>645</v>
+      </c>
+    </row>
+    <row r="104" spans="1:12" s="25" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A104" s="25" t="b">
         <v>1</v>
       </c>
@@ -20883,20 +20932,20 @@
       <c r="F104" s="25" t="s">
         <v>494</v>
       </c>
-      <c r="I104" s="25" t="s">
-        <v>645</v>
-      </c>
       <c r="J104" s="25" t="s">
         <v>645</v>
       </c>
       <c r="K104" s="25" t="s">
         <v>645</v>
       </c>
-    </row>
-    <row r="105" spans="1:11" s="25" customFormat="1" x14ac:dyDescent="0.2">
+      <c r="L104" s="25" t="s">
+        <v>645</v>
+      </c>
+    </row>
+    <row r="105" spans="1:12" s="25" customFormat="1" x14ac:dyDescent="0.2">
       <c r="D105" s="32"/>
     </row>
-    <row r="106" spans="1:11" s="25" customFormat="1" x14ac:dyDescent="0.2">
+    <row r="106" spans="1:12" s="25" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A106" s="25" t="b">
         <v>1</v>
       </c>
@@ -20918,17 +20967,17 @@
       <c r="H106" s="25" t="s">
         <v>846</v>
       </c>
-      <c r="I106" s="25" t="s">
-        <v>645</v>
-      </c>
       <c r="J106" s="25" t="s">
+        <v>645</v>
+      </c>
+      <c r="K106" s="25" t="s">
         <v>420</v>
       </c>
-      <c r="K106" s="25" t="s">
+      <c r="L106" s="25" t="s">
         <v>670</v>
       </c>
     </row>
-    <row r="107" spans="1:11" s="25" customFormat="1" x14ac:dyDescent="0.2">
+    <row r="107" spans="1:12" s="25" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A107" s="25" t="b">
         <v>1</v>
       </c>
@@ -20947,17 +20996,17 @@
       <c r="F107" s="25" t="s">
         <v>422</v>
       </c>
-      <c r="I107" s="25" t="s">
-        <v>645</v>
-      </c>
       <c r="J107" s="25" t="s">
         <v>645</v>
       </c>
       <c r="K107" s="25" t="s">
         <v>645</v>
       </c>
-    </row>
-    <row r="108" spans="1:11" s="25" customFormat="1" x14ac:dyDescent="0.2">
+      <c r="L107" s="25" t="s">
+        <v>645</v>
+      </c>
+    </row>
+    <row r="108" spans="1:12" s="25" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A108" s="25" t="b">
         <v>1</v>
       </c>
@@ -20976,17 +21025,17 @@
       <c r="F108" s="25" t="s">
         <v>423</v>
       </c>
-      <c r="I108" s="25" t="s">
-        <v>645</v>
-      </c>
       <c r="J108" s="25" t="s">
         <v>645</v>
       </c>
       <c r="K108" s="25" t="s">
         <v>645</v>
       </c>
-    </row>
-    <row r="109" spans="1:11" s="25" customFormat="1" x14ac:dyDescent="0.2">
+      <c r="L108" s="25" t="s">
+        <v>645</v>
+      </c>
+    </row>
+    <row r="109" spans="1:12" s="25" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A109" s="25" t="b">
         <v>1</v>
       </c>
@@ -21005,17 +21054,17 @@
       <c r="F109" s="25" t="s">
         <v>424</v>
       </c>
-      <c r="I109" s="25" t="s">
-        <v>645</v>
-      </c>
       <c r="J109" s="25" t="s">
         <v>645</v>
       </c>
       <c r="K109" s="25" t="s">
         <v>645</v>
       </c>
-    </row>
-    <row r="110" spans="1:11" s="25" customFormat="1" x14ac:dyDescent="0.2">
+      <c r="L109" s="25" t="s">
+        <v>645</v>
+      </c>
+    </row>
+    <row r="110" spans="1:12" s="25" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A110" s="25" t="b">
         <v>1</v>
       </c>
@@ -21031,13 +21080,13 @@
       <c r="E110" s="25" t="s">
         <v>151</v>
       </c>
-      <c r="I110" s="25" t="s">
-        <v>645</v>
-      </c>
       <c r="J110" s="25" t="s">
         <v>645</v>
       </c>
       <c r="K110" s="25" t="s">
+        <v>645</v>
+      </c>
+      <c r="L110" s="25" t="s">
         <v>645</v>
       </c>
     </row>
@@ -21048,7 +21097,7 @@
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{50F8335C-0B7A-174C-9395-80905662B1F5}">
-  <dimension ref="A1:P16"/>
+  <dimension ref="A1:Q16"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="10.5" bestFit="1" customWidth="1"/>
@@ -21058,17 +21107,17 @@
     <col min="5" max="5" width="19.1640625" bestFit="1" customWidth="1"/>
     <col min="6" max="6" width="12.1640625" bestFit="1" customWidth="1"/>
     <col min="7" max="7" width="15.83203125" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="31" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="27.5" bestFit="1" customWidth="1"/>
-    <col min="10" max="11" width="22.83203125" bestFit="1" customWidth="1"/>
-    <col min="12" max="12" width="20.1640625" bestFit="1" customWidth="1"/>
-    <col min="13" max="13" width="20.33203125" bestFit="1" customWidth="1"/>
-    <col min="14" max="14" width="22.33203125" bestFit="1" customWidth="1"/>
-    <col min="15" max="15" width="19.33203125" bestFit="1" customWidth="1"/>
-    <col min="16" max="16" width="12.5" bestFit="1" customWidth="1"/>
+    <col min="8" max="9" width="31" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="27.5" bestFit="1" customWidth="1"/>
+    <col min="11" max="12" width="22.83203125" bestFit="1" customWidth="1"/>
+    <col min="13" max="13" width="20.1640625" bestFit="1" customWidth="1"/>
+    <col min="14" max="14" width="20.33203125" bestFit="1" customWidth="1"/>
+    <col min="15" max="15" width="22.33203125" bestFit="1" customWidth="1"/>
+    <col min="16" max="16" width="19.33203125" bestFit="1" customWidth="1"/>
+    <col min="17" max="17" width="12.5" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:16" s="39" customFormat="1" ht="19" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:17" s="39" customFormat="1" ht="19" x14ac:dyDescent="0.25">
       <c r="A1" s="39" t="s">
         <v>666</v>
       </c>
@@ -21091,34 +21140,37 @@
         <v>682</v>
       </c>
       <c r="H1" s="39" t="s">
+        <v>989</v>
+      </c>
+      <c r="I1" s="39" t="s">
         <v>888</v>
       </c>
-      <c r="I1" s="40" t="s">
+      <c r="J1" s="40" t="s">
         <v>889</v>
       </c>
-      <c r="J1" s="40" t="s">
+      <c r="K1" s="40" t="s">
         <v>890</v>
       </c>
-      <c r="K1" s="40" t="s">
+      <c r="L1" s="40" t="s">
         <v>891</v>
       </c>
-      <c r="L1" s="40" t="s">
+      <c r="M1" s="40" t="s">
         <v>892</v>
       </c>
-      <c r="M1" s="40" t="s">
+      <c r="N1" s="40" t="s">
         <v>893</v>
       </c>
-      <c r="N1" s="40" t="s">
+      <c r="O1" s="40" t="s">
         <v>894</v>
       </c>
-      <c r="O1" s="40" t="s">
+      <c r="P1" s="40" t="s">
         <v>900</v>
       </c>
-      <c r="P1" s="39" t="s">
+      <c r="Q1" s="39" t="s">
         <v>848</v>
       </c>
     </row>
-    <row r="2" spans="1:16" x14ac:dyDescent="0.2">
+    <row r="2" spans="1:17" x14ac:dyDescent="0.2">
       <c r="A2" t="b">
         <v>1</v>
       </c>
@@ -21134,23 +21186,23 @@
       <c r="H2" t="s">
         <v>901</v>
       </c>
-      <c r="I2" t="s">
+      <c r="J2" t="s">
         <v>703</v>
       </c>
-      <c r="K2" t="s">
+      <c r="L2" t="s">
         <v>656</v>
       </c>
-      <c r="L2" t="s">
+      <c r="M2" t="s">
         <v>895</v>
       </c>
-      <c r="N2" t="s">
+      <c r="O2" t="s">
         <v>670</v>
       </c>
-      <c r="O2" t="s">
+      <c r="P2" t="s">
         <v>896</v>
       </c>
     </row>
-    <row r="3" spans="1:16" x14ac:dyDescent="0.2">
+    <row r="3" spans="1:17" x14ac:dyDescent="0.2">
       <c r="A3" t="b">
         <v>1</v>
       </c>
@@ -21166,23 +21218,23 @@
       <c r="H3" t="s">
         <v>902</v>
       </c>
-      <c r="I3" t="s">
+      <c r="J3" t="s">
         <v>703</v>
       </c>
-      <c r="K3" t="s">
+      <c r="L3" t="s">
         <v>670</v>
       </c>
-      <c r="L3" t="s">
+      <c r="M3" t="s">
         <v>895</v>
       </c>
-      <c r="N3" t="s">
+      <c r="O3" t="s">
         <v>649</v>
       </c>
-      <c r="O3" t="s">
+      <c r="P3" t="s">
         <v>896</v>
       </c>
     </row>
-    <row r="4" spans="1:16" x14ac:dyDescent="0.2">
+    <row r="4" spans="1:17" x14ac:dyDescent="0.2">
       <c r="A4" t="b">
         <v>1</v>
       </c>
@@ -21198,23 +21250,23 @@
       <c r="H4" t="s">
         <v>903</v>
       </c>
-      <c r="I4" t="s">
+      <c r="J4" t="s">
         <v>703</v>
       </c>
-      <c r="K4" t="s">
+      <c r="L4" t="s">
         <v>650</v>
       </c>
-      <c r="L4" t="s">
+      <c r="M4" t="s">
         <v>897</v>
       </c>
-      <c r="N4" t="s">
+      <c r="O4" t="s">
         <v>649</v>
       </c>
-      <c r="O4" t="s">
+      <c r="P4" t="s">
         <v>896</v>
       </c>
     </row>
-    <row r="5" spans="1:16" x14ac:dyDescent="0.2">
+    <row r="5" spans="1:17" x14ac:dyDescent="0.2">
       <c r="A5" t="b">
         <v>1</v>
       </c>
@@ -21230,23 +21282,23 @@
       <c r="H5" t="s">
         <v>904</v>
       </c>
-      <c r="I5" t="s">
+      <c r="J5" t="s">
         <v>703</v>
       </c>
-      <c r="K5" t="s">
+      <c r="L5" t="s">
         <v>649</v>
       </c>
-      <c r="L5" t="s">
+      <c r="M5" t="s">
         <v>895</v>
       </c>
-      <c r="N5" t="s">
+      <c r="O5" t="s">
         <v>671</v>
       </c>
-      <c r="O5" t="s">
+      <c r="P5" t="s">
         <v>896</v>
       </c>
     </row>
-    <row r="6" spans="1:16" x14ac:dyDescent="0.2">
+    <row r="6" spans="1:17" x14ac:dyDescent="0.2">
       <c r="A6" t="b">
         <v>1</v>
       </c>
@@ -21262,23 +21314,23 @@
       <c r="H6" t="s">
         <v>905</v>
       </c>
-      <c r="I6" t="s">
+      <c r="J6" t="s">
         <v>703</v>
       </c>
-      <c r="K6" t="s">
+      <c r="L6" t="s">
         <v>653</v>
       </c>
-      <c r="L6" t="s">
+      <c r="M6" t="s">
         <v>897</v>
       </c>
-      <c r="N6" t="s">
+      <c r="O6" t="s">
         <v>671</v>
       </c>
-      <c r="O6" t="s">
+      <c r="P6" t="s">
         <v>896</v>
       </c>
     </row>
-    <row r="7" spans="1:16" x14ac:dyDescent="0.2">
+    <row r="7" spans="1:17" x14ac:dyDescent="0.2">
       <c r="A7" t="b">
         <v>1</v>
       </c>
@@ -21294,23 +21346,23 @@
       <c r="H7" t="s">
         <v>906</v>
       </c>
-      <c r="I7" t="s">
+      <c r="J7" t="s">
         <v>703</v>
       </c>
-      <c r="K7" t="s">
+      <c r="L7" t="s">
         <v>671</v>
       </c>
-      <c r="L7" t="s">
+      <c r="M7" t="s">
         <v>895</v>
       </c>
-      <c r="N7" t="s">
+      <c r="O7" t="s">
         <v>651</v>
       </c>
-      <c r="O7" t="s">
+      <c r="P7" t="s">
         <v>896</v>
       </c>
     </row>
-    <row r="8" spans="1:16" x14ac:dyDescent="0.2">
+    <row r="8" spans="1:17" x14ac:dyDescent="0.2">
       <c r="A8" t="b">
         <v>1</v>
       </c>
@@ -21326,23 +21378,23 @@
       <c r="H8" t="s">
         <v>907</v>
       </c>
-      <c r="I8" t="s">
+      <c r="J8" t="s">
         <v>703</v>
       </c>
-      <c r="K8" t="s">
+      <c r="L8" t="s">
         <v>652</v>
       </c>
-      <c r="L8" t="s">
+      <c r="M8" t="s">
         <v>897</v>
       </c>
-      <c r="N8" t="s">
+      <c r="O8" t="s">
         <v>651</v>
       </c>
-      <c r="O8" t="s">
+      <c r="P8" t="s">
         <v>896</v>
       </c>
     </row>
-    <row r="9" spans="1:16" x14ac:dyDescent="0.2">
+    <row r="9" spans="1:17" x14ac:dyDescent="0.2">
       <c r="A9" t="b">
         <v>1</v>
       </c>
@@ -21358,23 +21410,23 @@
       <c r="H9" t="s">
         <v>908</v>
       </c>
-      <c r="I9" t="s">
+      <c r="J9" t="s">
         <v>703</v>
       </c>
-      <c r="K9" t="s">
+      <c r="L9" t="s">
         <v>651</v>
       </c>
-      <c r="L9" t="s">
+      <c r="M9" t="s">
         <v>895</v>
       </c>
-      <c r="N9" t="s">
+      <c r="O9" t="s">
         <v>672</v>
       </c>
-      <c r="O9" t="s">
+      <c r="P9" t="s">
         <v>896</v>
       </c>
     </row>
-    <row r="10" spans="1:16" x14ac:dyDescent="0.2">
+    <row r="10" spans="1:17" x14ac:dyDescent="0.2">
       <c r="A10" t="b">
         <v>1</v>
       </c>
@@ -21390,23 +21442,23 @@
       <c r="H10" t="s">
         <v>909</v>
       </c>
-      <c r="I10" t="s">
+      <c r="J10" t="s">
         <v>703</v>
       </c>
-      <c r="K10" t="s">
+      <c r="L10" t="s">
         <v>654</v>
       </c>
-      <c r="L10" t="s">
+      <c r="M10" t="s">
         <v>897</v>
       </c>
-      <c r="N10" t="s">
+      <c r="O10" t="s">
         <v>672</v>
       </c>
-      <c r="O10" t="s">
+      <c r="P10" t="s">
         <v>896</v>
       </c>
     </row>
-    <row r="11" spans="1:16" x14ac:dyDescent="0.2">
+    <row r="11" spans="1:17" x14ac:dyDescent="0.2">
       <c r="A11" t="b">
         <v>1</v>
       </c>
@@ -21422,23 +21474,23 @@
       <c r="H11" t="s">
         <v>910</v>
       </c>
-      <c r="I11" t="s">
+      <c r="J11" t="s">
         <v>703</v>
       </c>
-      <c r="K11" t="s">
+      <c r="L11" t="s">
         <v>673</v>
       </c>
-      <c r="L11" t="s">
+      <c r="M11" t="s">
         <v>897</v>
       </c>
-      <c r="N11" t="s">
+      <c r="O11" t="s">
         <v>654</v>
       </c>
-      <c r="O11" t="s">
+      <c r="P11" t="s">
         <v>896</v>
       </c>
     </row>
-    <row r="12" spans="1:16" x14ac:dyDescent="0.2">
+    <row r="12" spans="1:17" x14ac:dyDescent="0.2">
       <c r="A12" t="b">
         <v>1</v>
       </c>
@@ -21454,23 +21506,23 @@
       <c r="H12" t="s">
         <v>911</v>
       </c>
-      <c r="I12" t="s">
+      <c r="J12" t="s">
         <v>703</v>
       </c>
-      <c r="K12" t="s">
+      <c r="L12" t="s">
         <v>674</v>
       </c>
-      <c r="L12" t="s">
+      <c r="M12" t="s">
         <v>897</v>
       </c>
-      <c r="N12" t="s">
+      <c r="O12" t="s">
         <v>654</v>
       </c>
-      <c r="O12" t="s">
+      <c r="P12" t="s">
         <v>896</v>
       </c>
     </row>
-    <row r="13" spans="1:16" x14ac:dyDescent="0.2">
+    <row r="13" spans="1:17" x14ac:dyDescent="0.2">
       <c r="A13" t="b">
         <v>1</v>
       </c>
@@ -21486,23 +21538,23 @@
       <c r="H13" t="s">
         <v>912</v>
       </c>
-      <c r="I13" t="s">
+      <c r="J13" t="s">
         <v>703</v>
       </c>
-      <c r="K13" t="s">
+      <c r="L13" t="s">
         <v>672</v>
       </c>
-      <c r="L13" t="s">
+      <c r="M13" t="s">
         <v>895</v>
       </c>
-      <c r="N13" t="s">
+      <c r="O13" t="s">
         <v>675</v>
       </c>
-      <c r="O13" t="s">
+      <c r="P13" t="s">
         <v>896</v>
       </c>
     </row>
-    <row r="14" spans="1:16" x14ac:dyDescent="0.2">
+    <row r="14" spans="1:17" x14ac:dyDescent="0.2">
       <c r="A14" t="b">
         <v>1</v>
       </c>
@@ -21518,23 +21570,23 @@
       <c r="H14" t="s">
         <v>913</v>
       </c>
-      <c r="I14" t="s">
+      <c r="J14" t="s">
         <v>703</v>
       </c>
-      <c r="K14" t="s">
+      <c r="L14" t="s">
         <v>676</v>
       </c>
-      <c r="L14" t="s">
+      <c r="M14" t="s">
         <v>897</v>
       </c>
-      <c r="N14" t="s">
+      <c r="O14" t="s">
         <v>675</v>
       </c>
-      <c r="O14" t="s">
+      <c r="P14" t="s">
         <v>896</v>
       </c>
     </row>
-    <row r="15" spans="1:16" x14ac:dyDescent="0.2">
+    <row r="15" spans="1:17" x14ac:dyDescent="0.2">
       <c r="A15" t="b">
         <v>1</v>
       </c>
@@ -21550,23 +21602,23 @@
       <c r="H15" t="s">
         <v>914</v>
       </c>
-      <c r="I15" t="s">
+      <c r="J15" t="s">
         <v>703</v>
       </c>
-      <c r="K15" t="s">
+      <c r="L15" t="s">
         <v>899</v>
       </c>
-      <c r="L15" t="s">
+      <c r="M15" t="s">
         <v>897</v>
       </c>
-      <c r="N15" t="s">
+      <c r="O15" t="s">
         <v>675</v>
       </c>
-      <c r="O15" t="s">
+      <c r="P15" t="s">
         <v>896</v>
       </c>
     </row>
-    <row r="16" spans="1:16" x14ac:dyDescent="0.2">
+    <row r="16" spans="1:17" x14ac:dyDescent="0.2">
       <c r="A16" t="b">
         <v>1</v>
       </c>
@@ -21582,19 +21634,19 @@
       <c r="H16" t="s">
         <v>915</v>
       </c>
-      <c r="I16" t="s">
+      <c r="J16" t="s">
         <v>703</v>
       </c>
-      <c r="K16" t="s">
+      <c r="L16" t="s">
         <v>677</v>
       </c>
-      <c r="L16" t="s">
+      <c r="M16" t="s">
         <v>897</v>
       </c>
-      <c r="N16" t="s">
+      <c r="O16" t="s">
         <v>675</v>
       </c>
-      <c r="O16" t="s">
+      <c r="P16" t="s">
         <v>896</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Proper populationg of collNum in NWSS to ODM v2
</commit_message>
<xml_diff>
--- a/data/mapping_config_files/nwss_to_odm_v2_mapping.xlsx
+++ b/data/mapping_config_files/nwss_to_odm_v2_mapping.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/martinwellman/Documents/Health/Wastewater/PHES-ODM-MapGenerator/PHES-ODM-MapGenerator/data/mapping_config_files/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{AF19414E-9634-6646-B493-D7A48471653E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F3797779-CD3D-804A-A607-35746DC2EBA1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="500" windowWidth="40960" windowHeight="20860" xr2:uid="{77810E24-F86B-BC44-A0D5-8790E6EC60B4}"/>
   </bookViews>
@@ -53,7 +53,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3273" uniqueCount="992">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3272" uniqueCount="993">
   <si>
     <t>Reporter</t>
   </si>
@@ -3076,6 +3076,12 @@
   </si>
   <si>
     <t>The ID generator will convert this into a valid date/time/timezone string</t>
+  </si>
+  <si>
+    <t>if str(src.sample_type).endswith("time-weighted composite") and (src.composite_freq == "" or src.composite_freq is None):
+    target = 24
+else:
+    target = src.composite_freq</t>
   </si>
 </sst>
 </file>
@@ -3270,7 +3276,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="42">
+  <cellXfs count="46">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1"/>
@@ -3339,10 +3345,22 @@
     <xf numFmtId="0" fontId="4" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="13" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="6" fillId="6" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top"/>
+    </xf>
     <xf numFmtId="0" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment wrapText="1"/>
+      <alignment vertical="top"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="6" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" xfId="0" quotePrefix="1" applyFont="1" applyAlignment="1">
+      <alignment vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment vertical="top"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -14519,7 +14537,8 @@
     <col min="5" max="5" width="13" bestFit="1" customWidth="1"/>
     <col min="6" max="6" width="15.83203125" bestFit="1" customWidth="1"/>
     <col min="7" max="7" width="23.1640625" bestFit="1" customWidth="1"/>
-    <col min="8" max="9" width="20" customWidth="1"/>
+    <col min="8" max="8" width="20" style="43" customWidth="1"/>
+    <col min="9" max="9" width="20" customWidth="1"/>
     <col min="10" max="10" width="28.6640625" customWidth="1"/>
     <col min="11" max="11" width="47.6640625" customWidth="1"/>
   </cols>
@@ -14546,7 +14565,7 @@
       <c r="G1" s="37" t="s">
         <v>635</v>
       </c>
-      <c r="H1" s="37" t="s">
+      <c r="H1" s="41" t="s">
         <v>805</v>
       </c>
       <c r="I1" s="37" t="s">
@@ -14575,6 +14594,7 @@
       <c r="G2" s="25" t="s">
         <v>695</v>
       </c>
+      <c r="H2" s="42"/>
     </row>
     <row r="3" spans="1:10" s="25" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A3" s="25" t="b">
@@ -14595,6 +14615,7 @@
       <c r="G3" s="25" t="s">
         <v>701</v>
       </c>
+      <c r="H3" s="42"/>
     </row>
     <row r="4" spans="1:10" s="25" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A4" s="25" t="b">
@@ -14612,11 +14633,14 @@
       <c r="F4" s="25" t="s">
         <v>729</v>
       </c>
+      <c r="H4" s="42"/>
       <c r="J4" s="25" t="s">
         <v>875</v>
       </c>
     </row>
-    <row r="5" spans="1:10" s="25" customFormat="1" x14ac:dyDescent="0.2"/>
+    <row r="5" spans="1:10" s="25" customFormat="1" x14ac:dyDescent="0.2">
+      <c r="H5" s="42"/>
+    </row>
     <row r="6" spans="1:10" s="25" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A6" s="25" t="b">
         <v>1</v>
@@ -14636,6 +14660,7 @@
       <c r="G6" s="25" t="s">
         <v>693</v>
       </c>
+      <c r="H6" s="42"/>
     </row>
     <row r="7" spans="1:10" s="25" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A7" s="25" t="b">
@@ -14657,6 +14682,7 @@
       <c r="G7" s="26" t="s">
         <v>701</v>
       </c>
+      <c r="H7" s="42"/>
     </row>
     <row r="8" spans="1:10" s="25" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A8" s="25" t="b">
@@ -14677,6 +14703,7 @@
       <c r="G8" s="25" t="s">
         <v>701</v>
       </c>
+      <c r="H8" s="42"/>
     </row>
     <row r="9" spans="1:10" s="25" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A9" s="25" t="b">
@@ -14691,6 +14718,7 @@
       <c r="F9" s="25" t="s">
         <v>878</v>
       </c>
+      <c r="H9" s="42"/>
     </row>
     <row r="10" spans="1:10" s="25" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A10" s="25" t="b">
@@ -14705,6 +14733,7 @@
       <c r="F10" s="25" t="s">
         <v>879</v>
       </c>
+      <c r="H10" s="42"/>
     </row>
     <row r="11" spans="1:10" s="25" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A11" s="25" t="b">
@@ -14719,6 +14748,7 @@
       <c r="F11" s="25" t="s">
         <v>880</v>
       </c>
+      <c r="H11" s="42"/>
     </row>
     <row r="12" spans="1:10" s="25" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A12" s="25" t="b">
@@ -14733,6 +14763,7 @@
       <c r="F12" s="25" t="s">
         <v>881</v>
       </c>
+      <c r="H12" s="42"/>
     </row>
     <row r="13" spans="1:10" s="25" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A13" s="25" t="b">
@@ -14747,6 +14778,7 @@
       <c r="F13" s="25" t="s">
         <v>882</v>
       </c>
+      <c r="H13" s="42"/>
     </row>
     <row r="14" spans="1:10" s="25" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A14" s="25" t="b">
@@ -14761,6 +14793,7 @@
       <c r="F14" s="25" t="s">
         <v>874</v>
       </c>
+      <c r="H14" s="42"/>
     </row>
     <row r="15" spans="1:10" s="25" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A15" s="25" t="b">
@@ -14775,8 +14808,11 @@
       <c r="F15" s="25" t="s">
         <v>120</v>
       </c>
-    </row>
-    <row r="16" spans="1:10" s="25" customFormat="1" x14ac:dyDescent="0.2"/>
+      <c r="H15" s="42"/>
+    </row>
+    <row r="16" spans="1:10" s="25" customFormat="1" x14ac:dyDescent="0.2">
+      <c r="H16" s="42"/>
+    </row>
     <row r="17" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A17" s="25" t="b">
         <v>1</v>
@@ -14847,6 +14883,7 @@
       <c r="G20" s="25" t="s">
         <v>693</v>
       </c>
+      <c r="H20" s="42"/>
     </row>
     <row r="21" spans="1:11" s="25" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A21" s="25" t="b">
@@ -14864,6 +14901,7 @@
       <c r="F21" s="25" t="s">
         <v>735</v>
       </c>
+      <c r="H21" s="42"/>
       <c r="J21" s="25" t="s">
         <v>877</v>
       </c>
@@ -14887,8 +14925,11 @@
       <c r="G22" s="25" t="s">
         <v>701</v>
       </c>
-    </row>
-    <row r="23" spans="1:11" s="25" customFormat="1" x14ac:dyDescent="0.2"/>
+      <c r="H22" s="42"/>
+    </row>
+    <row r="23" spans="1:11" s="25" customFormat="1" x14ac:dyDescent="0.2">
+      <c r="H23" s="42"/>
+    </row>
     <row r="24" spans="1:11" s="25" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A24" s="25" t="b">
         <v>1</v>
@@ -14909,6 +14950,7 @@
       <c r="G24" s="26" t="s">
         <v>701</v>
       </c>
+      <c r="H24" s="42"/>
     </row>
     <row r="25" spans="1:11" s="25" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A25" s="25" t="b">
@@ -14929,6 +14971,7 @@
       <c r="G25" s="25" t="s">
         <v>876</v>
       </c>
+      <c r="H25" s="42"/>
     </row>
     <row r="26" spans="1:11" s="25" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A26" s="25" t="b">
@@ -14949,6 +14992,7 @@
       <c r="G26" s="25" t="s">
         <v>701</v>
       </c>
+      <c r="H26" s="42"/>
     </row>
     <row r="27" spans="1:11" s="25" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A27" s="25" t="b">
@@ -14969,6 +15013,7 @@
       <c r="G27" s="25" t="s">
         <v>703</v>
       </c>
+      <c r="H27" s="42"/>
     </row>
     <row r="28" spans="1:11" s="25" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A28" s="25" t="b">
@@ -14989,6 +15034,7 @@
       <c r="G28" s="25" t="s">
         <v>693</v>
       </c>
+      <c r="H28" s="42"/>
       <c r="K28" s="17"/>
     </row>
     <row r="29" spans="1:11" s="25" customFormat="1" x14ac:dyDescent="0.2">
@@ -15010,6 +15056,7 @@
       <c r="G29" s="25" t="s">
         <v>700</v>
       </c>
+      <c r="H29" s="42"/>
     </row>
     <row r="30" spans="1:11" s="25" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A30" s="25" t="b">
@@ -15030,6 +15077,7 @@
       <c r="G30" s="25" t="s">
         <v>702</v>
       </c>
+      <c r="H30" s="42"/>
     </row>
     <row r="31" spans="1:11" s="25" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A31" s="25" t="b">
@@ -15044,7 +15092,7 @@
       <c r="F31" s="25" t="s">
         <v>866</v>
       </c>
-      <c r="H31" s="28" t="s">
+      <c r="H31" s="44" t="s">
         <v>867</v>
       </c>
     </row>
@@ -15064,12 +15112,13 @@
       <c r="F32" s="25" t="s">
         <v>727</v>
       </c>
+      <c r="H32" s="42"/>
       <c r="J32" s="25" t="s">
         <v>985</v>
       </c>
     </row>
     <row r="33" spans="1:10" s="25" customFormat="1" x14ac:dyDescent="0.2">
-      <c r="H33" s="28"/>
+      <c r="H33" s="44"/>
     </row>
     <row r="34" spans="1:10" s="25" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A34" s="25" t="b">
@@ -15090,7 +15139,7 @@
       <c r="G34" s="25" t="s">
         <v>876</v>
       </c>
-      <c r="H34" s="28"/>
+      <c r="H34" s="44"/>
     </row>
     <row r="35" spans="1:10" s="25" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A35" s="25" t="b">
@@ -15111,7 +15160,7 @@
       <c r="G35" s="25" t="s">
         <v>703</v>
       </c>
-      <c r="H35" s="28"/>
+      <c r="H35" s="44"/>
     </row>
     <row r="36" spans="1:10" s="25" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A36" s="25" t="b">
@@ -15132,7 +15181,7 @@
       <c r="G36" s="25" t="s">
         <v>701</v>
       </c>
-      <c r="H36" s="28"/>
+      <c r="H36" s="44"/>
     </row>
     <row r="37" spans="1:10" s="25" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A37" s="25" t="b">
@@ -15153,10 +15202,10 @@
       <c r="G37" s="25" t="s">
         <v>693</v>
       </c>
-      <c r="H37" s="28"/>
+      <c r="H37" s="44"/>
     </row>
     <row r="38" spans="1:10" s="25" customFormat="1" x14ac:dyDescent="0.2">
-      <c r="H38" s="28"/>
+      <c r="H38" s="44"/>
     </row>
     <row r="39" spans="1:10" s="25" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A39" s="25" t="b">
@@ -15177,6 +15226,7 @@
       <c r="G39" s="25" t="s">
         <v>701</v>
       </c>
+      <c r="H39" s="42"/>
     </row>
     <row r="40" spans="1:10" s="25" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A40" s="25" t="b">
@@ -15191,6 +15241,7 @@
       <c r="F40" s="25" t="s">
         <v>115</v>
       </c>
+      <c r="H40" s="42"/>
     </row>
     <row r="41" spans="1:10" s="25" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A41" s="25" t="b">
@@ -15205,6 +15256,7 @@
       <c r="F41" s="25" t="s">
         <v>870</v>
       </c>
+      <c r="H41" s="42"/>
     </row>
     <row r="42" spans="1:10" s="25" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A42" s="25" t="b">
@@ -15222,6 +15274,7 @@
       <c r="F42" s="25" t="s">
         <v>729</v>
       </c>
+      <c r="H42" s="42"/>
       <c r="J42" s="25" t="s">
         <v>875</v>
       </c>
@@ -15246,6 +15299,7 @@
       <c r="G43" s="26" t="s">
         <v>701</v>
       </c>
+      <c r="H43" s="42"/>
     </row>
     <row r="44" spans="1:10" s="25" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A44" s="25" t="b">
@@ -15260,6 +15314,7 @@
       <c r="F44" s="25" t="s">
         <v>871</v>
       </c>
+      <c r="H44" s="42"/>
     </row>
     <row r="45" spans="1:10" s="25" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A45" s="25" t="b">
@@ -15274,6 +15329,7 @@
       <c r="F45" s="25" t="s">
         <v>872</v>
       </c>
+      <c r="H45" s="42"/>
     </row>
     <row r="46" spans="1:10" s="25" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A46" s="25" t="b">
@@ -15288,6 +15344,7 @@
       <c r="F46" s="25" t="s">
         <v>873</v>
       </c>
+      <c r="H46" s="42"/>
     </row>
     <row r="47" spans="1:10" s="25" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A47" s="25" t="b">
@@ -15302,6 +15359,7 @@
       <c r="F47" s="25" t="s">
         <v>874</v>
       </c>
+      <c r="H47" s="42"/>
     </row>
     <row r="48" spans="1:10" s="25" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A48" s="25" t="b">
@@ -15316,8 +15374,11 @@
       <c r="F48" s="25" t="s">
         <v>120</v>
       </c>
-    </row>
-    <row r="49" spans="1:11" s="25" customFormat="1" x14ac:dyDescent="0.2"/>
+      <c r="H48" s="42"/>
+    </row>
+    <row r="49" spans="1:11" s="25" customFormat="1" x14ac:dyDescent="0.2">
+      <c r="H49" s="42"/>
+    </row>
     <row r="50" spans="1:11" s="25" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A50" s="25" t="b">
         <v>0</v>
@@ -15334,6 +15395,7 @@
       <c r="F50" s="25" t="s">
         <v>727</v>
       </c>
+      <c r="H50" s="42"/>
       <c r="J50" s="25" t="s">
         <v>985</v>
       </c>
@@ -15358,6 +15420,7 @@
       <c r="G51" s="26" t="s">
         <v>701</v>
       </c>
+      <c r="H51" s="42"/>
     </row>
     <row r="52" spans="1:11" s="25" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A52" s="25" t="b">
@@ -15378,6 +15441,7 @@
       <c r="G52" s="25" t="s">
         <v>701</v>
       </c>
+      <c r="H52" s="42"/>
     </row>
     <row r="53" spans="1:11" s="25" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A53" s="25" t="b">
@@ -15398,8 +15462,11 @@
       <c r="G53" s="25" t="s">
         <v>693</v>
       </c>
-    </row>
-    <row r="54" spans="1:11" s="25" customFormat="1" x14ac:dyDescent="0.2"/>
+      <c r="H53" s="42"/>
+    </row>
+    <row r="54" spans="1:11" s="25" customFormat="1" x14ac:dyDescent="0.2">
+      <c r="H54" s="42"/>
+    </row>
     <row r="55" spans="1:11" s="25" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A55" s="25" t="b">
         <v>1</v>
@@ -15420,6 +15487,7 @@
       <c r="G55" s="26" t="s">
         <v>701</v>
       </c>
+      <c r="H55" s="42"/>
     </row>
     <row r="56" spans="1:11" s="25" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A56" s="25" t="b">
@@ -15440,6 +15508,7 @@
       <c r="G56" s="25" t="s">
         <v>701</v>
       </c>
+      <c r="H56" s="42"/>
     </row>
     <row r="57" spans="1:11" s="25" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A57" s="25" t="b">
@@ -15460,6 +15529,7 @@
       <c r="G57" s="25" t="s">
         <v>703</v>
       </c>
+      <c r="H57" s="42"/>
     </row>
     <row r="58" spans="1:11" s="25" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A58" s="25" t="b">
@@ -15480,6 +15550,7 @@
       <c r="G58" s="25" t="s">
         <v>704</v>
       </c>
+      <c r="H58" s="42"/>
       <c r="K58" s="17"/>
     </row>
     <row r="59" spans="1:11" s="25" customFormat="1" x14ac:dyDescent="0.2">
@@ -15501,9 +15572,12 @@
       <c r="G59" s="25" t="s">
         <v>693</v>
       </c>
+      <c r="H59" s="42"/>
       <c r="K59" s="17"/>
     </row>
-    <row r="60" spans="1:11" s="25" customFormat="1" x14ac:dyDescent="0.2"/>
+    <row r="60" spans="1:11" s="25" customFormat="1" x14ac:dyDescent="0.2">
+      <c r="H60" s="42"/>
+    </row>
     <row r="61" spans="1:11" s="25" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A61" s="25" t="b">
         <v>1</v>
@@ -15523,6 +15597,7 @@
       <c r="G61" s="25" t="s">
         <v>693</v>
       </c>
+      <c r="H61" s="42"/>
     </row>
     <row r="62" spans="1:11" s="25" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A62" s="25" t="b">
@@ -15543,6 +15618,7 @@
       <c r="G62" s="25" t="s">
         <v>701</v>
       </c>
+      <c r="H62" s="42"/>
     </row>
     <row r="63" spans="1:11" s="25" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A63" s="25" t="b">
@@ -15560,11 +15636,14 @@
       <c r="F63" s="25" t="s">
         <v>735</v>
       </c>
+      <c r="H63" s="42"/>
       <c r="J63" s="25" t="s">
         <v>877</v>
       </c>
     </row>
-    <row r="64" spans="1:11" s="25" customFormat="1" x14ac:dyDescent="0.2"/>
+    <row r="64" spans="1:11" s="25" customFormat="1" x14ac:dyDescent="0.2">
+      <c r="H64" s="42"/>
+    </row>
     <row r="65" spans="1:11" s="25" customFormat="1" ht="16" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A65" s="25" t="b">
         <v>1</v>
@@ -15602,15 +15681,12 @@
         <v>692</v>
       </c>
     </row>
-    <row r="67" spans="1:11" s="25" customFormat="1" x14ac:dyDescent="0.2">
+    <row r="67" spans="1:11" s="25" customFormat="1" ht="16" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A67" s="25" t="b">
         <v>1</v>
       </c>
       <c r="B67" s="25" t="s">
         <v>630</v>
-      </c>
-      <c r="C67" s="25" t="s">
-        <v>23</v>
       </c>
       <c r="D67" s="30"/>
       <c r="E67" s="25" t="s">
@@ -15619,8 +15695,8 @@
       <c r="F67" s="25" t="s">
         <v>119</v>
       </c>
-      <c r="G67" s="25" t="s">
-        <v>699</v>
+      <c r="H67" s="29" t="s">
+        <v>992</v>
       </c>
     </row>
     <row r="68" spans="1:11" s="25" customFormat="1" ht="17" customHeight="1" x14ac:dyDescent="0.2">
@@ -15637,7 +15713,7 @@
       <c r="F68" s="25" t="s">
         <v>137</v>
       </c>
-      <c r="H68" s="40" t="s">
+      <c r="H68" s="29" t="s">
         <v>990</v>
       </c>
       <c r="J68" s="25" t="s">
@@ -15660,7 +15736,7 @@
       <c r="F69" s="25" t="s">
         <v>144</v>
       </c>
-      <c r="H69" s="25" t="s">
+      <c r="H69" s="42" t="s">
         <v>921</v>
       </c>
     </row>
@@ -15683,6 +15759,7 @@
       <c r="G70" s="25" t="s">
         <v>701</v>
       </c>
+      <c r="H70" s="42"/>
     </row>
     <row r="71" spans="1:11" s="25" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A71" s="25" t="b">
@@ -15703,6 +15780,7 @@
       <c r="G71" s="25" t="s">
         <v>693</v>
       </c>
+      <c r="H71" s="42"/>
       <c r="K71" s="17"/>
     </row>
     <row r="72" spans="1:11" s="25" customFormat="1" x14ac:dyDescent="0.2">
@@ -15724,6 +15802,7 @@
       <c r="G72" s="25" t="s">
         <v>700</v>
       </c>
+      <c r="H72" s="42"/>
     </row>
     <row r="73" spans="1:11" s="25" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A73" s="25" t="b">
@@ -15744,6 +15823,7 @@
       <c r="G73" s="25" t="s">
         <v>694</v>
       </c>
+      <c r="H73" s="42"/>
     </row>
     <row r="74" spans="1:11" s="25" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A74" s="25" t="b">
@@ -15764,8 +15844,11 @@
       <c r="G74" s="25" t="s">
         <v>703</v>
       </c>
-    </row>
-    <row r="75" spans="1:11" s="25" customFormat="1" x14ac:dyDescent="0.2"/>
+      <c r="H74" s="42"/>
+    </row>
+    <row r="75" spans="1:11" s="25" customFormat="1" x14ac:dyDescent="0.2">
+      <c r="H75" s="42"/>
+    </row>
     <row r="76" spans="1:11" s="25" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A76" s="25" t="b">
         <v>1</v>
@@ -15786,6 +15869,7 @@
       <c r="G76" s="26" t="s">
         <v>701</v>
       </c>
+      <c r="H76" s="42"/>
     </row>
     <row r="77" spans="1:11" s="25" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A77" s="25" t="b">
@@ -15809,6 +15893,7 @@
       <c r="G77" s="25" t="s">
         <v>136</v>
       </c>
+      <c r="H77" s="42"/>
     </row>
     <row r="78" spans="1:11" s="25" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A78" s="25" t="b">
@@ -15832,6 +15917,7 @@
       <c r="G78" s="25" t="s">
         <v>134</v>
       </c>
+      <c r="H78" s="42"/>
     </row>
     <row r="79" spans="1:11" s="25" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A79" s="25" t="b">
@@ -15855,6 +15941,7 @@
       <c r="G79" s="25" t="s">
         <v>130</v>
       </c>
+      <c r="H79" s="42"/>
     </row>
     <row r="80" spans="1:11" s="25" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A80" s="25" t="b">
@@ -15878,6 +15965,7 @@
       <c r="G80" s="25" t="s">
         <v>131</v>
       </c>
+      <c r="H80" s="42"/>
     </row>
     <row r="81" spans="1:10" s="25" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A81" s="25" t="b">
@@ -15901,6 +15989,7 @@
       <c r="G81" s="25" t="s">
         <v>132</v>
       </c>
+      <c r="H81" s="42"/>
     </row>
     <row r="82" spans="1:10" s="25" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A82" s="25" t="b">
@@ -15924,6 +16013,7 @@
       <c r="G82" s="25" t="s">
         <v>133</v>
       </c>
+      <c r="H82" s="42"/>
     </row>
     <row r="83" spans="1:10" s="25" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A83" s="25" t="b">
@@ -15947,6 +16037,7 @@
       <c r="G83" s="25" t="s">
         <v>127</v>
       </c>
+      <c r="H83" s="42"/>
     </row>
     <row r="84" spans="1:10" s="25" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A84" s="25" t="b">
@@ -15970,9 +16061,11 @@
       <c r="G84" s="25" t="s">
         <v>135</v>
       </c>
+      <c r="H84" s="42"/>
     </row>
     <row r="85" spans="1:10" s="25" customFormat="1" x14ac:dyDescent="0.2">
       <c r="D85" s="30"/>
+      <c r="H85" s="42"/>
     </row>
     <row r="86" spans="1:10" s="25" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A86" s="25" t="b">
@@ -15990,7 +16083,7 @@
       <c r="F86" s="39" t="s">
         <v>120</v>
       </c>
-      <c r="H86" s="28" t="s">
+      <c r="H86" s="44" t="s">
         <v>722</v>
       </c>
     </row>
@@ -16013,6 +16106,7 @@
       <c r="G87" s="25" t="s">
         <v>696</v>
       </c>
+      <c r="H87" s="42"/>
     </row>
     <row r="88" spans="1:10" s="25" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A88" s="25" t="b">
@@ -16033,6 +16127,7 @@
       <c r="G88" s="25" t="s">
         <v>694</v>
       </c>
+      <c r="H88" s="42"/>
     </row>
     <row r="89" spans="1:10" s="25" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A89" s="25" t="b">
@@ -16053,6 +16148,7 @@
       <c r="G89" s="25" t="s">
         <v>701</v>
       </c>
+      <c r="H89" s="42"/>
     </row>
     <row r="90" spans="1:10" s="25" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A90" s="25" t="b">
@@ -16073,6 +16169,7 @@
       <c r="G90" s="25" t="s">
         <v>697</v>
       </c>
+      <c r="H90" s="42"/>
     </row>
     <row r="91" spans="1:10" s="25" customFormat="1" ht="17" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A91" s="25" t="b">
@@ -16091,7 +16188,7 @@
       <c r="F91" s="25" t="s">
         <v>83</v>
       </c>
-      <c r="H91" s="40" t="s">
+      <c r="H91" s="29" t="s">
         <v>862</v>
       </c>
     </row>
@@ -16115,6 +16212,7 @@
       <c r="G92" s="26" t="s">
         <v>701</v>
       </c>
+      <c r="H92" s="42"/>
     </row>
     <row r="93" spans="1:10" s="25" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A93" s="25" t="b">
@@ -16132,6 +16230,7 @@
       <c r="F93" s="25" t="s">
         <v>729</v>
       </c>
+      <c r="H93" s="42"/>
       <c r="J93" s="25" t="s">
         <v>875</v>
       </c>
@@ -16155,6 +16254,7 @@
       <c r="G94" s="25" t="s">
         <v>701</v>
       </c>
+      <c r="H94" s="42"/>
     </row>
     <row r="95" spans="1:10" s="25" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A95" s="25" t="b">
@@ -16175,6 +16275,7 @@
       <c r="G95" s="25" t="s">
         <v>693</v>
       </c>
+      <c r="H95" s="42"/>
     </row>
     <row r="96" spans="1:10" s="25" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A96" s="25" t="b">
@@ -16192,6 +16293,7 @@
       <c r="F96" s="25" t="s">
         <v>727</v>
       </c>
+      <c r="H96" s="42"/>
       <c r="J96" s="25" t="s">
         <v>985</v>
       </c>
@@ -16218,7 +16320,7 @@
       <c r="G97" s="25" t="s">
         <v>75</v>
       </c>
-      <c r="H97" s="25"/>
+      <c r="H97" s="42"/>
       <c r="I97" s="25"/>
       <c r="J97" s="25"/>
     </row>
@@ -16244,6 +16346,7 @@
       <c r="G98" s="25" t="s">
         <v>101</v>
       </c>
+      <c r="H98" s="42"/>
     </row>
     <row r="99" spans="1:11" s="25" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A99" s="25" t="b">
@@ -16267,6 +16370,7 @@
       <c r="G99" s="25" t="s">
         <v>102</v>
       </c>
+      <c r="H99" s="42"/>
     </row>
     <row r="100" spans="1:11" s="25" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A100" s="25" t="b">
@@ -16290,6 +16394,7 @@
       <c r="G100" s="25" t="s">
         <v>103</v>
       </c>
+      <c r="H100" s="42"/>
     </row>
     <row r="101" spans="1:11" s="25" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A101" s="25" t="b">
@@ -16313,6 +16418,7 @@
       <c r="G101" s="25" t="s">
         <v>104</v>
       </c>
+      <c r="H101" s="42"/>
     </row>
     <row r="102" spans="1:11" s="25" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A102" s="25" t="b">
@@ -16336,6 +16442,7 @@
       <c r="G102" s="25" t="s">
         <v>113</v>
       </c>
+      <c r="H102" s="42"/>
     </row>
     <row r="103" spans="1:11" s="25" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A103" s="25" t="b">
@@ -16359,6 +16466,7 @@
       <c r="G103" s="25" t="s">
         <v>112</v>
       </c>
+      <c r="H103" s="42"/>
     </row>
     <row r="104" spans="1:11" s="25" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A104" s="25" t="b">
@@ -16382,6 +16490,7 @@
       <c r="G104" s="25" t="s">
         <v>109</v>
       </c>
+      <c r="H104" s="42"/>
     </row>
     <row r="105" spans="1:11" s="25" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A105" s="25" t="b">
@@ -16405,6 +16514,7 @@
       <c r="G105" s="25" t="s">
         <v>108</v>
       </c>
+      <c r="H105" s="42"/>
     </row>
     <row r="106" spans="1:11" s="25" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A106" s="25" t="b">
@@ -16428,6 +16538,7 @@
       <c r="G106" s="25" t="s">
         <v>107</v>
       </c>
+      <c r="H106" s="42"/>
     </row>
     <row r="107" spans="1:11" s="25" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A107" s="25" t="b">
@@ -16451,6 +16562,7 @@
       <c r="G107" s="25" t="s">
         <v>106</v>
       </c>
+      <c r="H107" s="42"/>
     </row>
     <row r="108" spans="1:11" s="25" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A108" s="25" t="b">
@@ -16474,6 +16586,7 @@
       <c r="G108" s="25" t="s">
         <v>105</v>
       </c>
+      <c r="H108" s="42"/>
     </row>
     <row r="109" spans="1:11" s="25" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A109" s="25" t="b">
@@ -16497,6 +16610,7 @@
       <c r="G109" s="25" t="s">
         <v>110</v>
       </c>
+      <c r="H109" s="42"/>
     </row>
     <row r="110" spans="1:11" s="25" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A110" s="25" t="b">
@@ -16520,6 +16634,7 @@
       <c r="G110" s="25" t="s">
         <v>97</v>
       </c>
+      <c r="H110" s="42"/>
     </row>
     <row r="111" spans="1:11" s="25" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A111" s="25" t="b">
@@ -16543,6 +16658,7 @@
       <c r="G111" s="25" t="s">
         <v>111</v>
       </c>
+      <c r="H111" s="42"/>
     </row>
     <row r="112" spans="1:11" s="25" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A112" s="25" t="b">
@@ -16566,7 +16682,7 @@
       <c r="G112" s="39" t="s">
         <v>530</v>
       </c>
-      <c r="H112" s="27"/>
+      <c r="H112" s="45"/>
       <c r="I112" s="27"/>
       <c r="K112" s="39"/>
     </row>
@@ -25395,7 +25511,7 @@
       <c r="F68" s="23" t="s">
         <v>767</v>
       </c>
-      <c r="H68" s="41" t="s">
+      <c r="H68" s="40" t="s">
         <v>983</v>
       </c>
       <c r="I68" s="23" t="s">

</xml_diff>

<commit_message>
Change separator for date/time/timezone field (samples.collDT)
</commit_message>
<xml_diff>
--- a/data/mapping_config_files/nwss_to_odm_v2_mapping.xlsx
+++ b/data/mapping_config_files/nwss_to_odm_v2_mapping.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/martinwellman/Documents/Health/Wastewater/PHES-ODM-MapGenerator/PHES-ODM-MapGenerator/data/mapping_config_files/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F3797779-CD3D-804A-A607-35746DC2EBA1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4C137B89-7225-614A-A598-98BF8E16F133}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="500" windowWidth="40960" windowHeight="20860" xr2:uid="{77810E24-F86B-BC44-A0D5-8790E6EC60B4}"/>
   </bookViews>
@@ -3072,9 +3072,6 @@
     <t>old protocolRelationshipsID</t>
   </si>
   <si>
-    <t>sample_collect_date + '/' + sample_collect_time + '/' + time_zone</t>
-  </si>
-  <si>
     <t>The ID generator will convert this into a valid date/time/timezone string</t>
   </si>
   <si>
@@ -3082,6 +3079,9 @@
     target = 24
 else:
     target = src.composite_freq</t>
+  </si>
+  <si>
+    <t>sample_collect_date + '/!/' + sample_collect_time + '/!/' + time_zone</t>
   </si>
 </sst>
 </file>
@@ -15696,7 +15696,7 @@
         <v>119</v>
       </c>
       <c r="H67" s="29" t="s">
-        <v>992</v>
+        <v>991</v>
       </c>
     </row>
     <row r="68" spans="1:11" s="25" customFormat="1" ht="17" customHeight="1" x14ac:dyDescent="0.2">
@@ -15714,10 +15714,10 @@
         <v>137</v>
       </c>
       <c r="H68" s="29" t="s">
+        <v>992</v>
+      </c>
+      <c r="J68" s="25" t="s">
         <v>990</v>
-      </c>
-      <c r="J68" s="25" t="s">
-        <v>991</v>
       </c>
     </row>
     <row r="69" spans="1:11" s="25" customFormat="1" x14ac:dyDescent="0.2">
@@ -16703,8 +16703,7 @@
     <col min="5" max="5" width="12" bestFit="1" customWidth="1"/>
     <col min="6" max="6" width="12.1640625" bestFit="1" customWidth="1"/>
     <col min="7" max="7" width="15.83203125" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="15.83203125" customWidth="1"/>
-    <col min="9" max="9" width="35.33203125" bestFit="1" customWidth="1"/>
+    <col min="8" max="9" width="35.33203125" bestFit="1" customWidth="1"/>
     <col min="10" max="10" width="21.83203125" customWidth="1"/>
     <col min="11" max="11" width="16.83203125" bestFit="1" customWidth="1"/>
     <col min="12" max="12" width="22" bestFit="1" customWidth="1"/>

</xml_diff>